<commit_message>
📊 实时报告更新 Fri Apr 24 02:05:46 UTC 2026
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -425,13 +425,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>系统状态</t>
+          <t>状态</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -439,26 +439,16 @@
           <t>原因</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>建议</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>抓取失败</t>
+          <t>拦截失败</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Shape of passed values is (5846, 1), indices imply (5846, 10)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>稍后手动重试 Run Workflow</t>
+          <t>网络节点故障: Shape of passed values is (5846, 1), indices imply (5846, 10)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 实时报告更新 Fri Apr 24 02:40:09 UTC 2026
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,12 +493,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>V10.4</t>
+          <t>V10.5-Broad</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>T:2026-04-24 10:16:36</t>
+          <t>T:2026-04-24 10:40:09</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -507,7 +507,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>0.6817542197943519</v>
+        <v>0.09871477112681781</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>18.04</v>
+        <v>18</v>
       </c>
       <c r="E3" t="n">
         <v>18.16</v>
@@ -541,34 +541,34 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>442.7</v>
+        <v>332.6</v>
       </c>
       <c r="I3" t="n">
-        <v>1.98</v>
+        <v>1.75</v>
       </c>
       <c r="J3" t="n">
-        <v>20.58</v>
+        <v>22.38</v>
       </c>
       <c r="K3" t="n">
-        <v>19.32</v>
+        <v>14.01</v>
       </c>
       <c r="L3" t="n">
-        <v>5.18</v>
+        <v>5.62</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>600052</t>
+          <t>300890</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>东望时代</t>
+          <t>翔丰华</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -577,44 +577,44 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>4.68</v>
+        <v>43.77</v>
       </c>
       <c r="E4" t="n">
-        <v>4.7</v>
+        <v>43.41</v>
       </c>
       <c r="F4" t="n">
-        <v>4.27</v>
+        <v>40.59</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>252.9</v>
+        <v>220</v>
       </c>
       <c r="I4" t="n">
-        <v>2.18</v>
+        <v>2.65</v>
       </c>
       <c r="J4" t="n">
-        <v>8.48</v>
+        <v>23.04</v>
       </c>
       <c r="K4" t="n">
-        <v>10.7</v>
+        <v>4.4</v>
       </c>
       <c r="L4" t="n">
-        <v>3.36</v>
+        <v>10.87</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>002490</t>
+          <t>601101</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>山东墨龙</t>
+          <t>昊华能源</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -623,44 +623,44 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>10.11</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="E5" t="n">
-        <v>10.01</v>
+        <v>9.6</v>
       </c>
       <c r="F5" t="n">
-        <v>9.609999999999999</v>
+        <v>9.27</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>237</v>
+        <v>213.4</v>
       </c>
       <c r="I5" t="n">
-        <v>3.48</v>
+        <v>3.85</v>
       </c>
       <c r="J5" t="n">
-        <v>14</v>
+        <v>4.55</v>
       </c>
       <c r="K5" t="n">
-        <v>7.8</v>
+        <v>10.02</v>
       </c>
       <c r="L5" t="n">
-        <v>7.7</v>
+        <v>6.39</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>603198</t>
+          <t>002490</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>迎驾贡酒</t>
+          <t>山东墨龙</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -669,44 +669,44 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>40.54</v>
+        <v>10.11</v>
       </c>
       <c r="E6" t="n">
-        <v>39.73</v>
+        <v>10.01</v>
       </c>
       <c r="F6" t="n">
-        <v>37.88</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>235.2</v>
+        <v>207.5</v>
       </c>
       <c r="I6" t="n">
-        <v>3.9</v>
+        <v>3.48</v>
       </c>
       <c r="J6" t="n">
-        <v>1.75</v>
+        <v>15.61</v>
       </c>
       <c r="K6" t="n">
-        <v>11.76</v>
+        <v>5.84</v>
       </c>
       <c r="L6" t="n">
-        <v>5.57</v>
+        <v>8.59</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>002971</t>
+          <t>600052</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>和远气体</t>
+          <t>东望时代</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -715,44 +715,44 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>34.59</v>
+        <v>4.71</v>
       </c>
       <c r="E7" t="n">
-        <v>34.33</v>
+        <v>4.7</v>
       </c>
       <c r="F7" t="n">
-        <v>31.48</v>
+        <v>4.27</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>228.7</v>
+        <v>188.4</v>
       </c>
       <c r="I7" t="n">
-        <v>2.1</v>
+        <v>2.84</v>
       </c>
       <c r="J7" t="n">
-        <v>7.72</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="K7" t="n">
-        <v>9.34</v>
+        <v>7.66</v>
       </c>
       <c r="L7" t="n">
-        <v>4.11</v>
+        <v>3.61</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>002377</t>
+          <t>001314</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>国创高新</t>
+          <t>亿道信息</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -761,44 +761,44 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3.26</v>
+        <v>48.98</v>
       </c>
       <c r="E8" t="n">
-        <v>3.33</v>
+        <v>48.83</v>
       </c>
       <c r="F8" t="n">
-        <v>3.18</v>
+        <v>45.86</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>228</v>
+        <v>187</v>
       </c>
       <c r="I8" t="n">
-        <v>1.56</v>
+        <v>0.99</v>
       </c>
       <c r="J8" t="n">
-        <v>7.62</v>
+        <v>6.35</v>
       </c>
       <c r="K8" t="n">
-        <v>9.33</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="L8" t="n">
-        <v>2.27</v>
+        <v>3.81</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>002242</t>
+          <t>600722</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>九阳股份</t>
+          <t>金牛化工</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -807,44 +807,44 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>11.75</v>
+        <v>14.18</v>
       </c>
       <c r="E9" t="n">
-        <v>11.85</v>
+        <v>13.99</v>
       </c>
       <c r="F9" t="n">
-        <v>11.42</v>
+        <v>13.14</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>207.8</v>
+        <v>184.1</v>
       </c>
       <c r="I9" t="n">
-        <v>2.98</v>
+        <v>3.5</v>
       </c>
       <c r="J9" t="n">
-        <v>6.41</v>
+        <v>11.67</v>
       </c>
       <c r="K9" t="n">
-        <v>8.380000000000001</v>
+        <v>5.2</v>
       </c>
       <c r="L9" t="n">
-        <v>5.82</v>
+        <v>11.23</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>300357</t>
+          <t>002971</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>我武生物</t>
+          <t>和远气体</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -853,44 +853,44 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>26.97</v>
+        <v>34.35</v>
       </c>
       <c r="E10" t="n">
-        <v>26.74</v>
+        <v>34.33</v>
       </c>
       <c r="F10" t="n">
-        <v>25.94</v>
+        <v>31.48</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>199.2</v>
+        <v>178.9</v>
       </c>
       <c r="I10" t="n">
-        <v>3.73</v>
+        <v>1.39</v>
       </c>
       <c r="J10" t="n">
-        <v>2.93</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="K10" t="n">
-        <v>8.970000000000001</v>
+        <v>6.98</v>
       </c>
       <c r="L10" t="n">
-        <v>3.88</v>
+        <v>4.68</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>300654</t>
+          <t>002377</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>世纪天鸿</t>
+          <t>国创高新</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -899,44 +899,44 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>11.17</v>
+        <v>3.27</v>
       </c>
       <c r="E11" t="n">
-        <v>11.01</v>
+        <v>3.33</v>
       </c>
       <c r="F11" t="n">
-        <v>10.49</v>
+        <v>3.16</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>193.7</v>
+        <v>178.7</v>
       </c>
       <c r="I11" t="n">
-        <v>4.78</v>
+        <v>1.87</v>
       </c>
       <c r="J11" t="n">
-        <v>4.77</v>
+        <v>8.56</v>
       </c>
       <c r="K11" t="n">
-        <v>7.99</v>
+        <v>7.04</v>
       </c>
       <c r="L11" t="n">
-        <v>1.9</v>
+        <v>2.54</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>300443</t>
+          <t>000890</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>金雷股份</t>
+          <t>法尔胜</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -945,44 +945,44 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>31.31</v>
+        <v>17.23</v>
       </c>
       <c r="E12" t="n">
-        <v>30.99</v>
+        <v>17.04</v>
       </c>
       <c r="F12" t="n">
-        <v>29.13</v>
+        <v>15.34</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>187.5</v>
+        <v>174.4</v>
       </c>
       <c r="I12" t="n">
-        <v>4.16</v>
+        <v>2.8</v>
       </c>
       <c r="J12" t="n">
-        <v>6.58</v>
+        <v>16.89</v>
       </c>
       <c r="K12" t="n">
-        <v>6.97</v>
+        <v>2.65</v>
       </c>
       <c r="L12" t="n">
-        <v>5.04</v>
+        <v>11.73</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>600470</t>
+          <t>002242</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>六国化工</t>
+          <t>九阳股份</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -991,44 +991,44 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>7.13</v>
+        <v>11.7</v>
       </c>
       <c r="E13" t="n">
-        <v>7</v>
+        <v>11.85</v>
       </c>
       <c r="F13" t="n">
-        <v>6.64</v>
+        <v>11.38</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>187.2</v>
+        <v>174</v>
       </c>
       <c r="I13" t="n">
-        <v>4.24</v>
+        <v>2.54</v>
       </c>
       <c r="J13" t="n">
-        <v>6.43</v>
+        <v>6.81</v>
       </c>
       <c r="K13" t="n">
-        <v>7</v>
+        <v>5.98</v>
       </c>
       <c r="L13" t="n">
-        <v>2.37</v>
+        <v>6.18</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>600433</t>
+          <t>300865</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>冠豪高新</t>
+          <t>大宏立</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1037,44 +1037,44 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>4.1</v>
+        <v>30.78</v>
       </c>
       <c r="E14" t="n">
-        <v>4.07</v>
+        <v>30.47</v>
       </c>
       <c r="F14" t="n">
-        <v>3.95</v>
+        <v>28.52</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>186.7</v>
+        <v>173.4</v>
       </c>
       <c r="I14" t="n">
-        <v>4.59</v>
+        <v>3.18</v>
       </c>
       <c r="J14" t="n">
-        <v>6.27</v>
+        <v>9.08</v>
       </c>
       <c r="K14" t="n">
-        <v>7.02</v>
+        <v>6.42</v>
       </c>
       <c r="L14" t="n">
-        <v>4.55</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>300649</t>
+          <t>920159</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>杭州园林</t>
+          <t>农大科技</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1083,44 +1083,44 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>19.2</v>
+        <v>44.65</v>
       </c>
       <c r="E15" t="n">
-        <v>19.23</v>
+        <v>43.82</v>
       </c>
       <c r="F15" t="n">
-        <v>18.55</v>
+        <v>40.38</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>185.3</v>
+        <v>172.9</v>
       </c>
       <c r="I15" t="n">
-        <v>1.96</v>
+        <v>4.62</v>
       </c>
       <c r="J15" t="n">
-        <v>8.369999999999999</v>
+        <v>16.26</v>
       </c>
       <c r="K15" t="n">
-        <v>6.23</v>
+        <v>3.99</v>
       </c>
       <c r="L15" t="n">
-        <v>1.73</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>605268</t>
+          <t>002310</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>王力安防</t>
+          <t>东方新能</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1129,44 +1129,44 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>13.48</v>
+        <v>3.07</v>
       </c>
       <c r="E16" t="n">
-        <v>13.29</v>
+        <v>3.04</v>
       </c>
       <c r="F16" t="n">
-        <v>12.4</v>
+        <v>2.86</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>184.9</v>
+        <v>171.4</v>
       </c>
       <c r="I16" t="n">
-        <v>3.22</v>
+        <v>4.42</v>
       </c>
       <c r="J16" t="n">
-        <v>3.37</v>
+        <v>7.53</v>
       </c>
       <c r="K16" t="n">
-        <v>7.87</v>
+        <v>5.52</v>
       </c>
       <c r="L16" t="n">
-        <v>1.95</v>
+        <v>10.02</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>300111</t>
+          <t>603198</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>向日葵</t>
+          <t>迎驾贡酒</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1175,13 +1175,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3.9</v>
+        <v>40.62</v>
       </c>
       <c r="E17" t="n">
-        <v>3.87</v>
+        <v>39.73</v>
       </c>
       <c r="F17" t="n">
-        <v>3.68</v>
+        <v>37.88</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1189,30 +1189,30 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>182.5</v>
+        <v>169.7</v>
       </c>
       <c r="I17" t="n">
-        <v>3.72</v>
+        <v>4.1</v>
       </c>
       <c r="J17" t="n">
-        <v>3.91</v>
+        <v>2.03</v>
       </c>
       <c r="K17" t="n">
-        <v>7.53</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="L17" t="n">
-        <v>1.98</v>
+        <v>6.47</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>300200</t>
+          <t>000953</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>高盟新材</t>
+          <t>河化股份</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1221,33 +1221,33 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>10.56</v>
+        <v>6.75</v>
       </c>
       <c r="E18" t="n">
-        <v>10.4</v>
+        <v>6.72</v>
       </c>
       <c r="F18" t="n">
-        <v>9.91</v>
+        <v>6.58</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>181.4</v>
+        <v>167.4</v>
       </c>
       <c r="I18" t="n">
-        <v>3.33</v>
+        <v>3.69</v>
       </c>
       <c r="J18" t="n">
-        <v>6.03</v>
+        <v>3.41</v>
       </c>
       <c r="K18" t="n">
-        <v>6.75</v>
+        <v>7.81</v>
       </c>
       <c r="L18" t="n">
-        <v>2.67</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="19">
@@ -1267,7 +1267,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>5.44</v>
+        <v>5.38</v>
       </c>
       <c r="E19" t="n">
         <v>5.38</v>
@@ -1277,34 +1277,34 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>179.5</v>
+        <v>166.6</v>
       </c>
       <c r="I19" t="n">
-        <v>3.03</v>
+        <v>1.89</v>
       </c>
       <c r="J19" t="n">
-        <v>10.56</v>
+        <v>11.76</v>
       </c>
       <c r="K19" t="n">
-        <v>5.11</v>
+        <v>3.71</v>
       </c>
       <c r="L19" t="n">
-        <v>8.33</v>
+        <v>9.279999999999999</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>002658</t>
+          <t>002481</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>雪迪龙</t>
+          <t>双塔食品</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1313,13 +1313,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>9.119999999999999</v>
+        <v>4.62</v>
       </c>
       <c r="E20" t="n">
-        <v>9.01</v>
+        <v>4.54</v>
       </c>
       <c r="F20" t="n">
-        <v>8.720000000000001</v>
+        <v>4.42</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1327,30 +1327,30 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>178.7</v>
+        <v>162</v>
       </c>
       <c r="I20" t="n">
-        <v>2.7</v>
+        <v>4.76</v>
       </c>
       <c r="J20" t="n">
-        <v>6.98</v>
+        <v>2.53</v>
       </c>
       <c r="K20" t="n">
-        <v>6.25</v>
+        <v>9.32</v>
       </c>
       <c r="L20" t="n">
-        <v>2.26</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>600109</t>
+          <t>300443</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>国金证券</t>
+          <t>金雷股份</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1359,44 +1359,44 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>8.720000000000001</v>
+        <v>31.28</v>
       </c>
       <c r="E21" t="n">
-        <v>8.640000000000001</v>
+        <v>30.99</v>
       </c>
       <c r="F21" t="n">
-        <v>8.449999999999999</v>
+        <v>29.13</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>174.1</v>
+        <v>159.8</v>
       </c>
       <c r="I21" t="n">
-        <v>1.99</v>
+        <v>4.06</v>
       </c>
       <c r="J21" t="n">
-        <v>0.8</v>
+        <v>6.87</v>
       </c>
       <c r="K21" t="n">
-        <v>8.01</v>
+        <v>4.78</v>
       </c>
       <c r="L21" t="n">
-        <v>2.59</v>
+        <v>5.26</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>301630</t>
+          <t>002470</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>同宇新材</t>
+          <t>金正大</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1405,44 +1405,44 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>224.49</v>
+        <v>3.05</v>
       </c>
       <c r="E22" t="n">
-        <v>218.65</v>
+        <v>3.03</v>
       </c>
       <c r="F22" t="n">
-        <v>211.99</v>
+        <v>2.82</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>173.3</v>
+        <v>159.1</v>
       </c>
       <c r="I22" t="n">
-        <v>4.85</v>
+        <v>3.04</v>
       </c>
       <c r="J22" t="n">
-        <v>11.92</v>
+        <v>9.06</v>
       </c>
       <c r="K22" t="n">
-        <v>4.25</v>
+        <v>3.99</v>
       </c>
       <c r="L22" t="n">
-        <v>2.63</v>
+        <v>9.029999999999999</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>300057</t>
+          <t>603079</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>万顺新材</t>
+          <t>圣达生物</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1451,44 +1451,44 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>7.42</v>
+        <v>16.94</v>
       </c>
       <c r="E23" t="n">
-        <v>7.39</v>
+        <v>17.22</v>
       </c>
       <c r="F23" t="n">
-        <v>7.17</v>
+        <v>16.17</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>172.8</v>
+        <v>157.2</v>
       </c>
       <c r="I23" t="n">
-        <v>3.34</v>
+        <v>2.11</v>
       </c>
       <c r="J23" t="n">
-        <v>10.26</v>
+        <v>3.54</v>
       </c>
       <c r="K23" t="n">
-        <v>4.77</v>
+        <v>6.92</v>
       </c>
       <c r="L23" t="n">
-        <v>5.89</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>600323</t>
+          <t>300649</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>瀚蓝环境</t>
+          <t>杭州园林</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1497,44 +1497,44 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>29.84</v>
+        <v>19.18</v>
       </c>
       <c r="E24" t="n">
-        <v>29.84</v>
+        <v>19.23</v>
       </c>
       <c r="F24" t="n">
-        <v>28.93</v>
+        <v>18.5</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>170.1</v>
+        <v>155.5</v>
       </c>
       <c r="I24" t="n">
-        <v>1.53</v>
+        <v>1.86</v>
       </c>
       <c r="J24" t="n">
-        <v>0.86</v>
+        <v>9.59</v>
       </c>
       <c r="K24" t="n">
-        <v>7.72</v>
+        <v>4.76</v>
       </c>
       <c r="L24" t="n">
-        <v>2.11</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>600783</t>
+          <t>600470</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>鲁信创投</t>
+          <t>六国化工</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1543,44 +1543,44 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>22.19</v>
+        <v>7.1</v>
       </c>
       <c r="E25" t="n">
-        <v>22.25</v>
+        <v>7</v>
       </c>
       <c r="F25" t="n">
-        <v>21.26</v>
+        <v>6.64</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>166.2</v>
+        <v>154.9</v>
       </c>
       <c r="I25" t="n">
-        <v>2.35</v>
+        <v>3.8</v>
       </c>
       <c r="J25" t="n">
-        <v>3.16</v>
+        <v>7.58</v>
       </c>
       <c r="K25" t="n">
-        <v>6.69</v>
+        <v>5.38</v>
       </c>
       <c r="L25" t="n">
-        <v>5.3</v>
+        <v>2.79</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>300651</t>
+          <t>002201</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>金陵体育</t>
+          <t>九鼎新材</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1589,13 +1589,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>29.6</v>
+        <v>15.2</v>
       </c>
       <c r="E26" t="n">
-        <v>29.01</v>
+        <v>14.98</v>
       </c>
       <c r="F26" t="n">
-        <v>27.47</v>
+        <v>13.92</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1603,30 +1603,30 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>165.4</v>
+        <v>154.4</v>
       </c>
       <c r="I26" t="n">
-        <v>3.79</v>
+        <v>2.7</v>
       </c>
       <c r="J26" t="n">
-        <v>8.880000000000001</v>
+        <v>12.84</v>
       </c>
       <c r="K26" t="n">
-        <v>2.73</v>
+        <v>2.34</v>
       </c>
       <c r="L26" t="n">
-        <v>2.25</v>
+        <v>11.45</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>688813</t>
+          <t>600783</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>泰金新能</t>
+          <t>鲁信创投</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1635,44 +1635,44 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>77.89</v>
+        <v>22.28</v>
       </c>
       <c r="E27" t="n">
-        <v>77.28</v>
+        <v>22.25</v>
       </c>
       <c r="F27" t="n">
-        <v>74.75</v>
+        <v>21.26</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>164.8</v>
+        <v>150.2</v>
       </c>
       <c r="I27" t="n">
-        <v>3.6</v>
+        <v>2.77</v>
       </c>
       <c r="J27" t="n">
-        <v>15.55</v>
+        <v>3.66</v>
       </c>
       <c r="K27" t="n">
-        <v>2.47</v>
+        <v>5.05</v>
       </c>
       <c r="L27" t="n">
-        <v>3.67</v>
+        <v>6.11</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>301176</t>
+          <t>300607</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>逸豪新材</t>
+          <t>拓斯达</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1681,44 +1681,44 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>30.03</v>
+        <v>29.42</v>
       </c>
       <c r="E28" t="n">
-        <v>29.92</v>
+        <v>29.64</v>
       </c>
       <c r="F28" t="n">
-        <v>28.88</v>
+        <v>28.18</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>164.8</v>
+        <v>149.9</v>
       </c>
       <c r="I28" t="n">
-        <v>4.85</v>
+        <v>0.51</v>
       </c>
       <c r="J28" t="n">
-        <v>4.78</v>
+        <v>5.86</v>
       </c>
       <c r="K28" t="n">
-        <v>6.06</v>
+        <v>4.29</v>
       </c>
       <c r="L28" t="n">
-        <v>2.38</v>
+        <v>5.87</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>688117</t>
+          <t>300357</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>圣诺生物</t>
+          <t>我武生物</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1727,44 +1727,44 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>38.93</v>
+        <v>26.93</v>
       </c>
       <c r="E29" t="n">
-        <v>38.19</v>
+        <v>26.74</v>
       </c>
       <c r="F29" t="n">
-        <v>37.02</v>
+        <v>25.94</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>163.6</v>
+        <v>149.2</v>
       </c>
       <c r="I29" t="n">
-        <v>3.87</v>
+        <v>3.58</v>
       </c>
       <c r="J29" t="n">
-        <v>2.71</v>
+        <v>3.17</v>
       </c>
       <c r="K29" t="n">
-        <v>6.67</v>
+        <v>6.38</v>
       </c>
       <c r="L29" t="n">
-        <v>1.64</v>
+        <v>4.19</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>300480</t>
+          <t>001317</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>光力科技</t>
+          <t>三羊马</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1773,44 +1773,44 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>34.63</v>
+        <v>51.07</v>
       </c>
       <c r="E30" t="n">
-        <v>34.29</v>
+        <v>50.68</v>
       </c>
       <c r="F30" t="n">
-        <v>33.32</v>
+        <v>49.14</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>163.2</v>
+        <v>148.5</v>
       </c>
       <c r="I30" t="n">
-        <v>3.74</v>
+        <v>3.57</v>
       </c>
       <c r="J30" t="n">
-        <v>5.56</v>
+        <v>5.77</v>
       </c>
       <c r="K30" t="n">
-        <v>5.69</v>
+        <v>5.45</v>
       </c>
       <c r="L30" t="n">
-        <v>5.24</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>002165</t>
+          <t>002652</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>红 宝 丽</t>
+          <t>扬子新材</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1819,44 +1819,44 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>9.140000000000001</v>
+        <v>4.91</v>
       </c>
       <c r="E31" t="n">
-        <v>9.17</v>
+        <v>4.85</v>
       </c>
       <c r="F31" t="n">
-        <v>8.619999999999999</v>
+        <v>4.57</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>162.5</v>
+        <v>148.4</v>
       </c>
       <c r="I31" t="n">
-        <v>1.78</v>
+        <v>4.91</v>
       </c>
       <c r="J31" t="n">
-        <v>5.67</v>
+        <v>5</v>
       </c>
       <c r="K31" t="n">
-        <v>5.61</v>
+        <v>5.7</v>
       </c>
       <c r="L31" t="n">
-        <v>3.77</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>603520</t>
+          <t>605268</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>司太立</t>
+          <t>王力安防</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1865,44 +1865,44 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>10.92</v>
+        <v>13.34</v>
       </c>
       <c r="E32" t="n">
-        <v>10.88</v>
+        <v>13.29</v>
       </c>
       <c r="F32" t="n">
-        <v>10.34</v>
+        <v>12.4</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>161.5</v>
+        <v>148.1</v>
       </c>
       <c r="I32" t="n">
-        <v>3.21</v>
+        <v>2.14</v>
       </c>
       <c r="J32" t="n">
-        <v>3.88</v>
+        <v>3.9</v>
       </c>
       <c r="K32" t="n">
-        <v>6.14</v>
+        <v>6.04</v>
       </c>
       <c r="L32" t="n">
-        <v>1.87</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>000833</t>
+          <t>600408</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>粤桂股份</t>
+          <t>安泰集团</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1911,13 +1911,13 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>25.96</v>
+        <v>3.18</v>
       </c>
       <c r="E33" t="n">
-        <v>25.59</v>
+        <v>3.22</v>
       </c>
       <c r="F33" t="n">
-        <v>25.17</v>
+        <v>3.07</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1925,30 +1925,30 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>160.8</v>
+        <v>147.8</v>
       </c>
       <c r="I33" t="n">
-        <v>3.96</v>
+        <v>0.95</v>
       </c>
       <c r="J33" t="n">
-        <v>6.18</v>
+        <v>5.44</v>
       </c>
       <c r="K33" t="n">
-        <v>3.33</v>
+        <v>5.5</v>
       </c>
       <c r="L33" t="n">
-        <v>7.32</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>300589</t>
+          <t>000593</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>江龙船艇</t>
+          <t>德龙汇能</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1957,44 +1957,44 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>16.31</v>
+        <v>20.34</v>
       </c>
       <c r="E34" t="n">
-        <v>16.22</v>
+        <v>19.97</v>
       </c>
       <c r="F34" t="n">
-        <v>15.84</v>
+        <v>19.22</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>159.2</v>
+        <v>147.4</v>
       </c>
       <c r="I34" t="n">
-        <v>3.36</v>
+        <v>3.56</v>
       </c>
       <c r="J34" t="n">
-        <v>9.130000000000001</v>
+        <v>7.97</v>
       </c>
       <c r="K34" t="n">
-        <v>4.24</v>
+        <v>3.38</v>
       </c>
       <c r="L34" t="n">
-        <v>3.54</v>
+        <v>5.71</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>002213</t>
+          <t>600433</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>大为股份</t>
+          <t>冠豪高新</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2003,13 +2003,13 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>34.93</v>
+        <v>4.11</v>
       </c>
       <c r="E35" t="n">
-        <v>34.44</v>
+        <v>4.07</v>
       </c>
       <c r="F35" t="n">
-        <v>32.96</v>
+        <v>3.95</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2017,30 +2017,30 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>158.7</v>
+        <v>147.4</v>
       </c>
       <c r="I35" t="n">
-        <v>2.34</v>
+        <v>4.85</v>
       </c>
       <c r="J35" t="n">
-        <v>8.06</v>
+        <v>6.85</v>
       </c>
       <c r="K35" t="n">
-        <v>2.56</v>
+        <v>5</v>
       </c>
       <c r="L35" t="n">
-        <v>5.73</v>
+        <v>4.96</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>603158</t>
+          <t>300766</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>腾龙股份</t>
+          <t>每日互动</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2049,13 +2049,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>13.47</v>
+        <v>40.67</v>
       </c>
       <c r="E36" t="n">
-        <v>13.42</v>
+        <v>39.62</v>
       </c>
       <c r="F36" t="n">
-        <v>12.65</v>
+        <v>37.55</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2063,30 +2063,30 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>158</v>
+        <v>146.8</v>
       </c>
       <c r="I36" t="n">
-        <v>2.82</v>
+        <v>4.66</v>
       </c>
       <c r="J36" t="n">
-        <v>5.28</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="K36" t="n">
-        <v>3.44</v>
+        <v>3.2</v>
       </c>
       <c r="L36" t="n">
-        <v>3.52</v>
+        <v>11.93</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>001339</t>
+          <t>300200</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>智微智能</t>
+          <t>高盟新材</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2095,44 +2095,44 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>74.81999999999999</v>
+        <v>10.49</v>
       </c>
       <c r="E37" t="n">
-        <v>74.34999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="F37" t="n">
-        <v>71.55</v>
+        <v>9.91</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H37" t="n">
-        <v>156.8</v>
+        <v>146.6</v>
       </c>
       <c r="I37" t="n">
-        <v>1.93</v>
+        <v>2.64</v>
       </c>
       <c r="J37" t="n">
-        <v>6.7</v>
+        <v>6.75</v>
       </c>
       <c r="K37" t="n">
-        <v>4.89</v>
+        <v>4.97</v>
       </c>
       <c r="L37" t="n">
-        <v>6.24</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>003027</t>
+          <t>300106</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>同兴科技</t>
+          <t>西部牧业</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2141,44 +2141,44 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>24.84</v>
+        <v>10.73</v>
       </c>
       <c r="E38" t="n">
-        <v>24.81</v>
+        <v>10.74</v>
       </c>
       <c r="F38" t="n">
-        <v>23.14</v>
+        <v>10.19</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>156.5</v>
+        <v>144.8</v>
       </c>
       <c r="I38" t="n">
-        <v>2.86</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J38" t="n">
-        <v>10.41</v>
+        <v>6.89</v>
       </c>
       <c r="K38" t="n">
-        <v>3.63</v>
+        <v>4.77</v>
       </c>
       <c r="L38" t="n">
-        <v>2.73</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>300035</t>
+          <t>002658</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>中科电气</t>
+          <t>雪迪龙</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2187,13 +2187,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>24.63</v>
+        <v>9</v>
       </c>
       <c r="E39" t="n">
-        <v>24.28</v>
+        <v>9.01</v>
       </c>
       <c r="F39" t="n">
-        <v>23.12</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -2201,30 +2201,30 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>155.6</v>
+        <v>144.7</v>
       </c>
       <c r="I39" t="n">
-        <v>2.8</v>
+        <v>1.35</v>
       </c>
       <c r="J39" t="n">
-        <v>5.54</v>
+        <v>7.56</v>
       </c>
       <c r="K39" t="n">
-        <v>3.19</v>
+        <v>4.54</v>
       </c>
       <c r="L39" t="n">
-        <v>7.89</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>600678</t>
+          <t>300573</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>四川金顶</t>
+          <t>兴齐眼药</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2233,44 +2233,44 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>12.19</v>
+        <v>70.68000000000001</v>
       </c>
       <c r="E40" t="n">
-        <v>12.03</v>
+        <v>69.34</v>
       </c>
       <c r="F40" t="n">
-        <v>11.53</v>
+        <v>66.47</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>155.4</v>
+        <v>144.6</v>
       </c>
       <c r="I40" t="n">
-        <v>3.39</v>
+        <v>3.62</v>
       </c>
       <c r="J40" t="n">
-        <v>8.6</v>
+        <v>3.83</v>
       </c>
       <c r="K40" t="n">
-        <v>4.16</v>
+        <v>4.52</v>
       </c>
       <c r="L40" t="n">
-        <v>3.63</v>
+        <v>5.08</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>600844</t>
+          <t>600691</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>金煤科技</t>
+          <t>潞化科技</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2279,44 +2279,44 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>3.59</v>
+        <v>3.38</v>
       </c>
       <c r="E41" t="n">
-        <v>3.56</v>
+        <v>3.35</v>
       </c>
       <c r="F41" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>143.8</v>
+      </c>
+      <c r="I41" t="n">
+        <v>4</v>
+      </c>
+      <c r="J41" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="K41" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="L41" t="n">
         <v>3.36</v>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="H41" t="n">
-        <v>155</v>
-      </c>
-      <c r="I41" t="n">
-        <v>2.57</v>
-      </c>
-      <c r="J41" t="n">
-        <v>6.06</v>
-      </c>
-      <c r="K41" t="n">
-        <v>4.98</v>
-      </c>
-      <c r="L41" t="n">
-        <v>1.78</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>688059</t>
+          <t>002445</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>华锐精密</t>
+          <t>中南文化</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2325,44 +2325,44 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>121.48</v>
+        <v>3.64</v>
       </c>
       <c r="E42" t="n">
-        <v>121.28</v>
+        <v>3.55</v>
       </c>
       <c r="F42" t="n">
-        <v>116.62</v>
+        <v>3.36</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>153.6</v>
+        <v>143.6</v>
       </c>
       <c r="I42" t="n">
-        <v>3</v>
+        <v>4.3</v>
       </c>
       <c r="J42" t="n">
-        <v>3.62</v>
+        <v>5.99</v>
       </c>
       <c r="K42" t="n">
-        <v>5.7</v>
+        <v>3.72</v>
       </c>
       <c r="L42" t="n">
-        <v>4.19</v>
+        <v>5.08</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>600537</t>
+          <t>300025</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>亿晶光电</t>
+          <t>华星创业</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2371,13 +2371,13 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>3.49</v>
+        <v>5.38</v>
       </c>
       <c r="E43" t="n">
-        <v>3.45</v>
+        <v>5.32</v>
       </c>
       <c r="F43" t="n">
-        <v>3.23</v>
+        <v>5.08</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -2385,30 +2385,30 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>151.8</v>
+        <v>143.4</v>
       </c>
       <c r="I43" t="n">
-        <v>3.25</v>
+        <v>4.06</v>
       </c>
       <c r="J43" t="n">
-        <v>6.79</v>
+        <v>3.76</v>
       </c>
       <c r="K43" t="n">
-        <v>2.52</v>
+        <v>5.7</v>
       </c>
       <c r="L43" t="n">
-        <v>2.79</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>002937</t>
+          <t>688117</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>兴瑞科技</t>
+          <t>圣诺生物</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2417,44 +2417,44 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>33.4</v>
+        <v>38.8</v>
       </c>
       <c r="E44" t="n">
-        <v>32.58</v>
+        <v>38.19</v>
       </c>
       <c r="F44" t="n">
-        <v>30.18</v>
+        <v>37.02</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>151.7</v>
+        <v>143</v>
       </c>
       <c r="I44" t="n">
-        <v>4.28</v>
+        <v>3.52</v>
       </c>
       <c r="J44" t="n">
-        <v>2.32</v>
+        <v>3.52</v>
       </c>
       <c r="K44" t="n">
-        <v>6.01</v>
+        <v>5.74</v>
       </c>
       <c r="L44" t="n">
-        <v>2.22</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>300766</t>
+          <t>301248</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>每日互动</t>
+          <t>杰创智能</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2463,13 +2463,13 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>40.21</v>
+        <v>65.38</v>
       </c>
       <c r="E45" t="n">
-        <v>39.49</v>
+        <v>64.18000000000001</v>
       </c>
       <c r="F45" t="n">
-        <v>37.55</v>
+        <v>58.98</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2477,30 +2477,30 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>150.7</v>
+        <v>142.4</v>
       </c>
       <c r="I45" t="n">
-        <v>3.47</v>
+        <v>3.61</v>
       </c>
       <c r="J45" t="n">
-        <v>5.19</v>
+        <v>8.09</v>
       </c>
       <c r="K45" t="n">
-        <v>2.98</v>
+        <v>2.92</v>
       </c>
       <c r="L45" t="n">
-        <v>7.36</v>
+        <v>5.85</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>002256</t>
+          <t>300111</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>兆新股份</t>
+          <t>向日葵</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2509,13 +2509,13 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>4.53</v>
+        <v>3.9</v>
       </c>
       <c r="E46" t="n">
-        <v>4.51</v>
+        <v>3.87</v>
       </c>
       <c r="F46" t="n">
-        <v>4.29</v>
+        <v>3.68</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2523,30 +2523,30 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>150.3</v>
+        <v>141.9</v>
       </c>
       <c r="I46" t="n">
-        <v>1.57</v>
+        <v>3.72</v>
       </c>
       <c r="J46" t="n">
-        <v>5.01</v>
+        <v>4.27</v>
       </c>
       <c r="K46" t="n">
-        <v>3.02</v>
+        <v>5.4</v>
       </c>
       <c r="L46" t="n">
-        <v>4.42</v>
+        <v>2.16</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>000963</t>
+          <t>002975</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>华东医药</t>
+          <t>博杰股份</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2555,44 +2555,44 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>35.02</v>
+        <v>118</v>
       </c>
       <c r="E47" t="n">
-        <v>34.56</v>
+        <v>115.24</v>
       </c>
       <c r="F47" t="n">
-        <v>33.51</v>
+        <v>110.05</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H47" t="n">
-        <v>150.2</v>
+        <v>140.6</v>
       </c>
       <c r="I47" t="n">
-        <v>2.73</v>
+        <v>4.79</v>
       </c>
       <c r="J47" t="n">
-        <v>0.63</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="K47" t="n">
-        <v>6.47</v>
+        <v>2.34</v>
       </c>
       <c r="L47" t="n">
-        <v>3.83</v>
+        <v>11.49</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>300927</t>
+          <t>002165</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>江天化学</t>
+          <t>红 宝 丽</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2601,44 +2601,44 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>32.77</v>
+        <v>9.09</v>
       </c>
       <c r="E48" t="n">
-        <v>32.32</v>
+        <v>9.17</v>
       </c>
       <c r="F48" t="n">
-        <v>29.98</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H48" t="n">
-        <v>149.8</v>
+        <v>139.3</v>
       </c>
       <c r="I48" t="n">
-        <v>3.15</v>
+        <v>1.22</v>
       </c>
       <c r="J48" t="n">
-        <v>6.12</v>
+        <v>6.63</v>
       </c>
       <c r="K48" t="n">
-        <v>4.61</v>
+        <v>4.4</v>
       </c>
       <c r="L48" t="n">
-        <v>2.77</v>
+        <v>4.41</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>300069</t>
+          <t>920028</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>金利华电</t>
+          <t>新恒泰</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2647,13 +2647,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>25.32</v>
+        <v>16.9</v>
       </c>
       <c r="E49" t="n">
-        <v>25.06</v>
+        <v>16.55</v>
       </c>
       <c r="F49" t="n">
-        <v>23.67</v>
+        <v>15.74</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2661,30 +2661,30 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>148.9</v>
+        <v>138.9</v>
       </c>
       <c r="I49" t="n">
-        <v>2.06</v>
+        <v>4.39</v>
       </c>
       <c r="J49" t="n">
-        <v>5.27</v>
+        <v>11.66</v>
       </c>
       <c r="K49" t="n">
-        <v>2.84</v>
+        <v>2.69</v>
       </c>
       <c r="L49" t="n">
-        <v>1.53</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>000593</t>
+          <t>603811</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>德龙汇能</t>
+          <t>诚意药业</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2693,44 +2693,44 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>19.99</v>
+        <v>12.17</v>
       </c>
       <c r="E50" t="n">
-        <v>19.87</v>
+        <v>12.06</v>
       </c>
       <c r="F50" t="n">
-        <v>19.22</v>
+        <v>11.47</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H50" t="n">
-        <v>148.8</v>
+        <v>138.2</v>
       </c>
       <c r="I50" t="n">
-        <v>1.78</v>
+        <v>2.18</v>
       </c>
       <c r="J50" t="n">
-        <v>6.82</v>
+        <v>3.11</v>
       </c>
       <c r="K50" t="n">
-        <v>4.31</v>
+        <v>5.48</v>
       </c>
       <c r="L50" t="n">
-        <v>4.87</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>300867</t>
+          <t>300677</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>圣元环保</t>
+          <t>英科医疗</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2739,44 +2739,44 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>21.73</v>
+        <v>57.73</v>
       </c>
       <c r="E51" t="n">
-        <v>21.33</v>
+        <v>56.42</v>
       </c>
       <c r="F51" t="n">
-        <v>20.71</v>
+        <v>50.99</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H51" t="n">
-        <v>148.5</v>
+        <v>138</v>
       </c>
       <c r="I51" t="n">
-        <v>3.43</v>
+        <v>4.72</v>
       </c>
       <c r="J51" t="n">
-        <v>4.48</v>
+        <v>3.91</v>
       </c>
       <c r="K51" t="n">
-        <v>5.07</v>
+        <v>3.95</v>
       </c>
       <c r="L51" t="n">
-        <v>1.85</v>
+        <v>10.27</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>688707</t>
+          <t>003027</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>振华新材</t>
+          <t>同兴科技</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2785,13 +2785,13 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>16.93</v>
+        <v>24.96</v>
       </c>
       <c r="E52" t="n">
-        <v>16.95</v>
+        <v>24.81</v>
       </c>
       <c r="F52" t="n">
-        <v>15.83</v>
+        <v>23.14</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2799,30 +2799,30 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>147.3</v>
+        <v>137</v>
       </c>
       <c r="I52" t="n">
-        <v>2.73</v>
+        <v>3.35</v>
       </c>
       <c r="J52" t="n">
-        <v>4.68</v>
+        <v>11.42</v>
       </c>
       <c r="K52" t="n">
-        <v>2.93</v>
+        <v>2.61</v>
       </c>
       <c r="L52" t="n">
-        <v>4.04</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>301079</t>
+          <t>600488</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>邵阳液压</t>
+          <t>津药药业</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2831,44 +2831,44 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>44.7</v>
+        <v>6.83</v>
       </c>
       <c r="E53" t="n">
-        <v>45.06</v>
+        <v>6.84</v>
       </c>
       <c r="F53" t="n">
-        <v>43.4</v>
+        <v>6.21</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H53" t="n">
-        <v>147</v>
+        <v>136.6</v>
       </c>
       <c r="I53" t="n">
-        <v>2.29</v>
+        <v>1.34</v>
       </c>
       <c r="J53" t="n">
-        <v>11.51</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="K53" t="n">
-        <v>2.63</v>
+        <v>2.15</v>
       </c>
       <c r="L53" t="n">
-        <v>4.03</v>
+        <v>6.53</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>601128</t>
+          <t>603516</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>常熟银行</t>
+          <t>淳中科技</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2877,44 +2877,44 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>7.52</v>
+        <v>150.19</v>
       </c>
       <c r="E54" t="n">
-        <v>7.43</v>
+        <v>148.95</v>
       </c>
       <c r="F54" t="n">
-        <v>7.23</v>
+        <v>141.13</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H54" t="n">
-        <v>146.8</v>
+        <v>136.1</v>
       </c>
       <c r="I54" t="n">
-        <v>2.17</v>
+        <v>3.29</v>
       </c>
       <c r="J54" t="n">
-        <v>1.37</v>
+        <v>3.27</v>
       </c>
       <c r="K54" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L54" t="n">
-        <v>3.39</v>
+        <v>10.02</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>301587</t>
+          <t>002213</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>中瑞股份</t>
+          <t>大为股份</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2923,44 +2923,44 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>28.69</v>
+        <v>34.63</v>
       </c>
       <c r="E55" t="n">
-        <v>28.35</v>
+        <v>34.46</v>
       </c>
       <c r="F55" t="n">
-        <v>26.89</v>
+        <v>32.96</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H55" t="n">
-        <v>146.8</v>
+        <v>135.4</v>
       </c>
       <c r="I55" t="n">
-        <v>3.87</v>
+        <v>1.46</v>
       </c>
       <c r="J55" t="n">
-        <v>9.15</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="K55" t="n">
-        <v>3.4</v>
+        <v>1.96</v>
       </c>
       <c r="L55" t="n">
-        <v>1.94</v>
+        <v>6.57</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>300511</t>
+          <t>300589</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>雪榕生物</t>
+          <t>江龙船艇</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2969,13 +2969,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>7.7</v>
+        <v>16.35</v>
       </c>
       <c r="E56" t="n">
-        <v>7.66</v>
+        <v>16.22</v>
       </c>
       <c r="F56" t="n">
-        <v>7.3</v>
+        <v>15.84</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2983,30 +2983,30 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>146.2</v>
+        <v>135.2</v>
       </c>
       <c r="I56" t="n">
-        <v>1.99</v>
+        <v>3.61</v>
       </c>
       <c r="J56" t="n">
-        <v>4.19</v>
+        <v>9.75</v>
       </c>
       <c r="K56" t="n">
         <v>3.02</v>
       </c>
       <c r="L56" t="n">
-        <v>1.8</v>
+        <v>3.77</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>301529</t>
+          <t>300651</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>福赛科技</t>
+          <t>金陵体育</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3015,13 +3015,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>123.2</v>
+        <v>29.85</v>
       </c>
       <c r="E57" t="n">
-        <v>121.67</v>
+        <v>29.08</v>
       </c>
       <c r="F57" t="n">
-        <v>116.79</v>
+        <v>27.47</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -3029,30 +3029,30 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>146.2</v>
+        <v>135.1</v>
       </c>
       <c r="I57" t="n">
-        <v>3.35</v>
+        <v>4.66</v>
       </c>
       <c r="J57" t="n">
-        <v>4.5</v>
+        <v>11.63</v>
       </c>
       <c r="K57" t="n">
-        <v>2.91</v>
+        <v>2.38</v>
       </c>
       <c r="L57" t="n">
-        <v>2.51</v>
+        <v>2.96</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>300573</t>
+          <t>300615</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>兴齐眼药</t>
+          <t>欣天科技</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3061,44 +3061,44 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>70.77</v>
+        <v>13.61</v>
       </c>
       <c r="E58" t="n">
-        <v>69.28</v>
+        <v>13.63</v>
       </c>
       <c r="F58" t="n">
-        <v>66.47</v>
+        <v>12.7</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H58" t="n">
-        <v>146.2</v>
+        <v>134.4</v>
       </c>
       <c r="I58" t="n">
-        <v>3.75</v>
+        <v>1.49</v>
       </c>
       <c r="J58" t="n">
-        <v>3.02</v>
+        <v>5.29</v>
       </c>
       <c r="K58" t="n">
-        <v>5.41</v>
+        <v>4.44</v>
       </c>
       <c r="L58" t="n">
-        <v>3.98</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>002443</t>
+          <t>000089</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>金洲管道</t>
+          <t>深圳机场</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3107,44 +3107,44 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>11.31</v>
+        <v>7.02</v>
       </c>
       <c r="E59" t="n">
-        <v>11.22</v>
+        <v>6.95</v>
       </c>
       <c r="F59" t="n">
-        <v>10.8</v>
+        <v>6.79</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H59" t="n">
-        <v>144.7</v>
+        <v>134.4</v>
       </c>
       <c r="I59" t="n">
-        <v>1.53</v>
+        <v>2.03</v>
       </c>
       <c r="J59" t="n">
-        <v>4.39</v>
+        <v>0.6</v>
       </c>
       <c r="K59" t="n">
-        <v>2.85</v>
+        <v>7.67</v>
       </c>
       <c r="L59" t="n">
-        <v>2.55</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>002866</t>
+          <t>301176</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>传艺科技</t>
+          <t>逸豪新材</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3153,44 +3153,44 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>25.77</v>
+        <v>29.99</v>
       </c>
       <c r="E60" t="n">
-        <v>25.8</v>
+        <v>29.92</v>
       </c>
       <c r="F60" t="n">
-        <v>23.77</v>
+        <v>28.88</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H60" t="n">
-        <v>144.6</v>
+        <v>134.3</v>
       </c>
       <c r="I60" t="n">
-        <v>1.54</v>
+        <v>4.71</v>
       </c>
       <c r="J60" t="n">
-        <v>12.32</v>
+        <v>5.25</v>
       </c>
       <c r="K60" t="n">
-        <v>2.2</v>
+        <v>4.44</v>
       </c>
       <c r="L60" t="n">
-        <v>5.73</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>301248</t>
+          <t>300867</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>杰创智能</t>
+          <t>圣元环保</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3199,44 +3199,44 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>65.70999999999999</v>
+        <v>21.72</v>
       </c>
       <c r="E61" t="n">
-        <v>64.18000000000001</v>
+        <v>21.39</v>
       </c>
       <c r="F61" t="n">
-        <v>58.98</v>
+        <v>20.71</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H61" t="n">
-        <v>144.6</v>
+        <v>134.2</v>
       </c>
       <c r="I61" t="n">
-        <v>4.14</v>
+        <v>3.38</v>
       </c>
       <c r="J61" t="n">
-        <v>7.21</v>
+        <v>5.69</v>
       </c>
       <c r="K61" t="n">
-        <v>3.9</v>
+        <v>4.29</v>
       </c>
       <c r="L61" t="n">
-        <v>5.21</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>002177</t>
+          <t>600678</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>御银股份</t>
+          <t>四川金顶</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3245,13 +3245,13 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>7.5</v>
+        <v>12.15</v>
       </c>
       <c r="E62" t="n">
-        <v>7.45</v>
+        <v>12.03</v>
       </c>
       <c r="F62" t="n">
-        <v>7.28</v>
+        <v>11.53</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -3259,19 +3259,939 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>143.5</v>
+        <v>133.9</v>
       </c>
       <c r="I62" t="n">
-        <v>2.18</v>
+        <v>3.05</v>
       </c>
       <c r="J62" t="n">
-        <v>4.12</v>
+        <v>9.5</v>
       </c>
       <c r="K62" t="n">
-        <v>2.86</v>
+        <v>2.99</v>
       </c>
       <c r="L62" t="n">
-        <v>2.09</v>
+        <v>4.01</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>603127</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>昭衍新药</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>38.24</v>
+      </c>
+      <c r="E63" t="n">
+        <v>37.93</v>
+      </c>
+      <c r="F63" t="n">
+        <v>36.11</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H63" t="n">
+        <v>132.8</v>
+      </c>
+      <c r="I63" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="J63" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="K63" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="L63" t="n">
+        <v>9.380000000000001</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>300035</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>中科电气</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>24.81</v>
+      </c>
+      <c r="E64" t="n">
+        <v>24.31</v>
+      </c>
+      <c r="F64" t="n">
+        <v>23.12</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H64" t="n">
+        <v>132.8</v>
+      </c>
+      <c r="I64" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="J64" t="n">
+        <v>6.76</v>
+      </c>
+      <c r="K64" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="L64" t="n">
+        <v>9.65</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>600844</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>金煤科技</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="E65" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="F65" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H65" t="n">
+        <v>132.7</v>
+      </c>
+      <c r="I65" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="J65" t="n">
+        <v>6.96</v>
+      </c>
+      <c r="K65" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="L65" t="n">
+        <v>2.04</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>301079</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>邵阳液压</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>44.56</v>
+      </c>
+      <c r="E66" t="n">
+        <v>45.06</v>
+      </c>
+      <c r="F66" t="n">
+        <v>43.4</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H66" t="n">
+        <v>132.5</v>
+      </c>
+      <c r="I66" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="J66" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="K66" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="L66" t="n">
+        <v>4.34</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>000833</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>粤桂股份</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>25.99</v>
+      </c>
+      <c r="E67" t="n">
+        <v>25.59</v>
+      </c>
+      <c r="F67" t="n">
+        <v>25.17</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H67" t="n">
+        <v>130.6</v>
+      </c>
+      <c r="I67" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="J67" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="K67" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="L67" t="n">
+        <v>7.89</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>301587</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>中瑞股份</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>28.79</v>
+      </c>
+      <c r="E68" t="n">
+        <v>28.35</v>
+      </c>
+      <c r="F68" t="n">
+        <v>26.89</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H68" t="n">
+        <v>130.6</v>
+      </c>
+      <c r="I68" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="J68" t="n">
+        <v>10.13</v>
+      </c>
+      <c r="K68" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="L68" t="n">
+        <v>2.14</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>300927</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>江天化学</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>32.47</v>
+      </c>
+      <c r="E69" t="n">
+        <v>32.32</v>
+      </c>
+      <c r="F69" t="n">
+        <v>29.98</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H69" t="n">
+        <v>128.9</v>
+      </c>
+      <c r="I69" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="J69" t="n">
+        <v>6.87</v>
+      </c>
+      <c r="K69" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="L69" t="n">
+        <v>3.12</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>300505</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>川金诺</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>26.15</v>
+      </c>
+      <c r="E70" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="F70" t="n">
+        <v>24.81</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H70" t="n">
+        <v>128.6</v>
+      </c>
+      <c r="I70" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="J70" t="n">
+        <v>7.17</v>
+      </c>
+      <c r="K70" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="L70" t="n">
+        <v>4.07</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>688401</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>路维光电</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>65.81999999999999</v>
+      </c>
+      <c r="E71" t="n">
+        <v>64.91</v>
+      </c>
+      <c r="F71" t="n">
+        <v>61.05</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H71" t="n">
+        <v>128.6</v>
+      </c>
+      <c r="I71" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="J71" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="K71" t="n">
+        <v>3</v>
+      </c>
+      <c r="L71" t="n">
+        <v>5.57</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>000636</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>风华高科</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>22.58</v>
+      </c>
+      <c r="E72" t="n">
+        <v>22.55</v>
+      </c>
+      <c r="F72" t="n">
+        <v>21.57</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H72" t="n">
+        <v>127.4</v>
+      </c>
+      <c r="I72" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="J72" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="K72" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="L72" t="n">
+        <v>11.04</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>603936</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>博敏电子</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>16.54</v>
+      </c>
+      <c r="E73" t="n">
+        <v>16.28</v>
+      </c>
+      <c r="F73" t="n">
+        <v>15.24</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H73" t="n">
+        <v>126.3</v>
+      </c>
+      <c r="I73" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="J73" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="K73" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="L73" t="n">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>300961</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>深水海纳</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>13.98</v>
+      </c>
+      <c r="E74" t="n">
+        <v>13.93</v>
+      </c>
+      <c r="F74" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H74" t="n">
+        <v>125.9</v>
+      </c>
+      <c r="I74" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J74" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="K74" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="L74" t="n">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>688548</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>广钢气体</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>30.61</v>
+      </c>
+      <c r="E75" t="n">
+        <v>30.94</v>
+      </c>
+      <c r="F75" t="n">
+        <v>28.91</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H75" t="n">
+        <v>125</v>
+      </c>
+      <c r="I75" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="J75" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="K75" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="L75" t="n">
+        <v>8.699999999999999</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>605111</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>新洁能</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="E76" t="n">
+        <v>38.68</v>
+      </c>
+      <c r="F76" t="n">
+        <v>37.28</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H76" t="n">
+        <v>124.9</v>
+      </c>
+      <c r="I76" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="J76" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="K76" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="L76" t="n">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>688536</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>思瑞浦</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>221.49</v>
+      </c>
+      <c r="E77" t="n">
+        <v>218.54</v>
+      </c>
+      <c r="F77" t="n">
+        <v>213.65</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H77" t="n">
+        <v>124.7</v>
+      </c>
+      <c r="I77" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="J77" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="K77" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="L77" t="n">
+        <v>10.53</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>002922</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>伊戈尔</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>43.03</v>
+      </c>
+      <c r="E78" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="F78" t="n">
+        <v>40.06</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H78" t="n">
+        <v>124</v>
+      </c>
+      <c r="I78" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="J78" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="K78" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="L78" t="n">
+        <v>6.9</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>688059</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>华锐精密</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>121.84</v>
+      </c>
+      <c r="E79" t="n">
+        <v>121.28</v>
+      </c>
+      <c r="F79" t="n">
+        <v>116.62</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H79" t="n">
+        <v>123.5</v>
+      </c>
+      <c r="I79" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="J79" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="K79" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="L79" t="n">
+        <v>4.45</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>301003</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>江苏博云</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>65.48999999999999</v>
+      </c>
+      <c r="E80" t="n">
+        <v>65.86</v>
+      </c>
+      <c r="F80" t="n">
+        <v>62.34</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H80" t="n">
+        <v>123.4</v>
+      </c>
+      <c r="I80" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="J80" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="K80" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="L80" t="n">
+        <v>3.19</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>603002</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>宏昌电子</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="E81" t="n">
+        <v>14.21</v>
+      </c>
+      <c r="F81" t="n">
+        <v>13.38</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H81" t="n">
+        <v>122.8</v>
+      </c>
+      <c r="I81" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="J81" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="K81" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="L81" t="n">
+        <v>8.73</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>002380</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>科远智慧</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>💎 潜伏种子</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="E82" t="n">
+        <v>34.47</v>
+      </c>
+      <c r="F82" t="n">
+        <v>32.98</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>🔥 黄金堆积</t>
+        </is>
+      </c>
+      <c r="H82" t="n">
+        <v>122.7</v>
+      </c>
+      <c r="I82" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="J82" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="K82" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="L82" t="n">
+        <v>2.43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 实时报告更新 Fri Apr 24 03:38:29 UTC 2026
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>T:2026-04-24 10:40:09</t>
+          <t>T:2026-04-24 11:38:28</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -507,7 +507,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>0.09871477112681781</v>
+        <v>0.4601348875129807</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>18</v>
+        <v>17.87</v>
       </c>
       <c r="E3" t="n">
         <v>18.16</v>
@@ -545,30 +545,30 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>332.6</v>
+        <v>293</v>
       </c>
       <c r="I3" t="n">
-        <v>1.75</v>
+        <v>1.02</v>
       </c>
       <c r="J3" t="n">
-        <v>22.38</v>
+        <v>26.2</v>
       </c>
       <c r="K3" t="n">
-        <v>14.01</v>
+        <v>9.43</v>
       </c>
       <c r="L3" t="n">
-        <v>5.62</v>
+        <v>6.57</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>300890</t>
+          <t>300061</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>翔丰华</t>
+          <t>旗天科技</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -577,13 +577,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>43.77</v>
+        <v>10.21</v>
       </c>
       <c r="E4" t="n">
-        <v>43.41</v>
+        <v>10.22</v>
       </c>
       <c r="F4" t="n">
-        <v>40.59</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -591,30 +591,30 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>220</v>
+        <v>241</v>
       </c>
       <c r="I4" t="n">
-        <v>2.65</v>
+        <v>4.18</v>
       </c>
       <c r="J4" t="n">
-        <v>23.04</v>
+        <v>11.2</v>
       </c>
       <c r="K4" t="n">
-        <v>4.4</v>
+        <v>10.1</v>
       </c>
       <c r="L4" t="n">
-        <v>10.87</v>
+        <v>7.14</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>601101</t>
+          <t>300970</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>昊华能源</t>
+          <t>华绿生物</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -623,13 +623,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>9.720000000000001</v>
+        <v>43.23</v>
       </c>
       <c r="E5" t="n">
-        <v>9.6</v>
+        <v>45.21</v>
       </c>
       <c r="F5" t="n">
-        <v>9.27</v>
+        <v>42.14</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -637,30 +637,30 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>213.4</v>
+        <v>219.3</v>
       </c>
       <c r="I5" t="n">
-        <v>3.85</v>
+        <v>2.93</v>
       </c>
       <c r="J5" t="n">
-        <v>4.55</v>
+        <v>25.64</v>
       </c>
       <c r="K5" t="n">
-        <v>10.02</v>
+        <v>3.48</v>
       </c>
       <c r="L5" t="n">
-        <v>6.39</v>
+        <v>11.44</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>002490</t>
+          <t>301667</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>山东墨龙</t>
+          <t>纳百川</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -669,13 +669,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>10.11</v>
+        <v>120.18</v>
       </c>
       <c r="E6" t="n">
-        <v>10.01</v>
+        <v>117.57</v>
       </c>
       <c r="F6" t="n">
-        <v>9.609999999999999</v>
+        <v>105.84</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -683,30 +683,30 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>207.5</v>
+        <v>212.6</v>
       </c>
       <c r="I6" t="n">
-        <v>3.48</v>
+        <v>3.88</v>
       </c>
       <c r="J6" t="n">
-        <v>15.61</v>
+        <v>29.7</v>
       </c>
       <c r="K6" t="n">
-        <v>5.84</v>
+        <v>1.57</v>
       </c>
       <c r="L6" t="n">
-        <v>8.59</v>
+        <v>7.61</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>600052</t>
+          <t>301630</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>东望时代</t>
+          <t>同宇新材</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -715,13 +715,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>4.71</v>
+        <v>225.18</v>
       </c>
       <c r="E7" t="n">
-        <v>4.7</v>
+        <v>223.29</v>
       </c>
       <c r="F7" t="n">
-        <v>4.27</v>
+        <v>211.99</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -729,30 +729,30 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>188.4</v>
+        <v>205.4</v>
       </c>
       <c r="I7" t="n">
-        <v>2.84</v>
+        <v>5.18</v>
       </c>
       <c r="J7" t="n">
-        <v>9.109999999999999</v>
+        <v>23.12</v>
       </c>
       <c r="K7" t="n">
-        <v>7.66</v>
+        <v>3.16</v>
       </c>
       <c r="L7" t="n">
-        <v>3.61</v>
+        <v>5.21</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>001314</t>
+          <t>002490</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>亿道信息</t>
+          <t>山东墨龙</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -761,13 +761,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>48.98</v>
+        <v>10.17</v>
       </c>
       <c r="E8" t="n">
-        <v>48.83</v>
+        <v>10.01</v>
       </c>
       <c r="F8" t="n">
-        <v>45.86</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -775,30 +775,30 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>187</v>
+        <v>193.6</v>
       </c>
       <c r="I8" t="n">
-        <v>0.99</v>
+        <v>4.09</v>
       </c>
       <c r="J8" t="n">
-        <v>6.35</v>
+        <v>17.91</v>
       </c>
       <c r="K8" t="n">
-        <v>8.470000000000001</v>
+        <v>3.91</v>
       </c>
       <c r="L8" t="n">
-        <v>3.81</v>
+        <v>9.85</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>600722</t>
+          <t>601101</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>金牛化工</t>
+          <t>昊华能源</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -807,13 +807,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>14.18</v>
+        <v>9.69</v>
       </c>
       <c r="E9" t="n">
-        <v>13.99</v>
+        <v>9.6</v>
       </c>
       <c r="F9" t="n">
-        <v>13.14</v>
+        <v>9.27</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -821,30 +821,30 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>184.1</v>
+        <v>174.2</v>
       </c>
       <c r="I9" t="n">
-        <v>3.5</v>
+        <v>3.53</v>
       </c>
       <c r="J9" t="n">
-        <v>11.67</v>
+        <v>5.17</v>
       </c>
       <c r="K9" t="n">
-        <v>5.2</v>
+        <v>6.54</v>
       </c>
       <c r="L9" t="n">
-        <v>11.23</v>
+        <v>7.25</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>002971</t>
+          <t>920159</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>和远气体</t>
+          <t>农大科技</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -853,13 +853,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>34.35</v>
+        <v>43.55</v>
       </c>
       <c r="E10" t="n">
-        <v>34.33</v>
+        <v>43.82</v>
       </c>
       <c r="F10" t="n">
-        <v>31.48</v>
+        <v>40.38</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -867,30 +867,30 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>178.9</v>
+        <v>168.5</v>
       </c>
       <c r="I10" t="n">
-        <v>1.39</v>
+        <v>2.04</v>
       </c>
       <c r="J10" t="n">
-        <v>8.779999999999999</v>
+        <v>19.15</v>
       </c>
       <c r="K10" t="n">
-        <v>6.98</v>
+        <v>2.66</v>
       </c>
       <c r="L10" t="n">
-        <v>4.68</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>002377</t>
+          <t>920069</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>国创高新</t>
+          <t>普昂医疗</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -899,13 +899,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3.27</v>
+        <v>38.2</v>
       </c>
       <c r="E11" t="n">
-        <v>3.33</v>
+        <v>38.35</v>
       </c>
       <c r="F11" t="n">
-        <v>3.16</v>
+        <v>37.44</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -913,30 +913,30 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>178.7</v>
+        <v>166.2</v>
       </c>
       <c r="I11" t="n">
-        <v>1.87</v>
+        <v>3.44</v>
       </c>
       <c r="J11" t="n">
-        <v>8.56</v>
+        <v>18.34</v>
       </c>
       <c r="K11" t="n">
-        <v>7.04</v>
+        <v>2.74</v>
       </c>
       <c r="L11" t="n">
-        <v>2.54</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>000890</t>
+          <t>600052</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>法尔胜</t>
+          <t>东望时代</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -945,13 +945,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>17.23</v>
+        <v>4.61</v>
       </c>
       <c r="E12" t="n">
-        <v>17.04</v>
+        <v>4.7</v>
       </c>
       <c r="F12" t="n">
-        <v>15.34</v>
+        <v>4.27</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -959,30 +959,30 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>174.4</v>
+        <v>165.4</v>
       </c>
       <c r="I12" t="n">
-        <v>2.8</v>
+        <v>0.66</v>
       </c>
       <c r="J12" t="n">
-        <v>16.89</v>
+        <v>10.76</v>
       </c>
       <c r="K12" t="n">
-        <v>2.65</v>
+        <v>5.2</v>
       </c>
       <c r="L12" t="n">
-        <v>11.73</v>
+        <v>4.26</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>002242</t>
+          <t>688813</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>九阳股份</t>
+          <t>泰金新能</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -991,44 +991,44 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>11.7</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="E13" t="n">
-        <v>11.85</v>
+        <v>77.28</v>
       </c>
       <c r="F13" t="n">
-        <v>11.38</v>
+        <v>74.75</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>174</v>
+        <v>160.6</v>
       </c>
       <c r="I13" t="n">
-        <v>2.54</v>
+        <v>2.29</v>
       </c>
       <c r="J13" t="n">
-        <v>6.81</v>
+        <v>22.46</v>
       </c>
       <c r="K13" t="n">
-        <v>5.98</v>
+        <v>1.31</v>
       </c>
       <c r="L13" t="n">
-        <v>6.18</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>300865</t>
+          <t>600310</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>大宏立</t>
+          <t>广西能源</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1037,13 +1037,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>30.78</v>
+        <v>5.35</v>
       </c>
       <c r="E14" t="n">
-        <v>30.47</v>
+        <v>5.38</v>
       </c>
       <c r="F14" t="n">
-        <v>28.52</v>
+        <v>4.98</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1051,30 +1051,30 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>173.4</v>
+        <v>160.2</v>
       </c>
       <c r="I14" t="n">
-        <v>3.18</v>
+        <v>1.33</v>
       </c>
       <c r="J14" t="n">
-        <v>9.08</v>
+        <v>13.79</v>
       </c>
       <c r="K14" t="n">
-        <v>6.42</v>
+        <v>2.5</v>
       </c>
       <c r="L14" t="n">
-        <v>1.6</v>
+        <v>10.87</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>920159</t>
+          <t>300480</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>农大科技</t>
+          <t>光力科技</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1083,13 +1083,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>44.65</v>
+        <v>34.81</v>
       </c>
       <c r="E15" t="n">
-        <v>43.82</v>
+        <v>34.52</v>
       </c>
       <c r="F15" t="n">
-        <v>40.38</v>
+        <v>33.32</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1097,30 +1097,30 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>172.9</v>
+        <v>157.3</v>
       </c>
       <c r="I15" t="n">
-        <v>4.62</v>
+        <v>4.28</v>
       </c>
       <c r="J15" t="n">
-        <v>16.26</v>
+        <v>9.44</v>
       </c>
       <c r="K15" t="n">
-        <v>3.99</v>
+        <v>3.71</v>
       </c>
       <c r="L15" t="n">
-        <v>1.02</v>
+        <v>8.970000000000001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>002310</t>
+          <t>002377</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>东方新能</t>
+          <t>国创高新</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1129,13 +1129,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>3.07</v>
+        <v>3.27</v>
       </c>
       <c r="E16" t="n">
-        <v>3.04</v>
+        <v>3.33</v>
       </c>
       <c r="F16" t="n">
-        <v>2.86</v>
+        <v>3.16</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1143,30 +1143,30 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>171.4</v>
+        <v>153</v>
       </c>
       <c r="I16" t="n">
-        <v>4.42</v>
+        <v>1.87</v>
       </c>
       <c r="J16" t="n">
-        <v>7.53</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="K16" t="n">
-        <v>5.52</v>
+        <v>4.57</v>
       </c>
       <c r="L16" t="n">
-        <v>10.02</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>603198</t>
+          <t>300865</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>迎驾贡酒</t>
+          <t>大宏立</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1175,44 +1175,44 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>40.62</v>
+        <v>30.58</v>
       </c>
       <c r="E17" t="n">
-        <v>39.73</v>
+        <v>30.47</v>
       </c>
       <c r="F17" t="n">
-        <v>37.88</v>
+        <v>28.52</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>169.7</v>
+        <v>151.8</v>
       </c>
       <c r="I17" t="n">
-        <v>4.1</v>
+        <v>2.51</v>
       </c>
       <c r="J17" t="n">
-        <v>2.03</v>
+        <v>10.34</v>
       </c>
       <c r="K17" t="n">
-        <v>8.880000000000001</v>
+        <v>4.2</v>
       </c>
       <c r="L17" t="n">
-        <v>6.47</v>
+        <v>1.82</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>000953</t>
+          <t>002310</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>河化股份</t>
+          <t>东方新能</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1221,13 +1221,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>6.75</v>
+        <v>3.06</v>
       </c>
       <c r="E18" t="n">
-        <v>6.72</v>
+        <v>3.04</v>
       </c>
       <c r="F18" t="n">
-        <v>6.58</v>
+        <v>2.86</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1235,30 +1235,30 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>167.4</v>
+        <v>151.6</v>
       </c>
       <c r="I18" t="n">
-        <v>3.69</v>
+        <v>4.08</v>
       </c>
       <c r="J18" t="n">
-        <v>3.41</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>7.81</v>
+        <v>3.59</v>
       </c>
       <c r="L18" t="n">
-        <v>0.86</v>
+        <v>11.15</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>600310</t>
+          <t>301307</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>广西能源</t>
+          <t>美利信</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1267,13 +1267,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>5.38</v>
+        <v>43.92</v>
       </c>
       <c r="E19" t="n">
-        <v>5.38</v>
+        <v>43.56</v>
       </c>
       <c r="F19" t="n">
-        <v>4.98</v>
+        <v>41.08</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1281,30 +1281,30 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>166.6</v>
+        <v>149.4</v>
       </c>
       <c r="I19" t="n">
-        <v>1.89</v>
+        <v>5.15</v>
       </c>
       <c r="J19" t="n">
-        <v>11.76</v>
+        <v>11.23</v>
       </c>
       <c r="K19" t="n">
-        <v>3.71</v>
+        <v>2.46</v>
       </c>
       <c r="L19" t="n">
-        <v>9.279999999999999</v>
+        <v>5.46</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>002481</t>
+          <t>002470</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>双塔食品</t>
+          <t>金正大</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1313,44 +1313,44 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>4.62</v>
+        <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>4.54</v>
+        <v>3.03</v>
       </c>
       <c r="F20" t="n">
-        <v>4.42</v>
+        <v>2.82</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>162</v>
+        <v>148.6</v>
       </c>
       <c r="I20" t="n">
-        <v>4.76</v>
+        <v>1.35</v>
       </c>
       <c r="J20" t="n">
-        <v>2.53</v>
+        <v>10.38</v>
       </c>
       <c r="K20" t="n">
-        <v>9.32</v>
+        <v>2.67</v>
       </c>
       <c r="L20" t="n">
-        <v>1.32</v>
+        <v>10.35</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>300443</t>
+          <t>603496</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>金雷股份</t>
+          <t>恒为科技</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1359,13 +1359,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>31.28</v>
+        <v>32.52</v>
       </c>
       <c r="E21" t="n">
-        <v>30.99</v>
+        <v>32.21</v>
       </c>
       <c r="F21" t="n">
-        <v>29.13</v>
+        <v>30.04</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1373,30 +1373,30 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>159.8</v>
+        <v>147.8</v>
       </c>
       <c r="I21" t="n">
-        <v>4.06</v>
+        <v>2.07</v>
       </c>
       <c r="J21" t="n">
-        <v>6.87</v>
+        <v>10.57</v>
       </c>
       <c r="K21" t="n">
-        <v>4.78</v>
+        <v>2.54</v>
       </c>
       <c r="L21" t="n">
-        <v>5.26</v>
+        <v>10.71</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>002470</t>
+          <t>002866</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>金正大</t>
+          <t>传艺科技</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1405,44 +1405,44 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>3.05</v>
+        <v>26.14</v>
       </c>
       <c r="E22" t="n">
-        <v>3.03</v>
+        <v>26.08</v>
       </c>
       <c r="F22" t="n">
-        <v>2.82</v>
+        <v>23.77</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>159.1</v>
+        <v>147</v>
       </c>
       <c r="I22" t="n">
-        <v>3.04</v>
+        <v>2.99</v>
       </c>
       <c r="J22" t="n">
-        <v>9.06</v>
+        <v>19.07</v>
       </c>
       <c r="K22" t="n">
-        <v>3.99</v>
+        <v>1.31</v>
       </c>
       <c r="L22" t="n">
-        <v>9.029999999999999</v>
+        <v>8.970000000000001</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>603079</t>
+          <t>600433</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>圣达生物</t>
+          <t>冠豪高新</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1451,13 +1451,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>16.94</v>
+        <v>4.04</v>
       </c>
       <c r="E23" t="n">
-        <v>17.22</v>
+        <v>4.07</v>
       </c>
       <c r="F23" t="n">
-        <v>16.17</v>
+        <v>3.95</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1465,30 +1465,30 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>157.2</v>
+        <v>145.2</v>
       </c>
       <c r="I23" t="n">
-        <v>2.11</v>
+        <v>3.06</v>
       </c>
       <c r="J23" t="n">
-        <v>3.54</v>
+        <v>7.76</v>
       </c>
       <c r="K23" t="n">
-        <v>6.92</v>
+        <v>3.26</v>
       </c>
       <c r="L23" t="n">
-        <v>1.17</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>300649</t>
+          <t>002843</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>杭州园林</t>
+          <t>泰嘉股份</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1497,13 +1497,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>19.18</v>
+        <v>27.01</v>
       </c>
       <c r="E24" t="n">
-        <v>19.23</v>
+        <v>26.58</v>
       </c>
       <c r="F24" t="n">
-        <v>18.5</v>
+        <v>24.31</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1511,30 +1511,30 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>155.5</v>
+        <v>144.8</v>
       </c>
       <c r="I24" t="n">
-        <v>1.86</v>
+        <v>3.61</v>
       </c>
       <c r="J24" t="n">
-        <v>9.59</v>
+        <v>11.76</v>
       </c>
       <c r="K24" t="n">
-        <v>4.76</v>
+        <v>1.9</v>
       </c>
       <c r="L24" t="n">
-        <v>1.98</v>
+        <v>7.71</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>600470</t>
+          <t>002213</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>六国化工</t>
+          <t>大为股份</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1543,13 +1543,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>7.1</v>
+        <v>34.67</v>
       </c>
       <c r="E25" t="n">
-        <v>7</v>
+        <v>34.59</v>
       </c>
       <c r="F25" t="n">
-        <v>6.64</v>
+        <v>32.96</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1557,30 +1557,30 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>154.9</v>
+        <v>144</v>
       </c>
       <c r="I25" t="n">
-        <v>3.8</v>
+        <v>1.58</v>
       </c>
       <c r="J25" t="n">
-        <v>7.58</v>
+        <v>12.58</v>
       </c>
       <c r="K25" t="n">
-        <v>5.38</v>
+        <v>1.56</v>
       </c>
       <c r="L25" t="n">
-        <v>2.79</v>
+        <v>8.99</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>002201</t>
+          <t>301499</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>九鼎新材</t>
+          <t>维科精密</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1589,13 +1589,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>15.2</v>
+        <v>36.17</v>
       </c>
       <c r="E26" t="n">
-        <v>14.98</v>
+        <v>35.66</v>
       </c>
       <c r="F26" t="n">
-        <v>13.92</v>
+        <v>30.71</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1603,30 +1603,30 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>154.4</v>
+        <v>143.7</v>
       </c>
       <c r="I26" t="n">
-        <v>2.7</v>
+        <v>4.03</v>
       </c>
       <c r="J26" t="n">
-        <v>12.84</v>
+        <v>13.39</v>
       </c>
       <c r="K26" t="n">
-        <v>2.34</v>
+        <v>2.51</v>
       </c>
       <c r="L26" t="n">
-        <v>11.45</v>
+        <v>1.66</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>600783</t>
+          <t>300443</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>鲁信创投</t>
+          <t>金雷股份</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1635,13 +1635,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>22.28</v>
+        <v>31.05</v>
       </c>
       <c r="E27" t="n">
-        <v>22.25</v>
+        <v>30.99</v>
       </c>
       <c r="F27" t="n">
-        <v>21.26</v>
+        <v>29.13</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1649,30 +1649,30 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>150.2</v>
+        <v>141.4</v>
       </c>
       <c r="I27" t="n">
-        <v>2.77</v>
+        <v>3.29</v>
       </c>
       <c r="J27" t="n">
-        <v>3.66</v>
+        <v>7.49</v>
       </c>
       <c r="K27" t="n">
-        <v>5.05</v>
+        <v>3.04</v>
       </c>
       <c r="L27" t="n">
-        <v>6.11</v>
+        <v>5.73</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>300607</t>
+          <t>600470</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>拓斯达</t>
+          <t>六国化工</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1681,13 +1681,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>29.42</v>
+        <v>6.97</v>
       </c>
       <c r="E28" t="n">
-        <v>29.64</v>
+        <v>7</v>
       </c>
       <c r="F28" t="n">
-        <v>28.18</v>
+        <v>6.64</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1695,30 +1695,30 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>149.9</v>
+        <v>140.8</v>
       </c>
       <c r="I28" t="n">
-        <v>0.51</v>
+        <v>1.9</v>
       </c>
       <c r="J28" t="n">
-        <v>5.86</v>
+        <v>9.08</v>
       </c>
       <c r="K28" t="n">
-        <v>4.29</v>
+        <v>3.71</v>
       </c>
       <c r="L28" t="n">
-        <v>5.87</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>300357</t>
+          <t>000593</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>我武生物</t>
+          <t>德龙汇能</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1727,13 +1727,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>26.93</v>
+        <v>20.25</v>
       </c>
       <c r="E29" t="n">
-        <v>26.74</v>
+        <v>19.97</v>
       </c>
       <c r="F29" t="n">
-        <v>25.94</v>
+        <v>19.22</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1741,30 +1741,30 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>149.2</v>
+        <v>138.1</v>
       </c>
       <c r="I29" t="n">
-        <v>3.58</v>
+        <v>3.11</v>
       </c>
       <c r="J29" t="n">
-        <v>3.17</v>
+        <v>9.06</v>
       </c>
       <c r="K29" t="n">
-        <v>6.38</v>
+        <v>2.24</v>
       </c>
       <c r="L29" t="n">
-        <v>4.19</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>001317</t>
+          <t>002445</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>三羊马</t>
+          <t>中南文化</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1773,13 +1773,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>51.07</v>
+        <v>3.56</v>
       </c>
       <c r="E30" t="n">
-        <v>50.68</v>
+        <v>3.55</v>
       </c>
       <c r="F30" t="n">
-        <v>49.14</v>
+        <v>3.36</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1787,30 +1787,30 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>148.5</v>
+        <v>137</v>
       </c>
       <c r="I30" t="n">
-        <v>3.57</v>
+        <v>2.01</v>
       </c>
       <c r="J30" t="n">
-        <v>5.77</v>
+        <v>7.42</v>
       </c>
       <c r="K30" t="n">
-        <v>5.45</v>
+        <v>2.69</v>
       </c>
       <c r="L30" t="n">
-        <v>2.56</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>002652</t>
+          <t>002560</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>扬子新材</t>
+          <t>通达股份</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1819,44 +1819,44 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>4.91</v>
+        <v>14.36</v>
       </c>
       <c r="E31" t="n">
-        <v>4.85</v>
+        <v>14.43</v>
       </c>
       <c r="F31" t="n">
-        <v>4.57</v>
+        <v>13.36</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>148.4</v>
+        <v>136.7</v>
       </c>
       <c r="I31" t="n">
-        <v>4.91</v>
+        <v>0.63</v>
       </c>
       <c r="J31" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="K31" t="n">
-        <v>5.7</v>
+        <v>1.14</v>
       </c>
       <c r="L31" t="n">
-        <v>1.26</v>
+        <v>11.02</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>605268</t>
+          <t>300740</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>王力安防</t>
+          <t>水羊股份</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1865,13 +1865,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>13.34</v>
+        <v>24.36</v>
       </c>
       <c r="E32" t="n">
-        <v>13.29</v>
+        <v>23.89</v>
       </c>
       <c r="F32" t="n">
-        <v>12.4</v>
+        <v>23.23</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1879,30 +1879,30 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>148.1</v>
+        <v>136.4</v>
       </c>
       <c r="I32" t="n">
-        <v>2.14</v>
+        <v>5</v>
       </c>
       <c r="J32" t="n">
-        <v>3.9</v>
+        <v>6.15</v>
       </c>
       <c r="K32" t="n">
-        <v>6.04</v>
+        <v>3.07</v>
       </c>
       <c r="L32" t="n">
-        <v>2.27</v>
+        <v>5.44</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>600408</t>
+          <t>301292</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>安泰集团</t>
+          <t>海科新源</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1911,44 +1911,44 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>3.18</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="E33" t="n">
-        <v>3.22</v>
+        <v>85.2</v>
       </c>
       <c r="F33" t="n">
-        <v>3.07</v>
+        <v>77.81999999999999</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>147.8</v>
+        <v>135.8</v>
       </c>
       <c r="I33" t="n">
-        <v>0.95</v>
+        <v>2.55</v>
       </c>
       <c r="J33" t="n">
-        <v>5.44</v>
+        <v>16.25</v>
       </c>
       <c r="K33" t="n">
-        <v>5.5</v>
+        <v>1.32</v>
       </c>
       <c r="L33" t="n">
-        <v>1.77</v>
+        <v>11.51</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>000593</t>
+          <t>301248</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>德龙汇能</t>
+          <t>杰创智能</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1957,13 +1957,13 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>20.34</v>
+        <v>64.26000000000001</v>
       </c>
       <c r="E34" t="n">
-        <v>19.97</v>
+        <v>64.18000000000001</v>
       </c>
       <c r="F34" t="n">
-        <v>19.22</v>
+        <v>58.98</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1971,30 +1971,30 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>147.4</v>
+        <v>135.1</v>
       </c>
       <c r="I34" t="n">
-        <v>3.56</v>
+        <v>1.84</v>
       </c>
       <c r="J34" t="n">
-        <v>7.97</v>
+        <v>9.27</v>
       </c>
       <c r="K34" t="n">
-        <v>3.38</v>
+        <v>1.92</v>
       </c>
       <c r="L34" t="n">
-        <v>5.71</v>
+        <v>6.71</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>600433</t>
+          <t>600120</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>冠豪高新</t>
+          <t>浙江东方</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2003,13 +2003,13 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>4.11</v>
+        <v>5.95</v>
       </c>
       <c r="E35" t="n">
-        <v>4.07</v>
+        <v>5.86</v>
       </c>
       <c r="F35" t="n">
-        <v>3.95</v>
+        <v>5.49</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2017,30 +2017,30 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>147.4</v>
+        <v>134.9</v>
       </c>
       <c r="I35" t="n">
-        <v>4.85</v>
+        <v>3.3</v>
       </c>
       <c r="J35" t="n">
-        <v>6.85</v>
+        <v>3.04</v>
       </c>
       <c r="K35" t="n">
-        <v>5</v>
+        <v>3.98</v>
       </c>
       <c r="L35" t="n">
-        <v>4.96</v>
+        <v>6.02</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>300766</t>
+          <t>000953</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>每日互动</t>
+          <t>河化股份</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2049,13 +2049,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>40.67</v>
+        <v>6.73</v>
       </c>
       <c r="E36" t="n">
-        <v>39.62</v>
+        <v>6.72</v>
       </c>
       <c r="F36" t="n">
-        <v>37.55</v>
+        <v>6.58</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2063,30 +2063,30 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>146.8</v>
+        <v>134.5</v>
       </c>
       <c r="I36" t="n">
-        <v>4.66</v>
+        <v>3.38</v>
       </c>
       <c r="J36" t="n">
-        <v>8.359999999999999</v>
+        <v>3.72</v>
       </c>
       <c r="K36" t="n">
-        <v>3.2</v>
+        <v>4.97</v>
       </c>
       <c r="L36" t="n">
-        <v>11.93</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>300200</t>
+          <t>920028</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>高盟新材</t>
+          <t>新恒泰</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2095,13 +2095,13 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>10.49</v>
+        <v>16.81</v>
       </c>
       <c r="E37" t="n">
-        <v>10.4</v>
+        <v>16.55</v>
       </c>
       <c r="F37" t="n">
-        <v>9.91</v>
+        <v>15.74</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -2109,30 +2109,30 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>146.6</v>
+        <v>134.2</v>
       </c>
       <c r="I37" t="n">
-        <v>2.64</v>
+        <v>3.83</v>
       </c>
       <c r="J37" t="n">
-        <v>6.75</v>
+        <v>13.34</v>
       </c>
       <c r="K37" t="n">
-        <v>4.97</v>
+        <v>1.74</v>
       </c>
       <c r="L37" t="n">
-        <v>2.99</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>300106</t>
+          <t>603198</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>西部牧业</t>
+          <t>迎驾贡酒</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2141,44 +2141,44 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>10.73</v>
+        <v>40.45</v>
       </c>
       <c r="E38" t="n">
-        <v>10.74</v>
+        <v>39.73</v>
       </c>
       <c r="F38" t="n">
-        <v>10.19</v>
+        <v>37.88</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>144.8</v>
+        <v>134.1</v>
       </c>
       <c r="I38" t="n">
-        <v>0.9399999999999999</v>
+        <v>3.66</v>
       </c>
       <c r="J38" t="n">
-        <v>6.89</v>
+        <v>2.31</v>
       </c>
       <c r="K38" t="n">
-        <v>4.77</v>
+        <v>5.82</v>
       </c>
       <c r="L38" t="n">
-        <v>1.56</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>002658</t>
+          <t>300651</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>雪迪龙</t>
+          <t>金陵体育</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2187,13 +2187,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>9</v>
+        <v>29.48</v>
       </c>
       <c r="E39" t="n">
-        <v>9.01</v>
+        <v>29.08</v>
       </c>
       <c r="F39" t="n">
-        <v>8.720000000000001</v>
+        <v>27.47</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -2201,30 +2201,30 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>144.7</v>
+        <v>133.6</v>
       </c>
       <c r="I39" t="n">
-        <v>1.35</v>
+        <v>3.37</v>
       </c>
       <c r="J39" t="n">
-        <v>7.56</v>
+        <v>13.61</v>
       </c>
       <c r="K39" t="n">
-        <v>4.54</v>
+        <v>1.6</v>
       </c>
       <c r="L39" t="n">
-        <v>2.45</v>
+        <v>3.48</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>300573</t>
+          <t>003027</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>兴齐眼药</t>
+          <t>同兴科技</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2233,13 +2233,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>70.68000000000001</v>
+        <v>24.51</v>
       </c>
       <c r="E40" t="n">
-        <v>69.34</v>
+        <v>24.81</v>
       </c>
       <c r="F40" t="n">
-        <v>66.47</v>
+        <v>23.14</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -2247,30 +2247,30 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>144.6</v>
+        <v>133.1</v>
       </c>
       <c r="I40" t="n">
-        <v>3.62</v>
+        <v>1.49</v>
       </c>
       <c r="J40" t="n">
-        <v>3.83</v>
+        <v>13.06</v>
       </c>
       <c r="K40" t="n">
-        <v>4.52</v>
+        <v>1.74</v>
       </c>
       <c r="L40" t="n">
-        <v>5.08</v>
+        <v>3.41</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>600691</t>
+          <t>300200</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>潞化科技</t>
+          <t>高盟新材</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2279,13 +2279,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>3.38</v>
+        <v>10.36</v>
       </c>
       <c r="E41" t="n">
-        <v>3.35</v>
+        <v>10.4</v>
       </c>
       <c r="F41" t="n">
-        <v>3.19</v>
+        <v>9.91</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -2293,30 +2293,30 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>143.8</v>
+        <v>132.5</v>
       </c>
       <c r="I41" t="n">
-        <v>4</v>
+        <v>1.37</v>
       </c>
       <c r="J41" t="n">
-        <v>4.16</v>
+        <v>7.93</v>
       </c>
       <c r="K41" t="n">
-        <v>5.6</v>
+        <v>3.4</v>
       </c>
       <c r="L41" t="n">
-        <v>3.36</v>
+        <v>3.51</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>002445</t>
+          <t>688052</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>中南文化</t>
+          <t>纳芯微</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2325,13 +2325,13 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>3.64</v>
+        <v>186</v>
       </c>
       <c r="E42" t="n">
-        <v>3.55</v>
+        <v>182.41</v>
       </c>
       <c r="F42" t="n">
-        <v>3.36</v>
+        <v>178.73</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -2339,30 +2339,30 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>143.6</v>
+        <v>130.8</v>
       </c>
       <c r="I42" t="n">
-        <v>4.3</v>
+        <v>4.72</v>
       </c>
       <c r="J42" t="n">
-        <v>5.99</v>
+        <v>4.2</v>
       </c>
       <c r="K42" t="n">
-        <v>3.72</v>
+        <v>3.25</v>
       </c>
       <c r="L42" t="n">
-        <v>5.08</v>
+        <v>11.14</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>300025</t>
+          <t>300916</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>华星创业</t>
+          <t>朗特智能</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2371,13 +2371,13 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>5.38</v>
+        <v>36.17</v>
       </c>
       <c r="E43" t="n">
-        <v>5.32</v>
+        <v>35.98</v>
       </c>
       <c r="F43" t="n">
-        <v>5.08</v>
+        <v>32.5</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -2385,30 +2385,30 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>143.4</v>
+        <v>130.6</v>
       </c>
       <c r="I43" t="n">
-        <v>4.06</v>
+        <v>1.49</v>
       </c>
       <c r="J43" t="n">
-        <v>3.76</v>
+        <v>9.85</v>
       </c>
       <c r="K43" t="n">
-        <v>5.7</v>
+        <v>2.6</v>
       </c>
       <c r="L43" t="n">
-        <v>1.03</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>688117</t>
+          <t>600678</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>圣诺生物</t>
+          <t>四川金顶</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2417,13 +2417,13 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>38.8</v>
+        <v>11.96</v>
       </c>
       <c r="E44" t="n">
-        <v>38.19</v>
+        <v>12.03</v>
       </c>
       <c r="F44" t="n">
-        <v>37.02</v>
+        <v>11.53</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -2431,30 +2431,30 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="I44" t="n">
-        <v>3.52</v>
+        <v>1.44</v>
       </c>
       <c r="J44" t="n">
-        <v>3.52</v>
+        <v>11.34</v>
       </c>
       <c r="K44" t="n">
-        <v>5.74</v>
+        <v>2.05</v>
       </c>
       <c r="L44" t="n">
-        <v>2.14</v>
+        <v>4.78</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>301248</t>
+          <t>002799</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>杰创智能</t>
+          <t>环球印务</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2463,13 +2463,13 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>65.38</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E45" t="n">
-        <v>64.18000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="F45" t="n">
-        <v>58.98</v>
+        <v>7.87</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2477,30 +2477,30 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>142.4</v>
+        <v>129.8</v>
       </c>
       <c r="I45" t="n">
-        <v>3.61</v>
+        <v>4.93</v>
       </c>
       <c r="J45" t="n">
-        <v>8.09</v>
+        <v>3.57</v>
       </c>
       <c r="K45" t="n">
-        <v>2.92</v>
+        <v>4.63</v>
       </c>
       <c r="L45" t="n">
-        <v>5.85</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>300111</t>
+          <t>601921</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>向日葵</t>
+          <t>浙版传媒</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2509,44 +2509,44 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>3.9</v>
+        <v>8.27</v>
       </c>
       <c r="E46" t="n">
-        <v>3.87</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="F46" t="n">
-        <v>3.68</v>
+        <v>7.77</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>141.9</v>
+        <v>129.1</v>
       </c>
       <c r="I46" t="n">
-        <v>3.72</v>
+        <v>3.5</v>
       </c>
       <c r="J46" t="n">
-        <v>4.27</v>
+        <v>1.27</v>
       </c>
       <c r="K46" t="n">
-        <v>5.4</v>
+        <v>7</v>
       </c>
       <c r="L46" t="n">
-        <v>2.16</v>
+        <v>2.32</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>002975</t>
+          <t>002658</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>博杰股份</t>
+          <t>雪迪龙</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2555,13 +2555,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>118</v>
+        <v>8.94</v>
       </c>
       <c r="E47" t="n">
-        <v>115.24</v>
+        <v>9.01</v>
       </c>
       <c r="F47" t="n">
-        <v>110.05</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -2569,30 +2569,30 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>140.6</v>
+        <v>128.4</v>
       </c>
       <c r="I47" t="n">
-        <v>4.79</v>
+        <v>0.68</v>
       </c>
       <c r="J47" t="n">
-        <v>9.369999999999999</v>
+        <v>8.34</v>
       </c>
       <c r="K47" t="n">
-        <v>2.34</v>
+        <v>2.92</v>
       </c>
       <c r="L47" t="n">
-        <v>11.49</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>002165</t>
+          <t>300821</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>红 宝 丽</t>
+          <t>东岳硅材</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2601,13 +2601,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>9.09</v>
+        <v>14.97</v>
       </c>
       <c r="E48" t="n">
-        <v>9.17</v>
+        <v>14.64</v>
       </c>
       <c r="F48" t="n">
-        <v>8.619999999999999</v>
+        <v>13.81</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2615,30 +2615,30 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>139.3</v>
+        <v>128.2</v>
       </c>
       <c r="I48" t="n">
-        <v>1.22</v>
+        <v>4.76</v>
       </c>
       <c r="J48" t="n">
-        <v>6.63</v>
+        <v>6.56</v>
       </c>
       <c r="K48" t="n">
-        <v>4.4</v>
+        <v>2.25</v>
       </c>
       <c r="L48" t="n">
-        <v>4.41</v>
+        <v>11.64</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>920028</t>
+          <t>603186</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>新恒泰</t>
+          <t>华正新材</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2647,13 +2647,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>16.9</v>
+        <v>72.01000000000001</v>
       </c>
       <c r="E49" t="n">
-        <v>16.55</v>
+        <v>70.87</v>
       </c>
       <c r="F49" t="n">
-        <v>15.74</v>
+        <v>65.17</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2661,30 +2661,30 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>138.9</v>
+        <v>128.1</v>
       </c>
       <c r="I49" t="n">
-        <v>4.39</v>
+        <v>3.17</v>
       </c>
       <c r="J49" t="n">
-        <v>11.66</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="K49" t="n">
-        <v>2.69</v>
+        <v>1.71</v>
       </c>
       <c r="L49" t="n">
-        <v>0.83</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>603811</t>
+          <t>000833</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>诚意药业</t>
+          <t>粤桂股份</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2693,13 +2693,13 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>12.17</v>
+        <v>25.26</v>
       </c>
       <c r="E50" t="n">
-        <v>12.06</v>
+        <v>25.59</v>
       </c>
       <c r="F50" t="n">
-        <v>11.47</v>
+        <v>24.69</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2707,30 +2707,30 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>138.2</v>
+        <v>127.9</v>
       </c>
       <c r="I50" t="n">
-        <v>2.18</v>
+        <v>1.16</v>
       </c>
       <c r="J50" t="n">
-        <v>3.11</v>
+        <v>8.1</v>
       </c>
       <c r="K50" t="n">
-        <v>5.48</v>
+        <v>1.71</v>
       </c>
       <c r="L50" t="n">
-        <v>1.23</v>
+        <v>9.539999999999999</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>300677</t>
+          <t>300573</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>英科医疗</t>
+          <t>兴齐眼药</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2739,13 +2739,13 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>57.73</v>
+        <v>70.5</v>
       </c>
       <c r="E51" t="n">
-        <v>56.42</v>
+        <v>69.34</v>
       </c>
       <c r="F51" t="n">
-        <v>50.99</v>
+        <v>66.47</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2753,30 +2753,30 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>138</v>
+        <v>127.7</v>
       </c>
       <c r="I51" t="n">
-        <v>4.72</v>
+        <v>3.36</v>
       </c>
       <c r="J51" t="n">
-        <v>3.91</v>
+        <v>4.3</v>
       </c>
       <c r="K51" t="n">
-        <v>3.95</v>
+        <v>2.96</v>
       </c>
       <c r="L51" t="n">
-        <v>10.27</v>
+        <v>5.71</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>003027</t>
+          <t>002897</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>同兴科技</t>
+          <t>意华股份</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2785,13 +2785,13 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>24.96</v>
+        <v>67.95</v>
       </c>
       <c r="E52" t="n">
-        <v>24.81</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="F52" t="n">
-        <v>23.14</v>
+        <v>63.16</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2799,30 +2799,30 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>137</v>
+        <v>127.6</v>
       </c>
       <c r="I52" t="n">
-        <v>3.35</v>
+        <v>1.97</v>
       </c>
       <c r="J52" t="n">
-        <v>11.42</v>
+        <v>7.16</v>
       </c>
       <c r="K52" t="n">
-        <v>2.61</v>
+        <v>2</v>
       </c>
       <c r="L52" t="n">
-        <v>2.99</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>600488</t>
+          <t>603079</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>津药药业</t>
+          <t>圣达生物</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2831,13 +2831,13 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>6.83</v>
+        <v>16.93</v>
       </c>
       <c r="E53" t="n">
-        <v>6.84</v>
+        <v>17.22</v>
       </c>
       <c r="F53" t="n">
-        <v>6.21</v>
+        <v>16.17</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2845,30 +2845,30 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>136.6</v>
+        <v>127.2</v>
       </c>
       <c r="I53" t="n">
-        <v>1.34</v>
+        <v>2.05</v>
       </c>
       <c r="J53" t="n">
-        <v>8.949999999999999</v>
+        <v>3.84</v>
       </c>
       <c r="K53" t="n">
-        <v>2.15</v>
+        <v>4.32</v>
       </c>
       <c r="L53" t="n">
-        <v>6.53</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>603516</t>
+          <t>001317</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>淳中科技</t>
+          <t>三羊马</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2877,13 +2877,13 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>150.19</v>
+        <v>51.28</v>
       </c>
       <c r="E54" t="n">
-        <v>148.95</v>
+        <v>50.68</v>
       </c>
       <c r="F54" t="n">
-        <v>141.13</v>
+        <v>49.14</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2891,30 +2891,30 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>136.1</v>
+        <v>127.2</v>
       </c>
       <c r="I54" t="n">
-        <v>3.29</v>
+        <v>4</v>
       </c>
       <c r="J54" t="n">
-        <v>3.27</v>
+        <v>6.34</v>
       </c>
       <c r="K54" t="n">
-        <v>4</v>
+        <v>3.49</v>
       </c>
       <c r="L54" t="n">
-        <v>10.02</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>002213</t>
+          <t>301587</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>大为股份</t>
+          <t>中瑞股份</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2923,13 +2923,13 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>34.63</v>
+        <v>28.79</v>
       </c>
       <c r="E55" t="n">
-        <v>34.46</v>
+        <v>28.35</v>
       </c>
       <c r="F55" t="n">
-        <v>32.96</v>
+        <v>26.89</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2937,30 +2937,30 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>135.4</v>
+        <v>127.2</v>
       </c>
       <c r="I55" t="n">
-        <v>1.46</v>
+        <v>4.24</v>
       </c>
       <c r="J55" t="n">
-        <v>9.220000000000001</v>
+        <v>11.77</v>
       </c>
       <c r="K55" t="n">
-        <v>1.96</v>
+        <v>1.68</v>
       </c>
       <c r="L55" t="n">
-        <v>6.57</v>
+        <v>2.49</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>300589</t>
+          <t>603459</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>江龙船艇</t>
+          <t>红板科技</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2969,44 +2969,44 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>16.35</v>
+        <v>60.06</v>
       </c>
       <c r="E56" t="n">
-        <v>16.22</v>
+        <v>59.98</v>
       </c>
       <c r="F56" t="n">
-        <v>15.84</v>
+        <v>58.17</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H56" t="n">
-        <v>135.2</v>
+        <v>127.1</v>
       </c>
       <c r="I56" t="n">
-        <v>3.61</v>
+        <v>1.69</v>
       </c>
       <c r="J56" t="n">
-        <v>9.75</v>
+        <v>15.41</v>
       </c>
       <c r="K56" t="n">
-        <v>3.02</v>
+        <v>0.87</v>
       </c>
       <c r="L56" t="n">
-        <v>3.77</v>
+        <v>7.37</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>300651</t>
+          <t>300679</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>金陵体育</t>
+          <t>电连技术</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3015,13 +3015,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>29.85</v>
+        <v>44.09</v>
       </c>
       <c r="E57" t="n">
-        <v>29.08</v>
+        <v>43.79</v>
       </c>
       <c r="F57" t="n">
-        <v>27.47</v>
+        <v>41.33</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -3029,30 +3029,30 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>135.1</v>
+        <v>126.8</v>
       </c>
       <c r="I57" t="n">
-        <v>4.66</v>
+        <v>4.01</v>
       </c>
       <c r="J57" t="n">
-        <v>11.63</v>
+        <v>6.38</v>
       </c>
       <c r="K57" t="n">
-        <v>2.38</v>
+        <v>2.19</v>
       </c>
       <c r="L57" t="n">
-        <v>2.96</v>
+        <v>10.24</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>300615</t>
+          <t>301190</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>欣天科技</t>
+          <t>善水科技</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3061,13 +3061,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>13.61</v>
+        <v>24.78</v>
       </c>
       <c r="E58" t="n">
-        <v>13.63</v>
+        <v>24.27</v>
       </c>
       <c r="F58" t="n">
-        <v>12.7</v>
+        <v>22.42</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -3075,30 +3075,30 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>134.4</v>
+        <v>126.8</v>
       </c>
       <c r="I58" t="n">
-        <v>1.49</v>
+        <v>4.73</v>
       </c>
       <c r="J58" t="n">
-        <v>5.29</v>
+        <v>3.44</v>
       </c>
       <c r="K58" t="n">
-        <v>4.44</v>
+        <v>4.42</v>
       </c>
       <c r="L58" t="n">
-        <v>1.09</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>000089</t>
+          <t>300589</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>深圳机场</t>
+          <t>江龙船艇</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3107,44 +3107,44 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>7.02</v>
+        <v>16.32</v>
       </c>
       <c r="E59" t="n">
-        <v>6.95</v>
+        <v>16.22</v>
       </c>
       <c r="F59" t="n">
-        <v>6.79</v>
+        <v>15.84</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H59" t="n">
-        <v>134.4</v>
+        <v>126.6</v>
       </c>
       <c r="I59" t="n">
-        <v>2.03</v>
+        <v>3.42</v>
       </c>
       <c r="J59" t="n">
-        <v>0.6</v>
+        <v>10.86</v>
       </c>
       <c r="K59" t="n">
-        <v>7.67</v>
+        <v>1.93</v>
       </c>
       <c r="L59" t="n">
-        <v>0.86</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>301176</t>
+          <t>301116</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>逸豪新材</t>
+          <t>益客食品</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3153,44 +3153,44 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>29.99</v>
+        <v>10.8</v>
       </c>
       <c r="E60" t="n">
-        <v>29.92</v>
+        <v>10.77</v>
       </c>
       <c r="F60" t="n">
-        <v>28.88</v>
+        <v>10.48</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H60" t="n">
-        <v>134.3</v>
+        <v>126.6</v>
       </c>
       <c r="I60" t="n">
-        <v>4.71</v>
+        <v>4.45</v>
       </c>
       <c r="J60" t="n">
-        <v>5.25</v>
+        <v>2.02</v>
       </c>
       <c r="K60" t="n">
-        <v>4.44</v>
+        <v>6.54</v>
       </c>
       <c r="L60" t="n">
-        <v>2.62</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>300867</t>
+          <t>002652</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>圣元环保</t>
+          <t>扬子新材</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3199,13 +3199,13 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>21.72</v>
+        <v>4.92</v>
       </c>
       <c r="E61" t="n">
-        <v>21.39</v>
+        <v>4.85</v>
       </c>
       <c r="F61" t="n">
-        <v>20.71</v>
+        <v>4.57</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -3213,30 +3213,30 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>134.2</v>
+        <v>126.3</v>
       </c>
       <c r="I61" t="n">
-        <v>3.38</v>
+        <v>5.13</v>
       </c>
       <c r="J61" t="n">
-        <v>5.69</v>
+        <v>5.53</v>
       </c>
       <c r="K61" t="n">
-        <v>4.29</v>
+        <v>3.68</v>
       </c>
       <c r="L61" t="n">
-        <v>2.36</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>600678</t>
+          <t>600691</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>四川金顶</t>
+          <t>潞化科技</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3245,13 +3245,13 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>12.15</v>
+        <v>3.36</v>
       </c>
       <c r="E62" t="n">
-        <v>12.03</v>
+        <v>3.35</v>
       </c>
       <c r="F62" t="n">
-        <v>11.53</v>
+        <v>3.19</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -3259,30 +3259,30 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>133.9</v>
+        <v>125.7</v>
       </c>
       <c r="I62" t="n">
-        <v>3.05</v>
+        <v>3.38</v>
       </c>
       <c r="J62" t="n">
-        <v>9.5</v>
+        <v>4.94</v>
       </c>
       <c r="K62" t="n">
-        <v>2.99</v>
+        <v>3.83</v>
       </c>
       <c r="L62" t="n">
-        <v>4.01</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>603127</t>
+          <t>300025</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>昭衍新药</t>
+          <t>华星创业</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3291,13 +3291,13 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>38.24</v>
+        <v>5.33</v>
       </c>
       <c r="E63" t="n">
-        <v>37.93</v>
+        <v>5.32</v>
       </c>
       <c r="F63" t="n">
-        <v>36.11</v>
+        <v>5.08</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -3305,30 +3305,30 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>132.8</v>
+        <v>124.8</v>
       </c>
       <c r="I63" t="n">
-        <v>2.52</v>
+        <v>3.09</v>
       </c>
       <c r="J63" t="n">
-        <v>3.91</v>
+        <v>4.44</v>
       </c>
       <c r="K63" t="n">
-        <v>3.51</v>
+        <v>3.92</v>
       </c>
       <c r="L63" t="n">
-        <v>9.380000000000001</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>300035</t>
+          <t>600763</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>中科电气</t>
+          <t>通策医疗</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3337,13 +3337,13 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>24.81</v>
+        <v>43.56</v>
       </c>
       <c r="E64" t="n">
-        <v>24.31</v>
+        <v>43.36</v>
       </c>
       <c r="F64" t="n">
-        <v>23.12</v>
+        <v>41.26</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -3351,30 +3351,30 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>132.8</v>
+        <v>124.7</v>
       </c>
       <c r="I64" t="n">
-        <v>3.55</v>
+        <v>2.13</v>
       </c>
       <c r="J64" t="n">
-        <v>6.76</v>
+        <v>3.06</v>
       </c>
       <c r="K64" t="n">
-        <v>2.56</v>
+        <v>3.12</v>
       </c>
       <c r="L64" t="n">
-        <v>9.65</v>
+        <v>5.94</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>600844</t>
+          <t>300435</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>金煤科技</t>
+          <t>中泰股份</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3383,13 +3383,13 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>3.56</v>
+        <v>23.55</v>
       </c>
       <c r="E65" t="n">
-        <v>3.56</v>
+        <v>24.08</v>
       </c>
       <c r="F65" t="n">
-        <v>3.36</v>
+        <v>22.46</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -3397,30 +3397,30 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>132.7</v>
+        <v>124.4</v>
       </c>
       <c r="I65" t="n">
-        <v>1.71</v>
+        <v>1.07</v>
       </c>
       <c r="J65" t="n">
-        <v>6.96</v>
+        <v>5.99</v>
       </c>
       <c r="K65" t="n">
-        <v>3.74</v>
+        <v>2.12</v>
       </c>
       <c r="L65" t="n">
-        <v>2.04</v>
+        <v>5.38</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>301079</t>
+          <t>605268</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>邵阳液压</t>
+          <t>王力安防</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3429,13 +3429,13 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>44.56</v>
+        <v>13.37</v>
       </c>
       <c r="E66" t="n">
-        <v>45.06</v>
+        <v>13.29</v>
       </c>
       <c r="F66" t="n">
-        <v>43.4</v>
+        <v>12.4</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -3443,30 +3443,30 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>132.5</v>
+        <v>124</v>
       </c>
       <c r="I66" t="n">
-        <v>1.97</v>
+        <v>2.37</v>
       </c>
       <c r="J66" t="n">
-        <v>12.43</v>
+        <v>4.41</v>
       </c>
       <c r="K66" t="n">
-        <v>1.9</v>
+        <v>3.86</v>
       </c>
       <c r="L66" t="n">
-        <v>4.34</v>
+        <v>2.57</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>000833</t>
+          <t>300357</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>粤桂股份</t>
+          <t>我武生物</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3475,13 +3475,13 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>25.99</v>
+        <v>26.83</v>
       </c>
       <c r="E67" t="n">
-        <v>25.59</v>
+        <v>26.74</v>
       </c>
       <c r="F67" t="n">
-        <v>25.17</v>
+        <v>25.94</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -3489,30 +3489,30 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>130.6</v>
+        <v>123.8</v>
       </c>
       <c r="I67" t="n">
-        <v>4.08</v>
+        <v>3.19</v>
       </c>
       <c r="J67" t="n">
-        <v>6.67</v>
+        <v>3.53</v>
       </c>
       <c r="K67" t="n">
-        <v>2.41</v>
+        <v>4.14</v>
       </c>
       <c r="L67" t="n">
-        <v>7.89</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>301587</t>
+          <t>300671</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>中瑞股份</t>
+          <t>富满微</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3521,13 +3521,13 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>28.79</v>
+        <v>47.28</v>
       </c>
       <c r="E68" t="n">
-        <v>28.35</v>
+        <v>46.6</v>
       </c>
       <c r="F68" t="n">
-        <v>26.89</v>
+        <v>44.94</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -3535,30 +3535,30 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>130.6</v>
+        <v>123.6</v>
       </c>
       <c r="I68" t="n">
-        <v>4.24</v>
+        <v>3.21</v>
       </c>
       <c r="J68" t="n">
-        <v>10.13</v>
+        <v>6.18</v>
       </c>
       <c r="K68" t="n">
-        <v>2.51</v>
+        <v>1.99</v>
       </c>
       <c r="L68" t="n">
-        <v>2.14</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>300927</t>
+          <t>300677</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>江天化学</t>
+          <t>英科医疗</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3567,13 +3567,13 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>32.47</v>
+        <v>56.81</v>
       </c>
       <c r="E69" t="n">
-        <v>32.32</v>
+        <v>56.42</v>
       </c>
       <c r="F69" t="n">
-        <v>29.98</v>
+        <v>50.99</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -3581,30 +3581,30 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>128.9</v>
+        <v>123.5</v>
       </c>
       <c r="I69" t="n">
-        <v>2.2</v>
+        <v>3.05</v>
       </c>
       <c r="J69" t="n">
-        <v>6.87</v>
+        <v>4.42</v>
       </c>
       <c r="K69" t="n">
-        <v>3.45</v>
+        <v>2.57</v>
       </c>
       <c r="L69" t="n">
-        <v>3.12</v>
+        <v>11.62</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>300505</t>
+          <t>688117</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>川金诺</t>
+          <t>圣诺生物</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3613,13 +3613,13 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>26.15</v>
+        <v>38.95</v>
       </c>
       <c r="E70" t="n">
-        <v>25.9</v>
+        <v>38.19</v>
       </c>
       <c r="F70" t="n">
-        <v>24.81</v>
+        <v>37.02</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -3627,30 +3627,30 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>128.6</v>
+        <v>123</v>
       </c>
       <c r="I70" t="n">
-        <v>2.75</v>
+        <v>3.92</v>
       </c>
       <c r="J70" t="n">
-        <v>7.17</v>
+        <v>4.18</v>
       </c>
       <c r="K70" t="n">
-        <v>3.33</v>
+        <v>3.86</v>
       </c>
       <c r="L70" t="n">
-        <v>4.07</v>
+        <v>2.54</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>688401</t>
+          <t>002481</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>路维光电</t>
+          <t>双塔食品</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3659,44 +3659,44 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>65.81999999999999</v>
+        <v>4.6</v>
       </c>
       <c r="E71" t="n">
-        <v>64.91</v>
+        <v>4.54</v>
       </c>
       <c r="F71" t="n">
-        <v>61.05</v>
+        <v>4.42</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H71" t="n">
-        <v>128.6</v>
+        <v>122.9</v>
       </c>
       <c r="I71" t="n">
-        <v>3.98</v>
+        <v>4.31</v>
       </c>
       <c r="J71" t="n">
-        <v>4.41</v>
+        <v>2.78</v>
       </c>
       <c r="K71" t="n">
-        <v>3</v>
+        <v>5.98</v>
       </c>
       <c r="L71" t="n">
-        <v>5.57</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>000636</t>
+          <t>300505</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>风华高科</t>
+          <t>川金诺</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3705,13 +3705,13 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>22.58</v>
+        <v>25.78</v>
       </c>
       <c r="E72" t="n">
-        <v>22.55</v>
+        <v>25.9</v>
       </c>
       <c r="F72" t="n">
-        <v>21.57</v>
+        <v>24.81</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -3719,19 +3719,19 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>127.4</v>
+        <v>122.3</v>
       </c>
       <c r="I72" t="n">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
       <c r="J72" t="n">
-        <v>4.19</v>
+        <v>8.58</v>
       </c>
       <c r="K72" t="n">
-        <v>2.97</v>
+        <v>2.33</v>
       </c>
       <c r="L72" t="n">
-        <v>11.04</v>
+        <v>4.86</v>
       </c>
     </row>
     <row r="73">
@@ -3751,7 +3751,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>16.54</v>
+        <v>16.28</v>
       </c>
       <c r="E73" t="n">
         <v>16.28</v>
@@ -3765,30 +3765,30 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>126.3</v>
+        <v>122.2</v>
       </c>
       <c r="I73" t="n">
-        <v>3.12</v>
+        <v>1.5</v>
       </c>
       <c r="J73" t="n">
-        <v>5.8</v>
+        <v>7.01</v>
       </c>
       <c r="K73" t="n">
-        <v>2.34</v>
+        <v>1.6</v>
       </c>
       <c r="L73" t="n">
-        <v>5.9</v>
+        <v>7.15</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>300961</t>
+          <t>603516</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>深水海纳</t>
+          <t>淳中科技</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3797,13 +3797,13 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>13.98</v>
+        <v>147.3</v>
       </c>
       <c r="E74" t="n">
-        <v>13.93</v>
+        <v>148.95</v>
       </c>
       <c r="F74" t="n">
-        <v>13.25</v>
+        <v>141.13</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -3811,30 +3811,30 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>125.9</v>
+        <v>121.5</v>
       </c>
       <c r="I74" t="n">
-        <v>1.16</v>
+        <v>1.31</v>
       </c>
       <c r="J74" t="n">
-        <v>4.98</v>
+        <v>3.74</v>
       </c>
       <c r="K74" t="n">
-        <v>3.83</v>
+        <v>2.63</v>
       </c>
       <c r="L74" t="n">
-        <v>1.06</v>
+        <v>11.43</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>688548</t>
+          <t>300867</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>广钢气体</t>
+          <t>圣元环保</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3843,13 +3843,13 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>30.61</v>
+        <v>21.4</v>
       </c>
       <c r="E75" t="n">
-        <v>30.94</v>
+        <v>21.39</v>
       </c>
       <c r="F75" t="n">
-        <v>28.91</v>
+        <v>20.71</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -3857,30 +3857,30 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>125</v>
+        <v>121.4</v>
       </c>
       <c r="I75" t="n">
         <v>1.86</v>
       </c>
       <c r="J75" t="n">
-        <v>4.02</v>
+        <v>6.67</v>
       </c>
       <c r="K75" t="n">
-        <v>2.83</v>
+        <v>2.89</v>
       </c>
       <c r="L75" t="n">
-        <v>8.699999999999999</v>
+        <v>2.76</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>605111</t>
+          <t>688249</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>新洁能</t>
+          <t>晶合集成</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3889,13 +3889,13 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>38.9</v>
+        <v>30.33</v>
       </c>
       <c r="E76" t="n">
-        <v>38.68</v>
+        <v>30.24</v>
       </c>
       <c r="F76" t="n">
-        <v>37.28</v>
+        <v>27.78</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -3903,30 +3903,30 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>124.9</v>
+        <v>121.2</v>
       </c>
       <c r="I76" t="n">
-        <v>2.15</v>
+        <v>0.63</v>
       </c>
       <c r="J76" t="n">
-        <v>3.38</v>
+        <v>3.21</v>
       </c>
       <c r="K76" t="n">
-        <v>3.03</v>
+        <v>2.78</v>
       </c>
       <c r="L76" t="n">
-        <v>5.48</v>
+        <v>11.11</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>688536</t>
+          <t>301128</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>思瑞浦</t>
+          <t>强瑞技术</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3935,13 +3935,13 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>221.49</v>
+        <v>190.83</v>
       </c>
       <c r="E77" t="n">
-        <v>218.54</v>
+        <v>185.83</v>
       </c>
       <c r="F77" t="n">
-        <v>213.65</v>
+        <v>173.46</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -3949,30 +3949,30 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>124.7</v>
+        <v>121.1</v>
       </c>
       <c r="I77" t="n">
-        <v>4.07</v>
+        <v>5.14</v>
       </c>
       <c r="J77" t="n">
-        <v>3.48</v>
+        <v>6.75</v>
       </c>
       <c r="K77" t="n">
-        <v>2.98</v>
+        <v>1.59</v>
       </c>
       <c r="L77" t="n">
-        <v>10.53</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>002922</t>
+          <t>688312</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>伊戈尔</t>
+          <t>燕麦科技</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3981,13 +3981,13 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>43.03</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="E78" t="n">
-        <v>41.9</v>
+        <v>69.68000000000001</v>
       </c>
       <c r="F78" t="n">
-        <v>40.06</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -3995,30 +3995,30 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>124</v>
+        <v>120.9</v>
       </c>
       <c r="I78" t="n">
-        <v>4.67</v>
+        <v>2.61</v>
       </c>
       <c r="J78" t="n">
-        <v>4.38</v>
+        <v>5.84</v>
       </c>
       <c r="K78" t="n">
-        <v>2.62</v>
+        <v>1.88</v>
       </c>
       <c r="L78" t="n">
-        <v>6.9</v>
+        <v>5.96</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>688059</t>
+          <t>688401</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>华锐精密</t>
+          <t>路维光电</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -4027,13 +4027,13 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>121.84</v>
+        <v>65.61</v>
       </c>
       <c r="E79" t="n">
-        <v>121.28</v>
+        <v>64.91</v>
       </c>
       <c r="F79" t="n">
-        <v>116.62</v>
+        <v>61.05</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -4041,30 +4041,30 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>123.5</v>
+        <v>120.7</v>
       </c>
       <c r="I79" t="n">
-        <v>3.31</v>
+        <v>3.65</v>
       </c>
       <c r="J79" t="n">
-        <v>3.85</v>
+        <v>5.3</v>
       </c>
       <c r="K79" t="n">
-        <v>4.01</v>
+        <v>2.04</v>
       </c>
       <c r="L79" t="n">
-        <v>4.45</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>301003</t>
+          <t>603127</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>江苏博云</t>
+          <t>昭衍新药</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4073,13 +4073,13 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>65.48999999999999</v>
+        <v>38.15</v>
       </c>
       <c r="E80" t="n">
-        <v>65.86</v>
+        <v>37.93</v>
       </c>
       <c r="F80" t="n">
-        <v>62.34</v>
+        <v>36.11</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -4087,30 +4087,30 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>123.4</v>
+        <v>120.6</v>
       </c>
       <c r="I80" t="n">
-        <v>1.21</v>
+        <v>2.28</v>
       </c>
       <c r="J80" t="n">
-        <v>6.45</v>
+        <v>4.47</v>
       </c>
       <c r="K80" t="n">
-        <v>3.13</v>
+        <v>2.31</v>
       </c>
       <c r="L80" t="n">
-        <v>3.19</v>
+        <v>10.73</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>603002</t>
+          <t>002430</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>宏昌电子</t>
+          <t>杭氧股份</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4119,13 +4119,13 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>14.49</v>
+        <v>31.36</v>
       </c>
       <c r="E81" t="n">
-        <v>14.21</v>
+        <v>31.45</v>
       </c>
       <c r="F81" t="n">
-        <v>13.38</v>
+        <v>29.65</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -4133,30 +4133,30 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>122.8</v>
+        <v>120.4</v>
       </c>
       <c r="I81" t="n">
-        <v>4.47</v>
+        <v>2.82</v>
       </c>
       <c r="J81" t="n">
-        <v>5.37</v>
+        <v>3.39</v>
       </c>
       <c r="K81" t="n">
-        <v>2.19</v>
+        <v>2.65</v>
       </c>
       <c r="L81" t="n">
-        <v>8.73</v>
+        <v>10.57</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>002380</t>
+          <t>002922</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>科远智慧</t>
+          <t>伊戈尔</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4165,13 +4165,13 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>35.2</v>
+        <v>42.41</v>
       </c>
       <c r="E82" t="n">
-        <v>34.47</v>
+        <v>41.9</v>
       </c>
       <c r="F82" t="n">
-        <v>32.98</v>
+        <v>40.06</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -4179,19 +4179,19 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>122.7</v>
+        <v>120.1</v>
       </c>
       <c r="I82" t="n">
-        <v>3.65</v>
+        <v>3.16</v>
       </c>
       <c r="J82" t="n">
-        <v>4.9</v>
+        <v>5.51</v>
       </c>
       <c r="K82" t="n">
-        <v>3.59</v>
+        <v>1.92</v>
       </c>
       <c r="L82" t="n">
-        <v>2.43</v>
+        <v>8.710000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 实时报告更新 Fri Apr 24 04:39:46 UTC 2026
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>T:2026-04-24 11:38:28</t>
+          <t>T:2026-04-24 12:39:46</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -507,7 +507,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>0.4601348875129807</v>
+        <v>0.7947937967270495</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>

</xml_diff>

<commit_message>
📊 实时报告更新 Fri Apr 24 13:47:35 UTC 2026
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>T:2026-04-24 12:39:46</t>
+          <t>T:2026-04-24 21:47:35</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -507,7 +507,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>0.7947937967270495</v>
+        <v>0.9888782986371312</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
@@ -517,12 +517,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>300721</t>
+          <t>301667</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>怡达股份</t>
+          <t>纳百川</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -531,33 +531,33 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>17.87</v>
+        <v>120.65</v>
       </c>
       <c r="E3" t="n">
-        <v>18.16</v>
+        <v>118.79</v>
       </c>
       <c r="F3" t="n">
-        <v>16.81</v>
+        <v>105.84</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>293</v>
+        <v>242.5</v>
       </c>
       <c r="I3" t="n">
-        <v>1.02</v>
+        <v>4.29</v>
       </c>
       <c r="J3" t="n">
-        <v>26.2</v>
+        <v>43.42</v>
       </c>
       <c r="K3" t="n">
-        <v>9.43</v>
+        <v>1.15</v>
       </c>
       <c r="L3" t="n">
-        <v>6.57</v>
+        <v>11.32</v>
       </c>
     </row>
     <row r="4">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>10.21</v>
+        <v>10.13</v>
       </c>
       <c r="E4" t="n">
         <v>10.22</v>
@@ -591,30 +591,30 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>241</v>
+        <v>207.7</v>
       </c>
       <c r="I4" t="n">
-        <v>4.18</v>
+        <v>3.37</v>
       </c>
       <c r="J4" t="n">
-        <v>11.2</v>
+        <v>14.1</v>
       </c>
       <c r="K4" t="n">
-        <v>10.1</v>
+        <v>6.36</v>
       </c>
       <c r="L4" t="n">
-        <v>7.14</v>
+        <v>8.98</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>300970</t>
+          <t>688813</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>华绿生物</t>
+          <t>泰金新能</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -623,44 +623,44 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>43.23</v>
+        <v>77</v>
       </c>
       <c r="E5" t="n">
-        <v>45.21</v>
+        <v>77.28</v>
       </c>
       <c r="F5" t="n">
-        <v>42.14</v>
+        <v>74.48</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>219.3</v>
+        <v>185.3</v>
       </c>
       <c r="I5" t="n">
-        <v>2.93</v>
+        <v>2.42</v>
       </c>
       <c r="J5" t="n">
-        <v>25.64</v>
+        <v>29.96</v>
       </c>
       <c r="K5" t="n">
-        <v>3.48</v>
+        <v>0.87</v>
       </c>
       <c r="L5" t="n">
-        <v>11.44</v>
+        <v>7.05</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>301667</t>
+          <t>301560</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>纳百川</t>
+          <t>众捷汽车</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -669,13 +669,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>120.18</v>
+        <v>41.26</v>
       </c>
       <c r="E6" t="n">
-        <v>117.57</v>
+        <v>40.34</v>
       </c>
       <c r="F6" t="n">
-        <v>105.84</v>
+        <v>36.46</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -683,30 +683,30 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>212.6</v>
+        <v>180.7</v>
       </c>
       <c r="I6" t="n">
-        <v>3.88</v>
+        <v>4.64</v>
       </c>
       <c r="J6" t="n">
-        <v>29.7</v>
+        <v>24.98</v>
       </c>
       <c r="K6" t="n">
-        <v>1.57</v>
+        <v>1.73</v>
       </c>
       <c r="L6" t="n">
-        <v>7.61</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>301630</t>
+          <t>002866</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>同宇新材</t>
+          <t>传艺科技</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -715,44 +715,44 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>225.18</v>
+        <v>26.04</v>
       </c>
       <c r="E7" t="n">
-        <v>223.29</v>
+        <v>26.08</v>
       </c>
       <c r="F7" t="n">
-        <v>211.99</v>
+        <v>23.77</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>205.4</v>
+        <v>165.6</v>
       </c>
       <c r="I7" t="n">
-        <v>5.18</v>
+        <v>2.6</v>
       </c>
       <c r="J7" t="n">
-        <v>23.12</v>
+        <v>25.08</v>
       </c>
       <c r="K7" t="n">
-        <v>3.16</v>
+        <v>0.86</v>
       </c>
       <c r="L7" t="n">
-        <v>5.21</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>002490</t>
+          <t>920069</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>山东墨龙</t>
+          <t>普昂医疗</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -761,13 +761,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>10.17</v>
+        <v>38.17</v>
       </c>
       <c r="E8" t="n">
-        <v>10.01</v>
+        <v>38.35</v>
       </c>
       <c r="F8" t="n">
-        <v>9.609999999999999</v>
+        <v>37.34</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -775,30 +775,30 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>193.6</v>
+        <v>165.3</v>
       </c>
       <c r="I8" t="n">
-        <v>4.09</v>
+        <v>3.36</v>
       </c>
       <c r="J8" t="n">
-        <v>17.91</v>
+        <v>21.5</v>
       </c>
       <c r="K8" t="n">
-        <v>3.91</v>
+        <v>1.61</v>
       </c>
       <c r="L8" t="n">
-        <v>9.85</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>601101</t>
+          <t>688269</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>昊华能源</t>
+          <t>凯立新材</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -807,13 +807,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>9.69</v>
+        <v>41.21</v>
       </c>
       <c r="E9" t="n">
-        <v>9.6</v>
+        <v>41.39</v>
       </c>
       <c r="F9" t="n">
-        <v>9.27</v>
+        <v>40.18</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -821,30 +821,30 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>174.2</v>
+        <v>161.1</v>
       </c>
       <c r="I9" t="n">
-        <v>3.53</v>
+        <v>5.02</v>
       </c>
       <c r="J9" t="n">
-        <v>5.17</v>
+        <v>5.96</v>
       </c>
       <c r="K9" t="n">
-        <v>6.54</v>
+        <v>6.44</v>
       </c>
       <c r="L9" t="n">
-        <v>7.25</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>920159</t>
+          <t>688530</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>农大科技</t>
+          <t>欧莱新材</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -853,44 +853,44 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>43.55</v>
+        <v>38.5</v>
       </c>
       <c r="E10" t="n">
-        <v>43.82</v>
+        <v>37.94</v>
       </c>
       <c r="F10" t="n">
-        <v>40.38</v>
+        <v>34.31</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>168.5</v>
+        <v>155.4</v>
       </c>
       <c r="I10" t="n">
-        <v>2.04</v>
+        <v>5.02</v>
       </c>
       <c r="J10" t="n">
-        <v>19.15</v>
+        <v>22.54</v>
       </c>
       <c r="K10" t="n">
-        <v>2.66</v>
+        <v>0.85</v>
       </c>
       <c r="L10" t="n">
-        <v>1.2</v>
+        <v>5.71</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>920069</t>
+          <t>300865</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>普昂医疗</t>
+          <t>大宏立</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -899,13 +899,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>38.2</v>
+        <v>30.69</v>
       </c>
       <c r="E11" t="n">
-        <v>38.35</v>
+        <v>30.47</v>
       </c>
       <c r="F11" t="n">
-        <v>37.44</v>
+        <v>28.52</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -913,30 +913,30 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>166.2</v>
+        <v>155.3</v>
       </c>
       <c r="I11" t="n">
-        <v>3.44</v>
+        <v>2.88</v>
       </c>
       <c r="J11" t="n">
-        <v>18.34</v>
+        <v>14.8</v>
       </c>
       <c r="K11" t="n">
-        <v>2.74</v>
+        <v>3.01</v>
       </c>
       <c r="L11" t="n">
-        <v>1.08</v>
+        <v>2.61</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>600052</t>
+          <t>301499</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>东望时代</t>
+          <t>维科精密</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -945,13 +945,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>4.61</v>
+        <v>36.36</v>
       </c>
       <c r="E12" t="n">
-        <v>4.7</v>
+        <v>35.66</v>
       </c>
       <c r="F12" t="n">
-        <v>4.27</v>
+        <v>30.71</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -959,30 +959,30 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>165.4</v>
+        <v>153.6</v>
       </c>
       <c r="I12" t="n">
-        <v>0.66</v>
+        <v>4.57</v>
       </c>
       <c r="J12" t="n">
-        <v>10.76</v>
+        <v>18.26</v>
       </c>
       <c r="K12" t="n">
-        <v>5.2</v>
+        <v>1.71</v>
       </c>
       <c r="L12" t="n">
-        <v>4.26</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>688813</t>
+          <t>300480</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>泰金新能</t>
+          <t>光力科技</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -991,44 +991,44 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>76.90000000000001</v>
+        <v>34.55</v>
       </c>
       <c r="E13" t="n">
-        <v>77.28</v>
+        <v>34.52</v>
       </c>
       <c r="F13" t="n">
-        <v>74.75</v>
+        <v>33.32</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>160.6</v>
+        <v>151.8</v>
       </c>
       <c r="I13" t="n">
-        <v>2.29</v>
+        <v>3.51</v>
       </c>
       <c r="J13" t="n">
-        <v>22.46</v>
+        <v>12.08</v>
       </c>
       <c r="K13" t="n">
-        <v>1.31</v>
+        <v>2.37</v>
       </c>
       <c r="L13" t="n">
-        <v>5.3</v>
+        <v>11.44</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>600310</t>
+          <t>601101</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>广西能源</t>
+          <t>昊华能源</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1037,13 +1037,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>5.35</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="E14" t="n">
-        <v>5.38</v>
+        <v>9.6</v>
       </c>
       <c r="F14" t="n">
-        <v>4.98</v>
+        <v>9.27</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1051,30 +1051,30 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>160.2</v>
+        <v>150.3</v>
       </c>
       <c r="I14" t="n">
-        <v>1.33</v>
+        <v>4.49</v>
       </c>
       <c r="J14" t="n">
-        <v>13.79</v>
+        <v>6.5</v>
       </c>
       <c r="K14" t="n">
-        <v>2.5</v>
+        <v>4.11</v>
       </c>
       <c r="L14" t="n">
-        <v>10.87</v>
+        <v>9.109999999999999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>300480</t>
+          <t>300200</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>光力科技</t>
+          <t>高盟新材</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1083,13 +1083,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>34.81</v>
+        <v>10.68</v>
       </c>
       <c r="E15" t="n">
-        <v>34.52</v>
+        <v>10.42</v>
       </c>
       <c r="F15" t="n">
-        <v>33.32</v>
+        <v>9.91</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1097,30 +1097,30 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>157.3</v>
+        <v>149.8</v>
       </c>
       <c r="I15" t="n">
-        <v>4.28</v>
+        <v>4.5</v>
       </c>
       <c r="J15" t="n">
-        <v>9.44</v>
+        <v>11.38</v>
       </c>
       <c r="K15" t="n">
-        <v>3.71</v>
+        <v>2.44</v>
       </c>
       <c r="L15" t="n">
-        <v>8.970000000000001</v>
+        <v>5.05</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>002377</t>
+          <t>603336</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>国创高新</t>
+          <t>宏辉果蔬</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1129,13 +1129,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>3.27</v>
+        <v>11.28</v>
       </c>
       <c r="E16" t="n">
-        <v>3.33</v>
+        <v>11.24</v>
       </c>
       <c r="F16" t="n">
-        <v>3.16</v>
+        <v>10.59</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1143,30 +1143,30 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>153</v>
+        <v>148.5</v>
       </c>
       <c r="I16" t="n">
-        <v>1.87</v>
+        <v>4.16</v>
       </c>
       <c r="J16" t="n">
-        <v>9.539999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="K16" t="n">
-        <v>4.57</v>
+        <v>3.09</v>
       </c>
       <c r="L16" t="n">
-        <v>2.82</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>300865</t>
+          <t>603158</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>大宏立</t>
+          <t>腾龙股份</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1175,13 +1175,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>30.58</v>
+        <v>13.78</v>
       </c>
       <c r="E17" t="n">
-        <v>30.47</v>
+        <v>13.51</v>
       </c>
       <c r="F17" t="n">
-        <v>28.52</v>
+        <v>12.65</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1189,30 +1189,30 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>151.8</v>
+        <v>147.5</v>
       </c>
       <c r="I17" t="n">
-        <v>2.51</v>
+        <v>5.19</v>
       </c>
       <c r="J17" t="n">
-        <v>10.34</v>
+        <v>13.27</v>
       </c>
       <c r="K17" t="n">
-        <v>4.2</v>
+        <v>1.62</v>
       </c>
       <c r="L17" t="n">
-        <v>1.82</v>
+        <v>8.949999999999999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>002310</t>
+          <t>688693</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>东方新能</t>
+          <t>锴威特</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1221,44 +1221,44 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>3.06</v>
+        <v>83.47</v>
       </c>
       <c r="E18" t="n">
-        <v>3.04</v>
+        <v>84.36</v>
       </c>
       <c r="F18" t="n">
-        <v>2.86</v>
+        <v>79.06999999999999</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>151.6</v>
+        <v>146.6</v>
       </c>
       <c r="I18" t="n">
-        <v>4.08</v>
+        <v>1.42</v>
       </c>
       <c r="J18" t="n">
-        <v>8.390000000000001</v>
+        <v>19.5</v>
       </c>
       <c r="K18" t="n">
-        <v>3.59</v>
+        <v>1.13</v>
       </c>
       <c r="L18" t="n">
-        <v>11.15</v>
+        <v>6.34</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>301307</t>
+          <t>002380</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>美利信</t>
+          <t>科远智慧</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1267,13 +1267,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>43.92</v>
+        <v>35.6</v>
       </c>
       <c r="E19" t="n">
-        <v>43.56</v>
+        <v>34.64</v>
       </c>
       <c r="F19" t="n">
-        <v>41.08</v>
+        <v>32.98</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1281,30 +1281,30 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>149.4</v>
+        <v>146.5</v>
       </c>
       <c r="I19" t="n">
-        <v>5.15</v>
+        <v>4.83</v>
       </c>
       <c r="J19" t="n">
-        <v>11.23</v>
+        <v>10.88</v>
       </c>
       <c r="K19" t="n">
-        <v>2.46</v>
+        <v>2.33</v>
       </c>
       <c r="L19" t="n">
-        <v>5.46</v>
+        <v>5.43</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>002470</t>
+          <t>002165</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>金正大</t>
+          <t>红 宝 丽</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1313,13 +1313,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>9.09</v>
       </c>
       <c r="E20" t="n">
-        <v>3.03</v>
+        <v>9.17</v>
       </c>
       <c r="F20" t="n">
-        <v>2.82</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1327,30 +1327,30 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>148.6</v>
+        <v>144</v>
       </c>
       <c r="I20" t="n">
-        <v>1.35</v>
+        <v>1.22</v>
       </c>
       <c r="J20" t="n">
-        <v>10.38</v>
+        <v>10.92</v>
       </c>
       <c r="K20" t="n">
-        <v>2.67</v>
+        <v>2.11</v>
       </c>
       <c r="L20" t="n">
-        <v>10.35</v>
+        <v>7.22</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>603496</t>
+          <t>002377</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>恒为科技</t>
+          <t>国创高新</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1359,13 +1359,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>32.52</v>
+        <v>3.26</v>
       </c>
       <c r="E21" t="n">
-        <v>32.21</v>
+        <v>3.33</v>
       </c>
       <c r="F21" t="n">
-        <v>30.04</v>
+        <v>3.16</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1373,30 +1373,30 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>147.8</v>
+        <v>142.9</v>
       </c>
       <c r="I21" t="n">
-        <v>2.07</v>
+        <v>1.56</v>
       </c>
       <c r="J21" t="n">
-        <v>10.57</v>
+        <v>12.06</v>
       </c>
       <c r="K21" t="n">
-        <v>2.54</v>
+        <v>2.89</v>
       </c>
       <c r="L21" t="n">
-        <v>10.71</v>
+        <v>3.53</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>002866</t>
+          <t>603459</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>传艺科技</t>
+          <t>红板科技</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1405,13 +1405,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>26.14</v>
+        <v>60.1</v>
       </c>
       <c r="E22" t="n">
-        <v>26.08</v>
+        <v>59.98</v>
       </c>
       <c r="F22" t="n">
-        <v>23.77</v>
+        <v>58.17</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1419,30 +1419,30 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>147</v>
+        <v>141.6</v>
       </c>
       <c r="I22" t="n">
-        <v>2.99</v>
+        <v>1.76</v>
       </c>
       <c r="J22" t="n">
-        <v>19.07</v>
+        <v>19.97</v>
       </c>
       <c r="K22" t="n">
-        <v>1.31</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="L22" t="n">
-        <v>8.970000000000001</v>
+        <v>9.550000000000001</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>600433</t>
+          <t>301079</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>冠豪高新</t>
+          <t>邵阳液压</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1451,44 +1451,44 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>4.04</v>
+        <v>44.3</v>
       </c>
       <c r="E23" t="n">
-        <v>4.07</v>
+        <v>45.06</v>
       </c>
       <c r="F23" t="n">
-        <v>3.95</v>
+        <v>42.64</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>145.2</v>
+        <v>141.4</v>
       </c>
       <c r="I23" t="n">
-        <v>3.06</v>
+        <v>1.37</v>
       </c>
       <c r="J23" t="n">
-        <v>7.76</v>
+        <v>19.09</v>
       </c>
       <c r="K23" t="n">
-        <v>3.26</v>
+        <v>0.84</v>
       </c>
       <c r="L23" t="n">
-        <v>5.6</v>
+        <v>6.61</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>002843</t>
+          <t>600433</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>泰嘉股份</t>
+          <t>冠豪高新</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1497,13 +1497,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>27.01</v>
+        <v>4</v>
       </c>
       <c r="E24" t="n">
-        <v>26.58</v>
+        <v>4.07</v>
       </c>
       <c r="F24" t="n">
-        <v>24.31</v>
+        <v>3.9</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1511,30 +1511,30 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>144.8</v>
+        <v>141.2</v>
       </c>
       <c r="I24" t="n">
-        <v>3.61</v>
+        <v>2.04</v>
       </c>
       <c r="J24" t="n">
-        <v>11.76</v>
+        <v>10.17</v>
       </c>
       <c r="K24" t="n">
-        <v>1.9</v>
+        <v>2.13</v>
       </c>
       <c r="L24" t="n">
-        <v>7.71</v>
+        <v>7.29</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>002213</t>
+          <t>300106</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>大为股份</t>
+          <t>西部牧业</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1543,13 +1543,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>34.67</v>
+        <v>10.77</v>
       </c>
       <c r="E25" t="n">
-        <v>34.59</v>
+        <v>10.74</v>
       </c>
       <c r="F25" t="n">
-        <v>32.96</v>
+        <v>10.19</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1557,30 +1557,30 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>144</v>
+        <v>140.5</v>
       </c>
       <c r="I25" t="n">
-        <v>1.58</v>
+        <v>1.32</v>
       </c>
       <c r="J25" t="n">
-        <v>12.58</v>
+        <v>12.53</v>
       </c>
       <c r="K25" t="n">
-        <v>1.56</v>
+        <v>2.53</v>
       </c>
       <c r="L25" t="n">
-        <v>8.99</v>
+        <v>2.84</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>301499</t>
+          <t>600470</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>维科精密</t>
+          <t>六国化工</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1589,13 +1589,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>36.17</v>
+        <v>7.07</v>
       </c>
       <c r="E26" t="n">
-        <v>35.66</v>
+        <v>7</v>
       </c>
       <c r="F26" t="n">
-        <v>30.71</v>
+        <v>6.64</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1603,30 +1603,30 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>143.7</v>
+        <v>140.3</v>
       </c>
       <c r="I26" t="n">
-        <v>4.03</v>
+        <v>3.36</v>
       </c>
       <c r="J26" t="n">
-        <v>13.39</v>
+        <v>12.46</v>
       </c>
       <c r="K26" t="n">
-        <v>2.51</v>
+        <v>2.54</v>
       </c>
       <c r="L26" t="n">
-        <v>1.66</v>
+        <v>4.59</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>300443</t>
+          <t>300505</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>金雷股份</t>
+          <t>川金诺</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1635,13 +1635,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>31.05</v>
+        <v>26.13</v>
       </c>
       <c r="E27" t="n">
-        <v>30.99</v>
+        <v>25.9</v>
       </c>
       <c r="F27" t="n">
-        <v>29.13</v>
+        <v>24.81</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1649,30 +1649,30 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>141.4</v>
+        <v>140.2</v>
       </c>
       <c r="I27" t="n">
-        <v>3.29</v>
+        <v>2.67</v>
       </c>
       <c r="J27" t="n">
-        <v>7.49</v>
+        <v>11.58</v>
       </c>
       <c r="K27" t="n">
-        <v>3.04</v>
+        <v>1.57</v>
       </c>
       <c r="L27" t="n">
-        <v>5.73</v>
+        <v>6.56</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>600470</t>
+          <t>603221</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>六国化工</t>
+          <t>爱丽家居</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1681,13 +1681,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>6.97</v>
+        <v>11.98</v>
       </c>
       <c r="E28" t="n">
-        <v>7</v>
+        <v>11.72</v>
       </c>
       <c r="F28" t="n">
-        <v>6.64</v>
+        <v>11.07</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1695,30 +1695,30 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>140.8</v>
+        <v>139</v>
       </c>
       <c r="I28" t="n">
-        <v>1.9</v>
+        <v>5</v>
       </c>
       <c r="J28" t="n">
-        <v>9.08</v>
+        <v>3.93</v>
       </c>
       <c r="K28" t="n">
-        <v>3.71</v>
+        <v>5.27</v>
       </c>
       <c r="L28" t="n">
-        <v>3.34</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>000593</t>
+          <t>600678</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>德龙汇能</t>
+          <t>四川金顶</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1727,44 +1727,44 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>20.25</v>
+        <v>12.18</v>
       </c>
       <c r="E29" t="n">
-        <v>19.97</v>
+        <v>12.03</v>
       </c>
       <c r="F29" t="n">
-        <v>19.22</v>
+        <v>11.53</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>138.1</v>
+        <v>138</v>
       </c>
       <c r="I29" t="n">
-        <v>3.11</v>
+        <v>3.31</v>
       </c>
       <c r="J29" t="n">
-        <v>9.06</v>
+        <v>16.3</v>
       </c>
       <c r="K29" t="n">
-        <v>2.24</v>
+        <v>1.48</v>
       </c>
       <c r="L29" t="n">
-        <v>6.5</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>002445</t>
+          <t>002734</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>中南文化</t>
+          <t>利民股份</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1773,13 +1773,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>3.56</v>
+        <v>17.83</v>
       </c>
       <c r="E30" t="n">
-        <v>3.55</v>
+        <v>17.73</v>
       </c>
       <c r="F30" t="n">
-        <v>3.36</v>
+        <v>16.26</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1787,30 +1787,30 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>137</v>
+        <v>137.1</v>
       </c>
       <c r="I30" t="n">
-        <v>2.01</v>
+        <v>1.6</v>
       </c>
       <c r="J30" t="n">
-        <v>7.42</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="K30" t="n">
-        <v>2.69</v>
+        <v>1.89</v>
       </c>
       <c r="L30" t="n">
-        <v>6.3</v>
+        <v>7.45</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>002560</t>
+          <t>002445</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>通达股份</t>
+          <t>中南文化</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1819,44 +1819,44 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>14.36</v>
+        <v>3.55</v>
       </c>
       <c r="E31" t="n">
-        <v>14.43</v>
+        <v>3.55</v>
       </c>
       <c r="F31" t="n">
-        <v>13.36</v>
+        <v>3.36</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>136.7</v>
+        <v>136</v>
       </c>
       <c r="I31" t="n">
-        <v>0.63</v>
+        <v>1.72</v>
       </c>
       <c r="J31" t="n">
-        <v>17</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="K31" t="n">
-        <v>1.14</v>
+        <v>1.79</v>
       </c>
       <c r="L31" t="n">
-        <v>11.02</v>
+        <v>8.369999999999999</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>300740</t>
+          <t>300056</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>水羊股份</t>
+          <t>中创环保</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1865,13 +1865,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>24.36</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="E32" t="n">
-        <v>23.89</v>
+        <v>9.48</v>
       </c>
       <c r="F32" t="n">
-        <v>23.23</v>
+        <v>8.19</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1879,30 +1879,30 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>136.4</v>
+        <v>135.7</v>
       </c>
       <c r="I32" t="n">
-        <v>5</v>
+        <v>0.97</v>
       </c>
       <c r="J32" t="n">
-        <v>6.15</v>
+        <v>11.67</v>
       </c>
       <c r="K32" t="n">
-        <v>3.07</v>
+        <v>2.42</v>
       </c>
       <c r="L32" t="n">
-        <v>5.44</v>
+        <v>4.03</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>301292</t>
+          <t>603198</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>海科新源</t>
+          <t>迎驾贡酒</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1911,44 +1911,44 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>85.90000000000001</v>
+        <v>39.85</v>
       </c>
       <c r="E33" t="n">
-        <v>85.2</v>
+        <v>39.73</v>
       </c>
       <c r="F33" t="n">
-        <v>77.81999999999999</v>
+        <v>37.88</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>135.8</v>
+        <v>135</v>
       </c>
       <c r="I33" t="n">
-        <v>2.55</v>
+        <v>2.13</v>
       </c>
       <c r="J33" t="n">
-        <v>16.25</v>
+        <v>3.14</v>
       </c>
       <c r="K33" t="n">
-        <v>1.32</v>
+        <v>3.95</v>
       </c>
       <c r="L33" t="n">
-        <v>11.51</v>
+        <v>10.05</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>301248</t>
+          <t>300443</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>杰创智能</t>
+          <t>金雷股份</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1957,13 +1957,13 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>64.26000000000001</v>
+        <v>30.87</v>
       </c>
       <c r="E34" t="n">
-        <v>64.18000000000001</v>
+        <v>30.99</v>
       </c>
       <c r="F34" t="n">
-        <v>58.98</v>
+        <v>29.13</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1971,30 +1971,30 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>135.1</v>
+        <v>134</v>
       </c>
       <c r="I34" t="n">
-        <v>1.84</v>
+        <v>2.69</v>
       </c>
       <c r="J34" t="n">
-        <v>9.27</v>
+        <v>9.18</v>
       </c>
       <c r="K34" t="n">
-        <v>1.92</v>
+        <v>1.86</v>
       </c>
       <c r="L34" t="n">
-        <v>6.71</v>
+        <v>7.01</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>600120</t>
+          <t>300925</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>浙江东方</t>
+          <t>法本信息</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2003,13 +2003,13 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>5.95</v>
+        <v>19.85</v>
       </c>
       <c r="E35" t="n">
-        <v>5.86</v>
+        <v>19.98</v>
       </c>
       <c r="F35" t="n">
-        <v>5.49</v>
+        <v>17.95</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2017,30 +2017,30 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>134.9</v>
+        <v>133.8</v>
       </c>
       <c r="I35" t="n">
-        <v>3.3</v>
+        <v>3.66</v>
       </c>
       <c r="J35" t="n">
-        <v>3.04</v>
+        <v>9.43</v>
       </c>
       <c r="K35" t="n">
-        <v>3.98</v>
+        <v>1.76</v>
       </c>
       <c r="L35" t="n">
-        <v>6.02</v>
+        <v>6.51</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>000953</t>
+          <t>300607</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>河化股份</t>
+          <t>拓斯达</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2049,13 +2049,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>6.73</v>
+        <v>29.82</v>
       </c>
       <c r="E36" t="n">
-        <v>6.72</v>
+        <v>29.64</v>
       </c>
       <c r="F36" t="n">
-        <v>6.58</v>
+        <v>28.18</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2063,30 +2063,30 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>134.5</v>
+        <v>133.5</v>
       </c>
       <c r="I36" t="n">
-        <v>3.38</v>
+        <v>1.88</v>
       </c>
       <c r="J36" t="n">
-        <v>3.72</v>
+        <v>8.92</v>
       </c>
       <c r="K36" t="n">
-        <v>4.97</v>
+        <v>1.9</v>
       </c>
       <c r="L36" t="n">
-        <v>0.9399999999999999</v>
+        <v>8.93</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>920028</t>
+          <t>002752</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>新恒泰</t>
+          <t>昇兴股份</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2095,13 +2095,13 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>16.81</v>
+        <v>7.43</v>
       </c>
       <c r="E37" t="n">
-        <v>16.55</v>
+        <v>7.34</v>
       </c>
       <c r="F37" t="n">
-        <v>15.74</v>
+        <v>6.96</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -2109,30 +2109,30 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>134.2</v>
+        <v>132.9</v>
       </c>
       <c r="I37" t="n">
-        <v>3.83</v>
+        <v>2.48</v>
       </c>
       <c r="J37" t="n">
-        <v>13.34</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="K37" t="n">
-        <v>1.74</v>
+        <v>1.73</v>
       </c>
       <c r="L37" t="n">
-        <v>0.95</v>
+        <v>6.67</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>603198</t>
+          <t>300671</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>迎驾贡酒</t>
+          <t>富满微</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2141,44 +2141,44 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>40.45</v>
+        <v>47.65</v>
       </c>
       <c r="E38" t="n">
-        <v>39.73</v>
+        <v>46.6</v>
       </c>
       <c r="F38" t="n">
-        <v>37.88</v>
+        <v>44.94</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>134.1</v>
+        <v>130.6</v>
       </c>
       <c r="I38" t="n">
-        <v>3.66</v>
+        <v>4.02</v>
       </c>
       <c r="J38" t="n">
-        <v>2.31</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="K38" t="n">
-        <v>5.82</v>
+        <v>1.51</v>
       </c>
       <c r="L38" t="n">
-        <v>7.4</v>
+        <v>9.720000000000001</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>300651</t>
+          <t>300916</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>金陵体育</t>
+          <t>朗特智能</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2187,13 +2187,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>29.48</v>
+        <v>36</v>
       </c>
       <c r="E39" t="n">
-        <v>29.08</v>
+        <v>35.98</v>
       </c>
       <c r="F39" t="n">
-        <v>27.47</v>
+        <v>32.5</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -2201,19 +2201,19 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>133.6</v>
+        <v>129.7</v>
       </c>
       <c r="I39" t="n">
-        <v>3.37</v>
+        <v>1.01</v>
       </c>
       <c r="J39" t="n">
-        <v>13.61</v>
+        <v>12.48</v>
       </c>
       <c r="K39" t="n">
-        <v>1.6</v>
+        <v>1.65</v>
       </c>
       <c r="L39" t="n">
-        <v>3.48</v>
+        <v>4.11</v>
       </c>
     </row>
     <row r="40">
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>24.51</v>
+        <v>24.45</v>
       </c>
       <c r="E40" t="n">
         <v>24.81</v>
@@ -2243,34 +2243,34 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>133.1</v>
+        <v>129.4</v>
       </c>
       <c r="I40" t="n">
-        <v>1.49</v>
+        <v>1.24</v>
       </c>
       <c r="J40" t="n">
-        <v>13.06</v>
+        <v>18.64</v>
       </c>
       <c r="K40" t="n">
-        <v>1.74</v>
+        <v>1.24</v>
       </c>
       <c r="L40" t="n">
-        <v>3.41</v>
+        <v>4.85</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>300200</t>
+          <t>600691</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>高盟新材</t>
+          <t>潞化科技</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2279,13 +2279,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>10.36</v>
+        <v>3.38</v>
       </c>
       <c r="E41" t="n">
-        <v>10.4</v>
+        <v>3.35</v>
       </c>
       <c r="F41" t="n">
-        <v>9.91</v>
+        <v>3.19</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -2293,30 +2293,30 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>132.5</v>
+        <v>128.8</v>
       </c>
       <c r="I41" t="n">
-        <v>1.37</v>
+        <v>4</v>
       </c>
       <c r="J41" t="n">
-        <v>7.93</v>
+        <v>6.23</v>
       </c>
       <c r="K41" t="n">
-        <v>3.4</v>
+        <v>2.41</v>
       </c>
       <c r="L41" t="n">
-        <v>3.51</v>
+        <v>5.01</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>688052</t>
+          <t>300547</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>纳芯微</t>
+          <t>川环科技</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2325,44 +2325,44 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>186</v>
+        <v>37.4</v>
       </c>
       <c r="E42" t="n">
-        <v>182.41</v>
+        <v>37.05</v>
       </c>
       <c r="F42" t="n">
-        <v>178.73</v>
+        <v>33.76</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>130.8</v>
+        <v>127</v>
       </c>
       <c r="I42" t="n">
-        <v>4.72</v>
+        <v>3.43</v>
       </c>
       <c r="J42" t="n">
-        <v>4.2</v>
+        <v>14.42</v>
       </c>
       <c r="K42" t="n">
-        <v>3.25</v>
+        <v>1.19</v>
       </c>
       <c r="L42" t="n">
-        <v>11.14</v>
+        <v>9.390000000000001</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>300916</t>
+          <t>300589</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>朗特智能</t>
+          <t>江龙船艇</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2371,44 +2371,44 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>36.17</v>
+        <v>16.35</v>
       </c>
       <c r="E43" t="n">
-        <v>35.98</v>
+        <v>16.22</v>
       </c>
       <c r="F43" t="n">
-        <v>32.5</v>
+        <v>15.84</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>130.6</v>
+        <v>126.8</v>
       </c>
       <c r="I43" t="n">
-        <v>1.49</v>
+        <v>3.61</v>
       </c>
       <c r="J43" t="n">
-        <v>9.85</v>
+        <v>14.16</v>
       </c>
       <c r="K43" t="n">
-        <v>2.6</v>
+        <v>1.26</v>
       </c>
       <c r="L43" t="n">
-        <v>3.23</v>
+        <v>5.46</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>600678</t>
+          <t>300562</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>四川金顶</t>
+          <t>乐心医疗</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2417,13 +2417,13 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>11.96</v>
+        <v>14.47</v>
       </c>
       <c r="E44" t="n">
-        <v>12.03</v>
+        <v>14.48</v>
       </c>
       <c r="F44" t="n">
-        <v>11.53</v>
+        <v>13.46</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -2431,30 +2431,30 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>130</v>
+        <v>126.4</v>
       </c>
       <c r="I44" t="n">
-        <v>1.44</v>
+        <v>0.63</v>
       </c>
       <c r="J44" t="n">
-        <v>11.34</v>
+        <v>11.08</v>
       </c>
       <c r="K44" t="n">
-        <v>2.05</v>
+        <v>1.84</v>
       </c>
       <c r="L44" t="n">
-        <v>4.78</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>002799</t>
+          <t>300651</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>环球印务</t>
+          <t>金陵体育</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2463,44 +2463,44 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>8.300000000000001</v>
+        <v>28.79</v>
       </c>
       <c r="E45" t="n">
-        <v>8.1</v>
+        <v>29.08</v>
       </c>
       <c r="F45" t="n">
-        <v>7.87</v>
+        <v>27.47</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H45" t="n">
-        <v>129.8</v>
+        <v>126</v>
       </c>
       <c r="I45" t="n">
-        <v>4.93</v>
+        <v>0.95</v>
       </c>
       <c r="J45" t="n">
-        <v>3.57</v>
+        <v>18.27</v>
       </c>
       <c r="K45" t="n">
-        <v>4.63</v>
+        <v>1.08</v>
       </c>
       <c r="L45" t="n">
-        <v>0.9399999999999999</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>601921</t>
+          <t>003026</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>浙版传媒</t>
+          <t>中晶科技</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2509,33 +2509,33 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>8.27</v>
+        <v>39.32</v>
       </c>
       <c r="E46" t="n">
-        <v>8.140000000000001</v>
+        <v>38.6</v>
       </c>
       <c r="F46" t="n">
-        <v>7.77</v>
+        <v>36.9</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>129.1</v>
+        <v>124.4</v>
       </c>
       <c r="I46" t="n">
-        <v>3.5</v>
+        <v>3.31</v>
       </c>
       <c r="J46" t="n">
-        <v>1.27</v>
+        <v>11.04</v>
       </c>
       <c r="K46" t="n">
-        <v>7</v>
+        <v>1.69</v>
       </c>
       <c r="L46" t="n">
-        <v>2.32</v>
+        <v>4.11</v>
       </c>
     </row>
     <row r="47">
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>8.94</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="E47" t="n">
         <v>9.01</v>
@@ -2569,30 +2569,30 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>128.4</v>
+        <v>124.2</v>
       </c>
       <c r="I47" t="n">
-        <v>0.68</v>
+        <v>0.79</v>
       </c>
       <c r="J47" t="n">
-        <v>8.34</v>
+        <v>10.53</v>
       </c>
       <c r="K47" t="n">
-        <v>2.92</v>
+        <v>1.84</v>
       </c>
       <c r="L47" t="n">
-        <v>2.7</v>
+        <v>3.41</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>300821</t>
+          <t>920028</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>东岳硅材</t>
+          <t>新恒泰</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2601,44 +2601,44 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>14.97</v>
+        <v>16.96</v>
       </c>
       <c r="E48" t="n">
-        <v>14.64</v>
+        <v>16.55</v>
       </c>
       <c r="F48" t="n">
-        <v>13.81</v>
+        <v>15.74</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H48" t="n">
-        <v>128.2</v>
+        <v>123.7</v>
       </c>
       <c r="I48" t="n">
         <v>4.76</v>
       </c>
       <c r="J48" t="n">
-        <v>6.56</v>
+        <v>17.51</v>
       </c>
       <c r="K48" t="n">
-        <v>2.25</v>
+        <v>1.14</v>
       </c>
       <c r="L48" t="n">
-        <v>11.64</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>603186</t>
+          <t>300357</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>华正新材</t>
+          <t>我武生物</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2647,13 +2647,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>72.01000000000001</v>
+        <v>26.75</v>
       </c>
       <c r="E49" t="n">
-        <v>70.87</v>
+        <v>26.74</v>
       </c>
       <c r="F49" t="n">
-        <v>65.17</v>
+        <v>25.94</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2661,30 +2661,30 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>128.1</v>
+        <v>122.8</v>
       </c>
       <c r="I49" t="n">
-        <v>3.17</v>
+        <v>2.88</v>
       </c>
       <c r="J49" t="n">
-        <v>8.140000000000001</v>
+        <v>4.33</v>
       </c>
       <c r="K49" t="n">
-        <v>1.71</v>
+        <v>2.54</v>
       </c>
       <c r="L49" t="n">
-        <v>8.9</v>
+        <v>5.69</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>000833</t>
+          <t>001317</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>粤桂股份</t>
+          <t>三羊马</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2693,13 +2693,13 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>25.26</v>
+        <v>50.91</v>
       </c>
       <c r="E50" t="n">
-        <v>25.59</v>
+        <v>50.68</v>
       </c>
       <c r="F50" t="n">
-        <v>24.69</v>
+        <v>49.14</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2707,30 +2707,30 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>127.9</v>
+        <v>121.6</v>
       </c>
       <c r="I50" t="n">
-        <v>1.16</v>
+        <v>3.24</v>
       </c>
       <c r="J50" t="n">
-        <v>8.1</v>
+        <v>8.43</v>
       </c>
       <c r="K50" t="n">
-        <v>1.71</v>
+        <v>2.32</v>
       </c>
       <c r="L50" t="n">
-        <v>9.539999999999999</v>
+        <v>3.71</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>300573</t>
+          <t>600120</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>兴齐眼药</t>
+          <t>浙江东方</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2739,13 +2739,13 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>70.5</v>
+        <v>5.88</v>
       </c>
       <c r="E51" t="n">
-        <v>69.34</v>
+        <v>5.86</v>
       </c>
       <c r="F51" t="n">
-        <v>66.47</v>
+        <v>5.49</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2753,30 +2753,30 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>127.7</v>
+        <v>121.5</v>
       </c>
       <c r="I51" t="n">
-        <v>3.36</v>
+        <v>2.08</v>
       </c>
       <c r="J51" t="n">
-        <v>4.3</v>
+        <v>3.92</v>
       </c>
       <c r="K51" t="n">
-        <v>2.96</v>
+        <v>2.57</v>
       </c>
       <c r="L51" t="n">
-        <v>5.71</v>
+        <v>7.81</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>002897</t>
+          <t>600844</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>意华股份</t>
+          <t>金煤科技</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2785,13 +2785,13 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>67.95</v>
+        <v>3.53</v>
       </c>
       <c r="E52" t="n">
-        <v>67.40000000000001</v>
+        <v>3.56</v>
       </c>
       <c r="F52" t="n">
-        <v>63.16</v>
+        <v>3.36</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2799,30 +2799,30 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>127.6</v>
+        <v>121</v>
       </c>
       <c r="I52" t="n">
-        <v>1.97</v>
+        <v>0.86</v>
       </c>
       <c r="J52" t="n">
-        <v>7.16</v>
+        <v>10.42</v>
       </c>
       <c r="K52" t="n">
-        <v>2</v>
+        <v>1.61</v>
       </c>
       <c r="L52" t="n">
-        <v>8.699999999999999</v>
+        <v>3.04</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>603079</t>
+          <t>002386</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>圣达生物</t>
+          <t>天原股份</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2831,13 +2831,13 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>16.93</v>
+        <v>6.84</v>
       </c>
       <c r="E53" t="n">
-        <v>17.22</v>
+        <v>6.73</v>
       </c>
       <c r="F53" t="n">
-        <v>16.17</v>
+        <v>6.43</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2845,30 +2845,30 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>127.2</v>
+        <v>121</v>
       </c>
       <c r="I53" t="n">
-        <v>2.05</v>
+        <v>3.32</v>
       </c>
       <c r="J53" t="n">
-        <v>3.84</v>
+        <v>6.66</v>
       </c>
       <c r="K53" t="n">
-        <v>4.32</v>
+        <v>1.61</v>
       </c>
       <c r="L53" t="n">
-        <v>1.26</v>
+        <v>5.86</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>001317</t>
+          <t>300573</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>三羊马</t>
+          <t>兴齐眼药</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2877,13 +2877,13 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>51.28</v>
+        <v>70.84999999999999</v>
       </c>
       <c r="E54" t="n">
-        <v>50.68</v>
+        <v>69.34</v>
       </c>
       <c r="F54" t="n">
-        <v>49.14</v>
+        <v>66.47</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2891,30 +2891,30 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>127.2</v>
+        <v>120.8</v>
       </c>
       <c r="I54" t="n">
-        <v>4</v>
+        <v>3.87</v>
       </c>
       <c r="J54" t="n">
-        <v>6.34</v>
+        <v>5.64</v>
       </c>
       <c r="K54" t="n">
-        <v>3.49</v>
+        <v>1.94</v>
       </c>
       <c r="L54" t="n">
-        <v>2.8</v>
+        <v>7.51</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>301587</t>
+          <t>605268</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>中瑞股份</t>
+          <t>王力安防</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2923,13 +2923,13 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>28.79</v>
+        <v>13.72</v>
       </c>
       <c r="E55" t="n">
-        <v>28.35</v>
+        <v>13.31</v>
       </c>
       <c r="F55" t="n">
-        <v>26.89</v>
+        <v>12.4</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2937,30 +2937,30 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>127.2</v>
+        <v>120.6</v>
       </c>
       <c r="I55" t="n">
-        <v>4.24</v>
+        <v>5.05</v>
       </c>
       <c r="J55" t="n">
-        <v>11.77</v>
+        <v>6.54</v>
       </c>
       <c r="K55" t="n">
-        <v>1.68</v>
+        <v>2.87</v>
       </c>
       <c r="L55" t="n">
-        <v>2.49</v>
+        <v>3.83</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>603459</t>
+          <t>300615</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>红板科技</t>
+          <t>欣天科技</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2969,44 +2969,44 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>60.06</v>
+        <v>13.62</v>
       </c>
       <c r="E56" t="n">
-        <v>59.98</v>
+        <v>13.63</v>
       </c>
       <c r="F56" t="n">
-        <v>58.17</v>
+        <v>12.7</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H56" t="n">
-        <v>127.1</v>
+        <v>120.2</v>
       </c>
       <c r="I56" t="n">
-        <v>1.69</v>
+        <v>1.57</v>
       </c>
       <c r="J56" t="n">
-        <v>15.41</v>
+        <v>8.68</v>
       </c>
       <c r="K56" t="n">
-        <v>0.87</v>
+        <v>2.12</v>
       </c>
       <c r="L56" t="n">
-        <v>7.37</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>300679</t>
+          <t>002481</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>电连技术</t>
+          <t>双塔食品</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3015,13 +3015,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>44.09</v>
+        <v>4.63</v>
       </c>
       <c r="E57" t="n">
-        <v>43.79</v>
+        <v>4.54</v>
       </c>
       <c r="F57" t="n">
-        <v>41.33</v>
+        <v>4.42</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -3029,30 +3029,30 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>126.8</v>
+        <v>120.2</v>
       </c>
       <c r="I57" t="n">
-        <v>4.01</v>
+        <v>4.99</v>
       </c>
       <c r="J57" t="n">
-        <v>6.38</v>
+        <v>3.56</v>
       </c>
       <c r="K57" t="n">
-        <v>2.19</v>
+        <v>3.83</v>
       </c>
       <c r="L57" t="n">
-        <v>10.24</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>301190</t>
+          <t>300966</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>善水科技</t>
+          <t>共同药业</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3061,13 +3061,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>24.78</v>
+        <v>22.6</v>
       </c>
       <c r="E58" t="n">
-        <v>24.27</v>
+        <v>22.12</v>
       </c>
       <c r="F58" t="n">
-        <v>22.42</v>
+        <v>21.06</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -3075,30 +3075,30 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>126.8</v>
+        <v>120.1</v>
       </c>
       <c r="I58" t="n">
-        <v>4.73</v>
+        <v>4.29</v>
       </c>
       <c r="J58" t="n">
-        <v>3.44</v>
+        <v>6.17</v>
       </c>
       <c r="K58" t="n">
-        <v>4.42</v>
+        <v>2.95</v>
       </c>
       <c r="L58" t="n">
-        <v>1.3</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>300589</t>
+          <t>301587</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>江龙船艇</t>
+          <t>中瑞股份</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3107,44 +3107,44 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>16.32</v>
+        <v>28.76</v>
       </c>
       <c r="E59" t="n">
-        <v>16.22</v>
+        <v>28.35</v>
       </c>
       <c r="F59" t="n">
-        <v>15.84</v>
+        <v>26.89</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H59" t="n">
-        <v>126.6</v>
+        <v>120</v>
       </c>
       <c r="I59" t="n">
-        <v>3.42</v>
+        <v>4.13</v>
       </c>
       <c r="J59" t="n">
-        <v>10.86</v>
+        <v>16.49</v>
       </c>
       <c r="K59" t="n">
-        <v>1.93</v>
+        <v>1.17</v>
       </c>
       <c r="L59" t="n">
-        <v>4.2</v>
+        <v>3.48</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>301116</t>
+          <t>002079</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>益客食品</t>
+          <t>苏州固锝</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3153,44 +3153,44 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>10.8</v>
+        <v>10.68</v>
       </c>
       <c r="E60" t="n">
-        <v>10.77</v>
+        <v>10.7</v>
       </c>
       <c r="F60" t="n">
-        <v>10.48</v>
+        <v>10.24</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H60" t="n">
-        <v>126.6</v>
+        <v>119.7</v>
       </c>
       <c r="I60" t="n">
-        <v>4.45</v>
+        <v>1.42</v>
       </c>
       <c r="J60" t="n">
-        <v>2.02</v>
+        <v>6.62</v>
       </c>
       <c r="K60" t="n">
-        <v>6.54</v>
+        <v>1.52</v>
       </c>
       <c r="L60" t="n">
-        <v>1</v>
+        <v>5.79</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>002652</t>
+          <t>300867</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>扬子新材</t>
+          <t>圣元环保</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3199,13 +3199,13 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>4.92</v>
+        <v>21.34</v>
       </c>
       <c r="E61" t="n">
-        <v>4.85</v>
+        <v>21.39</v>
       </c>
       <c r="F61" t="n">
-        <v>4.57</v>
+        <v>20.71</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -3213,30 +3213,30 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>126.3</v>
+        <v>118.7</v>
       </c>
       <c r="I61" t="n">
-        <v>5.13</v>
+        <v>1.57</v>
       </c>
       <c r="J61" t="n">
-        <v>5.53</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="K61" t="n">
-        <v>3.68</v>
+        <v>1.93</v>
       </c>
       <c r="L61" t="n">
-        <v>1.4</v>
+        <v>3.67</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>600691</t>
+          <t>301106</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>潞化科技</t>
+          <t>骏成科技</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3245,13 +3245,13 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>3.36</v>
+        <v>33.32</v>
       </c>
       <c r="E62" t="n">
-        <v>3.35</v>
+        <v>33.41</v>
       </c>
       <c r="F62" t="n">
-        <v>3.19</v>
+        <v>30.82</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -3259,30 +3259,30 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>125.7</v>
+        <v>117.2</v>
       </c>
       <c r="I62" t="n">
-        <v>3.38</v>
+        <v>0.82</v>
       </c>
       <c r="J62" t="n">
-        <v>4.94</v>
+        <v>7.39</v>
       </c>
       <c r="K62" t="n">
-        <v>3.83</v>
+        <v>2.3</v>
       </c>
       <c r="L62" t="n">
-        <v>3.99</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>300025</t>
+          <t>002940</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>华星创业</t>
+          <t>昂利康</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3291,44 +3291,44 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>5.33</v>
+        <v>39.9</v>
       </c>
       <c r="E63" t="n">
-        <v>5.32</v>
+        <v>39.72</v>
       </c>
       <c r="F63" t="n">
-        <v>5.08</v>
+        <v>37.31</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="H63" t="n">
-        <v>124.8</v>
+        <v>116.5</v>
       </c>
       <c r="I63" t="n">
-        <v>3.09</v>
+        <v>1.79</v>
       </c>
       <c r="J63" t="n">
-        <v>4.44</v>
+        <v>13.36</v>
       </c>
       <c r="K63" t="n">
-        <v>3.92</v>
+        <v>0.67</v>
       </c>
       <c r="L63" t="n">
-        <v>1.22</v>
+        <v>9.74</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>600763</t>
+          <t>300726</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>通策医疗</t>
+          <t>宏达电子</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3337,13 +3337,13 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>43.56</v>
+        <v>48.51</v>
       </c>
       <c r="E64" t="n">
-        <v>43.36</v>
+        <v>48.26</v>
       </c>
       <c r="F64" t="n">
-        <v>41.26</v>
+        <v>47.01</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -3351,30 +3351,30 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>124.7</v>
+        <v>116.5</v>
       </c>
       <c r="I64" t="n">
-        <v>2.13</v>
+        <v>2.3</v>
       </c>
       <c r="J64" t="n">
-        <v>3.06</v>
+        <v>5.6</v>
       </c>
       <c r="K64" t="n">
-        <v>3.12</v>
+        <v>1.59</v>
       </c>
       <c r="L64" t="n">
-        <v>5.94</v>
+        <v>5.86</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>300435</t>
+          <t>301190</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>中泰股份</t>
+          <t>善水科技</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3383,13 +3383,13 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>23.55</v>
+        <v>24.35</v>
       </c>
       <c r="E65" t="n">
-        <v>24.08</v>
+        <v>24.27</v>
       </c>
       <c r="F65" t="n">
-        <v>22.46</v>
+        <v>22.42</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -3397,30 +3397,30 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>124.4</v>
+        <v>116.2</v>
       </c>
       <c r="I65" t="n">
-        <v>1.07</v>
+        <v>2.92</v>
       </c>
       <c r="J65" t="n">
-        <v>5.99</v>
+        <v>4.8</v>
       </c>
       <c r="K65" t="n">
-        <v>2.12</v>
+        <v>3.08</v>
       </c>
       <c r="L65" t="n">
-        <v>5.38</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>605268</t>
+          <t>000953</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>王力安防</t>
+          <t>河化股份</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3429,13 +3429,13 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>13.37</v>
+        <v>6.74</v>
       </c>
       <c r="E66" t="n">
-        <v>13.29</v>
+        <v>6.72</v>
       </c>
       <c r="F66" t="n">
-        <v>12.4</v>
+        <v>6.57</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -3443,30 +3443,30 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>124</v>
+        <v>115.8</v>
       </c>
       <c r="I66" t="n">
-        <v>2.37</v>
+        <v>3.53</v>
       </c>
       <c r="J66" t="n">
-        <v>4.41</v>
+        <v>4.64</v>
       </c>
       <c r="K66" t="n">
-        <v>3.86</v>
+        <v>3.1</v>
       </c>
       <c r="L66" t="n">
-        <v>2.57</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>300357</t>
+          <t>603290</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>我武生物</t>
+          <t>斯达半导</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3475,13 +3475,13 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>26.83</v>
+        <v>108.7</v>
       </c>
       <c r="E67" t="n">
-        <v>26.74</v>
+        <v>107.79</v>
       </c>
       <c r="F67" t="n">
-        <v>25.94</v>
+        <v>103.89</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -3489,30 +3489,30 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>123.8</v>
+        <v>115.6</v>
       </c>
       <c r="I67" t="n">
-        <v>3.19</v>
+        <v>2.55</v>
       </c>
       <c r="J67" t="n">
-        <v>3.53</v>
+        <v>4.23</v>
       </c>
       <c r="K67" t="n">
-        <v>4.14</v>
+        <v>1.97</v>
       </c>
       <c r="L67" t="n">
-        <v>4.66</v>
+        <v>10.97</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>300671</t>
+          <t>605122</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>富满微</t>
+          <t>四方新材</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3521,13 +3521,13 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>47.28</v>
+        <v>13.91</v>
       </c>
       <c r="E68" t="n">
-        <v>46.6</v>
+        <v>13.76</v>
       </c>
       <c r="F68" t="n">
-        <v>44.94</v>
+        <v>13.14</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -3535,30 +3535,30 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>123.6</v>
+        <v>115.2</v>
       </c>
       <c r="I68" t="n">
-        <v>3.21</v>
+        <v>2.2</v>
       </c>
       <c r="J68" t="n">
-        <v>6.18</v>
+        <v>4.83</v>
       </c>
       <c r="K68" t="n">
-        <v>1.99</v>
+        <v>2.99</v>
       </c>
       <c r="L68" t="n">
-        <v>6.4</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>300677</t>
+          <t>300025</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>英科医疗</t>
+          <t>华星创业</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3567,13 +3567,13 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>56.81</v>
+        <v>5.42</v>
       </c>
       <c r="E69" t="n">
-        <v>56.42</v>
+        <v>5.32</v>
       </c>
       <c r="F69" t="n">
-        <v>50.99</v>
+        <v>5.08</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -3581,30 +3581,30 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>123.5</v>
+        <v>115.1</v>
       </c>
       <c r="I69" t="n">
-        <v>3.05</v>
+        <v>4.84</v>
       </c>
       <c r="J69" t="n">
-        <v>4.42</v>
+        <v>5.92</v>
       </c>
       <c r="K69" t="n">
-        <v>2.57</v>
+        <v>2.62</v>
       </c>
       <c r="L69" t="n">
-        <v>11.62</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>688117</t>
+          <t>600423</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>圣诺生物</t>
+          <t>柳化股份</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3613,13 +3613,13 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>38.95</v>
+        <v>2.95</v>
       </c>
       <c r="E70" t="n">
-        <v>38.19</v>
+        <v>2.87</v>
       </c>
       <c r="F70" t="n">
-        <v>37.02</v>
+        <v>2.69</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -3627,30 +3627,30 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>123</v>
+        <v>114.9</v>
       </c>
       <c r="I70" t="n">
-        <v>3.92</v>
+        <v>4.98</v>
       </c>
       <c r="J70" t="n">
-        <v>4.18</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="K70" t="n">
-        <v>3.86</v>
+        <v>1.56</v>
       </c>
       <c r="L70" t="n">
-        <v>2.54</v>
+        <v>2.07</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>002481</t>
+          <t>603079</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>双塔食品</t>
+          <t>圣达生物</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3659,44 +3659,44 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>4.6</v>
+        <v>17.16</v>
       </c>
       <c r="E71" t="n">
-        <v>4.54</v>
+        <v>17.22</v>
       </c>
       <c r="F71" t="n">
-        <v>4.42</v>
+        <v>16.17</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="H71" t="n">
-        <v>122.9</v>
+        <v>114.5</v>
       </c>
       <c r="I71" t="n">
-        <v>4.31</v>
+        <v>3.44</v>
       </c>
       <c r="J71" t="n">
-        <v>2.78</v>
+        <v>5.08</v>
       </c>
       <c r="K71" t="n">
-        <v>5.98</v>
+        <v>2.85</v>
       </c>
       <c r="L71" t="n">
-        <v>1.45</v>
+        <v>1.66</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>300505</t>
+          <t>001287</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>川金诺</t>
+          <t>中电港</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3705,13 +3705,13 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>25.78</v>
+        <v>27.63</v>
       </c>
       <c r="E72" t="n">
-        <v>25.9</v>
+        <v>27.29</v>
       </c>
       <c r="F72" t="n">
-        <v>24.81</v>
+        <v>26.29</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -3719,30 +3719,30 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>122.3</v>
+        <v>114.2</v>
       </c>
       <c r="I72" t="n">
-        <v>1.3</v>
+        <v>3.1</v>
       </c>
       <c r="J72" t="n">
-        <v>8.58</v>
+        <v>5.04</v>
       </c>
       <c r="K72" t="n">
-        <v>2.33</v>
+        <v>1.59</v>
       </c>
       <c r="L72" t="n">
-        <v>4.86</v>
+        <v>10.56</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>603936</t>
+          <t>300961</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>博敏电子</t>
+          <t>深水海纳</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3751,13 +3751,13 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>16.28</v>
+        <v>13.9</v>
       </c>
       <c r="E73" t="n">
-        <v>16.28</v>
+        <v>13.93</v>
       </c>
       <c r="F73" t="n">
-        <v>15.24</v>
+        <v>13.25</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -3765,30 +3765,30 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>122.2</v>
+        <v>114.1</v>
       </c>
       <c r="I73" t="n">
-        <v>1.5</v>
+        <v>0.58</v>
       </c>
       <c r="J73" t="n">
-        <v>7.01</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="K73" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="L73" t="n">
-        <v>7.15</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>603516</t>
+          <t>600763</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>淳中科技</t>
+          <t>通策医疗</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3797,13 +3797,13 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>147.3</v>
+        <v>43.23</v>
       </c>
       <c r="E74" t="n">
-        <v>148.95</v>
+        <v>43.36</v>
       </c>
       <c r="F74" t="n">
-        <v>141.13</v>
+        <v>41.26</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -3811,30 +3811,30 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>121.5</v>
+        <v>113.5</v>
       </c>
       <c r="I74" t="n">
-        <v>1.31</v>
+        <v>1.36</v>
       </c>
       <c r="J74" t="n">
-        <v>3.74</v>
+        <v>3.81</v>
       </c>
       <c r="K74" t="n">
-        <v>2.63</v>
+        <v>1.94</v>
       </c>
       <c r="L74" t="n">
-        <v>11.43</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>300867</t>
+          <t>300591</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>圣元环保</t>
+          <t>万里马</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3843,13 +3843,13 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>21.4</v>
+        <v>6.96</v>
       </c>
       <c r="E75" t="n">
-        <v>21.39</v>
+        <v>6.84</v>
       </c>
       <c r="F75" t="n">
-        <v>20.71</v>
+        <v>6.55</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -3857,30 +3857,30 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>121.4</v>
+        <v>113.5</v>
       </c>
       <c r="I75" t="n">
-        <v>1.86</v>
+        <v>3.88</v>
       </c>
       <c r="J75" t="n">
-        <v>6.67</v>
+        <v>6.45</v>
       </c>
       <c r="K75" t="n">
-        <v>2.89</v>
+        <v>2.31</v>
       </c>
       <c r="L75" t="n">
-        <v>2.76</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>688249</t>
+          <t>600333</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>晶合集成</t>
+          <t>长春燃气</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3889,13 +3889,13 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>30.33</v>
+        <v>5.56</v>
       </c>
       <c r="E76" t="n">
-        <v>30.24</v>
+        <v>5.46</v>
       </c>
       <c r="F76" t="n">
-        <v>27.78</v>
+        <v>5.33</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -3903,30 +3903,30 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>121.2</v>
+        <v>112.5</v>
       </c>
       <c r="I76" t="n">
-        <v>0.63</v>
+        <v>3.93</v>
       </c>
       <c r="J76" t="n">
-        <v>3.21</v>
+        <v>4.31</v>
       </c>
       <c r="K76" t="n">
-        <v>2.78</v>
+        <v>2.94</v>
       </c>
       <c r="L76" t="n">
-        <v>11.11</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>301128</t>
+          <t>300229</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>强瑞技术</t>
+          <t>拓尔思</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3935,13 +3935,13 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>190.83</v>
+        <v>18.34</v>
       </c>
       <c r="E77" t="n">
-        <v>185.83</v>
+        <v>18.45</v>
       </c>
       <c r="F77" t="n">
-        <v>173.46</v>
+        <v>17.25</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -3949,30 +3949,30 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>121.1</v>
+        <v>112</v>
       </c>
       <c r="I77" t="n">
-        <v>5.14</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J77" t="n">
-        <v>6.75</v>
+        <v>4.5</v>
       </c>
       <c r="K77" t="n">
-        <v>1.59</v>
+        <v>1.58</v>
       </c>
       <c r="L77" t="n">
-        <v>11.5</v>
+        <v>7.16</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>688312</t>
+          <t>600216</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>燕麦科技</t>
+          <t>浙江医药</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3981,13 +3981,13 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>68.90000000000001</v>
+        <v>14.81</v>
       </c>
       <c r="E78" t="n">
-        <v>69.68000000000001</v>
+        <v>14.85</v>
       </c>
       <c r="F78" t="n">
-        <v>65.34999999999999</v>
+        <v>14.49</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -3995,30 +3995,30 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>120.9</v>
+        <v>112</v>
       </c>
       <c r="I78" t="n">
-        <v>2.61</v>
+        <v>1.09</v>
       </c>
       <c r="J78" t="n">
-        <v>5.84</v>
+        <v>3.75</v>
       </c>
       <c r="K78" t="n">
-        <v>1.88</v>
+        <v>1.83</v>
       </c>
       <c r="L78" t="n">
-        <v>5.96</v>
+        <v>5.32</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>688401</t>
+          <t>301176</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>路维光电</t>
+          <t>逸豪新材</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -4027,13 +4027,13 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>65.61</v>
+        <v>29.34</v>
       </c>
       <c r="E79" t="n">
-        <v>64.91</v>
+        <v>29.92</v>
       </c>
       <c r="F79" t="n">
-        <v>61.05</v>
+        <v>28.54</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -4041,30 +4041,30 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>120.7</v>
+        <v>112</v>
       </c>
       <c r="I79" t="n">
-        <v>3.65</v>
+        <v>2.44</v>
       </c>
       <c r="J79" t="n">
-        <v>5.3</v>
+        <v>7.51</v>
       </c>
       <c r="K79" t="n">
-        <v>2.04</v>
+        <v>1.83</v>
       </c>
       <c r="L79" t="n">
-        <v>6.7</v>
+        <v>3.71</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>603127</t>
+          <t>002164</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>昭衍新药</t>
+          <t>宁波东力</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4073,13 +4073,13 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>38.15</v>
+        <v>13.15</v>
       </c>
       <c r="E80" t="n">
-        <v>37.93</v>
+        <v>12.85</v>
       </c>
       <c r="F80" t="n">
-        <v>36.11</v>
+        <v>12.25</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -4087,30 +4087,30 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>120.6</v>
+        <v>111.8</v>
       </c>
       <c r="I80" t="n">
-        <v>2.28</v>
+        <v>4.28</v>
       </c>
       <c r="J80" t="n">
-        <v>4.47</v>
+        <v>4.31</v>
       </c>
       <c r="K80" t="n">
-        <v>2.31</v>
+        <v>2.88</v>
       </c>
       <c r="L80" t="n">
-        <v>10.73</v>
+        <v>2.69</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>002430</t>
+          <t>603990</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>杭氧股份</t>
+          <t>麦迪科技</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4119,13 +4119,13 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>31.36</v>
+        <v>15.42</v>
       </c>
       <c r="E81" t="n">
-        <v>31.45</v>
+        <v>15.12</v>
       </c>
       <c r="F81" t="n">
-        <v>29.65</v>
+        <v>14.41</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -4133,30 +4133,30 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>120.4</v>
+        <v>110.9</v>
       </c>
       <c r="I81" t="n">
-        <v>2.82</v>
+        <v>3.98</v>
       </c>
       <c r="J81" t="n">
-        <v>3.39</v>
+        <v>7.12</v>
       </c>
       <c r="K81" t="n">
-        <v>2.65</v>
+        <v>1.87</v>
       </c>
       <c r="L81" t="n">
-        <v>10.57</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>002922</t>
+          <t>688117</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>伊戈尔</t>
+          <t>圣诺生物</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4165,13 +4165,13 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>42.41</v>
+        <v>38.68</v>
       </c>
       <c r="E82" t="n">
-        <v>41.9</v>
+        <v>38.19</v>
       </c>
       <c r="F82" t="n">
-        <v>40.06</v>
+        <v>37.02</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -4179,19 +4179,19 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>120.1</v>
+        <v>110.6</v>
       </c>
       <c r="I82" t="n">
-        <v>3.16</v>
+        <v>3.2</v>
       </c>
       <c r="J82" t="n">
-        <v>5.51</v>
+        <v>5.3</v>
       </c>
       <c r="K82" t="n">
-        <v>1.92</v>
+        <v>2.45</v>
       </c>
       <c r="L82" t="n">
-        <v>8.710000000000001</v>
+        <v>3.23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 实时报告更新 Fri Apr 24 13:56:58 UTC 2026
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>T:2026-04-24 21:47:35</t>
+          <t>T:2026-04-24 21:56:58</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -507,7 +507,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>0.9888782986371312</v>
+        <v>0.05297701934565868</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>

</xml_diff>

<commit_message>
📊 实时报告更新 Fri Apr 24 14:08:43 UTC 2026
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>T:2026-04-24 21:56:58</t>
+          <t>T:2026-04-24 22:08:43</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -507,7 +507,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>0.05297701934565868</v>
+        <v>0.6862660001424312</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>

</xml_diff>

<commit_message>
📊 实时报告更新 Mon Apr 27 02:32:32 UTC 2026
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -436,19 +436,19 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>原因</t>
+          <t>诊断信息</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>系统波动</t>
+          <t>逻辑崩溃</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>数据源超时，请尝试重新运行 Actions</t>
+          <t>接口连接失败</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 实时报告更新 Mon Apr 27 03:16:22 UTC 2026
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K82"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,30 +456,35 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>止损参考</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>能量状态</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>综合评分</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>涨幅%</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>换手%</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>量比</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>额(亿)</t>
         </is>
@@ -488,15 +493,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>V10.8-Triple</t>
+          <t>V11.2-Full</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>T:2026-04-27 10:46:55</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>S:备用新浪</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>T:2026-04-27 11:16:22</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
@@ -505,6 +514,7 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -523,30 +533,33 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>94.3</v>
+        <v>94.44</v>
       </c>
       <c r="E3" t="n">
         <v>93.76000000000001</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>52</v>
+      <c r="F3" t="n">
+        <v>88.06999999999999</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H3" t="n">
-        <v>1.354</v>
+        <v>52</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1.505</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>3.9</v>
+        <v>1</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4.3</v>
       </c>
     </row>
     <row r="4">
@@ -566,41 +579,44 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>57.98</v>
+        <v>58</v>
       </c>
       <c r="E4" t="n">
         <v>57.41</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>52</v>
+      <c r="F4" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H4" t="n">
-        <v>2.619</v>
+        <v>52</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>2.655</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0.97</v>
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1.07</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>bj920028</t>
+          <t>bj920045</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>新恒泰</t>
+          <t>蘅东光</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -609,30 +625,33 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>17.78</v>
+        <v>562.39</v>
       </c>
       <c r="E5" t="n">
-        <v>17.39</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>52</v>
+        <v>549.22</v>
+      </c>
+      <c r="F5" t="n">
+        <v>527.24</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H5" t="n">
-        <v>4.835</v>
+        <v>52</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>5.12</v>
       </c>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>1.04</v>
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>4.72</v>
       </c>
     </row>
     <row r="6">
@@ -652,30 +671,33 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>35.45</v>
+        <v>35.5</v>
       </c>
       <c r="E6" t="n">
         <v>35.26</v>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>52</v>
+      <c r="F6" t="n">
+        <v>33.64</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H6" t="n">
-        <v>1.78</v>
+        <v>52</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>1.924</v>
       </c>
       <c r="J6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>1.85</v>
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>2.09</v>
       </c>
     </row>
     <row r="7">
@@ -695,30 +717,33 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>52.14</v>
+        <v>51</v>
       </c>
       <c r="E7" t="n">
         <v>50.91</v>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>52</v>
+      <c r="F7" t="n">
+        <v>48.68</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H7" t="n">
-        <v>4.405</v>
+        <v>52</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>2.123</v>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>1.33</v>
+        <v>1</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1.61</v>
       </c>
     </row>
     <row r="8">
@@ -738,30 +763,33 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>82.56</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="E8" t="n">
         <v>81.79000000000001</v>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>52</v>
+      <c r="F8" t="n">
+        <v>76.94</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H8" t="n">
-        <v>2.674</v>
+        <v>52</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>2.164</v>
       </c>
       <c r="J8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>1.17</v>
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1.26</v>
       </c>
     </row>
     <row r="9">
@@ -781,41 +809,44 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>9.98</v>
+        <v>9.94</v>
       </c>
       <c r="E9" t="n">
         <v>10.04</v>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>52</v>
+      <c r="F9" t="n">
+        <v>9.470000000000001</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H9" t="n">
-        <v>1.423</v>
+        <v>52</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1.016</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>0.86</v>
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.92</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>sz301529</t>
+          <t>bj920438</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>福赛科技</t>
+          <t>戈碧迦</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -824,41 +855,44 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>122.22</v>
+        <v>43.3</v>
       </c>
       <c r="E10" t="n">
-        <v>121.77</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>52</v>
+        <v>43.63</v>
+      </c>
+      <c r="F10" t="n">
+        <v>41.73</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H10" t="n">
-        <v>3.183</v>
+        <v>52</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>1.05</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>2.46</v>
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>sz301479</t>
+          <t>bj920809</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>弘景光电</t>
+          <t>安达科技</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -867,41 +901,44 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>109.2</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="E11" t="n">
-        <v>109.06</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
-        <v>52</v>
+        <v>8.24</v>
+      </c>
+      <c r="F11" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H11" t="n">
-        <v>1.534</v>
+        <v>52</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>1.222</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>1.36</v>
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1.11</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>sz301458</t>
+          <t>sz301536</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>钧崴电子</t>
+          <t>星宸科技</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -910,41 +947,44 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>40.35</v>
+        <v>83.39</v>
       </c>
       <c r="E12" t="n">
-        <v>39.93</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>52</v>
+        <v>82.44</v>
+      </c>
+      <c r="F12" t="n">
+        <v>79.68000000000001</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H12" t="n">
-        <v>2.437</v>
+        <v>52</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>2.194</v>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>1.87</v>
+        <v>1</v>
+      </c>
+      <c r="L12" t="n">
+        <v>7.79</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>sz301421</t>
+          <t>sz301529</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>波长光电</t>
+          <t>福赛科技</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -953,41 +993,44 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>99.51000000000001</v>
+        <v>121.39</v>
       </c>
       <c r="E13" t="n">
-        <v>97.95999999999999</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>52</v>
+        <v>121.77</v>
+      </c>
+      <c r="F13" t="n">
+        <v>116.08</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H13" t="n">
-        <v>3.57</v>
+        <v>52</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>2.482</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>3.19</v>
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2.72</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>sz301408</t>
+          <t>sz301479</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>华人健康</t>
+          <t>弘景光电</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -996,41 +1039,44 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>19.97</v>
+        <v>109.43</v>
       </c>
       <c r="E14" t="n">
-        <v>20.16</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>52</v>
+        <v>109.06</v>
+      </c>
+      <c r="F14" t="n">
+        <v>105.64</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H14" t="n">
-        <v>0.859</v>
+        <v>52</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>1.748</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>2.85</v>
+        <v>1</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1.52</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>sz301395</t>
+          <t>sz301458</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>仁信新材</t>
+          <t>钧崴电子</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1039,41 +1085,44 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>12.93</v>
+        <v>40.2</v>
       </c>
       <c r="E15" t="n">
-        <v>12.93</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>52</v>
+        <v>39.93</v>
+      </c>
+      <c r="F15" t="n">
+        <v>38.67</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H15" t="n">
-        <v>1.174</v>
+        <v>52</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>2.056</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>1.04</v>
+        <v>1</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2.07</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>sz301393</t>
+          <t>sz301421</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>昊帆生物</t>
+          <t>波长光电</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1082,41 +1131,44 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>60.56</v>
+        <v>99.66</v>
       </c>
       <c r="E16" t="n">
-        <v>60.94</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>52</v>
+        <v>97.95999999999999</v>
+      </c>
+      <c r="F16" t="n">
+        <v>94.02</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H16" t="n">
-        <v>1.051</v>
+        <v>52</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>3.726</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>0.99</v>
+        <v>1</v>
+      </c>
+      <c r="L16" t="n">
+        <v>3.55</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>sz301392</t>
+          <t>sz301419</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>汇成真空</t>
+          <t>阿莱德</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1125,41 +1177,44 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>162.5</v>
+        <v>41.95</v>
       </c>
       <c r="E17" t="n">
-        <v>162.53</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>52</v>
+        <v>41.95</v>
+      </c>
+      <c r="F17" t="n">
+        <v>40.48</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H17" t="n">
-        <v>0.925</v>
+        <v>52</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>3.27</v>
+        <v>1</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.93</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>sz301391</t>
+          <t>sz301408</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>卡莱特</t>
+          <t>华人健康</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1168,41 +1223,44 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>80.90000000000001</v>
+        <v>20.19</v>
       </c>
       <c r="E18" t="n">
-        <v>79.29000000000001</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>52</v>
+        <v>20.16</v>
+      </c>
+      <c r="F18" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H18" t="n">
-        <v>4.657</v>
+        <v>52</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>1.97</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>1.88</v>
+        <v>1</v>
+      </c>
+      <c r="L18" t="n">
+        <v>3.18</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>sz301382</t>
+          <t>sz301395</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>蜂助手</t>
+          <t>仁信新材</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1211,41 +1269,44 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>40.51</v>
+        <v>12.98</v>
       </c>
       <c r="E19" t="n">
-        <v>40.63</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>52</v>
+        <v>12.93</v>
+      </c>
+      <c r="F19" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H19" t="n">
-        <v>0.922</v>
+        <v>52</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>1.565</v>
       </c>
       <c r="J19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>3.26</v>
+        <v>1</v>
+      </c>
+      <c r="L19" t="n">
+        <v>1.09</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>sz301378</t>
+          <t>sz301393</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>通达海</t>
+          <t>昊帆生物</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1254,41 +1315,44 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>31.89</v>
+        <v>61.01</v>
       </c>
       <c r="E20" t="n">
-        <v>32.33</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
-        <v>52</v>
+        <v>60.94</v>
+      </c>
+      <c r="F20" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H20" t="n">
-        <v>1.82</v>
+        <v>52</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>1.802</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>1.35</v>
+        <v>1</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1.12</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>sz301371</t>
+          <t>sz301392</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>敷尔佳</t>
+          <t>汇成真空</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1297,41 +1361,44 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>29.14</v>
+        <v>162.35</v>
       </c>
       <c r="E21" t="n">
-        <v>28.54</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>52</v>
+        <v>162.53</v>
+      </c>
+      <c r="F21" t="n">
+        <v>155.15</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H21" t="n">
-        <v>4.183</v>
+        <v>52</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>0.832</v>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>2.01</v>
+        <v>1</v>
+      </c>
+      <c r="L21" t="n">
+        <v>3.74</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>sz301369</t>
+          <t>sz301382</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>联动科技</t>
+          <t>蜂助手</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1340,41 +1407,44 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>168.42</v>
+        <v>40.88</v>
       </c>
       <c r="E22" t="n">
-        <v>167.98</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G22" t="n">
-        <v>52</v>
+        <v>40.65</v>
+      </c>
+      <c r="F22" t="n">
+        <v>38.22</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H22" t="n">
-        <v>1.391</v>
+        <v>52</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>1.844</v>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K22" t="n">
-        <v>1.07</v>
+        <v>1</v>
+      </c>
+      <c r="L22" t="n">
+        <v>4.04</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>sz301365</t>
+          <t>sz301378</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>矩阵股份</t>
+          <t>通达海</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1383,41 +1453,44 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>34.11</v>
+        <v>31.68</v>
       </c>
       <c r="E23" t="n">
-        <v>33.97</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G23" t="n">
-        <v>52</v>
+        <v>32.33</v>
+      </c>
+      <c r="F23" t="n">
+        <v>30.85</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H23" t="n">
-        <v>2.279</v>
+        <v>52</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>1.149</v>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>1.11</v>
+        <v>1</v>
+      </c>
+      <c r="L23" t="n">
+        <v>1.49</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>sz301362</t>
+          <t>sz301371</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>民爆光电</t>
+          <t>敷尔佳</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1426,41 +1499,44 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>143.3</v>
+        <v>29.1</v>
       </c>
       <c r="E24" t="n">
-        <v>142.84</v>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
-        <v>52</v>
+        <v>28.54</v>
+      </c>
+      <c r="F24" t="n">
+        <v>27.41</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H24" t="n">
-        <v>1.179</v>
+        <v>52</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>4.04</v>
       </c>
       <c r="J24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>1.7</v>
+        <v>1</v>
+      </c>
+      <c r="L24" t="n">
+        <v>2.19</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>sz301349</t>
+          <t>sz301369</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>信德新材</t>
+          <t>联动科技</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1469,41 +1545,44 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>60.41</v>
+        <v>168.88</v>
       </c>
       <c r="E25" t="n">
-        <v>60.36</v>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G25" t="n">
-        <v>52</v>
+        <v>167.98</v>
+      </c>
+      <c r="F25" t="n">
+        <v>163.06</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H25" t="n">
-        <v>0.902</v>
+        <v>52</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>1.668</v>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>1.57</v>
+        <v>1</v>
+      </c>
+      <c r="L25" t="n">
+        <v>1.27</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sh600299</t>
+          <t>sz301365</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>安迪苏</t>
+          <t>矩阵股份</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1512,41 +1591,44 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>14.27</v>
+        <v>34.8</v>
       </c>
       <c r="E26" t="n">
-        <v>14.14</v>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G26" t="n">
-        <v>52</v>
+        <v>33.97</v>
+      </c>
+      <c r="F26" t="n">
+        <v>32.01</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H26" t="n">
-        <v>2.514</v>
+        <v>52</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>4.348</v>
       </c>
       <c r="J26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>1.22</v>
+        <v>1</v>
+      </c>
+      <c r="L26" t="n">
+        <v>1.24</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>sh600292</t>
+          <t>sz301362</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>电投水电</t>
+          <t>民爆光电</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1555,41 +1637,44 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>16.03</v>
+        <v>143.58</v>
       </c>
       <c r="E27" t="n">
-        <v>16.01</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G27" t="n">
-        <v>52</v>
+        <v>142.84</v>
+      </c>
+      <c r="F27" t="n">
+        <v>137.2</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H27" t="n">
-        <v>0.628</v>
+        <v>52</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>1.377</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>1.18</v>
+        <v>1</v>
+      </c>
+      <c r="L27" t="n">
+        <v>1.9</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>sh600256</t>
+          <t>sh600312</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>广汇能源</t>
+          <t>平高电气</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1598,41 +1683,44 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>6.22</v>
+        <v>22.17</v>
       </c>
       <c r="E28" t="n">
-        <v>6.13</v>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G28" t="n">
-        <v>52</v>
+        <v>22.09</v>
+      </c>
+      <c r="F28" t="n">
+        <v>21.23</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H28" t="n">
-        <v>3.667</v>
+        <v>52</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>1.325</v>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>11.66</v>
+        <v>1</v>
+      </c>
+      <c r="L28" t="n">
+        <v>3.74</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>sh600234</t>
+          <t>sh600310</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>科新发展</t>
+          <t>广西能源</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1641,41 +1729,44 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>24.02</v>
+        <v>5.34</v>
       </c>
       <c r="E29" t="n">
-        <v>23.45</v>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G29" t="n">
-        <v>52</v>
+        <v>5.19</v>
+      </c>
+      <c r="F29" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H29" t="n">
-        <v>5.12</v>
+        <v>52</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>4.912</v>
       </c>
       <c r="J29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>1.62</v>
+        <v>1</v>
+      </c>
+      <c r="L29" t="n">
+        <v>7.21</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>sh600233</t>
+          <t>sh600299</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>圆通速递</t>
+          <t>安迪苏</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1684,41 +1775,44 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>22.39</v>
+        <v>14.26</v>
       </c>
       <c r="E30" t="n">
-        <v>22.26</v>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G30" t="n">
-        <v>52</v>
+        <v>14.14</v>
+      </c>
+      <c r="F30" t="n">
+        <v>13.47</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H30" t="n">
-        <v>2.098</v>
+        <v>52</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>2.443</v>
       </c>
       <c r="J30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>3.43</v>
+        <v>1</v>
+      </c>
+      <c r="L30" t="n">
+        <v>1.33</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>sh600226</t>
+          <t>sh600292</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>亨通股份</t>
+          <t>电投水电</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1727,41 +1821,44 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>5.36</v>
+        <v>16.05</v>
       </c>
       <c r="E31" t="n">
-        <v>5.28</v>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G31" t="n">
-        <v>52</v>
+        <v>16.01</v>
+      </c>
+      <c r="F31" t="n">
+        <v>15.29</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H31" t="n">
-        <v>2.879</v>
+        <v>52</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>0.753</v>
       </c>
       <c r="J31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>1.92</v>
+        <v>1</v>
+      </c>
+      <c r="L31" t="n">
+        <v>1.44</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>sh600203</t>
+          <t>sh600267</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>福日电子</t>
+          <t>海正药业</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1770,41 +1867,44 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>12.51</v>
+        <v>11.46</v>
       </c>
       <c r="E32" t="n">
-        <v>12.24</v>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G32" t="n">
-        <v>52</v>
+        <v>11.42</v>
+      </c>
+      <c r="F32" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H32" t="n">
-        <v>4.077</v>
+        <v>52</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>0.792</v>
       </c>
       <c r="J32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>2.98</v>
+        <v>1</v>
+      </c>
+      <c r="L32" t="n">
+        <v>2.15</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>sh600188</t>
+          <t>sh600255</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>兖矿能源</t>
+          <t>鑫科材料</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1813,41 +1913,44 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>20.96</v>
+        <v>3.65</v>
       </c>
       <c r="E33" t="n">
-        <v>20.91</v>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G33" t="n">
-        <v>52</v>
+        <v>3.62</v>
+      </c>
+      <c r="F33" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H33" t="n">
-        <v>1.354</v>
+        <v>52</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>1.389</v>
       </c>
       <c r="J33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>5.48</v>
+        <v>1</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0.8</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>sh600172</t>
+          <t>sh600233</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>黄河旋风</t>
+          <t>圆通速递</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1856,41 +1959,44 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>8.449999999999999</v>
+        <v>22.48</v>
       </c>
       <c r="E34" t="n">
-        <v>8.41</v>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G34" t="n">
-        <v>52</v>
+        <v>22.26</v>
+      </c>
+      <c r="F34" t="n">
+        <v>21.45</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H34" t="n">
-        <v>1.807</v>
+        <v>52</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>2.508</v>
       </c>
       <c r="J34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>3.73</v>
+        <v>1</v>
+      </c>
+      <c r="L34" t="n">
+        <v>3.96</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>sh600171</t>
+          <t>sh600226</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>上海贝岭</t>
+          <t>亨通股份</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1899,41 +2005,44 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>29.34</v>
+        <v>5.44</v>
       </c>
       <c r="E35" t="n">
-        <v>28.91</v>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G35" t="n">
-        <v>52</v>
+        <v>5.3</v>
+      </c>
+      <c r="F35" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H35" t="n">
-        <v>3.165</v>
+        <v>52</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>4.415</v>
       </c>
       <c r="J35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>4.84</v>
+        <v>1</v>
+      </c>
+      <c r="L35" t="n">
+        <v>2.55</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>sh600160</t>
+          <t>sh600203</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>巨化股份</t>
+          <t>福日电子</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1942,41 +2051,44 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>35.75</v>
+        <v>12.52</v>
       </c>
       <c r="E36" t="n">
-        <v>35.46</v>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G36" t="n">
-        <v>52</v>
+        <v>12.24</v>
+      </c>
+      <c r="F36" t="n">
+        <v>11.58</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H36" t="n">
-        <v>1.997</v>
+        <v>52</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>4.16</v>
       </c>
       <c r="J36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>8.890000000000001</v>
+        <v>1</v>
+      </c>
+      <c r="L36" t="n">
+        <v>3.36</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>sh600158</t>
+          <t>sh600198</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>中体产业</t>
+          <t>大唐电信</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1985,41 +2097,44 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>10.67</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="E37" t="n">
-        <v>10.62</v>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G37" t="n">
-        <v>52</v>
+        <v>8.18</v>
+      </c>
+      <c r="F37" t="n">
+        <v>7.82</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H37" t="n">
-        <v>1.91</v>
+        <v>52</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>0.736</v>
       </c>
       <c r="J37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>4.79</v>
+        <v>1</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0.82</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>sh600157</t>
+          <t>sh600188</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>永泰能源</t>
+          <t>兖矿能源</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2028,41 +2143,44 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1.74</v>
+        <v>20.99</v>
       </c>
       <c r="E38" t="n">
-        <v>1.71</v>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G38" t="n">
-        <v>52</v>
+        <v>20.91</v>
+      </c>
+      <c r="F38" t="n">
+        <v>19.97</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H38" t="n">
-        <v>3.571</v>
+        <v>52</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>1.499</v>
       </c>
       <c r="J38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>9.619999999999999</v>
+        <v>1</v>
+      </c>
+      <c r="L38" t="n">
+        <v>6.13</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>sh600156</t>
+          <t>sh600185</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>华升股份</t>
+          <t>珠免集团</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2071,41 +2189,44 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>9.199999999999999</v>
+        <v>6.01</v>
       </c>
       <c r="E39" t="n">
-        <v>9.279999999999999</v>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G39" t="n">
-        <v>52</v>
+        <v>5.96</v>
+      </c>
+      <c r="F39" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H39" t="n">
-        <v>0.877</v>
+        <v>52</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>1.52</v>
       </c>
       <c r="J39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>3.42</v>
+        <v>1</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0.89</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>sh600148</t>
+          <t>sh600177</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>长春一东</t>
+          <t>雅戈尔</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2114,41 +2235,44 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>18.81</v>
+        <v>7.63</v>
       </c>
       <c r="E40" t="n">
-        <v>18.54</v>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G40" t="n">
-        <v>52</v>
+        <v>7.61</v>
+      </c>
+      <c r="F40" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H40" t="n">
-        <v>5.143</v>
+        <v>52</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>0.66</v>
       </c>
       <c r="J40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K40" t="n">
-        <v>0.9399999999999999</v>
+        <v>1</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0.89</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>sh600143</t>
+          <t>sh600172</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>金发科技</t>
+          <t>黄河旋风</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2157,41 +2281,44 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>16.99</v>
+        <v>8.41</v>
       </c>
       <c r="E41" t="n">
-        <v>16.84</v>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G41" t="n">
-        <v>52</v>
+        <v>8.41</v>
+      </c>
+      <c r="F41" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H41" t="n">
-        <v>1.676</v>
+        <v>52</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>1.325</v>
       </c>
       <c r="J41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K41" t="n">
-        <v>4.02</v>
+        <v>1</v>
+      </c>
+      <c r="L41" t="n">
+        <v>4.05</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>sh600501</t>
+          <t>sh600171</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>航天晨光</t>
+          <t>上海贝岭</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2200,41 +2327,44 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>23.24</v>
+        <v>29.33</v>
       </c>
       <c r="E42" t="n">
-        <v>23.22</v>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>52</v>
+        <v>28.91</v>
+      </c>
+      <c r="F42" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H42" t="n">
-        <v>1.796</v>
+        <v>52</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>3.129</v>
       </c>
       <c r="J42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K42" t="n">
-        <v>1.27</v>
+        <v>1</v>
+      </c>
+      <c r="L42" t="n">
+        <v>5.22</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>sh600499</t>
+          <t>sh600160</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>科达制造</t>
+          <t>巨化股份</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2243,41 +2373,44 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>20.21</v>
+        <v>35.99</v>
       </c>
       <c r="E43" t="n">
-        <v>20.18</v>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G43" t="n">
-        <v>52</v>
+        <v>35.49</v>
+      </c>
+      <c r="F43" t="n">
+        <v>34.21</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H43" t="n">
-        <v>2.019</v>
+        <v>52</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>2.682</v>
       </c>
       <c r="J43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K43" t="n">
-        <v>8.34</v>
+        <v>1</v>
+      </c>
+      <c r="L43" t="n">
+        <v>11.16</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>sh600489</t>
+          <t>sh600483</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>中金黄金</t>
+          <t>福能股份</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2286,30 +2419,33 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>25.75</v>
+        <v>9.98</v>
       </c>
       <c r="E44" t="n">
-        <v>25.66</v>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G44" t="n">
-        <v>52</v>
+        <v>9.91</v>
+      </c>
+      <c r="F44" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H44" t="n">
-        <v>0.862</v>
+        <v>52</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>1.217</v>
       </c>
       <c r="J44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>6.1</v>
+        <v>1</v>
+      </c>
+      <c r="L44" t="n">
+        <v>1.14</v>
       </c>
     </row>
     <row r="45">
@@ -2329,30 +2465,33 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>28.25</v>
+        <v>28.17</v>
       </c>
       <c r="E45" t="n">
         <v>28.04</v>
       </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G45" t="n">
-        <v>52</v>
+      <c r="F45" t="n">
+        <v>27.15</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H45" t="n">
-        <v>1.546</v>
+        <v>52</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>1.258</v>
       </c>
       <c r="J45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K45" t="n">
-        <v>6.58</v>
+        <v>1</v>
+      </c>
+      <c r="L45" t="n">
+        <v>7.36</v>
       </c>
     </row>
     <row r="46">
@@ -2372,41 +2511,44 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>13.55</v>
+        <v>13.68</v>
       </c>
       <c r="E46" t="n">
         <v>13.5</v>
       </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G46" t="n">
-        <v>52</v>
+      <c r="F46" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H46" t="n">
-        <v>1.65</v>
+        <v>52</v>
       </c>
       <c r="I46" t="n">
-        <v>0</v>
+        <v>2.626</v>
       </c>
       <c r="J46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K46" t="n">
-        <v>2.37</v>
+        <v>1</v>
+      </c>
+      <c r="L46" t="n">
+        <v>2.66</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>sh600415</t>
+          <t>sh600429</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>小商品城</t>
+          <t>三元股份</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2415,41 +2557,44 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>13.64</v>
+        <v>6.15</v>
       </c>
       <c r="E47" t="n">
-        <v>13.44</v>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G47" t="n">
-        <v>52</v>
+        <v>6.11</v>
+      </c>
+      <c r="F47" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H47" t="n">
-        <v>2.943</v>
+        <v>52</v>
       </c>
       <c r="I47" t="n">
-        <v>0</v>
+        <v>2.329</v>
       </c>
       <c r="J47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K47" t="n">
-        <v>11.83</v>
+        <v>1</v>
+      </c>
+      <c r="L47" t="n">
+        <v>2.58</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>sh600366</t>
+          <t>sh600426</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>宁波韵升</t>
+          <t>华鲁恒升</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2458,41 +2603,44 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>13.08</v>
+        <v>38.04</v>
       </c>
       <c r="E48" t="n">
-        <v>12.92</v>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G48" t="n">
-        <v>52</v>
+        <v>37.83</v>
+      </c>
+      <c r="F48" t="n">
+        <v>36.31</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H48" t="n">
-        <v>2.267</v>
+        <v>52</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
+        <v>1.116</v>
       </c>
       <c r="J48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K48" t="n">
-        <v>2.01</v>
+        <v>1</v>
+      </c>
+      <c r="L48" t="n">
+        <v>5.22</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>sh600363</t>
+          <t>sh600395</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>联创光电</t>
+          <t>盘江股份</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2501,41 +2649,44 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>53.46</v>
+        <v>5.75</v>
       </c>
       <c r="E49" t="n">
-        <v>52.56</v>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G49" t="n">
-        <v>52</v>
+        <v>5.74</v>
+      </c>
+      <c r="F49" t="n">
+        <v>5.54</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H49" t="n">
-        <v>2.827</v>
+        <v>52</v>
       </c>
       <c r="I49" t="n">
-        <v>0</v>
+        <v>0.524</v>
       </c>
       <c r="J49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K49" t="n">
-        <v>2.09</v>
+        <v>1</v>
+      </c>
+      <c r="L49" t="n">
+        <v>1.13</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>sh600361</t>
+          <t>sh600378</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>创新新材</t>
+          <t>昊华科技</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2544,41 +2695,44 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>4.66</v>
+        <v>35.61</v>
       </c>
       <c r="E50" t="n">
-        <v>4.58</v>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G50" t="n">
-        <v>52</v>
+        <v>35.52</v>
+      </c>
+      <c r="F50" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H50" t="n">
-        <v>3.786</v>
+        <v>52</v>
       </c>
       <c r="I50" t="n">
-        <v>0</v>
+        <v>1.021</v>
       </c>
       <c r="J50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K50" t="n">
-        <v>2.11</v>
+        <v>1</v>
+      </c>
+      <c r="L50" t="n">
+        <v>3.58</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>sh600351</t>
+          <t>sh600366</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>亚宝药业</t>
+          <t>宁波韵升</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2587,41 +2741,44 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>6.71</v>
+        <v>13.08</v>
       </c>
       <c r="E51" t="n">
-        <v>6.55</v>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G51" t="n">
-        <v>52</v>
+        <v>12.92</v>
+      </c>
+      <c r="F51" t="n">
+        <v>12.55</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H51" t="n">
-        <v>4.517</v>
+        <v>52</v>
       </c>
       <c r="I51" t="n">
-        <v>0</v>
+        <v>2.267</v>
       </c>
       <c r="J51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K51" t="n">
-        <v>1.58</v>
+        <v>1</v>
+      </c>
+      <c r="L51" t="n">
+        <v>2.33</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>sh600345</t>
+          <t>sh600363</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>长江通信</t>
+          <t>联创光电</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2630,41 +2787,44 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>52.8</v>
+        <v>53.13</v>
       </c>
       <c r="E52" t="n">
-        <v>51.57</v>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G52" t="n">
-        <v>52</v>
+        <v>52.59</v>
+      </c>
+      <c r="F52" t="n">
+        <v>50.66</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H52" t="n">
-        <v>4.762</v>
+        <v>52</v>
       </c>
       <c r="I52" t="n">
-        <v>0</v>
+        <v>2.193</v>
       </c>
       <c r="J52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K52" t="n">
-        <v>4.6</v>
+        <v>1</v>
+      </c>
+      <c r="L52" t="n">
+        <v>2.4</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>sh600333</t>
+          <t>sh600362</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>长春燃气</t>
+          <t>江西铜业</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2673,41 +2833,44 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>5.73</v>
+        <v>45.1</v>
       </c>
       <c r="E53" t="n">
-        <v>5.68</v>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G53" t="n">
-        <v>52</v>
+        <v>44.96</v>
+      </c>
+      <c r="F53" t="n">
+        <v>43.71</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H53" t="n">
-        <v>3.058</v>
+        <v>52</v>
       </c>
       <c r="I53" t="n">
-        <v>0</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="J53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K53" t="n">
-        <v>0.87</v>
+        <v>1</v>
+      </c>
+      <c r="L53" t="n">
+        <v>7.36</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>sh600331</t>
+          <t>sh600361</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>宏达股份</t>
+          <t>创新新材</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2716,41 +2879,44 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>18.55</v>
+        <v>4.65</v>
       </c>
       <c r="E54" t="n">
-        <v>18.4</v>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G54" t="n">
-        <v>52</v>
+        <v>4.58</v>
+      </c>
+      <c r="F54" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H54" t="n">
-        <v>1.7</v>
+        <v>52</v>
       </c>
       <c r="I54" t="n">
-        <v>0</v>
+        <v>3.563</v>
       </c>
       <c r="J54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K54" t="n">
-        <v>6.12</v>
+        <v>1</v>
+      </c>
+      <c r="L54" t="n">
+        <v>2.57</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>sh600323</t>
+          <t>sh600351</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>瀚蓝环境</t>
+          <t>亚宝药业</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2759,41 +2925,44 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>31.16</v>
+        <v>6.75</v>
       </c>
       <c r="E55" t="n">
-        <v>30.86</v>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G55" t="n">
-        <v>52</v>
+        <v>6.6</v>
+      </c>
+      <c r="F55" t="n">
+        <v>6.35</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H55" t="n">
-        <v>3.213</v>
+        <v>52</v>
       </c>
       <c r="I55" t="n">
-        <v>0</v>
+        <v>5.14</v>
       </c>
       <c r="J55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K55" t="n">
-        <v>2.27</v>
+        <v>1</v>
+      </c>
+      <c r="L55" t="n">
+        <v>2.08</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>sh600312</t>
+          <t>sh600345</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>平高电气</t>
+          <t>长江通信</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2802,41 +2971,44 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>22.15</v>
+        <v>52.62</v>
       </c>
       <c r="E56" t="n">
-        <v>22.09</v>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G56" t="n">
-        <v>52</v>
+        <v>51.57</v>
+      </c>
+      <c r="F56" t="n">
+        <v>49.54</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H56" t="n">
-        <v>1.234</v>
+        <v>52</v>
       </c>
       <c r="I56" t="n">
-        <v>0</v>
+        <v>4.405</v>
       </c>
       <c r="J56" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K56" t="n">
-        <v>3.3</v>
+        <v>1</v>
+      </c>
+      <c r="L56" t="n">
+        <v>5.21</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>sh600310</t>
+          <t>sh600333</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>广西能源</t>
+          <t>长春燃气</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2845,41 +3017,44 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>5.25</v>
+        <v>5.73</v>
       </c>
       <c r="E57" t="n">
-        <v>5.15</v>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G57" t="n">
-        <v>52</v>
+        <v>5.68</v>
+      </c>
+      <c r="F57" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H57" t="n">
-        <v>3.143</v>
+        <v>52</v>
       </c>
       <c r="I57" t="n">
-        <v>0</v>
+        <v>3.058</v>
       </c>
       <c r="J57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K57" t="n">
-        <v>6.1</v>
+        <v>1</v>
+      </c>
+      <c r="L57" t="n">
+        <v>0.95</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>sh600629</t>
+          <t>sh600331</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>华建集团</t>
+          <t>宏达股份</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2888,41 +3063,44 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>20.46</v>
+        <v>18.72</v>
       </c>
       <c r="E58" t="n">
-        <v>20.26</v>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G58" t="n">
-        <v>52</v>
+        <v>18.44</v>
+      </c>
+      <c r="F58" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H58" t="n">
-        <v>2.505</v>
+        <v>52</v>
       </c>
       <c r="I58" t="n">
-        <v>0</v>
+        <v>2.632</v>
       </c>
       <c r="J58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K58" t="n">
-        <v>2.48</v>
+        <v>1</v>
+      </c>
+      <c r="L58" t="n">
+        <v>7.08</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>sh600617</t>
+          <t>sh600323</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>国新能源</t>
+          <t>瀚蓝环境</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2931,41 +3109,44 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>3.36</v>
+        <v>30.99</v>
       </c>
       <c r="E59" t="n">
-        <v>3.35</v>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G59" t="n">
-        <v>52</v>
+        <v>30.86</v>
+      </c>
+      <c r="F59" t="n">
+        <v>29.14</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H59" t="n">
-        <v>1.205</v>
+        <v>52</v>
       </c>
       <c r="I59" t="n">
-        <v>0</v>
+        <v>2.65</v>
       </c>
       <c r="J59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K59" t="n">
-        <v>0.96</v>
+        <v>1</v>
+      </c>
+      <c r="L59" t="n">
+        <v>2.5</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>sh600605</t>
+          <t>sh600600</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>汇通能源</t>
+          <t>青岛啤酒</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2974,41 +3155,44 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>32.8</v>
+        <v>62.05</v>
       </c>
       <c r="E60" t="n">
-        <v>32.73</v>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G60" t="n">
-        <v>52</v>
+        <v>61.88</v>
+      </c>
+      <c r="F60" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H60" t="n">
-        <v>3.08</v>
+        <v>52</v>
       </c>
       <c r="I60" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="J60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K60" t="n">
-        <v>1.78</v>
+        <v>1</v>
+      </c>
+      <c r="L60" t="n">
+        <v>1.48</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>sh600603</t>
+          <t>sh600580</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>广汇物流</t>
+          <t>卧龙电驱</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3017,41 +3201,44 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>6.12</v>
+        <v>38.07</v>
       </c>
       <c r="E61" t="n">
-        <v>6.11</v>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G61" t="n">
-        <v>52</v>
+        <v>37.96</v>
+      </c>
+      <c r="F61" t="n">
+        <v>36.68</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H61" t="n">
-        <v>0.658</v>
+        <v>52</v>
       </c>
       <c r="I61" t="n">
-        <v>0</v>
+        <v>0.981</v>
       </c>
       <c r="J61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K61" t="n">
-        <v>1.03</v>
+        <v>1</v>
+      </c>
+      <c r="L61" t="n">
+        <v>5.71</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>sh600602</t>
+          <t>sh600575</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>云赛智联</t>
+          <t>淮河能源</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3060,41 +3247,44 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>22.61</v>
+        <v>3.84</v>
       </c>
       <c r="E62" t="n">
-        <v>22.4</v>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G62" t="n">
-        <v>52</v>
+        <v>3.74</v>
+      </c>
+      <c r="F62" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H62" t="n">
-        <v>1.755</v>
+        <v>52</v>
       </c>
       <c r="I62" t="n">
-        <v>0</v>
+        <v>4.632</v>
       </c>
       <c r="J62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K62" t="n">
-        <v>6.65</v>
+        <v>1</v>
+      </c>
+      <c r="L62" t="n">
+        <v>2.81</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>sh600580</t>
+          <t>sh600573</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>卧龙电驱</t>
+          <t>惠泉啤酒</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3103,41 +3293,44 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>38.11</v>
+        <v>13.3</v>
       </c>
       <c r="E63" t="n">
-        <v>37.96</v>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G63" t="n">
-        <v>52</v>
+        <v>13.15</v>
+      </c>
+      <c r="F63" t="n">
+        <v>12.66</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H63" t="n">
-        <v>1.088</v>
+        <v>52</v>
       </c>
       <c r="I63" t="n">
-        <v>0</v>
+        <v>3.583</v>
       </c>
       <c r="J63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K63" t="n">
-        <v>4.94</v>
+        <v>1</v>
+      </c>
+      <c r="L63" t="n">
+        <v>1.37</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>sh600575</t>
+          <t>sh600570</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>淮河能源</t>
+          <t>恒生电子</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3146,41 +3339,44 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>3.81</v>
+        <v>26.49</v>
       </c>
       <c r="E64" t="n">
-        <v>3.73</v>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G64" t="n">
-        <v>52</v>
+        <v>26.35</v>
+      </c>
+      <c r="F64" t="n">
+        <v>25.55</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H64" t="n">
-        <v>3.815</v>
+        <v>52</v>
       </c>
       <c r="I64" t="n">
-        <v>0</v>
+        <v>1.107</v>
       </c>
       <c r="J64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K64" t="n">
-        <v>2.37</v>
+        <v>1</v>
+      </c>
+      <c r="L64" t="n">
+        <v>3.09</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>sh600573</t>
+          <t>sh600550</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>惠泉啤酒</t>
+          <t>保变电气</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3189,41 +3385,44 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>13.16</v>
+        <v>15.33</v>
       </c>
       <c r="E65" t="n">
-        <v>13.15</v>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G65" t="n">
-        <v>52</v>
+        <v>15.17</v>
+      </c>
+      <c r="F65" t="n">
+        <v>14.48</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H65" t="n">
-        <v>2.492</v>
+        <v>52</v>
       </c>
       <c r="I65" t="n">
-        <v>0</v>
+        <v>2.064</v>
       </c>
       <c r="J65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K65" t="n">
-        <v>1.25</v>
+        <v>1</v>
+      </c>
+      <c r="L65" t="n">
+        <v>4.64</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>sh600570</t>
+          <t>sh600546</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>恒生电子</t>
+          <t>山煤国际</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3232,41 +3431,44 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>26.4</v>
+        <v>12.9</v>
       </c>
       <c r="E66" t="n">
-        <v>26.35</v>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G66" t="n">
-        <v>52</v>
+        <v>12.73</v>
+      </c>
+      <c r="F66" t="n">
+        <v>12.32</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H66" t="n">
-        <v>0.763</v>
+        <v>52</v>
       </c>
       <c r="I66" t="n">
-        <v>0</v>
+        <v>2.625</v>
       </c>
       <c r="J66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K66" t="n">
-        <v>2.65</v>
+        <v>1</v>
+      </c>
+      <c r="L66" t="n">
+        <v>2.41</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>sh600552</t>
+          <t>sh600545</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>凯盛科技</t>
+          <t>卓郎智能</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3275,41 +3477,44 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>15.77</v>
+        <v>4.89</v>
       </c>
       <c r="E67" t="n">
-        <v>15.42</v>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G67" t="n">
-        <v>52</v>
+        <v>4.82</v>
+      </c>
+      <c r="F67" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H67" t="n">
-        <v>4.576</v>
+        <v>52</v>
       </c>
       <c r="I67" t="n">
-        <v>0</v>
+        <v>3.165</v>
       </c>
       <c r="J67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K67" t="n">
-        <v>6.19</v>
+        <v>1</v>
+      </c>
+      <c r="L67" t="n">
+        <v>7.25</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>sh600546</t>
+          <t>sh600535</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>山煤国际</t>
+          <t>天士力</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3318,41 +3523,44 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>12.84</v>
+        <v>14.99</v>
       </c>
       <c r="E68" t="n">
-        <v>12.73</v>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G68" t="n">
-        <v>52</v>
+        <v>14.94</v>
+      </c>
+      <c r="F68" t="n">
+        <v>14.68</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H68" t="n">
-        <v>2.148</v>
+        <v>52</v>
       </c>
       <c r="I68" t="n">
-        <v>0</v>
+        <v>2.531</v>
       </c>
       <c r="J68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K68" t="n">
-        <v>2.04</v>
+        <v>1</v>
+      </c>
+      <c r="L68" t="n">
+        <v>4.19</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>sh600545</t>
+          <t>sh600531</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>卓郎智能</t>
+          <t>豫光金铅</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3361,41 +3569,44 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>4.92</v>
+        <v>16.06</v>
       </c>
       <c r="E69" t="n">
-        <v>4.82</v>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G69" t="n">
-        <v>52</v>
+        <v>15.79</v>
+      </c>
+      <c r="F69" t="n">
+        <v>15.07</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H69" t="n">
-        <v>3.797</v>
+        <v>52</v>
       </c>
       <c r="I69" t="n">
-        <v>0</v>
+        <v>3.213</v>
       </c>
       <c r="J69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K69" t="n">
-        <v>6.85</v>
+        <v>1</v>
+      </c>
+      <c r="L69" t="n">
+        <v>7.35</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>sh600539</t>
+          <t>sh600515</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>狮头股份</t>
+          <t>海南机场</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3404,41 +3615,44 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>17.7</v>
+        <v>3.43</v>
       </c>
       <c r="E70" t="n">
-        <v>17.41</v>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G70" t="n">
-        <v>52</v>
+        <v>3.42</v>
+      </c>
+      <c r="F70" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H70" t="n">
-        <v>4.92</v>
+        <v>52</v>
       </c>
       <c r="I70" t="n">
-        <v>0</v>
+        <v>0.587</v>
       </c>
       <c r="J70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K70" t="n">
-        <v>2.63</v>
+        <v>1</v>
+      </c>
+      <c r="L70" t="n">
+        <v>1.31</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>sh600535</t>
+          <t>sh600513</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>天士力</t>
+          <t>联环药业</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3447,41 +3661,44 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>14.99</v>
+        <v>20.4</v>
       </c>
       <c r="E71" t="n">
-        <v>14.94</v>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G71" t="n">
-        <v>52</v>
+        <v>20.29</v>
+      </c>
+      <c r="F71" t="n">
+        <v>19.53</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H71" t="n">
-        <v>2.531</v>
+        <v>52</v>
       </c>
       <c r="I71" t="n">
-        <v>0</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K71" t="n">
-        <v>3.97</v>
+        <v>1</v>
+      </c>
+      <c r="L71" t="n">
+        <v>1.28</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>sh600531</t>
+          <t>sh600510</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>豫光金铅</t>
+          <t>黑牡丹</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3490,41 +3707,44 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>15.93</v>
+        <v>11.28</v>
       </c>
       <c r="E72" t="n">
-        <v>15.72</v>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G72" t="n">
-        <v>52</v>
+        <v>11.08</v>
+      </c>
+      <c r="F72" t="n">
+        <v>10.56</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H72" t="n">
-        <v>2.378</v>
+        <v>52</v>
       </c>
       <c r="I72" t="n">
-        <v>0</v>
+        <v>3.014</v>
       </c>
       <c r="J72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K72" t="n">
-        <v>5.86</v>
+        <v>1</v>
+      </c>
+      <c r="L72" t="n">
+        <v>1.42</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>sh600510</t>
+          <t>sh600501</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>黑牡丹</t>
+          <t>航天晨光</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3533,41 +3753,44 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>11.12</v>
+        <v>23.15</v>
       </c>
       <c r="E73" t="n">
-        <v>11.04</v>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G73" t="n">
-        <v>52</v>
+        <v>23.22</v>
+      </c>
+      <c r="F73" t="n">
+        <v>22.54</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H73" t="n">
-        <v>1.553</v>
+        <v>52</v>
       </c>
       <c r="I73" t="n">
-        <v>0</v>
+        <v>1.402</v>
       </c>
       <c r="J73" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K73" t="n">
-        <v>1.14</v>
+        <v>1</v>
+      </c>
+      <c r="L73" t="n">
+        <v>1.43</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>sh600867</t>
+          <t>sh600499</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>通化东宝</t>
+          <t>科达制造</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3576,41 +3799,44 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>10.02</v>
+        <v>20.23</v>
       </c>
       <c r="E74" t="n">
-        <v>9.789999999999999</v>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G74" t="n">
-        <v>52</v>
+        <v>20.18</v>
+      </c>
+      <c r="F74" t="n">
+        <v>19.58</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H74" t="n">
-        <v>4.266</v>
+        <v>52</v>
       </c>
       <c r="I74" t="n">
-        <v>0</v>
+        <v>2.12</v>
       </c>
       <c r="J74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K74" t="n">
-        <v>5.15</v>
+        <v>1</v>
+      </c>
+      <c r="L74" t="n">
+        <v>9.460000000000001</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>sh600835</t>
+          <t>sh600489</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>上海机电</t>
+          <t>中金黄金</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3619,41 +3845,44 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>23.59</v>
+        <v>25.89</v>
       </c>
       <c r="E75" t="n">
-        <v>23.65</v>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G75" t="n">
-        <v>52</v>
+        <v>25.7</v>
+      </c>
+      <c r="F75" t="n">
+        <v>24.84</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H75" t="n">
-        <v>0.554</v>
+        <v>52</v>
       </c>
       <c r="I75" t="n">
-        <v>0</v>
+        <v>1.41</v>
       </c>
       <c r="J75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K75" t="n">
-        <v>1.29</v>
+        <v>1</v>
+      </c>
+      <c r="L75" t="n">
+        <v>7.64</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>sh600776</t>
+          <t>sh600759</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>东方通信</t>
+          <t>洲际油气</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3662,41 +3891,44 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>16.63</v>
+        <v>5.22</v>
       </c>
       <c r="E76" t="n">
-        <v>16.57</v>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G76" t="n">
-        <v>52</v>
+        <v>5.2</v>
+      </c>
+      <c r="F76" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H76" t="n">
-        <v>1.094</v>
+        <v>52</v>
       </c>
       <c r="I76" t="n">
-        <v>0</v>
+        <v>0.967</v>
       </c>
       <c r="J76" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K76" t="n">
-        <v>3.57</v>
+        <v>1</v>
+      </c>
+      <c r="L76" t="n">
+        <v>8.4</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>sh600773</t>
+          <t>sh600758</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>西藏城投</t>
+          <t>辽宁能源</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3705,41 +3937,44 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>25.6</v>
+        <v>4.08</v>
       </c>
       <c r="E77" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G77" t="n">
-        <v>52</v>
+        <v>4.03</v>
+      </c>
+      <c r="F77" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H77" t="n">
-        <v>3.812</v>
+        <v>52</v>
       </c>
       <c r="I77" t="n">
-        <v>0</v>
+        <v>2.513</v>
       </c>
       <c r="J77" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K77" t="n">
-        <v>5.87</v>
+        <v>1</v>
+      </c>
+      <c r="L77" t="n">
+        <v>2.09</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>sh600761</t>
+          <t>sh600745</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>安徽合力</t>
+          <t>闻泰科技</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3748,41 +3983,44 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>17.82</v>
+        <v>28.12</v>
       </c>
       <c r="E78" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G78" t="n">
-        <v>52</v>
+        <v>28</v>
+      </c>
+      <c r="F78" t="n">
+        <v>26.38</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H78" t="n">
-        <v>4.028</v>
+        <v>52</v>
       </c>
       <c r="I78" t="n">
-        <v>0</v>
+        <v>1.115</v>
       </c>
       <c r="J78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K78" t="n">
-        <v>2.65</v>
+        <v>1</v>
+      </c>
+      <c r="L78" t="n">
+        <v>7.61</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>sh600759</t>
+          <t>sh600733</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>洲际油气</t>
+          <t>北汽蓝谷</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3791,41 +4029,44 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>5.2</v>
+        <v>7.52</v>
       </c>
       <c r="E79" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G79" t="n">
-        <v>52</v>
+        <v>7.3</v>
+      </c>
+      <c r="F79" t="n">
+        <v>7.11</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H79" t="n">
-        <v>0.58</v>
+        <v>52</v>
       </c>
       <c r="I79" t="n">
-        <v>0</v>
+        <v>5.175</v>
       </c>
       <c r="J79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K79" t="n">
-        <v>7.53</v>
+        <v>1</v>
+      </c>
+      <c r="L79" t="n">
+        <v>8.26</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>sh600758</t>
+          <t>sh600707</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>辽宁能源</t>
+          <t>彩虹股份</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3834,41 +4075,44 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>4.05</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="E80" t="n">
-        <v>4.01</v>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G80" t="n">
-        <v>52</v>
+        <v>8.23</v>
+      </c>
+      <c r="F80" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H80" t="n">
-        <v>1.759</v>
+        <v>52</v>
       </c>
       <c r="I80" t="n">
-        <v>0</v>
+        <v>2.726</v>
       </c>
       <c r="J80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K80" t="n">
-        <v>1.58</v>
+        <v>1</v>
+      </c>
+      <c r="L80" t="n">
+        <v>7.25</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>sh600745</t>
+          <t>sh600698</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>闻泰科技</t>
+          <t>湖南天雁</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3877,41 +4121,44 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>28.15</v>
+        <v>7.32</v>
       </c>
       <c r="E81" t="n">
-        <v>28</v>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G81" t="n">
-        <v>52</v>
+        <v>7.16</v>
+      </c>
+      <c r="F81" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H81" t="n">
-        <v>1.223</v>
+        <v>52</v>
       </c>
       <c r="I81" t="n">
-        <v>0</v>
+        <v>3.977</v>
       </c>
       <c r="J81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K81" t="n">
-        <v>7.15</v>
+        <v>1</v>
+      </c>
+      <c r="L81" t="n">
+        <v>0.86</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>sh600733</t>
+          <t>sh600694</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>北汽蓝谷</t>
+          <t>大商股份</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3920,30 +4167,33 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>7.44</v>
+        <v>18.34</v>
       </c>
       <c r="E82" t="n">
-        <v>7.26</v>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>潜伏蓄势</t>
-        </is>
-      </c>
-      <c r="G82" t="n">
-        <v>52</v>
+        <v>18.15</v>
+      </c>
+      <c r="F82" t="n">
+        <v>17.52</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>潜伏蓄势</t>
+        </is>
       </c>
       <c r="H82" t="n">
-        <v>4.056</v>
+        <v>52</v>
       </c>
       <c r="I82" t="n">
-        <v>0</v>
+        <v>1.719</v>
       </c>
       <c r="J82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K82" t="n">
-        <v>6.6</v>
+        <v>1</v>
+      </c>
+      <c r="L82" t="n">
+        <v>1.06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 实时报告更新 Mon Apr 27 04:50:32 UTC 2026
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>T:2026-04-27 11:16:22</t>
+          <t>T:2026-04-27 12:50:32</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>94.44</v>
+        <v>94.33</v>
       </c>
       <c r="E3" t="n">
         <v>93.76000000000001</v>
@@ -550,7 +550,7 @@
         <v>52</v>
       </c>
       <c r="I3" t="n">
-        <v>1.505</v>
+        <v>1.387</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -559,7 +559,7 @@
         <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>4.3</v>
+        <v>4.44</v>
       </c>
     </row>
     <row r="4">
@@ -579,7 +579,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>58</v>
+        <v>58.06</v>
       </c>
       <c r="E4" t="n">
         <v>57.41</v>
@@ -596,7 +596,7 @@
         <v>52</v>
       </c>
       <c r="I4" t="n">
-        <v>2.655</v>
+        <v>2.761</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -605,7 +605,7 @@
         <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>1.07</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="5">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>562.39</v>
+        <v>562.6799999999999</v>
       </c>
       <c r="E5" t="n">
         <v>549.22</v>
@@ -642,7 +642,7 @@
         <v>52</v>
       </c>
       <c r="I5" t="n">
-        <v>5.12</v>
+        <v>5.174</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -651,18 +651,18 @@
         <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>4.72</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>bj920111</t>
+          <t>sz301529</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>聚星科技</t>
+          <t>福赛科技</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -671,13 +671,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>35.5</v>
+        <v>121.44</v>
       </c>
       <c r="E6" t="n">
-        <v>35.26</v>
+        <v>121.77</v>
       </c>
       <c r="F6" t="n">
-        <v>33.64</v>
+        <v>116.08</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         <v>52</v>
       </c>
       <c r="I6" t="n">
-        <v>1.924</v>
+        <v>2.524</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -697,18 +697,18 @@
         <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>2.09</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>bj920179</t>
+          <t>sz301479</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>凯德石英</t>
+          <t>弘景光电</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -717,13 +717,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>51</v>
+        <v>108.75</v>
       </c>
       <c r="E7" t="n">
-        <v>50.91</v>
+        <v>109.06</v>
       </c>
       <c r="F7" t="n">
-        <v>48.68</v>
+        <v>105.64</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -734,7 +734,7 @@
         <v>52</v>
       </c>
       <c r="I7" t="n">
-        <v>2.123</v>
+        <v>1.116</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -749,12 +749,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>bj920181</t>
+          <t>sz301458</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>赛英电子</t>
+          <t>钧崴电子</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -763,13 +763,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>82.15000000000001</v>
+        <v>40.08</v>
       </c>
       <c r="E8" t="n">
-        <v>81.79000000000001</v>
+        <v>39.93</v>
       </c>
       <c r="F8" t="n">
-        <v>76.94</v>
+        <v>38.67</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -780,7 +780,7 @@
         <v>52</v>
       </c>
       <c r="I8" t="n">
-        <v>2.164</v>
+        <v>1.752</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -789,18 +789,18 @@
         <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>1.26</v>
+        <v>2.16</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>bj920402</t>
+          <t>sz301421</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>硅烷科技</t>
+          <t>波长光电</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -809,13 +809,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>9.94</v>
+        <v>99.67</v>
       </c>
       <c r="E9" t="n">
-        <v>10.04</v>
+        <v>97.95999999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>9.470000000000001</v>
+        <v>94.02</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -826,7 +826,7 @@
         <v>52</v>
       </c>
       <c r="I9" t="n">
-        <v>1.016</v>
+        <v>3.736</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -835,18 +835,18 @@
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>0.92</v>
+        <v>3.66</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>bj920438</t>
+          <t>sz301419</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>戈碧迦</t>
+          <t>阿莱德</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -855,13 +855,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>43.3</v>
+        <v>42.09</v>
       </c>
       <c r="E10" t="n">
-        <v>43.63</v>
+        <v>41.95</v>
       </c>
       <c r="F10" t="n">
-        <v>41.73</v>
+        <v>40.48</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -872,7 +872,7 @@
         <v>52</v>
       </c>
       <c r="I10" t="n">
-        <v>1.05</v>
+        <v>1.275</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -881,18 +881,18 @@
         <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>bj920809</t>
+          <t>sz301408</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>安达科技</t>
+          <t>华人健康</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -901,13 +901,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>8.279999999999999</v>
+        <v>20.13</v>
       </c>
       <c r="E11" t="n">
-        <v>8.24</v>
+        <v>20.16</v>
       </c>
       <c r="F11" t="n">
-        <v>7.99</v>
+        <v>19.21</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -918,7 +918,7 @@
         <v>52</v>
       </c>
       <c r="I11" t="n">
-        <v>1.222</v>
+        <v>1.667</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -927,18 +927,18 @@
         <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>1.11</v>
+        <v>3.32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>sz301536</t>
+          <t>sz301395</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>星宸科技</t>
+          <t>仁信新材</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -947,13 +947,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>83.39</v>
+        <v>12.98</v>
       </c>
       <c r="E12" t="n">
-        <v>82.44</v>
+        <v>12.93</v>
       </c>
       <c r="F12" t="n">
-        <v>79.68000000000001</v>
+        <v>11.76</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         <v>52</v>
       </c>
       <c r="I12" t="n">
-        <v>2.194</v>
+        <v>1.565</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -973,18 +973,18 @@
         <v>1</v>
       </c>
       <c r="L12" t="n">
-        <v>7.79</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>sz301529</t>
+          <t>sz301393</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>福赛科技</t>
+          <t>昊帆生物</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -993,13 +993,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>121.39</v>
+        <v>61.02</v>
       </c>
       <c r="E13" t="n">
-        <v>121.77</v>
+        <v>60.94</v>
       </c>
       <c r="F13" t="n">
-        <v>116.08</v>
+        <v>58.39</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
         <v>52</v>
       </c>
       <c r="I13" t="n">
-        <v>2.482</v>
+        <v>1.819</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -1019,18 +1019,18 @@
         <v>1</v>
       </c>
       <c r="L13" t="n">
-        <v>2.72</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>sz301479</t>
+          <t>sz301382</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>弘景光电</t>
+          <t>蜂助手</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1039,13 +1039,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>109.43</v>
+        <v>40.96</v>
       </c>
       <c r="E14" t="n">
-        <v>109.06</v>
+        <v>40.65</v>
       </c>
       <c r="F14" t="n">
-        <v>105.64</v>
+        <v>38.22</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
         <v>52</v>
       </c>
       <c r="I14" t="n">
-        <v>1.748</v>
+        <v>2.043</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -1065,18 +1065,18 @@
         <v>1</v>
       </c>
       <c r="L14" t="n">
-        <v>1.52</v>
+        <v>4.22</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>sz301458</t>
+          <t>sz301378</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>钧崴电子</t>
+          <t>通达海</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1085,13 +1085,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>40.2</v>
+        <v>31.56</v>
       </c>
       <c r="E15" t="n">
-        <v>39.93</v>
+        <v>32.33</v>
       </c>
       <c r="F15" t="n">
-        <v>38.67</v>
+        <v>30.85</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1102,7 +1102,7 @@
         <v>52</v>
       </c>
       <c r="I15" t="n">
-        <v>2.056</v>
+        <v>0.766</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -1111,18 +1111,18 @@
         <v>1</v>
       </c>
       <c r="L15" t="n">
-        <v>2.07</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>sz301421</t>
+          <t>sz301371</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>波长光电</t>
+          <t>敷尔佳</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1131,13 +1131,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>99.66</v>
+        <v>29.07</v>
       </c>
       <c r="E16" t="n">
-        <v>97.95999999999999</v>
+        <v>28.54</v>
       </c>
       <c r="F16" t="n">
-        <v>94.02</v>
+        <v>27.41</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
         <v>52</v>
       </c>
       <c r="I16" t="n">
-        <v>3.726</v>
+        <v>3.933</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1157,18 +1157,18 @@
         <v>1</v>
       </c>
       <c r="L16" t="n">
-        <v>3.55</v>
+        <v>2.28</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>sz301419</t>
+          <t>sz301369</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>阿莱德</t>
+          <t>联动科技</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1177,13 +1177,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>41.95</v>
+        <v>168.67</v>
       </c>
       <c r="E17" t="n">
-        <v>41.95</v>
+        <v>167.98</v>
       </c>
       <c r="F17" t="n">
-        <v>40.48</v>
+        <v>163.06</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1194,7 +1194,7 @@
         <v>52</v>
       </c>
       <c r="I17" t="n">
-        <v>0.9379999999999999</v>
+        <v>1.541</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1203,18 +1203,18 @@
         <v>1</v>
       </c>
       <c r="L17" t="n">
-        <v>0.93</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>sz301408</t>
+          <t>sz301366</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>华人健康</t>
+          <t>一博科技</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1223,13 +1223,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>20.19</v>
+        <v>37.41</v>
       </c>
       <c r="E18" t="n">
-        <v>20.16</v>
+        <v>37.31</v>
       </c>
       <c r="F18" t="n">
-        <v>19.21</v>
+        <v>36.11</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1240,7 +1240,7 @@
         <v>52</v>
       </c>
       <c r="I18" t="n">
-        <v>1.97</v>
+        <v>1.382</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1249,18 +1249,18 @@
         <v>1</v>
       </c>
       <c r="L18" t="n">
-        <v>3.18</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>sz301395</t>
+          <t>sz301365</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>仁信新材</t>
+          <t>矩阵股份</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1269,13 +1269,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>12.98</v>
+        <v>34.75</v>
       </c>
       <c r="E19" t="n">
-        <v>12.93</v>
+        <v>33.97</v>
       </c>
       <c r="F19" t="n">
-        <v>11.76</v>
+        <v>32.01</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1286,7 +1286,7 @@
         <v>52</v>
       </c>
       <c r="I19" t="n">
-        <v>1.565</v>
+        <v>4.198</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1295,18 +1295,18 @@
         <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>1.09</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>sz301393</t>
+          <t>sz301362</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>昊帆生物</t>
+          <t>民爆光电</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1315,13 +1315,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>61.01</v>
+        <v>143.21</v>
       </c>
       <c r="E20" t="n">
-        <v>60.94</v>
+        <v>142.84</v>
       </c>
       <c r="F20" t="n">
-        <v>58.39</v>
+        <v>137.2</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1332,7 +1332,7 @@
         <v>52</v>
       </c>
       <c r="I20" t="n">
-        <v>1.802</v>
+        <v>1.116</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1341,18 +1341,18 @@
         <v>1</v>
       </c>
       <c r="L20" t="n">
-        <v>1.12</v>
+        <v>2.03</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>sz301392</t>
+          <t>sz301348</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>汇成真空</t>
+          <t>蓝箭电子</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1361,13 +1361,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>162.35</v>
+        <v>24.18</v>
       </c>
       <c r="E21" t="n">
-        <v>162.53</v>
+        <v>24.01</v>
       </c>
       <c r="F21" t="n">
-        <v>155.15</v>
+        <v>22.94</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1378,7 +1378,7 @@
         <v>52</v>
       </c>
       <c r="I21" t="n">
-        <v>0.832</v>
+        <v>1.469</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1387,18 +1387,18 @@
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>3.74</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>sz301382</t>
+          <t>sh600207</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>蜂助手</t>
+          <t>安彩高科</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1407,13 +1407,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>40.88</v>
+        <v>5.88</v>
       </c>
       <c r="E22" t="n">
-        <v>40.65</v>
+        <v>5.9</v>
       </c>
       <c r="F22" t="n">
-        <v>38.22</v>
+        <v>5.69</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1424,7 +1424,7 @@
         <v>52</v>
       </c>
       <c r="I22" t="n">
-        <v>1.844</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1433,18 +1433,18 @@
         <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>4.04</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>sz301378</t>
+          <t>sh600203</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>通达海</t>
+          <t>福日电子</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1453,13 +1453,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>31.68</v>
+        <v>12.53</v>
       </c>
       <c r="E23" t="n">
-        <v>32.33</v>
+        <v>12.24</v>
       </c>
       <c r="F23" t="n">
-        <v>30.85</v>
+        <v>11.58</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1470,7 +1470,7 @@
         <v>52</v>
       </c>
       <c r="I23" t="n">
-        <v>1.149</v>
+        <v>4.243</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1479,18 +1479,18 @@
         <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>1.49</v>
+        <v>3.47</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>sz301371</t>
+          <t>sh600198</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>敷尔佳</t>
+          <t>大唐电信</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1499,13 +1499,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>29.1</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="E24" t="n">
-        <v>28.54</v>
+        <v>8.18</v>
       </c>
       <c r="F24" t="n">
-        <v>27.41</v>
+        <v>7.82</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1516,7 +1516,7 @@
         <v>52</v>
       </c>
       <c r="I24" t="n">
-        <v>4.04</v>
+        <v>0.736</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1525,18 +1525,18 @@
         <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>2.19</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>sz301369</t>
+          <t>sh600188</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>联动科技</t>
+          <t>兖矿能源</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1545,13 +1545,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>168.88</v>
+        <v>20.98</v>
       </c>
       <c r="E25" t="n">
-        <v>167.98</v>
+        <v>20.91</v>
       </c>
       <c r="F25" t="n">
-        <v>163.06</v>
+        <v>19.97</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1562,7 +1562,7 @@
         <v>52</v>
       </c>
       <c r="I25" t="n">
-        <v>1.668</v>
+        <v>1.451</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1571,18 +1571,18 @@
         <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>1.27</v>
+        <v>6.34</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sz301365</t>
+          <t>sh600185</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>矩阵股份</t>
+          <t>珠免集团</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1591,13 +1591,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>34.8</v>
+        <v>5.99</v>
       </c>
       <c r="E26" t="n">
-        <v>33.97</v>
+        <v>5.96</v>
       </c>
       <c r="F26" t="n">
-        <v>32.01</v>
+        <v>5.71</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1608,7 +1608,7 @@
         <v>52</v>
       </c>
       <c r="I26" t="n">
-        <v>4.348</v>
+        <v>1.182</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1617,18 +1617,18 @@
         <v>1</v>
       </c>
       <c r="L26" t="n">
-        <v>1.24</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>sz301362</t>
+          <t>sh600172</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>民爆光电</t>
+          <t>黄河旋风</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1637,13 +1637,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>143.58</v>
+        <v>8.4</v>
       </c>
       <c r="E27" t="n">
-        <v>142.84</v>
+        <v>8.41</v>
       </c>
       <c r="F27" t="n">
-        <v>137.2</v>
+        <v>8.1</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1654,7 +1654,7 @@
         <v>52</v>
       </c>
       <c r="I27" t="n">
-        <v>1.377</v>
+        <v>1.205</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1663,18 +1663,18 @@
         <v>1</v>
       </c>
       <c r="L27" t="n">
-        <v>1.9</v>
+        <v>4.23</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>sh600312</t>
+          <t>sh600171</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>平高电气</t>
+          <t>上海贝岭</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1683,13 +1683,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>22.17</v>
+        <v>29.3</v>
       </c>
       <c r="E28" t="n">
-        <v>22.09</v>
+        <v>28.91</v>
       </c>
       <c r="F28" t="n">
-        <v>21.23</v>
+        <v>27.5</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1700,7 +1700,7 @@
         <v>52</v>
       </c>
       <c r="I28" t="n">
-        <v>1.325</v>
+        <v>3.024</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1709,18 +1709,18 @@
         <v>1</v>
       </c>
       <c r="L28" t="n">
-        <v>3.74</v>
+        <v>5.34</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>sh600310</t>
+          <t>sh600160</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>广西能源</t>
+          <t>巨化股份</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1729,13 +1729,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>5.34</v>
+        <v>36.01</v>
       </c>
       <c r="E29" t="n">
-        <v>5.19</v>
+        <v>35.49</v>
       </c>
       <c r="F29" t="n">
-        <v>4.72</v>
+        <v>34.21</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1746,7 +1746,7 @@
         <v>52</v>
       </c>
       <c r="I29" t="n">
-        <v>4.912</v>
+        <v>2.739</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1755,18 +1755,18 @@
         <v>1</v>
       </c>
       <c r="L29" t="n">
-        <v>7.21</v>
+        <v>11.61</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>sh600299</t>
+          <t>sh600158</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>安迪苏</t>
+          <t>中体产业</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1775,13 +1775,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>14.26</v>
+        <v>10.72</v>
       </c>
       <c r="E30" t="n">
-        <v>14.14</v>
+        <v>10.62</v>
       </c>
       <c r="F30" t="n">
-        <v>13.47</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1792,7 +1792,7 @@
         <v>52</v>
       </c>
       <c r="I30" t="n">
-        <v>2.443</v>
+        <v>2.388</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1801,18 +1801,18 @@
         <v>1</v>
       </c>
       <c r="L30" t="n">
-        <v>1.33</v>
+        <v>5.13</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>sh600292</t>
+          <t>sh600157</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>电投水电</t>
+          <t>永泰能源</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1821,13 +1821,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>16.05</v>
+        <v>1.73</v>
       </c>
       <c r="E31" t="n">
-        <v>16.01</v>
+        <v>1.71</v>
       </c>
       <c r="F31" t="n">
-        <v>15.29</v>
+        <v>1.64</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1838,7 +1838,7 @@
         <v>52</v>
       </c>
       <c r="I31" t="n">
-        <v>0.753</v>
+        <v>2.976</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1847,18 +1847,18 @@
         <v>1</v>
       </c>
       <c r="L31" t="n">
-        <v>1.44</v>
+        <v>10.86</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>sh600267</t>
+          <t>sh600156</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>海正药业</t>
+          <t>华升股份</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1867,13 +1867,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>11.46</v>
+        <v>9.26</v>
       </c>
       <c r="E32" t="n">
-        <v>11.42</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="F32" t="n">
-        <v>10.99</v>
+        <v>8.43</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         <v>52</v>
       </c>
       <c r="I32" t="n">
-        <v>0.792</v>
+        <v>1.535</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1893,18 +1893,18 @@
         <v>1</v>
       </c>
       <c r="L32" t="n">
-        <v>2.15</v>
+        <v>3.67</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>sh600255</t>
+          <t>sh600143</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>鑫科材料</t>
+          <t>金发科技</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1913,13 +1913,13 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>3.65</v>
+        <v>16.95</v>
       </c>
       <c r="E33" t="n">
-        <v>3.62</v>
+        <v>16.84</v>
       </c>
       <c r="F33" t="n">
-        <v>3.5</v>
+        <v>16.25</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1930,7 +1930,7 @@
         <v>52</v>
       </c>
       <c r="I33" t="n">
-        <v>1.389</v>
+        <v>1.436</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1939,18 +1939,18 @@
         <v>1</v>
       </c>
       <c r="L33" t="n">
-        <v>0.8</v>
+        <v>4.51</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>sh600233</t>
+          <t>sh600132</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>圆通速递</t>
+          <t>重庆啤酒</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1959,13 +1959,13 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>22.48</v>
+        <v>55.08</v>
       </c>
       <c r="E34" t="n">
-        <v>22.26</v>
+        <v>54.56</v>
       </c>
       <c r="F34" t="n">
-        <v>21.45</v>
+        <v>52.81</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1976,7 +1976,7 @@
         <v>52</v>
       </c>
       <c r="I34" t="n">
-        <v>2.508</v>
+        <v>1.68</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1985,18 +1985,18 @@
         <v>1</v>
       </c>
       <c r="L34" t="n">
-        <v>3.96</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>sh600226</t>
+          <t>sh600123</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>亨通股份</t>
+          <t>兰花科创</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2005,13 +2005,13 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>5.44</v>
+        <v>6.73</v>
       </c>
       <c r="E35" t="n">
-        <v>5.3</v>
+        <v>6.59</v>
       </c>
       <c r="F35" t="n">
-        <v>5.03</v>
+        <v>6.27</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2022,7 +2022,7 @@
         <v>52</v>
       </c>
       <c r="I35" t="n">
-        <v>4.415</v>
+        <v>4.18</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -2031,18 +2031,18 @@
         <v>1</v>
       </c>
       <c r="L35" t="n">
-        <v>2.55</v>
+        <v>2.74</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>sh600203</t>
+          <t>sh600114</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>福日电子</t>
+          <t>东睦股份</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2051,13 +2051,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>12.52</v>
+        <v>33.95</v>
       </c>
       <c r="E36" t="n">
-        <v>12.24</v>
+        <v>33.61</v>
       </c>
       <c r="F36" t="n">
-        <v>11.58</v>
+        <v>32.38</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2068,7 +2068,7 @@
         <v>52</v>
       </c>
       <c r="I36" t="n">
-        <v>4.16</v>
+        <v>2.136</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -2077,18 +2077,18 @@
         <v>1</v>
       </c>
       <c r="L36" t="n">
-        <v>3.36</v>
+        <v>3.12</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>sh600198</t>
+          <t>sh600109</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>大唐电信</t>
+          <t>国金证券</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2097,13 +2097,13 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>8.210000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="E37" t="n">
-        <v>8.18</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="F37" t="n">
-        <v>7.82</v>
+        <v>8.49</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -2114,7 +2114,7 @@
         <v>52</v>
       </c>
       <c r="I37" t="n">
-        <v>0.736</v>
+        <v>1.387</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -2123,18 +2123,18 @@
         <v>1</v>
       </c>
       <c r="L37" t="n">
-        <v>0.82</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>sh600188</t>
+          <t>sh600370</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>兖矿能源</t>
+          <t>三房巷</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2143,13 +2143,13 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>20.99</v>
+        <v>2.68</v>
       </c>
       <c r="E38" t="n">
-        <v>20.91</v>
+        <v>2.69</v>
       </c>
       <c r="F38" t="n">
-        <v>19.97</v>
+        <v>2.51</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -2160,7 +2160,7 @@
         <v>52</v>
       </c>
       <c r="I38" t="n">
-        <v>1.499</v>
+        <v>1.515</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -2169,18 +2169,18 @@
         <v>1</v>
       </c>
       <c r="L38" t="n">
-        <v>6.13</v>
+        <v>4.14</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>sh600185</t>
+          <t>sh600366</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>珠免集团</t>
+          <t>宁波韵升</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2189,13 +2189,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>6.01</v>
+        <v>13.08</v>
       </c>
       <c r="E39" t="n">
-        <v>5.96</v>
+        <v>12.92</v>
       </c>
       <c r="F39" t="n">
-        <v>5.71</v>
+        <v>12.55</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -2206,7 +2206,7 @@
         <v>52</v>
       </c>
       <c r="I39" t="n">
-        <v>1.52</v>
+        <v>2.267</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2215,18 +2215,18 @@
         <v>1</v>
       </c>
       <c r="L39" t="n">
-        <v>0.89</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>sh600177</t>
+          <t>sh600363</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>雅戈尔</t>
+          <t>联创光电</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2235,13 +2235,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>7.63</v>
+        <v>53.05</v>
       </c>
       <c r="E40" t="n">
-        <v>7.61</v>
+        <v>52.59</v>
       </c>
       <c r="F40" t="n">
-        <v>7.4</v>
+        <v>50.66</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -2252,7 +2252,7 @@
         <v>52</v>
       </c>
       <c r="I40" t="n">
-        <v>0.66</v>
+        <v>2.039</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2261,18 +2261,18 @@
         <v>1</v>
       </c>
       <c r="L40" t="n">
-        <v>0.89</v>
+        <v>2.46</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>sh600172</t>
+          <t>sh600361</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>黄河旋风</t>
+          <t>创新新材</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2281,13 +2281,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>8.41</v>
+        <v>4.65</v>
       </c>
       <c r="E41" t="n">
-        <v>8.41</v>
+        <v>4.58</v>
       </c>
       <c r="F41" t="n">
-        <v>8.1</v>
+        <v>4.4</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -2298,7 +2298,7 @@
         <v>52</v>
       </c>
       <c r="I41" t="n">
-        <v>1.325</v>
+        <v>3.563</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2307,18 +2307,18 @@
         <v>1</v>
       </c>
       <c r="L41" t="n">
-        <v>4.05</v>
+        <v>2.66</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>sh600171</t>
+          <t>sh600351</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>上海贝岭</t>
+          <t>亚宝药业</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2327,13 +2327,13 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>29.33</v>
+        <v>6.74</v>
       </c>
       <c r="E42" t="n">
-        <v>28.91</v>
+        <v>6.6</v>
       </c>
       <c r="F42" t="n">
-        <v>27.5</v>
+        <v>6.35</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -2344,7 +2344,7 @@
         <v>52</v>
       </c>
       <c r="I42" t="n">
-        <v>3.129</v>
+        <v>4.984</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
@@ -2353,18 +2353,18 @@
         <v>1</v>
       </c>
       <c r="L42" t="n">
-        <v>5.22</v>
+        <v>2.12</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>sh600160</t>
+          <t>sh600345</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>巨化股份</t>
+          <t>长江通信</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2373,13 +2373,13 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>35.99</v>
+        <v>52.58</v>
       </c>
       <c r="E43" t="n">
-        <v>35.49</v>
+        <v>51.57</v>
       </c>
       <c r="F43" t="n">
-        <v>34.21</v>
+        <v>49.54</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -2390,7 +2390,7 @@
         <v>52</v>
       </c>
       <c r="I43" t="n">
-        <v>2.682</v>
+        <v>4.325</v>
       </c>
       <c r="J43" t="n">
         <v>0</v>
@@ -2399,18 +2399,18 @@
         <v>1</v>
       </c>
       <c r="L43" t="n">
-        <v>11.16</v>
+        <v>5.31</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>sh600483</t>
+          <t>sh600333</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>福能股份</t>
+          <t>长春燃气</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2419,13 +2419,13 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>9.98</v>
+        <v>5.73</v>
       </c>
       <c r="E44" t="n">
-        <v>9.91</v>
+        <v>5.68</v>
       </c>
       <c r="F44" t="n">
-        <v>9.5</v>
+        <v>5.49</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -2436,7 +2436,7 @@
         <v>52</v>
       </c>
       <c r="I44" t="n">
-        <v>1.217</v>
+        <v>3.058</v>
       </c>
       <c r="J44" t="n">
         <v>0</v>
@@ -2445,18 +2445,18 @@
         <v>1</v>
       </c>
       <c r="L44" t="n">
-        <v>1.14</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>sh600460</t>
+          <t>sh600331</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>士兰微</t>
+          <t>宏达股份</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2465,13 +2465,13 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>28.17</v>
+        <v>18.57</v>
       </c>
       <c r="E45" t="n">
-        <v>28.04</v>
+        <v>18.44</v>
       </c>
       <c r="F45" t="n">
-        <v>27.15</v>
+        <v>17.72</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2482,7 +2482,7 @@
         <v>52</v>
       </c>
       <c r="I45" t="n">
-        <v>1.258</v>
+        <v>1.809</v>
       </c>
       <c r="J45" t="n">
         <v>0</v>
@@ -2491,18 +2491,18 @@
         <v>1</v>
       </c>
       <c r="L45" t="n">
-        <v>7.36</v>
+        <v>7.42</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>sh600446</t>
+          <t>sh600323</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>金证股份</t>
+          <t>瀚蓝环境</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2511,13 +2511,13 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>13.68</v>
+        <v>31</v>
       </c>
       <c r="E46" t="n">
-        <v>13.5</v>
+        <v>30.86</v>
       </c>
       <c r="F46" t="n">
-        <v>12.9</v>
+        <v>29.14</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2528,7 +2528,7 @@
         <v>52</v>
       </c>
       <c r="I46" t="n">
-        <v>2.626</v>
+        <v>2.683</v>
       </c>
       <c r="J46" t="n">
         <v>0</v>
@@ -2537,18 +2537,18 @@
         <v>1</v>
       </c>
       <c r="L46" t="n">
-        <v>2.66</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>sh600429</t>
+          <t>sh600312</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>三元股份</t>
+          <t>平高电气</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2557,13 +2557,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>6.15</v>
+        <v>22.16</v>
       </c>
       <c r="E47" t="n">
-        <v>6.11</v>
+        <v>22.09</v>
       </c>
       <c r="F47" t="n">
-        <v>5.89</v>
+        <v>21.23</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -2574,7 +2574,7 @@
         <v>52</v>
       </c>
       <c r="I47" t="n">
-        <v>2.329</v>
+        <v>1.28</v>
       </c>
       <c r="J47" t="n">
         <v>0</v>
@@ -2583,18 +2583,18 @@
         <v>1</v>
       </c>
       <c r="L47" t="n">
-        <v>2.58</v>
+        <v>3.86</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>sh600426</t>
+          <t>sh600310</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>华鲁恒升</t>
+          <t>广西能源</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2603,13 +2603,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>38.04</v>
+        <v>5.29</v>
       </c>
       <c r="E48" t="n">
-        <v>37.83</v>
+        <v>5.2</v>
       </c>
       <c r="F48" t="n">
-        <v>36.31</v>
+        <v>4.72</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2620,7 +2620,7 @@
         <v>52</v>
       </c>
       <c r="I48" t="n">
-        <v>1.116</v>
+        <v>3.929</v>
       </c>
       <c r="J48" t="n">
         <v>0</v>
@@ -2629,18 +2629,18 @@
         <v>1</v>
       </c>
       <c r="L48" t="n">
-        <v>5.22</v>
+        <v>7.71</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>sh600395</t>
+          <t>sh600299</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>盘江股份</t>
+          <t>安迪苏</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2649,13 +2649,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>5.75</v>
+        <v>14.28</v>
       </c>
       <c r="E49" t="n">
-        <v>5.74</v>
+        <v>14.14</v>
       </c>
       <c r="F49" t="n">
-        <v>5.54</v>
+        <v>13.47</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2666,7 +2666,7 @@
         <v>52</v>
       </c>
       <c r="I49" t="n">
-        <v>0.524</v>
+        <v>2.586</v>
       </c>
       <c r="J49" t="n">
         <v>0</v>
@@ -2675,18 +2675,18 @@
         <v>1</v>
       </c>
       <c r="L49" t="n">
-        <v>1.13</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>sh600378</t>
+          <t>sh600292</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>昊华科技</t>
+          <t>电投水电</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2695,13 +2695,13 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>35.61</v>
+        <v>16.02</v>
       </c>
       <c r="E50" t="n">
-        <v>35.52</v>
+        <v>16.01</v>
       </c>
       <c r="F50" t="n">
-        <v>34.3</v>
+        <v>15.29</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2712,7 +2712,7 @@
         <v>52</v>
       </c>
       <c r="I50" t="n">
-        <v>1.021</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="J50" t="n">
         <v>0</v>
@@ -2721,18 +2721,18 @@
         <v>1</v>
       </c>
       <c r="L50" t="n">
-        <v>3.58</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>sh600366</t>
+          <t>sh600255</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>宁波韵升</t>
+          <t>鑫科材料</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2741,13 +2741,13 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>13.08</v>
+        <v>3.65</v>
       </c>
       <c r="E51" t="n">
-        <v>12.92</v>
+        <v>3.63</v>
       </c>
       <c r="F51" t="n">
-        <v>12.55</v>
+        <v>3.5</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2758,7 +2758,7 @@
         <v>52</v>
       </c>
       <c r="I51" t="n">
-        <v>2.267</v>
+        <v>1.389</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
@@ -2767,18 +2767,18 @@
         <v>1</v>
       </c>
       <c r="L51" t="n">
-        <v>2.33</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>sh600363</t>
+          <t>sh600233</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>联创光电</t>
+          <t>圆通速递</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2787,13 +2787,13 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>53.13</v>
+        <v>22.51</v>
       </c>
       <c r="E52" t="n">
-        <v>52.59</v>
+        <v>22.26</v>
       </c>
       <c r="F52" t="n">
-        <v>50.66</v>
+        <v>21.45</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2804,7 +2804,7 @@
         <v>52</v>
       </c>
       <c r="I52" t="n">
-        <v>2.193</v>
+        <v>2.645</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -2813,18 +2813,18 @@
         <v>1</v>
       </c>
       <c r="L52" t="n">
-        <v>2.4</v>
+        <v>4.15</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>sh600362</t>
+          <t>sh600226</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>江西铜业</t>
+          <t>亨通股份</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2833,13 +2833,13 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>45.1</v>
+        <v>5.39</v>
       </c>
       <c r="E53" t="n">
-        <v>44.96</v>
+        <v>5.3</v>
       </c>
       <c r="F53" t="n">
-        <v>43.71</v>
+        <v>5.03</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2850,7 +2850,7 @@
         <v>52</v>
       </c>
       <c r="I53" t="n">
-        <v>0.6919999999999999</v>
+        <v>3.455</v>
       </c>
       <c r="J53" t="n">
         <v>0</v>
@@ -2859,18 +2859,18 @@
         <v>1</v>
       </c>
       <c r="L53" t="n">
-        <v>7.36</v>
+        <v>2.65</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>sh600361</t>
+          <t>sh600546</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>创新新材</t>
+          <t>山煤国际</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2879,13 +2879,13 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>4.65</v>
+        <v>12.94</v>
       </c>
       <c r="E54" t="n">
-        <v>4.58</v>
+        <v>12.73</v>
       </c>
       <c r="F54" t="n">
-        <v>4.4</v>
+        <v>12.32</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2896,7 +2896,7 @@
         <v>52</v>
       </c>
       <c r="I54" t="n">
-        <v>3.563</v>
+        <v>2.944</v>
       </c>
       <c r="J54" t="n">
         <v>0</v>
@@ -2905,18 +2905,18 @@
         <v>1</v>
       </c>
       <c r="L54" t="n">
-        <v>2.57</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>sh600351</t>
+          <t>sh600545</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>亚宝药业</t>
+          <t>卓郎智能</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2925,13 +2925,13 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>6.75</v>
+        <v>4.88</v>
       </c>
       <c r="E55" t="n">
-        <v>6.6</v>
+        <v>4.82</v>
       </c>
       <c r="F55" t="n">
-        <v>6.35</v>
+        <v>4.41</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2942,7 +2942,7 @@
         <v>52</v>
       </c>
       <c r="I55" t="n">
-        <v>5.14</v>
+        <v>2.954</v>
       </c>
       <c r="J55" t="n">
         <v>0</v>
@@ -2951,18 +2951,18 @@
         <v>1</v>
       </c>
       <c r="L55" t="n">
-        <v>2.08</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>sh600345</t>
+          <t>sh600535</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>长江通信</t>
+          <t>天士力</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2971,13 +2971,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>52.62</v>
+        <v>14.99</v>
       </c>
       <c r="E56" t="n">
-        <v>51.57</v>
+        <v>14.94</v>
       </c>
       <c r="F56" t="n">
-        <v>49.54</v>
+        <v>14.67</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2988,7 +2988,7 @@
         <v>52</v>
       </c>
       <c r="I56" t="n">
-        <v>4.405</v>
+        <v>2.531</v>
       </c>
       <c r="J56" t="n">
         <v>0</v>
@@ -2997,18 +2997,18 @@
         <v>1</v>
       </c>
       <c r="L56" t="n">
-        <v>5.21</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>sh600333</t>
+          <t>sh600531</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>长春燃气</t>
+          <t>豫光金铅</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3017,13 +3017,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>5.73</v>
+        <v>16</v>
       </c>
       <c r="E57" t="n">
-        <v>5.68</v>
+        <v>15.79</v>
       </c>
       <c r="F57" t="n">
-        <v>5.49</v>
+        <v>15.07</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -3034,7 +3034,7 @@
         <v>52</v>
       </c>
       <c r="I57" t="n">
-        <v>3.058</v>
+        <v>2.828</v>
       </c>
       <c r="J57" t="n">
         <v>0</v>
@@ -3043,18 +3043,18 @@
         <v>1</v>
       </c>
       <c r="L57" t="n">
-        <v>0.95</v>
+        <v>7.71</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>sh600331</t>
+          <t>sh600515</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>宏达股份</t>
+          <t>海南机场</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3063,13 +3063,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>18.72</v>
+        <v>3.44</v>
       </c>
       <c r="E58" t="n">
-        <v>18.44</v>
+        <v>3.42</v>
       </c>
       <c r="F58" t="n">
-        <v>17.72</v>
+        <v>3.3</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -3080,7 +3080,7 @@
         <v>52</v>
       </c>
       <c r="I58" t="n">
-        <v>2.632</v>
+        <v>0.88</v>
       </c>
       <c r="J58" t="n">
         <v>0</v>
@@ -3089,18 +3089,18 @@
         <v>1</v>
       </c>
       <c r="L58" t="n">
-        <v>7.08</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>sh600323</t>
+          <t>sh600513</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>瀚蓝环境</t>
+          <t>联环药业</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3109,13 +3109,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>30.99</v>
+        <v>20.34</v>
       </c>
       <c r="E59" t="n">
-        <v>30.86</v>
+        <v>20.3</v>
       </c>
       <c r="F59" t="n">
-        <v>29.14</v>
+        <v>19.53</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -3126,7 +3126,7 @@
         <v>52</v>
       </c>
       <c r="I59" t="n">
-        <v>2.65</v>
+        <v>0.643</v>
       </c>
       <c r="J59" t="n">
         <v>0</v>
@@ -3135,18 +3135,18 @@
         <v>1</v>
       </c>
       <c r="L59" t="n">
-        <v>2.5</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>sh600600</t>
+          <t>sh600510</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>青岛啤酒</t>
+          <t>黑牡丹</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3155,13 +3155,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>62.05</v>
+        <v>11.28</v>
       </c>
       <c r="E60" t="n">
-        <v>61.88</v>
+        <v>11.08</v>
       </c>
       <c r="F60" t="n">
-        <v>60.52</v>
+        <v>10.56</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -3172,7 +3172,7 @@
         <v>52</v>
       </c>
       <c r="I60" t="n">
-        <v>0.6</v>
+        <v>3.014</v>
       </c>
       <c r="J60" t="n">
         <v>0</v>
@@ -3181,18 +3181,18 @@
         <v>1</v>
       </c>
       <c r="L60" t="n">
-        <v>1.48</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>sh600580</t>
+          <t>sh600501</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>卧龙电驱</t>
+          <t>航天晨光</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3201,13 +3201,13 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>38.07</v>
+        <v>23.09</v>
       </c>
       <c r="E61" t="n">
-        <v>37.96</v>
+        <v>23.22</v>
       </c>
       <c r="F61" t="n">
-        <v>36.68</v>
+        <v>22.54</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -3218,7 +3218,7 @@
         <v>52</v>
       </c>
       <c r="I61" t="n">
-        <v>0.981</v>
+        <v>1.139</v>
       </c>
       <c r="J61" t="n">
         <v>0</v>
@@ -3227,18 +3227,18 @@
         <v>1</v>
       </c>
       <c r="L61" t="n">
-        <v>5.71</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>sh600575</t>
+          <t>sh600499</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>淮河能源</t>
+          <t>科达制造</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3247,13 +3247,13 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>3.84</v>
+        <v>20.17</v>
       </c>
       <c r="E62" t="n">
-        <v>3.74</v>
+        <v>20.18</v>
       </c>
       <c r="F62" t="n">
-        <v>3.58</v>
+        <v>19.58</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -3264,7 +3264,7 @@
         <v>52</v>
       </c>
       <c r="I62" t="n">
-        <v>4.632</v>
+        <v>1.817</v>
       </c>
       <c r="J62" t="n">
         <v>0</v>
@@ -3273,18 +3273,18 @@
         <v>1</v>
       </c>
       <c r="L62" t="n">
-        <v>2.81</v>
+        <v>9.75</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>sh600573</t>
+          <t>sh600489</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>惠泉啤酒</t>
+          <t>中金黄金</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3293,13 +3293,13 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>13.3</v>
+        <v>25.77</v>
       </c>
       <c r="E63" t="n">
-        <v>13.15</v>
+        <v>25.7</v>
       </c>
       <c r="F63" t="n">
-        <v>12.66</v>
+        <v>24.84</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -3310,7 +3310,7 @@
         <v>52</v>
       </c>
       <c r="I63" t="n">
-        <v>3.583</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J63" t="n">
         <v>0</v>
@@ -3319,18 +3319,18 @@
         <v>1</v>
       </c>
       <c r="L63" t="n">
-        <v>1.37</v>
+        <v>8.06</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>sh600570</t>
+          <t>sh600483</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>恒生电子</t>
+          <t>福能股份</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3339,13 +3339,13 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>26.49</v>
+        <v>9.94</v>
       </c>
       <c r="E64" t="n">
-        <v>26.35</v>
+        <v>9.91</v>
       </c>
       <c r="F64" t="n">
-        <v>25.55</v>
+        <v>9.5</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -3356,7 +3356,7 @@
         <v>52</v>
       </c>
       <c r="I64" t="n">
-        <v>1.107</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="J64" t="n">
         <v>0</v>
@@ -3365,18 +3365,18 @@
         <v>1</v>
       </c>
       <c r="L64" t="n">
-        <v>3.09</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>sh600550</t>
+          <t>sh600460</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>保变电气</t>
+          <t>士兰微</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3385,13 +3385,13 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>15.33</v>
+        <v>28.19</v>
       </c>
       <c r="E65" t="n">
-        <v>15.17</v>
+        <v>28.04</v>
       </c>
       <c r="F65" t="n">
-        <v>14.48</v>
+        <v>27.15</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -3402,7 +3402,7 @@
         <v>52</v>
       </c>
       <c r="I65" t="n">
-        <v>2.064</v>
+        <v>1.33</v>
       </c>
       <c r="J65" t="n">
         <v>0</v>
@@ -3411,18 +3411,18 @@
         <v>1</v>
       </c>
       <c r="L65" t="n">
-        <v>4.64</v>
+        <v>7.62</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>sh600546</t>
+          <t>sh600446</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>山煤国际</t>
+          <t>金证股份</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3431,14 +3431,14 @@
         </is>
       </c>
       <c r="D66" t="n">
+        <v>13.66</v>
+      </c>
+      <c r="E66" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F66" t="n">
         <v>12.9</v>
       </c>
-      <c r="E66" t="n">
-        <v>12.73</v>
-      </c>
-      <c r="F66" t="n">
-        <v>12.32</v>
-      </c>
       <c r="G66" t="inlineStr">
         <is>
           <t>潜伏蓄势</t>
@@ -3448,7 +3448,7 @@
         <v>52</v>
       </c>
       <c r="I66" t="n">
-        <v>2.625</v>
+        <v>2.476</v>
       </c>
       <c r="J66" t="n">
         <v>0</v>
@@ -3457,18 +3457,18 @@
         <v>1</v>
       </c>
       <c r="L66" t="n">
-        <v>2.41</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>sh600545</t>
+          <t>sh600429</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>卓郎智能</t>
+          <t>三元股份</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3477,13 +3477,13 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>4.89</v>
+        <v>6.1</v>
       </c>
       <c r="E67" t="n">
-        <v>4.82</v>
+        <v>6.11</v>
       </c>
       <c r="F67" t="n">
-        <v>4.41</v>
+        <v>5.89</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -3494,7 +3494,7 @@
         <v>52</v>
       </c>
       <c r="I67" t="n">
-        <v>3.165</v>
+        <v>1.498</v>
       </c>
       <c r="J67" t="n">
         <v>0</v>
@@ -3503,18 +3503,18 @@
         <v>1</v>
       </c>
       <c r="L67" t="n">
-        <v>7.25</v>
+        <v>2.66</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>sh600535</t>
+          <t>sh600426</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>天士力</t>
+          <t>华鲁恒升</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3523,13 +3523,13 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>14.99</v>
+        <v>37.96</v>
       </c>
       <c r="E68" t="n">
-        <v>14.94</v>
+        <v>37.83</v>
       </c>
       <c r="F68" t="n">
-        <v>14.68</v>
+        <v>36.31</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -3540,7 +3540,7 @@
         <v>52</v>
       </c>
       <c r="I68" t="n">
-        <v>2.531</v>
+        <v>0.904</v>
       </c>
       <c r="J68" t="n">
         <v>0</v>
@@ -3549,18 +3549,18 @@
         <v>1</v>
       </c>
       <c r="L68" t="n">
-        <v>4.19</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>sh600531</t>
+          <t>sh600378</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>豫光金铅</t>
+          <t>昊华科技</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3569,13 +3569,13 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>16.06</v>
+        <v>35.57</v>
       </c>
       <c r="E69" t="n">
-        <v>15.79</v>
+        <v>35.52</v>
       </c>
       <c r="F69" t="n">
-        <v>15.07</v>
+        <v>34.3</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -3586,7 +3586,7 @@
         <v>52</v>
       </c>
       <c r="I69" t="n">
-        <v>3.213</v>
+        <v>0.908</v>
       </c>
       <c r="J69" t="n">
         <v>0</v>
@@ -3595,18 +3595,18 @@
         <v>1</v>
       </c>
       <c r="L69" t="n">
-        <v>7.35</v>
+        <v>3.69</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>sh600515</t>
+          <t>sh600698</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>海南机场</t>
+          <t>湖南天雁</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3615,13 +3615,13 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>3.43</v>
+        <v>7.3</v>
       </c>
       <c r="E70" t="n">
-        <v>3.42</v>
+        <v>7.16</v>
       </c>
       <c r="F70" t="n">
-        <v>3.3</v>
+        <v>7.05</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -3632,7 +3632,7 @@
         <v>52</v>
       </c>
       <c r="I70" t="n">
-        <v>0.587</v>
+        <v>3.693</v>
       </c>
       <c r="J70" t="n">
         <v>0</v>
@@ -3641,18 +3641,18 @@
         <v>1</v>
       </c>
       <c r="L70" t="n">
-        <v>1.31</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>sh600513</t>
+          <t>sh600694</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>联环药业</t>
+          <t>大商股份</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3661,13 +3661,13 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>20.4</v>
+        <v>18.37</v>
       </c>
       <c r="E71" t="n">
-        <v>20.29</v>
+        <v>18.18</v>
       </c>
       <c r="F71" t="n">
-        <v>19.53</v>
+        <v>17.52</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -3678,7 +3678,7 @@
         <v>52</v>
       </c>
       <c r="I71" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.886</v>
       </c>
       <c r="J71" t="n">
         <v>0</v>
@@ -3687,18 +3687,18 @@
         <v>1</v>
       </c>
       <c r="L71" t="n">
-        <v>1.28</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>sh600510</t>
+          <t>sh600686</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>黑牡丹</t>
+          <t>金龙汽车</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3707,13 +3707,13 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>11.28</v>
+        <v>17.35</v>
       </c>
       <c r="E72" t="n">
-        <v>11.08</v>
+        <v>17.37</v>
       </c>
       <c r="F72" t="n">
-        <v>10.56</v>
+        <v>16.76</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -3724,7 +3724,7 @@
         <v>52</v>
       </c>
       <c r="I72" t="n">
-        <v>3.014</v>
+        <v>0.931</v>
       </c>
       <c r="J72" t="n">
         <v>0</v>
@@ -3733,18 +3733,18 @@
         <v>1</v>
       </c>
       <c r="L72" t="n">
-        <v>1.42</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>sh600501</t>
+          <t>sh600674</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>航天晨光</t>
+          <t>川投能源</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3753,13 +3753,13 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>23.15</v>
+        <v>15.03</v>
       </c>
       <c r="E73" t="n">
-        <v>23.22</v>
+        <v>14.99</v>
       </c>
       <c r="F73" t="n">
-        <v>22.54</v>
+        <v>14.5</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -3770,7 +3770,7 @@
         <v>52</v>
       </c>
       <c r="I73" t="n">
-        <v>1.402</v>
+        <v>0.67</v>
       </c>
       <c r="J73" t="n">
         <v>0</v>
@@ -3779,18 +3779,18 @@
         <v>1</v>
       </c>
       <c r="L73" t="n">
-        <v>1.43</v>
+        <v>2.08</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>sh600499</t>
+          <t>sh600667</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>科达制造</t>
+          <t>太极实业</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3799,13 +3799,13 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>20.23</v>
+        <v>9.85</v>
       </c>
       <c r="E74" t="n">
-        <v>20.18</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F74" t="n">
-        <v>19.58</v>
+        <v>9.51</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -3816,7 +3816,7 @@
         <v>52</v>
       </c>
       <c r="I74" t="n">
-        <v>2.12</v>
+        <v>1.442</v>
       </c>
       <c r="J74" t="n">
         <v>0</v>
@@ -3825,18 +3825,18 @@
         <v>1</v>
       </c>
       <c r="L74" t="n">
-        <v>9.460000000000001</v>
+        <v>6.27</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>sh600489</t>
+          <t>sh600660</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>中金黄金</t>
+          <t>福耀玻璃</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3845,13 +3845,13 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>25.89</v>
+        <v>60.55</v>
       </c>
       <c r="E75" t="n">
-        <v>25.7</v>
+        <v>59.81</v>
       </c>
       <c r="F75" t="n">
-        <v>24.84</v>
+        <v>57.47</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -3862,7 +3862,7 @@
         <v>52</v>
       </c>
       <c r="I75" t="n">
-        <v>1.41</v>
+        <v>2.575</v>
       </c>
       <c r="J75" t="n">
         <v>0</v>
@@ -3871,18 +3871,18 @@
         <v>1</v>
       </c>
       <c r="L75" t="n">
-        <v>7.64</v>
+        <v>6.38</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>sh600759</t>
+          <t>sh600629</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>洲际油气</t>
+          <t>华建集团</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3891,13 +3891,13 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>5.22</v>
+        <v>20.44</v>
       </c>
       <c r="E76" t="n">
-        <v>5.2</v>
+        <v>20.26</v>
       </c>
       <c r="F76" t="n">
-        <v>4.95</v>
+        <v>19.28</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -3908,7 +3908,7 @@
         <v>52</v>
       </c>
       <c r="I76" t="n">
-        <v>0.967</v>
+        <v>2.405</v>
       </c>
       <c r="J76" t="n">
         <v>0</v>
@@ -3917,18 +3917,18 @@
         <v>1</v>
       </c>
       <c r="L76" t="n">
-        <v>8.4</v>
+        <v>2.86</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>sh600758</t>
+          <t>sh600617</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>辽宁能源</t>
+          <t>国新能源</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3937,13 +3937,13 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>4.08</v>
+        <v>3.38</v>
       </c>
       <c r="E77" t="n">
-        <v>4.03</v>
+        <v>3.35</v>
       </c>
       <c r="F77" t="n">
-        <v>3.82</v>
+        <v>3.2</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -3954,7 +3954,7 @@
         <v>52</v>
       </c>
       <c r="I77" t="n">
-        <v>2.513</v>
+        <v>1.807</v>
       </c>
       <c r="J77" t="n">
         <v>0</v>
@@ -3963,18 +3963,18 @@
         <v>1</v>
       </c>
       <c r="L77" t="n">
-        <v>2.09</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>sh600745</t>
+          <t>sh600605</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>闻泰科技</t>
+          <t>汇通能源</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3983,13 +3983,13 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>28.12</v>
+        <v>32.99</v>
       </c>
       <c r="E78" t="n">
-        <v>28</v>
+        <v>32.73</v>
       </c>
       <c r="F78" t="n">
-        <v>26.38</v>
+        <v>31.21</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -4000,7 +4000,7 @@
         <v>52</v>
       </c>
       <c r="I78" t="n">
-        <v>1.115</v>
+        <v>3.677</v>
       </c>
       <c r="J78" t="n">
         <v>0</v>
@@ -4009,18 +4009,18 @@
         <v>1</v>
       </c>
       <c r="L78" t="n">
-        <v>7.61</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>sh600733</t>
+          <t>sh600602</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>北汽蓝谷</t>
+          <t>云赛智联</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -4029,13 +4029,13 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>7.52</v>
+        <v>22.6</v>
       </c>
       <c r="E79" t="n">
-        <v>7.3</v>
+        <v>22.42</v>
       </c>
       <c r="F79" t="n">
-        <v>7.11</v>
+        <v>21.17</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -4046,7 +4046,7 @@
         <v>52</v>
       </c>
       <c r="I79" t="n">
-        <v>5.175</v>
+        <v>1.71</v>
       </c>
       <c r="J79" t="n">
         <v>0</v>
@@ -4055,18 +4055,18 @@
         <v>1</v>
       </c>
       <c r="L79" t="n">
-        <v>8.26</v>
+        <v>7.78</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>sh600707</t>
+          <t>sh600600</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>彩虹股份</t>
+          <t>青岛啤酒</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4075,13 +4075,13 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>8.289999999999999</v>
+        <v>62.07</v>
       </c>
       <c r="E80" t="n">
-        <v>8.23</v>
+        <v>61.88</v>
       </c>
       <c r="F80" t="n">
-        <v>7.85</v>
+        <v>60.52</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -4092,7 +4092,7 @@
         <v>52</v>
       </c>
       <c r="I80" t="n">
-        <v>2.726</v>
+        <v>0.632</v>
       </c>
       <c r="J80" t="n">
         <v>0</v>
@@ -4101,18 +4101,18 @@
         <v>1</v>
       </c>
       <c r="L80" t="n">
-        <v>7.25</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>sh600698</t>
+          <t>sh600580</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>湖南天雁</t>
+          <t>卧龙电驱</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4121,13 +4121,13 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>7.32</v>
+        <v>38.02</v>
       </c>
       <c r="E81" t="n">
-        <v>7.16</v>
+        <v>37.96</v>
       </c>
       <c r="F81" t="n">
-        <v>7.05</v>
+        <v>36.68</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -4138,7 +4138,7 @@
         <v>52</v>
       </c>
       <c r="I81" t="n">
-        <v>3.977</v>
+        <v>0.849</v>
       </c>
       <c r="J81" t="n">
         <v>0</v>
@@ -4147,18 +4147,18 @@
         <v>1</v>
       </c>
       <c r="L81" t="n">
-        <v>0.86</v>
+        <v>5.91</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>sh600694</t>
+          <t>sh600575</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>大商股份</t>
+          <t>淮河能源</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4167,13 +4167,13 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>18.34</v>
+        <v>3.82</v>
       </c>
       <c r="E82" t="n">
-        <v>18.15</v>
+        <v>3.74</v>
       </c>
       <c r="F82" t="n">
-        <v>17.52</v>
+        <v>3.58</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -4184,7 +4184,7 @@
         <v>52</v>
       </c>
       <c r="I82" t="n">
-        <v>1.719</v>
+        <v>4.087</v>
       </c>
       <c r="J82" t="n">
         <v>0</v>
@@ -4193,7 +4193,7 @@
         <v>1</v>
       </c>
       <c r="L82" t="n">
-        <v>1.06</v>
+        <v>2.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 实时报告更新 Tue Apr 28 04:56:02 UTC 2026
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>T:2026-04-27 12:50:32</t>
+          <t>T:2026-04-28 12:56:01</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -519,12 +519,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>sz301696</t>
+          <t>sz301389</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>三瑞智能</t>
+          <t>隆扬电子</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -533,13 +533,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>94.33</v>
+        <v>64.36</v>
       </c>
       <c r="E3" t="n">
-        <v>93.76000000000001</v>
+        <v>62.46</v>
       </c>
       <c r="F3" t="n">
-        <v>88.06999999999999</v>
+        <v>59.12</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -550,7 +550,7 @@
         <v>52</v>
       </c>
       <c r="I3" t="n">
-        <v>1.387</v>
+        <v>5.009</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -559,18 +559,18 @@
         <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>4.44</v>
+        <v>4.74</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>bj920012</t>
+          <t>sz301387</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>创达新材</t>
+          <t>光大同创</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -579,13 +579,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>58.06</v>
+        <v>62.88</v>
       </c>
       <c r="E4" t="n">
-        <v>57.41</v>
+        <v>61.92</v>
       </c>
       <c r="F4" t="n">
-        <v>54.9</v>
+        <v>58.33</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
         <v>52</v>
       </c>
       <c r="I4" t="n">
-        <v>2.761</v>
+        <v>3.167</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -605,18 +605,18 @@
         <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>1.1</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>bj920045</t>
+          <t>sz301382</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>蘅东光</t>
+          <t>蜂助手</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -625,13 +625,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>562.6799999999999</v>
+        <v>42.28</v>
       </c>
       <c r="E5" t="n">
-        <v>549.22</v>
+        <v>41.71</v>
       </c>
       <c r="F5" t="n">
-        <v>527.24</v>
+        <v>39.2</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
         <v>52</v>
       </c>
       <c r="I5" t="n">
-        <v>5.174</v>
+        <v>3.78</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -651,18 +651,18 @@
         <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>4.8</v>
+        <v>7.05</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>sz301529</t>
+          <t>sz301365</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>福赛科技</t>
+          <t>矩阵股份</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -671,13 +671,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>121.44</v>
+        <v>34.95</v>
       </c>
       <c r="E6" t="n">
-        <v>121.77</v>
+        <v>35.37</v>
       </c>
       <c r="F6" t="n">
-        <v>116.08</v>
+        <v>33.63</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         <v>52</v>
       </c>
       <c r="I6" t="n">
-        <v>2.524</v>
+        <v>0.518</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -697,18 +697,18 @@
         <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>2.78</v>
+        <v>1.59</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>sz301479</t>
+          <t>sz301360</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>弘景光电</t>
+          <t>荣旗科技</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -717,13 +717,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>108.75</v>
+        <v>83.45999999999999</v>
       </c>
       <c r="E7" t="n">
-        <v>109.06</v>
+        <v>83.59</v>
       </c>
       <c r="F7" t="n">
-        <v>105.64</v>
+        <v>80.41</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -734,7 +734,7 @@
         <v>52</v>
       </c>
       <c r="I7" t="n">
-        <v>1.116</v>
+        <v>1.041</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -743,18 +743,18 @@
         <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>1.61</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>sz301458</t>
+          <t>sz301348</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>钧崴电子</t>
+          <t>蓝箭电子</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -763,13 +763,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>40.08</v>
+        <v>24.5</v>
       </c>
       <c r="E8" t="n">
-        <v>39.93</v>
+        <v>24.61</v>
       </c>
       <c r="F8" t="n">
-        <v>38.67</v>
+        <v>23.55</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -780,7 +780,7 @@
         <v>52</v>
       </c>
       <c r="I8" t="n">
-        <v>1.752</v>
+        <v>0.699</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -789,18 +789,18 @@
         <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>2.16</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>sz301421</t>
+          <t>sz301328</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>波长光电</t>
+          <t>维峰电子</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -809,13 +809,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>99.67</v>
+        <v>61.09</v>
       </c>
       <c r="E9" t="n">
-        <v>97.95999999999999</v>
+        <v>60.49</v>
       </c>
       <c r="F9" t="n">
-        <v>94.02</v>
+        <v>58.32</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -826,7 +826,7 @@
         <v>52</v>
       </c>
       <c r="I9" t="n">
-        <v>3.736</v>
+        <v>2.157</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -835,18 +835,18 @@
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>3.66</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>sz301419</t>
+          <t>sz301327</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>阿莱德</t>
+          <t>华宝新能</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -855,13 +855,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>42.09</v>
+        <v>62.03</v>
       </c>
       <c r="E10" t="n">
-        <v>41.95</v>
+        <v>61.93</v>
       </c>
       <c r="F10" t="n">
-        <v>40.48</v>
+        <v>59.49</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -872,7 +872,7 @@
         <v>52</v>
       </c>
       <c r="I10" t="n">
-        <v>1.275</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -881,18 +881,18 @@
         <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>1.02</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>sz301408</t>
+          <t>sz301326</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>华人健康</t>
+          <t>捷邦科技</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -901,13 +901,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>20.13</v>
+        <v>159.86</v>
       </c>
       <c r="E11" t="n">
-        <v>20.16</v>
+        <v>160.23</v>
       </c>
       <c r="F11" t="n">
-        <v>19.21</v>
+        <v>153.86</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -918,7 +918,7 @@
         <v>52</v>
       </c>
       <c r="I11" t="n">
-        <v>1.667</v>
+        <v>0.775</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -927,18 +927,18 @@
         <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>3.32</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>sz301395</t>
+          <t>sz301323</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>仁信新材</t>
+          <t>新莱福</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -947,13 +947,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>12.98</v>
+        <v>67.79000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>12.93</v>
+        <v>67.95</v>
       </c>
       <c r="F12" t="n">
-        <v>11.76</v>
+        <v>65.93000000000001</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         <v>52</v>
       </c>
       <c r="I12" t="n">
-        <v>1.565</v>
+        <v>1.361</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -973,18 +973,18 @@
         <v>1</v>
       </c>
       <c r="L12" t="n">
-        <v>1.13</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>sz301393</t>
+          <t>sz301321</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>昊帆生物</t>
+          <t>翰博高新</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -993,13 +993,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>61.02</v>
+        <v>24.46</v>
       </c>
       <c r="E13" t="n">
-        <v>60.94</v>
+        <v>23.98</v>
       </c>
       <c r="F13" t="n">
-        <v>58.39</v>
+        <v>22.94</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
         <v>52</v>
       </c>
       <c r="I13" t="n">
-        <v>1.819</v>
+        <v>3.556</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -1019,18 +1019,18 @@
         <v>1</v>
       </c>
       <c r="L13" t="n">
-        <v>1.18</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>sz301382</t>
+          <t>sz301317</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>蜂助手</t>
+          <t>鑫磊股份</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1039,13 +1039,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>40.96</v>
+        <v>56.89</v>
       </c>
       <c r="E14" t="n">
-        <v>40.65</v>
+        <v>56.12</v>
       </c>
       <c r="F14" t="n">
-        <v>38.22</v>
+        <v>53.53</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
         <v>52</v>
       </c>
       <c r="I14" t="n">
-        <v>2.043</v>
+        <v>4.366</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -1065,18 +1065,18 @@
         <v>1</v>
       </c>
       <c r="L14" t="n">
-        <v>4.22</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>sz301378</t>
+          <t>sz301312</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>通达海</t>
+          <t>智立方</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1085,13 +1085,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>31.56</v>
+        <v>118.34</v>
       </c>
       <c r="E15" t="n">
-        <v>32.33</v>
+        <v>116.42</v>
       </c>
       <c r="F15" t="n">
-        <v>30.85</v>
+        <v>107.41</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1102,7 +1102,7 @@
         <v>52</v>
       </c>
       <c r="I15" t="n">
-        <v>0.766</v>
+        <v>2.779</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -1111,18 +1111,18 @@
         <v>1</v>
       </c>
       <c r="L15" t="n">
-        <v>1.53</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>sz301371</t>
+          <t>sz301285</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>敷尔佳</t>
+          <t>鸿日达</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1131,13 +1131,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>29.07</v>
+        <v>107.39</v>
       </c>
       <c r="E16" t="n">
-        <v>28.54</v>
+        <v>107.36</v>
       </c>
       <c r="F16" t="n">
-        <v>27.41</v>
+        <v>100.98</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
         <v>52</v>
       </c>
       <c r="I16" t="n">
-        <v>3.933</v>
+        <v>1.283</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1157,18 +1157,18 @@
         <v>1</v>
       </c>
       <c r="L16" t="n">
-        <v>2.28</v>
+        <v>2.06</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>sz301369</t>
+          <t>sz301282</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>联动科技</t>
+          <t>金禄电子</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1177,13 +1177,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>168.67</v>
+        <v>45.22</v>
       </c>
       <c r="E17" t="n">
-        <v>167.98</v>
+        <v>45.55</v>
       </c>
       <c r="F17" t="n">
-        <v>163.06</v>
+        <v>43.23</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1194,7 +1194,7 @@
         <v>52</v>
       </c>
       <c r="I17" t="n">
-        <v>1.541</v>
+        <v>0.713</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1203,18 +1203,18 @@
         <v>1</v>
       </c>
       <c r="L17" t="n">
-        <v>1.31</v>
+        <v>3.07</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>sz301366</t>
+          <t>sz301281</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>一博科技</t>
+          <t>科源制药</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1223,13 +1223,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>37.41</v>
+        <v>39</v>
       </c>
       <c r="E18" t="n">
-        <v>37.31</v>
+        <v>38.21</v>
       </c>
       <c r="F18" t="n">
-        <v>36.11</v>
+        <v>36.34</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1240,7 +1240,7 @@
         <v>52</v>
       </c>
       <c r="I18" t="n">
-        <v>1.382</v>
+        <v>4.028</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1249,18 +1249,18 @@
         <v>1</v>
       </c>
       <c r="L18" t="n">
-        <v>0.8</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>sz301365</t>
+          <t>sh600325</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>矩阵股份</t>
+          <t>华发股份</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1269,13 +1269,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>34.75</v>
+        <v>3.41</v>
       </c>
       <c r="E19" t="n">
-        <v>33.97</v>
+        <v>3.44</v>
       </c>
       <c r="F19" t="n">
-        <v>32.01</v>
+        <v>3.29</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1286,7 +1286,7 @@
         <v>52</v>
       </c>
       <c r="I19" t="n">
-        <v>4.198</v>
+        <v>0.888</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1295,18 +1295,18 @@
         <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>1.29</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>sz301362</t>
+          <t>sh600323</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>民爆光电</t>
+          <t>瀚蓝环境</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1315,13 +1315,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>143.21</v>
+        <v>31.25</v>
       </c>
       <c r="E20" t="n">
-        <v>142.84</v>
+        <v>31.03</v>
       </c>
       <c r="F20" t="n">
-        <v>137.2</v>
+        <v>29.9</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1332,7 +1332,7 @@
         <v>52</v>
       </c>
       <c r="I20" t="n">
-        <v>1.116</v>
+        <v>1.395</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1341,18 +1341,18 @@
         <v>1</v>
       </c>
       <c r="L20" t="n">
-        <v>2.03</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>sz301348</t>
+          <t>sh600315</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>蓝箭电子</t>
+          <t>上海家化</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1361,13 +1361,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>24.18</v>
+        <v>20.82</v>
       </c>
       <c r="E21" t="n">
-        <v>24.01</v>
+        <v>21.12</v>
       </c>
       <c r="F21" t="n">
-        <v>22.94</v>
+        <v>20.36</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1378,7 +1378,7 @@
         <v>52</v>
       </c>
       <c r="I21" t="n">
-        <v>1.469</v>
+        <v>0.823</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1387,18 +1387,18 @@
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>1.53</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>sh600207</t>
+          <t>sh600285</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>安彩高科</t>
+          <t>羚锐制药</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1407,13 +1407,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>5.88</v>
+        <v>22.5</v>
       </c>
       <c r="E22" t="n">
-        <v>5.9</v>
+        <v>21.98</v>
       </c>
       <c r="F22" t="n">
-        <v>5.69</v>
+        <v>21.89</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1424,7 +1424,7 @@
         <v>52</v>
       </c>
       <c r="I22" t="n">
-        <v>0.6850000000000001</v>
+        <v>4.895</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1433,18 +1433,18 @@
         <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>0.8100000000000001</v>
+        <v>4.43</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>sh600203</t>
+          <t>sh600282</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>福日电子</t>
+          <t>南钢股份</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1453,13 +1453,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>12.53</v>
+        <v>5.32</v>
       </c>
       <c r="E23" t="n">
-        <v>12.24</v>
+        <v>5.27</v>
       </c>
       <c r="F23" t="n">
-        <v>11.58</v>
+        <v>5.08</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1470,7 +1470,7 @@
         <v>52</v>
       </c>
       <c r="I23" t="n">
-        <v>4.243</v>
+        <v>1.916</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1479,18 +1479,18 @@
         <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>3.47</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>sh600198</t>
+          <t>sh600262</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>大唐电信</t>
+          <t>北方股份</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1499,13 +1499,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>8.210000000000001</v>
+        <v>23.61</v>
       </c>
       <c r="E24" t="n">
-        <v>8.18</v>
+        <v>23.43</v>
       </c>
       <c r="F24" t="n">
-        <v>7.82</v>
+        <v>22.26</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1516,7 +1516,7 @@
         <v>52</v>
       </c>
       <c r="I24" t="n">
-        <v>0.736</v>
+        <v>2.697</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1525,18 +1525,18 @@
         <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>0.87</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>sh600188</t>
+          <t>sh600256</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>兖矿能源</t>
+          <t>广汇能源</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1545,13 +1545,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>20.98</v>
+        <v>6.4</v>
       </c>
       <c r="E25" t="n">
-        <v>20.91</v>
+        <v>6.31</v>
       </c>
       <c r="F25" t="n">
-        <v>19.97</v>
+        <v>6.07</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1562,7 +1562,7 @@
         <v>52</v>
       </c>
       <c r="I25" t="n">
-        <v>1.451</v>
+        <v>2.564</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1571,18 +1571,18 @@
         <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>6.34</v>
+        <v>7.69</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sh600185</t>
+          <t>sh600236</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>珠免集团</t>
+          <t>桂冠电力</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1591,13 +1591,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>5.99</v>
+        <v>9.76</v>
       </c>
       <c r="E26" t="n">
-        <v>5.96</v>
+        <v>9.66</v>
       </c>
       <c r="F26" t="n">
-        <v>5.71</v>
+        <v>9.31</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1608,7 +1608,7 @@
         <v>52</v>
       </c>
       <c r="I26" t="n">
-        <v>1.182</v>
+        <v>2.413</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1617,18 +1617,18 @@
         <v>1</v>
       </c>
       <c r="L26" t="n">
-        <v>0.97</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>sh600172</t>
+          <t>sh600234</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>黄河旋风</t>
+          <t>科新发展</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1637,13 +1637,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>8.4</v>
+        <v>23.97</v>
       </c>
       <c r="E27" t="n">
-        <v>8.41</v>
+        <v>24</v>
       </c>
       <c r="F27" t="n">
-        <v>8.1</v>
+        <v>22.64</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1654,7 +1654,7 @@
         <v>52</v>
       </c>
       <c r="I27" t="n">
-        <v>1.205</v>
+        <v>1.697</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1663,18 +1663,18 @@
         <v>1</v>
       </c>
       <c r="L27" t="n">
-        <v>4.23</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>sh600171</t>
+          <t>sh600230</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>上海贝岭</t>
+          <t>沧州大化</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1683,13 +1683,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>29.3</v>
+        <v>19.17</v>
       </c>
       <c r="E28" t="n">
-        <v>28.91</v>
+        <v>19.07</v>
       </c>
       <c r="F28" t="n">
-        <v>27.5</v>
+        <v>18.38</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1700,7 +1700,7 @@
         <v>52</v>
       </c>
       <c r="I28" t="n">
-        <v>3.024</v>
+        <v>1.375</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1709,18 +1709,18 @@
         <v>1</v>
       </c>
       <c r="L28" t="n">
-        <v>5.34</v>
+        <v>1.39</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>sh600160</t>
+          <t>sh600216</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>巨化股份</t>
+          <t>浙江医药</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1729,13 +1729,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>36.01</v>
+        <v>14.67</v>
       </c>
       <c r="E29" t="n">
-        <v>35.49</v>
+        <v>14.63</v>
       </c>
       <c r="F29" t="n">
-        <v>34.21</v>
+        <v>14.24</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1746,7 +1746,7 @@
         <v>52</v>
       </c>
       <c r="I29" t="n">
-        <v>2.739</v>
+        <v>0.755</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1755,18 +1755,18 @@
         <v>1</v>
       </c>
       <c r="L29" t="n">
-        <v>11.61</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>sh600158</t>
+          <t>sh600188</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>中体产业</t>
+          <t>兖矿能源</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1775,13 +1775,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>10.72</v>
+        <v>21.36</v>
       </c>
       <c r="E30" t="n">
-        <v>10.62</v>
+        <v>21.08</v>
       </c>
       <c r="F30" t="n">
-        <v>9.960000000000001</v>
+        <v>20.22</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1792,7 +1792,7 @@
         <v>52</v>
       </c>
       <c r="I30" t="n">
-        <v>2.388</v>
+        <v>2.692</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1801,18 +1801,18 @@
         <v>1</v>
       </c>
       <c r="L30" t="n">
-        <v>5.13</v>
+        <v>6.56</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>sh600157</t>
+          <t>sh600170</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>永泰能源</t>
+          <t>上海建工</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1821,13 +1821,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1.73</v>
+        <v>2.65</v>
       </c>
       <c r="E31" t="n">
-        <v>1.71</v>
+        <v>2.65</v>
       </c>
       <c r="F31" t="n">
-        <v>1.64</v>
+        <v>2.57</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1838,7 +1838,7 @@
         <v>52</v>
       </c>
       <c r="I31" t="n">
-        <v>2.976</v>
+        <v>0.76</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1847,18 +1847,18 @@
         <v>1</v>
       </c>
       <c r="L31" t="n">
-        <v>10.86</v>
+        <v>1.82</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>sh600156</t>
+          <t>sh600160</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>华升股份</t>
+          <t>巨化股份</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1867,13 +1867,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>9.26</v>
+        <v>36.44</v>
       </c>
       <c r="E32" t="n">
-        <v>9.279999999999999</v>
+        <v>36.18</v>
       </c>
       <c r="F32" t="n">
-        <v>8.43</v>
+        <v>34.59</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         <v>52</v>
       </c>
       <c r="I32" t="n">
-        <v>1.535</v>
+        <v>1.561</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1893,18 +1893,18 @@
         <v>1</v>
       </c>
       <c r="L32" t="n">
-        <v>3.67</v>
+        <v>10.04</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>sh600143</t>
+          <t>sh600157</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>金发科技</t>
+          <t>永泰能源</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1913,13 +1913,13 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>16.95</v>
+        <v>1.75</v>
       </c>
       <c r="E33" t="n">
-        <v>16.84</v>
+        <v>1.75</v>
       </c>
       <c r="F33" t="n">
-        <v>16.25</v>
+        <v>1.69</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1930,7 +1930,7 @@
         <v>52</v>
       </c>
       <c r="I33" t="n">
-        <v>1.436</v>
+        <v>0.575</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1939,18 +1939,18 @@
         <v>1</v>
       </c>
       <c r="L33" t="n">
-        <v>4.51</v>
+        <v>9.220000000000001</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>sh600132</t>
+          <t>sh600155</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>重庆啤酒</t>
+          <t>华创云信</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1959,13 +1959,13 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>55.08</v>
+        <v>6.12</v>
       </c>
       <c r="E34" t="n">
-        <v>54.56</v>
+        <v>6.1</v>
       </c>
       <c r="F34" t="n">
-        <v>52.81</v>
+        <v>5.92</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1976,7 +1976,7 @@
         <v>52</v>
       </c>
       <c r="I34" t="n">
-        <v>1.68</v>
+        <v>0.824</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1985,18 +1985,18 @@
         <v>1</v>
       </c>
       <c r="L34" t="n">
-        <v>1.72</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>sh600123</t>
+          <t>sh600478</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>兰花科创</t>
+          <t>科力远</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2005,13 +2005,13 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>6.73</v>
+        <v>7.85</v>
       </c>
       <c r="E35" t="n">
-        <v>6.59</v>
+        <v>7.79</v>
       </c>
       <c r="F35" t="n">
-        <v>6.27</v>
+        <v>7.41</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2022,7 +2022,7 @@
         <v>52</v>
       </c>
       <c r="I35" t="n">
-        <v>4.18</v>
+        <v>1.29</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -2031,18 +2031,18 @@
         <v>1</v>
       </c>
       <c r="L35" t="n">
-        <v>2.74</v>
+        <v>3.06</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>sh600114</t>
+          <t>sh600470</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>东睦股份</t>
+          <t>六国化工</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2051,13 +2051,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>33.95</v>
+        <v>6.99</v>
       </c>
       <c r="E36" t="n">
-        <v>33.61</v>
+        <v>7.01</v>
       </c>
       <c r="F36" t="n">
-        <v>32.38</v>
+        <v>6.64</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2068,7 +2068,7 @@
         <v>52</v>
       </c>
       <c r="I36" t="n">
-        <v>2.136</v>
+        <v>1.158</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -2077,18 +2077,18 @@
         <v>1</v>
       </c>
       <c r="L36" t="n">
-        <v>3.12</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>sh600109</t>
+          <t>sh600433</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>国金证券</t>
+          <t>冠豪高新</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2097,13 +2097,13 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>8.77</v>
+        <v>4.58</v>
       </c>
       <c r="E37" t="n">
-        <v>8.710000000000001</v>
+        <v>4.47</v>
       </c>
       <c r="F37" t="n">
-        <v>8.49</v>
+        <v>4.18</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -2114,7 +2114,7 @@
         <v>52</v>
       </c>
       <c r="I37" t="n">
-        <v>1.387</v>
+        <v>4.091</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -2123,18 +2123,18 @@
         <v>1</v>
       </c>
       <c r="L37" t="n">
-        <v>2.11</v>
+        <v>7.88</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>sh600370</t>
+          <t>sh600426</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>三房巷</t>
+          <t>华鲁恒升</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2143,13 +2143,13 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>2.68</v>
+        <v>39.31</v>
       </c>
       <c r="E38" t="n">
-        <v>2.69</v>
+        <v>38.6</v>
       </c>
       <c r="F38" t="n">
-        <v>2.51</v>
+        <v>37</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -2160,7 +2160,7 @@
         <v>52</v>
       </c>
       <c r="I38" t="n">
-        <v>1.515</v>
+        <v>3.611</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -2169,18 +2169,18 @@
         <v>1</v>
       </c>
       <c r="L38" t="n">
-        <v>4.14</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>sh600366</t>
+          <t>sh600409</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>宁波韵升</t>
+          <t>三友化工</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2189,13 +2189,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>13.08</v>
+        <v>7.81</v>
       </c>
       <c r="E39" t="n">
-        <v>12.92</v>
+        <v>7.7</v>
       </c>
       <c r="F39" t="n">
-        <v>12.55</v>
+        <v>7.32</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -2206,7 +2206,7 @@
         <v>52</v>
       </c>
       <c r="I39" t="n">
-        <v>2.267</v>
+        <v>2.628</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2215,18 +2215,18 @@
         <v>1</v>
       </c>
       <c r="L39" t="n">
-        <v>2.5</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>sh600363</t>
+          <t>sh600395</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>联创光电</t>
+          <t>盘江股份</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2235,13 +2235,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>53.05</v>
+        <v>5.76</v>
       </c>
       <c r="E40" t="n">
-        <v>52.59</v>
+        <v>5.73</v>
       </c>
       <c r="F40" t="n">
-        <v>50.66</v>
+        <v>5.57</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -2252,7 +2252,7 @@
         <v>52</v>
       </c>
       <c r="I40" t="n">
-        <v>2.039</v>
+        <v>0.876</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2261,18 +2261,18 @@
         <v>1</v>
       </c>
       <c r="L40" t="n">
-        <v>2.46</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>sh600361</t>
+          <t>sh600383</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>创新新材</t>
+          <t>金地集团</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2281,13 +2281,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>4.65</v>
+        <v>2.71</v>
       </c>
       <c r="E41" t="n">
-        <v>4.58</v>
+        <v>2.71</v>
       </c>
       <c r="F41" t="n">
-        <v>4.4</v>
+        <v>2.63</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -2298,7 +2298,7 @@
         <v>52</v>
       </c>
       <c r="I41" t="n">
-        <v>3.563</v>
+        <v>0.743</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2307,18 +2307,18 @@
         <v>1</v>
       </c>
       <c r="L41" t="n">
-        <v>2.66</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>sh600351</t>
+          <t>sh600375</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>亚宝药业</t>
+          <t>汉马科技</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2327,13 +2327,13 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>6.74</v>
+        <v>5.33</v>
       </c>
       <c r="E42" t="n">
-        <v>6.6</v>
+        <v>5.3</v>
       </c>
       <c r="F42" t="n">
-        <v>6.35</v>
+        <v>5.16</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -2344,7 +2344,7 @@
         <v>52</v>
       </c>
       <c r="I42" t="n">
-        <v>4.984</v>
+        <v>1.718</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
@@ -2353,18 +2353,18 @@
         <v>1</v>
       </c>
       <c r="L42" t="n">
-        <v>2.12</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>sh600345</t>
+          <t>sh600369</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>长江通信</t>
+          <t>西南证券</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2373,13 +2373,13 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>52.58</v>
+        <v>4.17</v>
       </c>
       <c r="E43" t="n">
-        <v>51.57</v>
+        <v>4.17</v>
       </c>
       <c r="F43" t="n">
-        <v>49.54</v>
+        <v>4.05</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -2390,7 +2390,7 @@
         <v>52</v>
       </c>
       <c r="I43" t="n">
-        <v>4.325</v>
+        <v>0.725</v>
       </c>
       <c r="J43" t="n">
         <v>0</v>
@@ -2399,18 +2399,18 @@
         <v>1</v>
       </c>
       <c r="L43" t="n">
-        <v>5.31</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>sh600333</t>
+          <t>sh600352</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>长春燃气</t>
+          <t>浙江龙盛</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2419,13 +2419,13 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>5.73</v>
+        <v>13.23</v>
       </c>
       <c r="E44" t="n">
-        <v>5.68</v>
+        <v>13.17</v>
       </c>
       <c r="F44" t="n">
-        <v>5.49</v>
+        <v>12.4</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -2436,7 +2436,7 @@
         <v>52</v>
       </c>
       <c r="I44" t="n">
-        <v>3.058</v>
+        <v>1.535</v>
       </c>
       <c r="J44" t="n">
         <v>0</v>
@@ -2445,18 +2445,18 @@
         <v>1</v>
       </c>
       <c r="L44" t="n">
-        <v>1</v>
+        <v>4.39</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>sh600331</t>
+          <t>sh600351</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>宏达股份</t>
+          <t>亚宝药业</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2465,13 +2465,13 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>18.57</v>
+        <v>6.87</v>
       </c>
       <c r="E45" t="n">
-        <v>18.44</v>
+        <v>6.85</v>
       </c>
       <c r="F45" t="n">
-        <v>17.72</v>
+        <v>6.58</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2482,7 +2482,7 @@
         <v>52</v>
       </c>
       <c r="I45" t="n">
-        <v>1.809</v>
+        <v>1.178</v>
       </c>
       <c r="J45" t="n">
         <v>0</v>
@@ -2491,18 +2491,18 @@
         <v>1</v>
       </c>
       <c r="L45" t="n">
-        <v>7.42</v>
+        <v>1.87</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>sh600323</t>
+          <t>sh600348</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>瀚蓝环境</t>
+          <t>华阳股份</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2511,13 +2511,13 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>31</v>
+        <v>10.17</v>
       </c>
       <c r="E46" t="n">
-        <v>30.86</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="F46" t="n">
-        <v>29.14</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2528,7 +2528,7 @@
         <v>52</v>
       </c>
       <c r="I46" t="n">
-        <v>2.683</v>
+        <v>3.776</v>
       </c>
       <c r="J46" t="n">
         <v>0</v>
@@ -2537,18 +2537,18 @@
         <v>1</v>
       </c>
       <c r="L46" t="n">
-        <v>2.59</v>
+        <v>4.17</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>sh600312</t>
+          <t>sh600345</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>平高电气</t>
+          <t>长江通信</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2557,13 +2557,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>22.16</v>
+        <v>52.9</v>
       </c>
       <c r="E47" t="n">
-        <v>22.09</v>
+        <v>52.87</v>
       </c>
       <c r="F47" t="n">
-        <v>21.23</v>
+        <v>49.56</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -2574,7 +2574,7 @@
         <v>52</v>
       </c>
       <c r="I47" t="n">
-        <v>1.28</v>
+        <v>1.399</v>
       </c>
       <c r="J47" t="n">
         <v>0</v>
@@ -2583,18 +2583,18 @@
         <v>1</v>
       </c>
       <c r="L47" t="n">
-        <v>3.86</v>
+        <v>6.12</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>sh600310</t>
+          <t>sh600340</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>广西能源</t>
+          <t>华夏幸福</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2603,13 +2603,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>5.29</v>
+        <v>1.26</v>
       </c>
       <c r="E48" t="n">
-        <v>5.2</v>
+        <v>1.26</v>
       </c>
       <c r="F48" t="n">
-        <v>4.72</v>
+        <v>1.2</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2620,7 +2620,7 @@
         <v>52</v>
       </c>
       <c r="I48" t="n">
-        <v>3.929</v>
+        <v>1.613</v>
       </c>
       <c r="J48" t="n">
         <v>0</v>
@@ -2629,18 +2629,18 @@
         <v>1</v>
       </c>
       <c r="L48" t="n">
-        <v>7.71</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>sh600299</t>
+          <t>sh600332</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>安迪苏</t>
+          <t>白云山</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2649,13 +2649,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>14.28</v>
+        <v>22.95</v>
       </c>
       <c r="E49" t="n">
-        <v>14.14</v>
+        <v>22.62</v>
       </c>
       <c r="F49" t="n">
-        <v>13.47</v>
+        <v>22.19</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2666,7 +2666,7 @@
         <v>52</v>
       </c>
       <c r="I49" t="n">
-        <v>2.586</v>
+        <v>2.961</v>
       </c>
       <c r="J49" t="n">
         <v>0</v>
@@ -2675,18 +2675,18 @@
         <v>1</v>
       </c>
       <c r="L49" t="n">
-        <v>1.36</v>
+        <v>4.23</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>sh600292</t>
+          <t>sh600328</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>电投水电</t>
+          <t>中盐化工</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2695,13 +2695,13 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>16.02</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="E50" t="n">
-        <v>16.01</v>
+        <v>8.68</v>
       </c>
       <c r="F50" t="n">
-        <v>15.29</v>
+        <v>8.41</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2712,7 +2712,7 @@
         <v>52</v>
       </c>
       <c r="I50" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="J50" t="n">
         <v>0</v>
@@ -2721,18 +2721,18 @@
         <v>1</v>
       </c>
       <c r="L50" t="n">
-        <v>1.48</v>
+        <v>1.39</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>sh600255</t>
+          <t>sh600600</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>鑫科材料</t>
+          <t>青岛啤酒</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2741,13 +2741,13 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>3.65</v>
+        <v>62.89</v>
       </c>
       <c r="E51" t="n">
-        <v>3.63</v>
+        <v>62.43</v>
       </c>
       <c r="F51" t="n">
-        <v>3.5</v>
+        <v>60.91</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2758,7 +2758,7 @@
         <v>52</v>
       </c>
       <c r="I51" t="n">
-        <v>1.389</v>
+        <v>1.599</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
@@ -2767,18 +2767,18 @@
         <v>1</v>
       </c>
       <c r="L51" t="n">
-        <v>0.97</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>sh600233</t>
+          <t>sh600573</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>圆通速递</t>
+          <t>惠泉啤酒</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2787,13 +2787,13 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>22.51</v>
+        <v>13.42</v>
       </c>
       <c r="E52" t="n">
-        <v>22.26</v>
+        <v>13.39</v>
       </c>
       <c r="F52" t="n">
-        <v>21.45</v>
+        <v>12.84</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2804,7 +2804,7 @@
         <v>52</v>
       </c>
       <c r="I52" t="n">
-        <v>2.645</v>
+        <v>1.054</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -2813,18 +2813,18 @@
         <v>1</v>
       </c>
       <c r="L52" t="n">
-        <v>4.15</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>sh600226</t>
+          <t>sh600566</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>亨通股份</t>
+          <t>济川药业</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2833,13 +2833,13 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>5.39</v>
+        <v>26.97</v>
       </c>
       <c r="E53" t="n">
-        <v>5.3</v>
+        <v>26.86</v>
       </c>
       <c r="F53" t="n">
-        <v>5.03</v>
+        <v>25.96</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2850,7 +2850,7 @@
         <v>52</v>
       </c>
       <c r="I53" t="n">
-        <v>3.455</v>
+        <v>1.087</v>
       </c>
       <c r="J53" t="n">
         <v>0</v>
@@ -2859,18 +2859,18 @@
         <v>1</v>
       </c>
       <c r="L53" t="n">
-        <v>2.65</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>sh600546</t>
+          <t>sh600558</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>山煤国际</t>
+          <t>大西洋</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2879,13 +2879,13 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>12.94</v>
+        <v>5.57</v>
       </c>
       <c r="E54" t="n">
-        <v>12.73</v>
+        <v>5.47</v>
       </c>
       <c r="F54" t="n">
-        <v>12.32</v>
+        <v>5.38</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2896,7 +2896,7 @@
         <v>52</v>
       </c>
       <c r="I54" t="n">
-        <v>2.944</v>
+        <v>4.112</v>
       </c>
       <c r="J54" t="n">
         <v>0</v>
@@ -2905,18 +2905,18 @@
         <v>1</v>
       </c>
       <c r="L54" t="n">
-        <v>2.62</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>sh600545</t>
+          <t>sh600546</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>卓郎智能</t>
+          <t>山煤国际</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2925,13 +2925,13 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>4.88</v>
+        <v>13.4</v>
       </c>
       <c r="E55" t="n">
-        <v>4.82</v>
+        <v>13.16</v>
       </c>
       <c r="F55" t="n">
-        <v>4.41</v>
+        <v>12.56</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2942,7 +2942,7 @@
         <v>52</v>
       </c>
       <c r="I55" t="n">
-        <v>2.954</v>
+        <v>3.957</v>
       </c>
       <c r="J55" t="n">
         <v>0</v>
@@ -2951,18 +2951,18 @@
         <v>1</v>
       </c>
       <c r="L55" t="n">
-        <v>7.4</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>sh600535</t>
+          <t>sh600545</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>天士力</t>
+          <t>卓郎智能</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2971,13 +2971,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>14.99</v>
+        <v>5.02</v>
       </c>
       <c r="E56" t="n">
-        <v>14.94</v>
+        <v>5.03</v>
       </c>
       <c r="F56" t="n">
-        <v>14.67</v>
+        <v>4.71</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2988,7 +2988,7 @@
         <v>52</v>
       </c>
       <c r="I56" t="n">
-        <v>2.531</v>
+        <v>1.414</v>
       </c>
       <c r="J56" t="n">
         <v>0</v>
@@ -2997,18 +2997,18 @@
         <v>1</v>
       </c>
       <c r="L56" t="n">
-        <v>4.3</v>
+        <v>5.33</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>sh600531</t>
+          <t>sh600535</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>豫光金铅</t>
+          <t>天士力</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3017,13 +3017,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>16</v>
+        <v>15.13</v>
       </c>
       <c r="E57" t="n">
-        <v>15.79</v>
+        <v>15.08</v>
       </c>
       <c r="F57" t="n">
-        <v>15.07</v>
+        <v>14.65</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -3034,7 +3034,7 @@
         <v>52</v>
       </c>
       <c r="I57" t="n">
-        <v>2.828</v>
+        <v>1.001</v>
       </c>
       <c r="J57" t="n">
         <v>0</v>
@@ -3043,18 +3043,18 @@
         <v>1</v>
       </c>
       <c r="L57" t="n">
-        <v>7.71</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>sh600515</t>
+          <t>sh600516</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>海南机场</t>
+          <t>方大炭素</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3063,13 +3063,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>3.44</v>
+        <v>5.43</v>
       </c>
       <c r="E58" t="n">
-        <v>3.42</v>
+        <v>5.42</v>
       </c>
       <c r="F58" t="n">
-        <v>3.3</v>
+        <v>5.2</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -3080,7 +3080,7 @@
         <v>52</v>
       </c>
       <c r="I58" t="n">
-        <v>0.88</v>
+        <v>0.556</v>
       </c>
       <c r="J58" t="n">
         <v>0</v>
@@ -3089,18 +3089,18 @@
         <v>1</v>
       </c>
       <c r="L58" t="n">
-        <v>1.36</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>sh600513</t>
+          <t>sh600515</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>联环药业</t>
+          <t>海南机场</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3109,13 +3109,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>20.34</v>
+        <v>3.53</v>
       </c>
       <c r="E59" t="n">
-        <v>20.3</v>
+        <v>3.53</v>
       </c>
       <c r="F59" t="n">
-        <v>19.53</v>
+        <v>3.43</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -3126,7 +3126,7 @@
         <v>52</v>
       </c>
       <c r="I59" t="n">
-        <v>0.643</v>
+        <v>1.437</v>
       </c>
       <c r="J59" t="n">
         <v>0</v>
@@ -3135,18 +3135,18 @@
         <v>1</v>
       </c>
       <c r="L59" t="n">
-        <v>1.41</v>
+        <v>4.31</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>sh600510</t>
+          <t>sh600511</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>黑牡丹</t>
+          <t>国药股份</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3155,13 +3155,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>11.28</v>
+        <v>28.71</v>
       </c>
       <c r="E60" t="n">
-        <v>11.08</v>
+        <v>28.66</v>
       </c>
       <c r="F60" t="n">
-        <v>10.56</v>
+        <v>27.94</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -3172,7 +3172,7 @@
         <v>52</v>
       </c>
       <c r="I60" t="n">
-        <v>3.014</v>
+        <v>0.525</v>
       </c>
       <c r="J60" t="n">
         <v>0</v>
@@ -3181,18 +3181,18 @@
         <v>1</v>
       </c>
       <c r="L60" t="n">
-        <v>1.52</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>sh600501</t>
+          <t>sh600510</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>航天晨光</t>
+          <t>黑牡丹</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3201,13 +3201,13 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>23.09</v>
+        <v>11.29</v>
       </c>
       <c r="E61" t="n">
-        <v>23.22</v>
+        <v>11.25</v>
       </c>
       <c r="F61" t="n">
-        <v>22.54</v>
+        <v>10.8</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -3218,7 +3218,7 @@
         <v>52</v>
       </c>
       <c r="I61" t="n">
-        <v>1.139</v>
+        <v>1.529</v>
       </c>
       <c r="J61" t="n">
         <v>0</v>
@@ -3227,18 +3227,18 @@
         <v>1</v>
       </c>
       <c r="L61" t="n">
-        <v>1.48</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>sh600499</t>
+          <t>sh600508</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>科达制造</t>
+          <t>上海能源</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3247,13 +3247,13 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>20.17</v>
+        <v>13.66</v>
       </c>
       <c r="E62" t="n">
-        <v>20.18</v>
+        <v>13.52</v>
       </c>
       <c r="F62" t="n">
-        <v>19.58</v>
+        <v>12.92</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -3264,7 +3264,7 @@
         <v>52</v>
       </c>
       <c r="I62" t="n">
-        <v>1.817</v>
+        <v>1.788</v>
       </c>
       <c r="J62" t="n">
         <v>0</v>
@@ -3273,18 +3273,18 @@
         <v>1</v>
       </c>
       <c r="L62" t="n">
-        <v>9.75</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>sh600489</t>
+          <t>sh600503</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>中金黄金</t>
+          <t>华丽家族</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3293,13 +3293,13 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>25.77</v>
+        <v>2.48</v>
       </c>
       <c r="E63" t="n">
-        <v>25.7</v>
+        <v>2.47</v>
       </c>
       <c r="F63" t="n">
-        <v>24.84</v>
+        <v>2.35</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -3310,7 +3310,7 @@
         <v>52</v>
       </c>
       <c r="I63" t="n">
-        <v>0.9399999999999999</v>
+        <v>2.058</v>
       </c>
       <c r="J63" t="n">
         <v>0</v>
@@ -3319,18 +3319,18 @@
         <v>1</v>
       </c>
       <c r="L63" t="n">
-        <v>8.06</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>sh600483</t>
+          <t>sh600496</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>福能股份</t>
+          <t>精工钢构</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3339,13 +3339,13 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>9.94</v>
+        <v>3.75</v>
       </c>
       <c r="E64" t="n">
-        <v>9.91</v>
+        <v>3.75</v>
       </c>
       <c r="F64" t="n">
-        <v>9.5</v>
+        <v>3.62</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -3356,7 +3356,7 @@
         <v>52</v>
       </c>
       <c r="I64" t="n">
-        <v>0.8110000000000001</v>
+        <v>0.806</v>
       </c>
       <c r="J64" t="n">
         <v>0</v>
@@ -3365,18 +3365,18 @@
         <v>1</v>
       </c>
       <c r="L64" t="n">
-        <v>1.21</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>sh600460</t>
+          <t>sh600491</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>士兰微</t>
+          <t>龙元建设</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3385,13 +3385,13 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>28.19</v>
+        <v>1.91</v>
       </c>
       <c r="E65" t="n">
-        <v>28.04</v>
+        <v>1.91</v>
       </c>
       <c r="F65" t="n">
-        <v>27.15</v>
+        <v>1.82</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -3402,7 +3402,7 @@
         <v>52</v>
       </c>
       <c r="I65" t="n">
-        <v>1.33</v>
+        <v>3.243</v>
       </c>
       <c r="J65" t="n">
         <v>0</v>
@@ -3411,18 +3411,18 @@
         <v>1</v>
       </c>
       <c r="L65" t="n">
-        <v>7.62</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>sh600446</t>
+          <t>sh600486</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>金证股份</t>
+          <t>扬农化工</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3431,13 +3431,13 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>13.66</v>
+        <v>73.75</v>
       </c>
       <c r="E66" t="n">
-        <v>13.5</v>
+        <v>72.47</v>
       </c>
       <c r="F66" t="n">
-        <v>12.9</v>
+        <v>68.76000000000001</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
         <v>52</v>
       </c>
       <c r="I66" t="n">
-        <v>2.476</v>
+        <v>3.99</v>
       </c>
       <c r="J66" t="n">
         <v>0</v>
@@ -3457,18 +3457,18 @@
         <v>1</v>
       </c>
       <c r="L66" t="n">
-        <v>2.78</v>
+        <v>5.79</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>sh600429</t>
+          <t>sh600761</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>三元股份</t>
+          <t>安徽合力</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3477,13 +3477,13 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>6.1</v>
+        <v>18.1</v>
       </c>
       <c r="E67" t="n">
-        <v>6.11</v>
+        <v>18.02</v>
       </c>
       <c r="F67" t="n">
-        <v>5.89</v>
+        <v>17.36</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -3494,7 +3494,7 @@
         <v>52</v>
       </c>
       <c r="I67" t="n">
-        <v>1.498</v>
+        <v>1.8</v>
       </c>
       <c r="J67" t="n">
         <v>0</v>
@@ -3503,18 +3503,18 @@
         <v>1</v>
       </c>
       <c r="L67" t="n">
-        <v>2.66</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>sh600426</t>
+          <t>sh600751</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>华鲁恒升</t>
+          <t>海航科技</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3523,13 +3523,13 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>37.96</v>
+        <v>3.71</v>
       </c>
       <c r="E68" t="n">
-        <v>37.83</v>
+        <v>3.73</v>
       </c>
       <c r="F68" t="n">
-        <v>36.31</v>
+        <v>3.59</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -3540,7 +3540,7 @@
         <v>52</v>
       </c>
       <c r="I68" t="n">
-        <v>0.904</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="J68" t="n">
         <v>0</v>
@@ -3549,18 +3549,18 @@
         <v>1</v>
       </c>
       <c r="L68" t="n">
-        <v>5.4</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>sh600378</t>
+          <t>sh600744</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>昊华科技</t>
+          <t>华银电力</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3569,13 +3569,13 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>35.57</v>
+        <v>8.01</v>
       </c>
       <c r="E69" t="n">
-        <v>35.52</v>
+        <v>7.99</v>
       </c>
       <c r="F69" t="n">
-        <v>34.3</v>
+        <v>7.59</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -3586,7 +3586,7 @@
         <v>52</v>
       </c>
       <c r="I69" t="n">
-        <v>0.908</v>
+        <v>1.65</v>
       </c>
       <c r="J69" t="n">
         <v>0</v>
@@ -3595,18 +3595,18 @@
         <v>1</v>
       </c>
       <c r="L69" t="n">
-        <v>3.69</v>
+        <v>6.44</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>sh600698</t>
+          <t>sh600740</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>湖南天雁</t>
+          <t>山西焦化</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3615,13 +3615,13 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>7.3</v>
+        <v>4.25</v>
       </c>
       <c r="E70" t="n">
-        <v>7.16</v>
+        <v>4.23</v>
       </c>
       <c r="F70" t="n">
-        <v>7.05</v>
+        <v>4.09</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -3632,7 +3632,7 @@
         <v>52</v>
       </c>
       <c r="I70" t="n">
-        <v>3.693</v>
+        <v>0.95</v>
       </c>
       <c r="J70" t="n">
         <v>0</v>
@@ -3641,18 +3641,18 @@
         <v>1</v>
       </c>
       <c r="L70" t="n">
-        <v>0.88</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>sh600694</t>
+          <t>sh600739</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>大商股份</t>
+          <t>辽宁成大</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3661,13 +3661,13 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>18.37</v>
+        <v>11.84</v>
       </c>
       <c r="E71" t="n">
-        <v>18.18</v>
+        <v>11.66</v>
       </c>
       <c r="F71" t="n">
-        <v>17.52</v>
+        <v>11.36</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -3678,7 +3678,7 @@
         <v>52</v>
       </c>
       <c r="I71" t="n">
-        <v>1.886</v>
+        <v>3.226</v>
       </c>
       <c r="J71" t="n">
         <v>0</v>
@@ -3687,18 +3687,18 @@
         <v>1</v>
       </c>
       <c r="L71" t="n">
-        <v>1.16</v>
+        <v>1.93</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>sh600686</t>
+          <t>sh600699</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>金龙汽车</t>
+          <t>均胜电子</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3707,13 +3707,13 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>17.35</v>
+        <v>28.77</v>
       </c>
       <c r="E72" t="n">
-        <v>17.37</v>
+        <v>28.87</v>
       </c>
       <c r="F72" t="n">
-        <v>16.76</v>
+        <v>28.13</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -3724,7 +3724,7 @@
         <v>52</v>
       </c>
       <c r="I72" t="n">
-        <v>0.931</v>
+        <v>0.63</v>
       </c>
       <c r="J72" t="n">
         <v>0</v>
@@ -3733,18 +3733,18 @@
         <v>1</v>
       </c>
       <c r="L72" t="n">
-        <v>1.98</v>
+        <v>9.109999999999999</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>sh600674</t>
+          <t>sh600691</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>川投能源</t>
+          <t>潞化科技</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3753,13 +3753,13 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>15.03</v>
+        <v>3.29</v>
       </c>
       <c r="E73" t="n">
-        <v>14.99</v>
+        <v>3.29</v>
       </c>
       <c r="F73" t="n">
-        <v>14.5</v>
+        <v>3.16</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -3770,7 +3770,7 @@
         <v>52</v>
       </c>
       <c r="I73" t="n">
-        <v>0.67</v>
+        <v>1.231</v>
       </c>
       <c r="J73" t="n">
         <v>0</v>
@@ -3779,18 +3779,18 @@
         <v>1</v>
       </c>
       <c r="L73" t="n">
-        <v>2.08</v>
+        <v>1.39</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>sh600667</t>
+          <t>sh600688</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>太极实业</t>
+          <t>上海石化</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3799,13 +3799,13 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>9.85</v>
+        <v>2.81</v>
       </c>
       <c r="E74" t="n">
-        <v>9.800000000000001</v>
+        <v>2.79</v>
       </c>
       <c r="F74" t="n">
-        <v>9.51</v>
+        <v>2.7</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -3816,7 +3816,7 @@
         <v>52</v>
       </c>
       <c r="I74" t="n">
-        <v>1.442</v>
+        <v>1.444</v>
       </c>
       <c r="J74" t="n">
         <v>0</v>
@@ -3825,18 +3825,18 @@
         <v>1</v>
       </c>
       <c r="L74" t="n">
-        <v>6.27</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>sh600660</t>
+          <t>sh600685</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>福耀玻璃</t>
+          <t>中船防务</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3845,13 +3845,13 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>60.55</v>
+        <v>32.04</v>
       </c>
       <c r="E75" t="n">
-        <v>59.81</v>
+        <v>31.47</v>
       </c>
       <c r="F75" t="n">
-        <v>57.47</v>
+        <v>29.95</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -3862,7 +3862,7 @@
         <v>52</v>
       </c>
       <c r="I75" t="n">
-        <v>2.575</v>
+        <v>4.263</v>
       </c>
       <c r="J75" t="n">
         <v>0</v>
@@ -3871,18 +3871,18 @@
         <v>1</v>
       </c>
       <c r="L75" t="n">
-        <v>6.38</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>sh600629</t>
+          <t>sh600674</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>华建集团</t>
+          <t>川投能源</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3891,13 +3891,13 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>20.44</v>
+        <v>15.25</v>
       </c>
       <c r="E76" t="n">
-        <v>20.26</v>
+        <v>15.17</v>
       </c>
       <c r="F76" t="n">
-        <v>19.28</v>
+        <v>14.75</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -3908,7 +3908,7 @@
         <v>52</v>
       </c>
       <c r="I76" t="n">
-        <v>2.405</v>
+        <v>1.262</v>
       </c>
       <c r="J76" t="n">
         <v>0</v>
@@ -3917,18 +3917,18 @@
         <v>1</v>
       </c>
       <c r="L76" t="n">
-        <v>2.86</v>
+        <v>4.18</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>sh600617</t>
+          <t>sh600664</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>国新能源</t>
+          <t>哈药股份</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3937,13 +3937,13 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>3.38</v>
+        <v>3.69</v>
       </c>
       <c r="E77" t="n">
-        <v>3.35</v>
+        <v>3.71</v>
       </c>
       <c r="F77" t="n">
-        <v>3.2</v>
+        <v>3.58</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -3954,7 +3954,7 @@
         <v>52</v>
       </c>
       <c r="I77" t="n">
-        <v>1.807</v>
+        <v>0.545</v>
       </c>
       <c r="J77" t="n">
         <v>0</v>
@@ -3963,18 +3963,18 @@
         <v>1</v>
       </c>
       <c r="L77" t="n">
-        <v>1.14</v>
+        <v>2.94</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>sh600605</t>
+          <t>sh600642</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>汇通能源</t>
+          <t>申能股份</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3983,13 +3983,13 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>32.99</v>
+        <v>9.06</v>
       </c>
       <c r="E78" t="n">
-        <v>32.73</v>
+        <v>9</v>
       </c>
       <c r="F78" t="n">
-        <v>31.21</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -4000,7 +4000,7 @@
         <v>52</v>
       </c>
       <c r="I78" t="n">
-        <v>3.677</v>
+        <v>1.229</v>
       </c>
       <c r="J78" t="n">
         <v>0</v>
@@ -4009,18 +4009,18 @@
         <v>1</v>
       </c>
       <c r="L78" t="n">
-        <v>1.95</v>
+        <v>1.59</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>sh600602</t>
+          <t>sh600641</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>云赛智联</t>
+          <t>先导基电</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -4029,13 +4029,13 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>22.6</v>
+        <v>27.6</v>
       </c>
       <c r="E79" t="n">
-        <v>22.42</v>
+        <v>26.95</v>
       </c>
       <c r="F79" t="n">
-        <v>21.17</v>
+        <v>24.99</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -4046,7 +4046,7 @@
         <v>52</v>
       </c>
       <c r="I79" t="n">
-        <v>1.71</v>
+        <v>4.072</v>
       </c>
       <c r="J79" t="n">
         <v>0</v>
@@ -4055,18 +4055,18 @@
         <v>1</v>
       </c>
       <c r="L79" t="n">
-        <v>7.78</v>
+        <v>11.51</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>sh600600</t>
+          <t>sh600621</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>青岛啤酒</t>
+          <t>华鑫股份</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4075,13 +4075,13 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>62.07</v>
+        <v>14.1</v>
       </c>
       <c r="E80" t="n">
-        <v>61.88</v>
+        <v>14.02</v>
       </c>
       <c r="F80" t="n">
-        <v>60.52</v>
+        <v>13.62</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -4092,7 +4092,7 @@
         <v>52</v>
       </c>
       <c r="I80" t="n">
-        <v>0.632</v>
+        <v>1.293</v>
       </c>
       <c r="J80" t="n">
         <v>0</v>
@@ -4101,18 +4101,18 @@
         <v>1</v>
       </c>
       <c r="L80" t="n">
-        <v>1.55</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>sh600580</t>
+          <t>sh600619</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>卧龙电驱</t>
+          <t>海立股份</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4121,13 +4121,13 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>38.02</v>
+        <v>17.5</v>
       </c>
       <c r="E81" t="n">
-        <v>37.96</v>
+        <v>17.41</v>
       </c>
       <c r="F81" t="n">
-        <v>36.68</v>
+        <v>16.73</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -4138,7 +4138,7 @@
         <v>52</v>
       </c>
       <c r="I81" t="n">
-        <v>0.849</v>
+        <v>1.744</v>
       </c>
       <c r="J81" t="n">
         <v>0</v>
@@ -4147,18 +4147,18 @@
         <v>1</v>
       </c>
       <c r="L81" t="n">
-        <v>5.91</v>
+        <v>3.15</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>sh600575</t>
+          <t>sh600617</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>淮河能源</t>
+          <t>国新能源</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4167,13 +4167,13 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>3.82</v>
+        <v>3.4</v>
       </c>
       <c r="E82" t="n">
-        <v>3.74</v>
+        <v>3.42</v>
       </c>
       <c r="F82" t="n">
-        <v>3.58</v>
+        <v>3.29</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -4184,7 +4184,7 @@
         <v>52</v>
       </c>
       <c r="I82" t="n">
-        <v>4.087</v>
+        <v>0.592</v>
       </c>
       <c r="J82" t="n">
         <v>0</v>
@@ -4193,7 +4193,7 @@
         <v>1</v>
       </c>
       <c r="L82" t="n">
-        <v>2.9</v>
+        <v>1.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 实时报告更新 Wed Apr 29 02:46:24 UTC 2026
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>T:2026-04-28 12:56:01</t>
+          <t>T:2026-04-29 10:46:24</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -519,12 +519,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>sz301389</t>
+          <t>sz301468</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>隆扬电子</t>
+          <t>博盈特焊</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -533,13 +533,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>64.36</v>
+        <v>50.6</v>
       </c>
       <c r="E3" t="n">
-        <v>62.46</v>
+        <v>50.6</v>
       </c>
       <c r="F3" t="n">
-        <v>59.12</v>
+        <v>48.34</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -550,7 +550,7 @@
         <v>52</v>
       </c>
       <c r="I3" t="n">
-        <v>5.009</v>
+        <v>0.576</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -559,18 +559,18 @@
         <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>4.74</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>sz301387</t>
+          <t>sz301413</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>光大同创</t>
+          <t>安培龙</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -579,13 +579,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>62.88</v>
+        <v>97.66</v>
       </c>
       <c r="E4" t="n">
-        <v>61.92</v>
+        <v>97.67</v>
       </c>
       <c r="F4" t="n">
-        <v>58.33</v>
+        <v>94.67</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
         <v>52</v>
       </c>
       <c r="I4" t="n">
-        <v>3.167</v>
+        <v>0.525</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -605,18 +605,18 @@
         <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>1.35</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>sz301382</t>
+          <t>sz301408</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>蜂助手</t>
+          <t>华人健康</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -625,13 +625,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>42.28</v>
+        <v>20.84</v>
       </c>
       <c r="E5" t="n">
-        <v>41.71</v>
+        <v>20.73</v>
       </c>
       <c r="F5" t="n">
-        <v>39.2</v>
+        <v>19.11</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
         <v>52</v>
       </c>
       <c r="I5" t="n">
-        <v>3.78</v>
+        <v>1.758</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -651,18 +651,18 @@
         <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>7.05</v>
+        <v>4.05</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>sz301365</t>
+          <t>sz301392</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>矩阵股份</t>
+          <t>汇成真空</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -671,13 +671,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>34.95</v>
+        <v>159.26</v>
       </c>
       <c r="E6" t="n">
-        <v>35.37</v>
+        <v>158.16</v>
       </c>
       <c r="F6" t="n">
-        <v>33.63</v>
+        <v>149.94</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         <v>52</v>
       </c>
       <c r="I6" t="n">
-        <v>0.518</v>
+        <v>1.783</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -697,18 +697,18 @@
         <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>1.59</v>
+        <v>3.35</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>sz301360</t>
+          <t>sz301389</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>荣旗科技</t>
+          <t>隆扬电子</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -717,13 +717,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>83.45999999999999</v>
+        <v>64.05</v>
       </c>
       <c r="E7" t="n">
-        <v>83.59</v>
+        <v>63.54</v>
       </c>
       <c r="F7" t="n">
-        <v>80.41</v>
+        <v>60.02</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -734,7 +734,7 @@
         <v>52</v>
       </c>
       <c r="I7" t="n">
-        <v>1.041</v>
+        <v>2.153</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -743,18 +743,18 @@
         <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>0.85</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>sz301348</t>
+          <t>sz301382</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>蓝箭电子</t>
+          <t>蜂助手</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -763,13 +763,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>24.5</v>
+        <v>42.8</v>
       </c>
       <c r="E8" t="n">
-        <v>24.61</v>
+        <v>42.27</v>
       </c>
       <c r="F8" t="n">
-        <v>23.55</v>
+        <v>39.96</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -780,7 +780,7 @@
         <v>52</v>
       </c>
       <c r="I8" t="n">
-        <v>0.699</v>
+        <v>2.638</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -789,18 +789,18 @@
         <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>2.41</v>
+        <v>3.92</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>sz301328</t>
+          <t>sz301378</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>维峰电子</t>
+          <t>通达海</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -809,13 +809,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>61.09</v>
+        <v>31.89</v>
       </c>
       <c r="E9" t="n">
-        <v>60.49</v>
+        <v>31.54</v>
       </c>
       <c r="F9" t="n">
-        <v>58.32</v>
+        <v>29.86</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -826,7 +826,7 @@
         <v>52</v>
       </c>
       <c r="I9" t="n">
-        <v>2.157</v>
+        <v>3.237</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -835,18 +835,18 @@
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>sz301327</t>
+          <t>sz301377</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>华宝新能</t>
+          <t>鼎泰高科</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -855,13 +855,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>62.03</v>
+        <v>227.85</v>
       </c>
       <c r="E10" t="n">
-        <v>61.93</v>
+        <v>225.24</v>
       </c>
       <c r="F10" t="n">
-        <v>59.49</v>
+        <v>216.4</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -872,7 +872,7 @@
         <v>52</v>
       </c>
       <c r="I10" t="n">
-        <v>0.5669999999999999</v>
+        <v>2.175</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -881,18 +881,18 @@
         <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>1.07</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>sz301326</t>
+          <t>sz301373</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>捷邦科技</t>
+          <t>凌玮科技</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -901,13 +901,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>159.86</v>
+        <v>116.56</v>
       </c>
       <c r="E11" t="n">
-        <v>160.23</v>
+        <v>114.85</v>
       </c>
       <c r="F11" t="n">
-        <v>153.86</v>
+        <v>108.9</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -918,7 +918,7 @@
         <v>52</v>
       </c>
       <c r="I11" t="n">
-        <v>0.775</v>
+        <v>2.47</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -927,18 +927,18 @@
         <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>1.51</v>
+        <v>3.09</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>sz301323</t>
+          <t>sz301372</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>新莱福</t>
+          <t>科净源</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -947,13 +947,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>67.79000000000001</v>
+        <v>35.53</v>
       </c>
       <c r="E12" t="n">
-        <v>67.95</v>
+        <v>35</v>
       </c>
       <c r="F12" t="n">
-        <v>65.93000000000001</v>
+        <v>33.33</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         <v>52</v>
       </c>
       <c r="I12" t="n">
-        <v>1.361</v>
+        <v>4.408</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -973,18 +973,18 @@
         <v>1</v>
       </c>
       <c r="L12" t="n">
-        <v>0.82</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>sz301321</t>
+          <t>sz301371</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>翰博高新</t>
+          <t>敷尔佳</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -993,13 +993,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>24.46</v>
+        <v>29.45</v>
       </c>
       <c r="E13" t="n">
-        <v>23.98</v>
+        <v>29.13</v>
       </c>
       <c r="F13" t="n">
-        <v>22.94</v>
+        <v>27.6</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
         <v>52</v>
       </c>
       <c r="I13" t="n">
-        <v>3.556</v>
+        <v>2.506</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -1019,18 +1019,18 @@
         <v>1</v>
       </c>
       <c r="L13" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>sz301317</t>
+          <t>sz301362</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>鑫磊股份</t>
+          <t>民爆光电</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1039,13 +1039,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>56.89</v>
+        <v>142.82</v>
       </c>
       <c r="E14" t="n">
-        <v>56.12</v>
+        <v>140.19</v>
       </c>
       <c r="F14" t="n">
-        <v>53.53</v>
+        <v>130.69</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
         <v>52</v>
       </c>
       <c r="I14" t="n">
-        <v>4.366</v>
+        <v>3.854</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -1065,18 +1065,18 @@
         <v>1</v>
       </c>
       <c r="L14" t="n">
-        <v>2.3</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>sz301312</t>
+          <t>sz301360</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>智立方</t>
+          <t>荣旗科技</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1085,13 +1085,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>118.34</v>
+        <v>87.3</v>
       </c>
       <c r="E15" t="n">
-        <v>116.42</v>
+        <v>85.33</v>
       </c>
       <c r="F15" t="n">
-        <v>107.41</v>
+        <v>81.23</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1102,7 +1102,7 @@
         <v>52</v>
       </c>
       <c r="I15" t="n">
-        <v>2.779</v>
+        <v>4.314</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -1111,18 +1111,18 @@
         <v>1</v>
       </c>
       <c r="L15" t="n">
-        <v>4.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>sz301285</t>
+          <t>sz301317</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>鸿日达</t>
+          <t>鑫磊股份</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1131,13 +1131,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>107.39</v>
+        <v>60.48</v>
       </c>
       <c r="E16" t="n">
-        <v>107.36</v>
+        <v>61.21</v>
       </c>
       <c r="F16" t="n">
-        <v>100.98</v>
+        <v>55.24</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
         <v>52</v>
       </c>
       <c r="I16" t="n">
-        <v>1.283</v>
+        <v>0.666</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1157,18 +1157,18 @@
         <v>1</v>
       </c>
       <c r="L16" t="n">
-        <v>2.06</v>
+        <v>3.96</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>sz301282</t>
+          <t>sz301316</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>金禄电子</t>
+          <t>慧博云通</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1177,13 +1177,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>45.22</v>
+        <v>47.47</v>
       </c>
       <c r="E17" t="n">
-        <v>45.55</v>
+        <v>47.37</v>
       </c>
       <c r="F17" t="n">
-        <v>43.23</v>
+        <v>44.98</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1194,7 +1194,7 @@
         <v>52</v>
       </c>
       <c r="I17" t="n">
-        <v>0.713</v>
+        <v>2.416</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1203,18 +1203,18 @@
         <v>1</v>
       </c>
       <c r="L17" t="n">
-        <v>3.07</v>
+        <v>3.86</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>sz301281</t>
+          <t>sz301302</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>科源制药</t>
+          <t>华如科技</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1223,13 +1223,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>39</v>
+        <v>24.25</v>
       </c>
       <c r="E18" t="n">
-        <v>38.21</v>
+        <v>24.13</v>
       </c>
       <c r="F18" t="n">
-        <v>36.34</v>
+        <v>23.46</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1240,7 +1240,7 @@
         <v>52</v>
       </c>
       <c r="I18" t="n">
-        <v>4.028</v>
+        <v>1.38</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1249,18 +1249,18 @@
         <v>1</v>
       </c>
       <c r="L18" t="n">
-        <v>1.12</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>sh600325</t>
+          <t>sh600133</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>华发股份</t>
+          <t>东湖高新</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1269,13 +1269,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3.41</v>
+        <v>8.84</v>
       </c>
       <c r="E19" t="n">
-        <v>3.44</v>
+        <v>8.82</v>
       </c>
       <c r="F19" t="n">
-        <v>3.29</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1286,7 +1286,7 @@
         <v>52</v>
       </c>
       <c r="I19" t="n">
-        <v>0.888</v>
+        <v>0.569</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1295,18 +1295,18 @@
         <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>2.02</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>sh600323</t>
+          <t>sh600131</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>瀚蓝环境</t>
+          <t>国网信通</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1315,13 +1315,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>31.25</v>
+        <v>17.22</v>
       </c>
       <c r="E20" t="n">
-        <v>31.03</v>
+        <v>17.03</v>
       </c>
       <c r="F20" t="n">
-        <v>29.9</v>
+        <v>16.47</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1332,7 +1332,7 @@
         <v>52</v>
       </c>
       <c r="I20" t="n">
-        <v>1.395</v>
+        <v>2.439</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1341,18 +1341,18 @@
         <v>1</v>
       </c>
       <c r="L20" t="n">
-        <v>1.41</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>sh600315</t>
+          <t>sh600127</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>上海家化</t>
+          <t>金健米业</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1361,13 +1361,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>20.82</v>
+        <v>6.84</v>
       </c>
       <c r="E21" t="n">
-        <v>21.12</v>
+        <v>6.81</v>
       </c>
       <c r="F21" t="n">
-        <v>20.36</v>
+        <v>6.59</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1378,7 +1378,7 @@
         <v>52</v>
       </c>
       <c r="I21" t="n">
-        <v>0.823</v>
+        <v>1.034</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1387,18 +1387,18 @@
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>1.86</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>sh600285</t>
+          <t>sh600126</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>羚锐制药</t>
+          <t>杭钢股份</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1407,13 +1407,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>22.5</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>21.98</v>
+        <v>9.26</v>
       </c>
       <c r="F22" t="n">
-        <v>21.89</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1424,7 +1424,7 @@
         <v>52</v>
       </c>
       <c r="I22" t="n">
-        <v>4.895</v>
+        <v>1.639</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1433,18 +1433,18 @@
         <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>4.43</v>
+        <v>7.32</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>sh600282</t>
+          <t>sh600121</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>南钢股份</t>
+          <t>郑州煤电</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1453,13 +1453,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>5.32</v>
+        <v>4.31</v>
       </c>
       <c r="E23" t="n">
-        <v>5.27</v>
+        <v>4.25</v>
       </c>
       <c r="F23" t="n">
-        <v>5.08</v>
+        <v>4.09</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1470,7 +1470,7 @@
         <v>52</v>
       </c>
       <c r="I23" t="n">
-        <v>1.916</v>
+        <v>2.619</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1479,18 +1479,18 @@
         <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>1.69</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>sh600262</t>
+          <t>sh600116</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>北方股份</t>
+          <t>三峡水利</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1499,13 +1499,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>23.61</v>
+        <v>6.61</v>
       </c>
       <c r="E24" t="n">
-        <v>23.43</v>
+        <v>6.59</v>
       </c>
       <c r="F24" t="n">
-        <v>22.26</v>
+        <v>6.36</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1516,7 +1516,7 @@
         <v>52</v>
       </c>
       <c r="I24" t="n">
-        <v>2.697</v>
+        <v>0.916</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1525,18 +1525,18 @@
         <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>1.77</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>sh600256</t>
+          <t>sh600114</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>广汇能源</t>
+          <t>东睦股份</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1545,13 +1545,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>6.4</v>
+        <v>32.87</v>
       </c>
       <c r="E25" t="n">
-        <v>6.31</v>
+        <v>32.75</v>
       </c>
       <c r="F25" t="n">
-        <v>6.07</v>
+        <v>31.66</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1562,7 +1562,7 @@
         <v>52</v>
       </c>
       <c r="I25" t="n">
-        <v>2.564</v>
+        <v>0.828</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1571,18 +1571,18 @@
         <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>7.69</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sh600236</t>
+          <t>sh600110</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>桂冠电力</t>
+          <t>诺德股份</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1591,13 +1591,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>9.76</v>
+        <v>10.74</v>
       </c>
       <c r="E26" t="n">
-        <v>9.66</v>
+        <v>10.67</v>
       </c>
       <c r="F26" t="n">
-        <v>9.31</v>
+        <v>10.19</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1608,7 +1608,7 @@
         <v>52</v>
       </c>
       <c r="I26" t="n">
-        <v>2.413</v>
+        <v>1.705</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1617,18 +1617,18 @@
         <v>1</v>
       </c>
       <c r="L26" t="n">
-        <v>1.18</v>
+        <v>9.44</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>sh600234</t>
+          <t>sh600109</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>科新发展</t>
+          <t>国金证券</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1637,13 +1637,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>23.97</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="E27" t="n">
-        <v>24</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="F27" t="n">
-        <v>22.64</v>
+        <v>8.6</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1654,7 +1654,7 @@
         <v>52</v>
       </c>
       <c r="I27" t="n">
-        <v>1.697</v>
+        <v>1.474</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1663,18 +1663,18 @@
         <v>1</v>
       </c>
       <c r="L27" t="n">
-        <v>1.46</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>sh600230</t>
+          <t>sh600108</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>沧州大化</t>
+          <t>亚盛集团</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1683,13 +1683,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>19.17</v>
+        <v>4.27</v>
       </c>
       <c r="E28" t="n">
-        <v>19.07</v>
+        <v>4.23</v>
       </c>
       <c r="F28" t="n">
-        <v>18.38</v>
+        <v>4.06</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1700,7 +1700,7 @@
         <v>52</v>
       </c>
       <c r="I28" t="n">
-        <v>1.375</v>
+        <v>2.153</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1709,18 +1709,18 @@
         <v>1</v>
       </c>
       <c r="L28" t="n">
-        <v>1.39</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>sh600216</t>
+          <t>sh600103</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>浙江医药</t>
+          <t>青山纸业</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1729,13 +1729,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>14.67</v>
+        <v>4.72</v>
       </c>
       <c r="E29" t="n">
-        <v>14.63</v>
+        <v>4.63</v>
       </c>
       <c r="F29" t="n">
-        <v>14.24</v>
+        <v>4.41</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1746,7 +1746,7 @@
         <v>52</v>
       </c>
       <c r="I29" t="n">
-        <v>0.755</v>
+        <v>3.965</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1755,18 +1755,18 @@
         <v>1</v>
       </c>
       <c r="L29" t="n">
-        <v>1.15</v>
+        <v>6.77</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>sh600188</t>
+          <t>sh600101</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>兖矿能源</t>
+          <t>明星电力</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1775,13 +1775,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>21.36</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="E30" t="n">
-        <v>21.08</v>
+        <v>9.69</v>
       </c>
       <c r="F30" t="n">
-        <v>20.22</v>
+        <v>9.32</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1792,7 +1792,7 @@
         <v>52</v>
       </c>
       <c r="I30" t="n">
-        <v>2.692</v>
+        <v>3.455</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1801,18 +1801,18 @@
         <v>1</v>
       </c>
       <c r="L30" t="n">
-        <v>6.56</v>
+        <v>1.81</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>sh600170</t>
+          <t>sh600095</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>上海建工</t>
+          <t>湘财股份</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1821,13 +1821,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2.65</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="E31" t="n">
-        <v>2.65</v>
+        <v>8.85</v>
       </c>
       <c r="F31" t="n">
-        <v>2.57</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1838,7 +1838,7 @@
         <v>52</v>
       </c>
       <c r="I31" t="n">
-        <v>0.76</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1847,18 +1847,18 @@
         <v>1</v>
       </c>
       <c r="L31" t="n">
-        <v>1.82</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>sh600160</t>
+          <t>sh600078</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>巨化股份</t>
+          <t>澄星股份</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1867,13 +1867,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>36.44</v>
+        <v>12.89</v>
       </c>
       <c r="E32" t="n">
-        <v>36.18</v>
+        <v>12.79</v>
       </c>
       <c r="F32" t="n">
-        <v>34.59</v>
+        <v>12.31</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         <v>52</v>
       </c>
       <c r="I32" t="n">
-        <v>1.561</v>
+        <v>1.257</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1893,18 +1893,18 @@
         <v>1</v>
       </c>
       <c r="L32" t="n">
-        <v>10.04</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>sh600157</t>
+          <t>sh600063</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>永泰能源</t>
+          <t>皖维高新</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1913,13 +1913,13 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1.75</v>
+        <v>7.1</v>
       </c>
       <c r="E33" t="n">
-        <v>1.75</v>
+        <v>7.01</v>
       </c>
       <c r="F33" t="n">
-        <v>1.69</v>
+        <v>6.75</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1930,7 +1930,7 @@
         <v>52</v>
       </c>
       <c r="I33" t="n">
-        <v>0.575</v>
+        <v>2.011</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1939,18 +1939,18 @@
         <v>1</v>
       </c>
       <c r="L33" t="n">
-        <v>9.220000000000001</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>sh600155</t>
+          <t>sh600060</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>华创云信</t>
+          <t>海信视像</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1959,13 +1959,13 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>6.12</v>
+        <v>24.88</v>
       </c>
       <c r="E34" t="n">
-        <v>6.1</v>
+        <v>24.77</v>
       </c>
       <c r="F34" t="n">
-        <v>5.92</v>
+        <v>23.84</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1976,7 +1976,7 @@
         <v>52</v>
       </c>
       <c r="I34" t="n">
-        <v>0.824</v>
+        <v>1.51</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1985,18 +1985,18 @@
         <v>1</v>
       </c>
       <c r="L34" t="n">
-        <v>0.87</v>
+        <v>1.74</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>sh600478</t>
+          <t>sh600219</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>科力远</t>
+          <t>南山铝业</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2005,13 +2005,13 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>7.85</v>
+        <v>5.34</v>
       </c>
       <c r="E35" t="n">
-        <v>7.79</v>
+        <v>5.31</v>
       </c>
       <c r="F35" t="n">
-        <v>7.41</v>
+        <v>5.1</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2022,7 +2022,7 @@
         <v>52</v>
       </c>
       <c r="I35" t="n">
-        <v>1.29</v>
+        <v>0.945</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -2031,18 +2031,18 @@
         <v>1</v>
       </c>
       <c r="L35" t="n">
-        <v>3.06</v>
+        <v>6.36</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>sh600470</t>
+          <t>sh600211</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>六国化工</t>
+          <t>西藏药业</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2051,13 +2051,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>6.99</v>
+        <v>41.25</v>
       </c>
       <c r="E36" t="n">
-        <v>7.01</v>
+        <v>40.64</v>
       </c>
       <c r="F36" t="n">
-        <v>6.64</v>
+        <v>39.74</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2068,7 +2068,7 @@
         <v>52</v>
       </c>
       <c r="I36" t="n">
-        <v>1.158</v>
+        <v>2.996</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -2077,18 +2077,18 @@
         <v>1</v>
       </c>
       <c r="L36" t="n">
-        <v>1.78</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>sh600433</t>
+          <t>sh600210</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>冠豪高新</t>
+          <t>紫江企业</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2097,13 +2097,13 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4.58</v>
+        <v>7.15</v>
       </c>
       <c r="E37" t="n">
-        <v>4.47</v>
+        <v>7.04</v>
       </c>
       <c r="F37" t="n">
-        <v>4.18</v>
+        <v>6.96</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -2114,7 +2114,7 @@
         <v>52</v>
       </c>
       <c r="I37" t="n">
-        <v>4.091</v>
+        <v>4.227</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -2123,18 +2123,18 @@
         <v>1</v>
       </c>
       <c r="L37" t="n">
-        <v>7.88</v>
+        <v>2.81</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>sh600426</t>
+          <t>sh600208</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>华鲁恒升</t>
+          <t>衢州发展</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2143,13 +2143,13 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>39.31</v>
+        <v>4.16</v>
       </c>
       <c r="E38" t="n">
-        <v>38.6</v>
+        <v>4.17</v>
       </c>
       <c r="F38" t="n">
-        <v>37</v>
+        <v>3.99</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -2160,7 +2160,7 @@
         <v>52</v>
       </c>
       <c r="I38" t="n">
-        <v>3.611</v>
+        <v>1.217</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -2169,18 +2169,18 @@
         <v>1</v>
       </c>
       <c r="L38" t="n">
-        <v>8.300000000000001</v>
+        <v>6.12</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>sh600409</t>
+          <t>sh600206</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>三友化工</t>
+          <t>有研新材</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2189,13 +2189,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>7.81</v>
+        <v>26.88</v>
       </c>
       <c r="E39" t="n">
-        <v>7.7</v>
+        <v>26.8</v>
       </c>
       <c r="F39" t="n">
-        <v>7.32</v>
+        <v>25.67</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -2206,7 +2206,7 @@
         <v>52</v>
       </c>
       <c r="I39" t="n">
-        <v>2.628</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2215,18 +2215,18 @@
         <v>1</v>
       </c>
       <c r="L39" t="n">
-        <v>2.56</v>
+        <v>9.08</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>sh600395</t>
+          <t>sh600201</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>盘江股份</t>
+          <t>生物股份</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2235,13 +2235,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>5.76</v>
+        <v>13.89</v>
       </c>
       <c r="E40" t="n">
-        <v>5.73</v>
+        <v>13.8</v>
       </c>
       <c r="F40" t="n">
-        <v>5.57</v>
+        <v>13.33</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -2252,7 +2252,7 @@
         <v>52</v>
       </c>
       <c r="I40" t="n">
-        <v>0.876</v>
+        <v>2.283</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2261,18 +2261,18 @@
         <v>1</v>
       </c>
       <c r="L40" t="n">
-        <v>1.06</v>
+        <v>2.18</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>sh600383</t>
+          <t>sh600187</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>金地集团</t>
+          <t>国中水务</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2281,13 +2281,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>2.71</v>
+        <v>1.83</v>
       </c>
       <c r="E41" t="n">
-        <v>2.71</v>
+        <v>1.8</v>
       </c>
       <c r="F41" t="n">
-        <v>2.63</v>
+        <v>1.71</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -2298,7 +2298,7 @@
         <v>52</v>
       </c>
       <c r="I41" t="n">
-        <v>0.743</v>
+        <v>3.977</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2307,18 +2307,18 @@
         <v>1</v>
       </c>
       <c r="L41" t="n">
-        <v>1.04</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>sh600375</t>
+          <t>sh600177</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>汉马科技</t>
+          <t>雅戈尔</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2327,13 +2327,13 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>5.33</v>
+        <v>7.63</v>
       </c>
       <c r="E42" t="n">
-        <v>5.3</v>
+        <v>7.55</v>
       </c>
       <c r="F42" t="n">
-        <v>5.16</v>
+        <v>7.29</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -2344,7 +2344,7 @@
         <v>52</v>
       </c>
       <c r="I42" t="n">
-        <v>1.718</v>
+        <v>2.416</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
@@ -2353,18 +2353,18 @@
         <v>1</v>
       </c>
       <c r="L42" t="n">
-        <v>1.23</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>sh600369</t>
+          <t>sh600172</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>西南证券</t>
+          <t>黄河旋风</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2373,13 +2373,13 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>4.17</v>
+        <v>8.26</v>
       </c>
       <c r="E43" t="n">
-        <v>4.17</v>
+        <v>8.1</v>
       </c>
       <c r="F43" t="n">
-        <v>4.05</v>
+        <v>7.75</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -2390,7 +2390,7 @@
         <v>52</v>
       </c>
       <c r="I43" t="n">
-        <v>0.725</v>
+        <v>3.379</v>
       </c>
       <c r="J43" t="n">
         <v>0</v>
@@ -2399,18 +2399,18 @@
         <v>1</v>
       </c>
       <c r="L43" t="n">
-        <v>1.07</v>
+        <v>2.86</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>sh600352</t>
+          <t>sh600170</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>浙江龙盛</t>
+          <t>上海建工</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2419,13 +2419,13 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>13.23</v>
+        <v>2.67</v>
       </c>
       <c r="E44" t="n">
-        <v>13.17</v>
+        <v>2.67</v>
       </c>
       <c r="F44" t="n">
-        <v>12.4</v>
+        <v>2.6</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -2436,7 +2436,7 @@
         <v>52</v>
       </c>
       <c r="I44" t="n">
-        <v>1.535</v>
+        <v>0.755</v>
       </c>
       <c r="J44" t="n">
         <v>0</v>
@@ -2445,18 +2445,18 @@
         <v>1</v>
       </c>
       <c r="L44" t="n">
-        <v>4.39</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>sh600351</t>
+          <t>sh600160</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>亚宝药业</t>
+          <t>巨化股份</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2465,13 +2465,13 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>6.87</v>
+        <v>36.79</v>
       </c>
       <c r="E45" t="n">
-        <v>6.85</v>
+        <v>36.67</v>
       </c>
       <c r="F45" t="n">
-        <v>6.58</v>
+        <v>35.6</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2482,7 +2482,7 @@
         <v>52</v>
       </c>
       <c r="I45" t="n">
-        <v>1.178</v>
+        <v>1.574</v>
       </c>
       <c r="J45" t="n">
         <v>0</v>
@@ -2491,18 +2491,18 @@
         <v>1</v>
       </c>
       <c r="L45" t="n">
-        <v>1.87</v>
+        <v>8.859999999999999</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>sh600348</t>
+          <t>sh600158</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>华阳股份</t>
+          <t>中体产业</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2511,13 +2511,13 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>10.17</v>
+        <v>10.66</v>
       </c>
       <c r="E46" t="n">
-        <v>9.960000000000001</v>
+        <v>10.42</v>
       </c>
       <c r="F46" t="n">
-        <v>9.550000000000001</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2528,7 +2528,7 @@
         <v>52</v>
       </c>
       <c r="I46" t="n">
-        <v>3.776</v>
+        <v>4.51</v>
       </c>
       <c r="J46" t="n">
         <v>0</v>
@@ -2537,18 +2537,18 @@
         <v>1</v>
       </c>
       <c r="L46" t="n">
-        <v>4.17</v>
+        <v>4.65</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>sh600345</t>
+          <t>sh600157</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>长江通信</t>
+          <t>永泰能源</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2557,13 +2557,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>52.9</v>
+        <v>1.79</v>
       </c>
       <c r="E47" t="n">
-        <v>52.87</v>
+        <v>1.77</v>
       </c>
       <c r="F47" t="n">
-        <v>49.56</v>
+        <v>1.71</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -2574,7 +2574,7 @@
         <v>52</v>
       </c>
       <c r="I47" t="n">
-        <v>1.399</v>
+        <v>2.286</v>
       </c>
       <c r="J47" t="n">
         <v>0</v>
@@ -2583,18 +2583,18 @@
         <v>1</v>
       </c>
       <c r="L47" t="n">
-        <v>6.12</v>
+        <v>10.94</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>sh600340</t>
+          <t>sh600151</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>华夏幸福</t>
+          <t>航天机电</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2603,13 +2603,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>1.26</v>
+        <v>13.98</v>
       </c>
       <c r="E48" t="n">
-        <v>1.26</v>
+        <v>13.87</v>
       </c>
       <c r="F48" t="n">
-        <v>1.2</v>
+        <v>13.08</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2620,7 +2620,7 @@
         <v>52</v>
       </c>
       <c r="I48" t="n">
-        <v>1.613</v>
+        <v>2.044</v>
       </c>
       <c r="J48" t="n">
         <v>0</v>
@@ -2629,18 +2629,18 @@
         <v>1</v>
       </c>
       <c r="L48" t="n">
-        <v>0.88</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>sh600332</t>
+          <t>sh600143</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>白云山</t>
+          <t>金发科技</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2649,13 +2649,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>22.95</v>
+        <v>16.91</v>
       </c>
       <c r="E49" t="n">
-        <v>22.62</v>
+        <v>16.73</v>
       </c>
       <c r="F49" t="n">
-        <v>22.19</v>
+        <v>16.17</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2666,7 +2666,7 @@
         <v>52</v>
       </c>
       <c r="I49" t="n">
-        <v>2.961</v>
+        <v>1.806</v>
       </c>
       <c r="J49" t="n">
         <v>0</v>
@@ -2675,18 +2675,18 @@
         <v>1</v>
       </c>
       <c r="L49" t="n">
-        <v>4.23</v>
+        <v>2.89</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>sh600328</t>
+          <t>sh600141</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>中盐化工</t>
+          <t>兴发集团</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2695,13 +2695,13 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>8.710000000000001</v>
+        <v>33.16</v>
       </c>
       <c r="E50" t="n">
-        <v>8.68</v>
+        <v>32.88</v>
       </c>
       <c r="F50" t="n">
-        <v>8.41</v>
+        <v>29.95</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2712,7 +2712,7 @@
         <v>52</v>
       </c>
       <c r="I50" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.438</v>
       </c>
       <c r="J50" t="n">
         <v>0</v>
@@ -2721,18 +2721,18 @@
         <v>1</v>
       </c>
       <c r="L50" t="n">
-        <v>1.39</v>
+        <v>9.19</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>sh600600</t>
+          <t>sh600309</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>青岛啤酒</t>
+          <t>万华化学</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2741,13 +2741,13 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>62.89</v>
+        <v>90</v>
       </c>
       <c r="E51" t="n">
-        <v>62.43</v>
+        <v>89.81999999999999</v>
       </c>
       <c r="F51" t="n">
-        <v>60.91</v>
+        <v>86.76000000000001</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2758,7 +2758,7 @@
         <v>52</v>
       </c>
       <c r="I51" t="n">
-        <v>1.599</v>
+        <v>0.581</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
@@ -2767,18 +2767,18 @@
         <v>1</v>
       </c>
       <c r="L51" t="n">
-        <v>3.58</v>
+        <v>10.11</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>sh600573</t>
+          <t>sh600307</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>惠泉啤酒</t>
+          <t>酒钢宏兴</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2787,13 +2787,13 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>13.42</v>
+        <v>1.79</v>
       </c>
       <c r="E52" t="n">
-        <v>13.39</v>
+        <v>1.77</v>
       </c>
       <c r="F52" t="n">
-        <v>12.84</v>
+        <v>1.7</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2804,7 +2804,7 @@
         <v>52</v>
       </c>
       <c r="I52" t="n">
-        <v>1.054</v>
+        <v>2.286</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -2813,18 +2813,18 @@
         <v>1</v>
       </c>
       <c r="L52" t="n">
-        <v>1.23</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>sh600566</t>
+          <t>sh600301</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>济川药业</t>
+          <t>华锡有色</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2833,13 +2833,13 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>26.97</v>
+        <v>49.49</v>
       </c>
       <c r="E53" t="n">
-        <v>26.86</v>
+        <v>49.34</v>
       </c>
       <c r="F53" t="n">
-        <v>25.96</v>
+        <v>47.63</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2850,7 +2850,7 @@
         <v>52</v>
       </c>
       <c r="I53" t="n">
-        <v>1.087</v>
+        <v>0.63</v>
       </c>
       <c r="J53" t="n">
         <v>0</v>
@@ -2859,18 +2859,18 @@
         <v>1</v>
       </c>
       <c r="L53" t="n">
-        <v>1</v>
+        <v>2.53</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>sh600558</t>
+          <t>sh600299</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>大西洋</t>
+          <t>安迪苏</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2879,13 +2879,13 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>5.57</v>
+        <v>13.87</v>
       </c>
       <c r="E54" t="n">
-        <v>5.47</v>
+        <v>13.95</v>
       </c>
       <c r="F54" t="n">
-        <v>5.38</v>
+        <v>13.43</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2896,7 +2896,7 @@
         <v>52</v>
       </c>
       <c r="I54" t="n">
-        <v>4.112</v>
+        <v>0.507</v>
       </c>
       <c r="J54" t="n">
         <v>0</v>
@@ -2905,18 +2905,18 @@
         <v>1</v>
       </c>
       <c r="L54" t="n">
-        <v>1.8</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>sh600546</t>
+          <t>sh600298</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>山煤国际</t>
+          <t>安琪酵母</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2925,13 +2925,13 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>13.4</v>
+        <v>38.5</v>
       </c>
       <c r="E55" t="n">
-        <v>13.16</v>
+        <v>38.44</v>
       </c>
       <c r="F55" t="n">
-        <v>12.56</v>
+        <v>37.45</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2942,7 +2942,7 @@
         <v>52</v>
       </c>
       <c r="I55" t="n">
-        <v>3.957</v>
+        <v>0.575</v>
       </c>
       <c r="J55" t="n">
         <v>0</v>
@@ -2951,18 +2951,18 @@
         <v>1</v>
       </c>
       <c r="L55" t="n">
-        <v>3.55</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>sh600545</t>
+          <t>sh600282</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>卓郎智能</t>
+          <t>南钢股份</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2971,13 +2971,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>5.02</v>
+        <v>5.44</v>
       </c>
       <c r="E56" t="n">
-        <v>5.03</v>
+        <v>5.43</v>
       </c>
       <c r="F56" t="n">
-        <v>4.71</v>
+        <v>5.25</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2988,7 +2988,7 @@
         <v>52</v>
       </c>
       <c r="I56" t="n">
-        <v>1.414</v>
+        <v>1.493</v>
       </c>
       <c r="J56" t="n">
         <v>0</v>
@@ -2997,18 +2997,18 @@
         <v>1</v>
       </c>
       <c r="L56" t="n">
-        <v>5.33</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>sh600535</t>
+          <t>sh600271</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>天士力</t>
+          <t>航天信息</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3017,13 +3017,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>15.13</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="E57" t="n">
-        <v>15.08</v>
+        <v>8.15</v>
       </c>
       <c r="F57" t="n">
-        <v>14.65</v>
+        <v>7.87</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -3034,7 +3034,7 @@
         <v>52</v>
       </c>
       <c r="I57" t="n">
-        <v>1.001</v>
+        <v>2.602</v>
       </c>
       <c r="J57" t="n">
         <v>0</v>
@@ -3043,18 +3043,18 @@
         <v>1</v>
       </c>
       <c r="L57" t="n">
-        <v>1.79</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>sh600516</t>
+          <t>sh600268</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>方大炭素</t>
+          <t>国电南自</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3063,13 +3063,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>5.43</v>
+        <v>15.11</v>
       </c>
       <c r="E58" t="n">
-        <v>5.42</v>
+        <v>14.86</v>
       </c>
       <c r="F58" t="n">
-        <v>5.2</v>
+        <v>14.39</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -3080,7 +3080,7 @@
         <v>52</v>
       </c>
       <c r="I58" t="n">
-        <v>0.556</v>
+        <v>2.999</v>
       </c>
       <c r="J58" t="n">
         <v>0</v>
@@ -3089,18 +3089,18 @@
         <v>1</v>
       </c>
       <c r="L58" t="n">
-        <v>1.57</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>sh600515</t>
+          <t>sh600262</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>海南机场</t>
+          <t>北方股份</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3109,13 +3109,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>3.53</v>
+        <v>24.36</v>
       </c>
       <c r="E59" t="n">
-        <v>3.53</v>
+        <v>23.91</v>
       </c>
       <c r="F59" t="n">
-        <v>3.43</v>
+        <v>23.63</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -3126,7 +3126,7 @@
         <v>52</v>
       </c>
       <c r="I59" t="n">
-        <v>1.437</v>
+        <v>4.281</v>
       </c>
       <c r="J59" t="n">
         <v>0</v>
@@ -3135,18 +3135,18 @@
         <v>1</v>
       </c>
       <c r="L59" t="n">
-        <v>4.31</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>sh600511</t>
+          <t>sh600256</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>国药股份</t>
+          <t>广汇能源</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3155,13 +3155,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>28.71</v>
+        <v>6.55</v>
       </c>
       <c r="E60" t="n">
-        <v>28.66</v>
+        <v>6.56</v>
       </c>
       <c r="F60" t="n">
-        <v>27.94</v>
+        <v>6.34</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -3172,7 +3172,7 @@
         <v>52</v>
       </c>
       <c r="I60" t="n">
-        <v>0.525</v>
+        <v>0.769</v>
       </c>
       <c r="J60" t="n">
         <v>0</v>
@@ -3181,18 +3181,18 @@
         <v>1</v>
       </c>
       <c r="L60" t="n">
-        <v>0.84</v>
+        <v>6.54</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>sh600510</t>
+          <t>sh600251</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>黑牡丹</t>
+          <t>冠农股份</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3201,13 +3201,13 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>11.29</v>
+        <v>12.27</v>
       </c>
       <c r="E61" t="n">
-        <v>11.25</v>
+        <v>12.23</v>
       </c>
       <c r="F61" t="n">
-        <v>10.8</v>
+        <v>11.76</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -3218,7 +3218,7 @@
         <v>52</v>
       </c>
       <c r="I61" t="n">
-        <v>1.529</v>
+        <v>1.91</v>
       </c>
       <c r="J61" t="n">
         <v>0</v>
@@ -3227,18 +3227,18 @@
         <v>1</v>
       </c>
       <c r="L61" t="n">
-        <v>1.16</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>sh600508</t>
+          <t>sh600234</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>上海能源</t>
+          <t>科新发展</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3247,13 +3247,13 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>13.66</v>
+        <v>24.35</v>
       </c>
       <c r="E62" t="n">
-        <v>13.52</v>
+        <v>24.25</v>
       </c>
       <c r="F62" t="n">
-        <v>12.92</v>
+        <v>22.89</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -3264,7 +3264,7 @@
         <v>52</v>
       </c>
       <c r="I62" t="n">
-        <v>1.788</v>
+        <v>2.397</v>
       </c>
       <c r="J62" t="n">
         <v>0</v>
@@ -3273,18 +3273,18 @@
         <v>1</v>
       </c>
       <c r="L62" t="n">
-        <v>0.98</v>
+        <v>1.24</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>sh600503</t>
+          <t>sh600230</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>华丽家族</t>
+          <t>沧州大化</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3293,13 +3293,13 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>2.48</v>
+        <v>19.6</v>
       </c>
       <c r="E63" t="n">
-        <v>2.47</v>
+        <v>19.47</v>
       </c>
       <c r="F63" t="n">
-        <v>2.35</v>
+        <v>18.54</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -3310,7 +3310,7 @@
         <v>52</v>
       </c>
       <c r="I63" t="n">
-        <v>2.058</v>
+        <v>1.924</v>
       </c>
       <c r="J63" t="n">
         <v>0</v>
@@ -3319,18 +3319,18 @@
         <v>1</v>
       </c>
       <c r="L63" t="n">
-        <v>1.04</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>sh600496</t>
+          <t>sh600227</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>精工钢构</t>
+          <t>赤天化</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3339,13 +3339,13 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>3.75</v>
+        <v>4.25</v>
       </c>
       <c r="E64" t="n">
-        <v>3.75</v>
+        <v>4.15</v>
       </c>
       <c r="F64" t="n">
-        <v>3.62</v>
+        <v>3.92</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -3356,7 +3356,7 @@
         <v>52</v>
       </c>
       <c r="I64" t="n">
-        <v>0.806</v>
+        <v>4.938</v>
       </c>
       <c r="J64" t="n">
         <v>0</v>
@@ -3365,18 +3365,18 @@
         <v>1</v>
       </c>
       <c r="L64" t="n">
-        <v>0.9</v>
+        <v>11.08</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>sh600491</t>
+          <t>sh600226</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>龙元建设</t>
+          <t>亨通股份</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3385,13 +3385,13 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>1.91</v>
+        <v>5.28</v>
       </c>
       <c r="E65" t="n">
-        <v>1.91</v>
+        <v>5.27</v>
       </c>
       <c r="F65" t="n">
-        <v>1.82</v>
+        <v>5.05</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -3402,7 +3402,7 @@
         <v>52</v>
       </c>
       <c r="I65" t="n">
-        <v>3.243</v>
+        <v>0.571</v>
       </c>
       <c r="J65" t="n">
         <v>0</v>
@@ -3411,18 +3411,18 @@
         <v>1</v>
       </c>
       <c r="L65" t="n">
-        <v>1.57</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>sh600486</t>
+          <t>sh600221</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>扬农化工</t>
+          <t>海航控股</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3431,13 +3431,13 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>73.75</v>
+        <v>1.44</v>
       </c>
       <c r="E66" t="n">
-        <v>72.47</v>
+        <v>1.44</v>
       </c>
       <c r="F66" t="n">
-        <v>68.76000000000001</v>
+        <v>1.39</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
         <v>52</v>
       </c>
       <c r="I66" t="n">
-        <v>3.99</v>
+        <v>0.699</v>
       </c>
       <c r="J66" t="n">
         <v>0</v>
@@ -3457,18 +3457,18 @@
         <v>1</v>
       </c>
       <c r="L66" t="n">
-        <v>5.79</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>sh600761</t>
+          <t>sh600376</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>安徽合力</t>
+          <t>首开股份</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3477,13 +3477,13 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>18.1</v>
+        <v>4.45</v>
       </c>
       <c r="E67" t="n">
-        <v>18.02</v>
+        <v>4.34</v>
       </c>
       <c r="F67" t="n">
-        <v>17.36</v>
+        <v>4.13</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -3494,7 +3494,7 @@
         <v>52</v>
       </c>
       <c r="I67" t="n">
-        <v>1.8</v>
+        <v>3.972</v>
       </c>
       <c r="J67" t="n">
         <v>0</v>
@@ -3503,18 +3503,18 @@
         <v>1</v>
       </c>
       <c r="L67" t="n">
-        <v>2.44</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>sh600751</t>
+          <t>sh600372</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>海航科技</t>
+          <t>中航机载</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3523,13 +3523,13 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>3.71</v>
+        <v>13</v>
       </c>
       <c r="E68" t="n">
-        <v>3.73</v>
+        <v>12.98</v>
       </c>
       <c r="F68" t="n">
-        <v>3.59</v>
+        <v>12.62</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -3540,7 +3540,7 @@
         <v>52</v>
       </c>
       <c r="I68" t="n">
-        <v>0.8149999999999999</v>
+        <v>0.541</v>
       </c>
       <c r="J68" t="n">
         <v>0</v>
@@ -3549,18 +3549,18 @@
         <v>1</v>
       </c>
       <c r="L68" t="n">
-        <v>1.04</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>sh600744</t>
+          <t>sh600366</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>华银电力</t>
+          <t>宁波韵升</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3569,13 +3569,13 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>8.01</v>
+        <v>13.2</v>
       </c>
       <c r="E69" t="n">
-        <v>7.99</v>
+        <v>12.99</v>
       </c>
       <c r="F69" t="n">
-        <v>7.59</v>
+        <v>12.46</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -3586,7 +3586,7 @@
         <v>52</v>
       </c>
       <c r="I69" t="n">
-        <v>1.65</v>
+        <v>3.125</v>
       </c>
       <c r="J69" t="n">
         <v>0</v>
@@ -3595,18 +3595,18 @@
         <v>1</v>
       </c>
       <c r="L69" t="n">
-        <v>6.44</v>
+        <v>2.65</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>sh600740</t>
+          <t>sh600362</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>山西焦化</t>
+          <t>江西铜业</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3615,13 +3615,13 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>4.25</v>
+        <v>44.89</v>
       </c>
       <c r="E70" t="n">
-        <v>4.23</v>
+        <v>44.61</v>
       </c>
       <c r="F70" t="n">
-        <v>4.09</v>
+        <v>43.07</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -3632,7 +3632,7 @@
         <v>52</v>
       </c>
       <c r="I70" t="n">
-        <v>0.95</v>
+        <v>1.378</v>
       </c>
       <c r="J70" t="n">
         <v>0</v>
@@ -3641,18 +3641,18 @@
         <v>1</v>
       </c>
       <c r="L70" t="n">
-        <v>1.16</v>
+        <v>7.23</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>sh600739</t>
+          <t>sh600353</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>辽宁成大</t>
+          <t>旭光电子</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3661,13 +3661,13 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>11.84</v>
+        <v>17.82</v>
       </c>
       <c r="E71" t="n">
-        <v>11.66</v>
+        <v>17.85</v>
       </c>
       <c r="F71" t="n">
-        <v>11.36</v>
+        <v>17.05</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -3678,7 +3678,7 @@
         <v>52</v>
       </c>
       <c r="I71" t="n">
-        <v>3.226</v>
+        <v>0.678</v>
       </c>
       <c r="J71" t="n">
         <v>0</v>
@@ -3687,18 +3687,18 @@
         <v>1</v>
       </c>
       <c r="L71" t="n">
-        <v>1.93</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>sh600699</t>
+          <t>sh600348</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>均胜电子</t>
+          <t>华阳股份</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3707,13 +3707,13 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>28.77</v>
+        <v>10.33</v>
       </c>
       <c r="E72" t="n">
-        <v>28.87</v>
+        <v>10.29</v>
       </c>
       <c r="F72" t="n">
-        <v>28.13</v>
+        <v>9.91</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -3724,7 +3724,7 @@
         <v>52</v>
       </c>
       <c r="I72" t="n">
-        <v>0.63</v>
+        <v>1.175</v>
       </c>
       <c r="J72" t="n">
         <v>0</v>
@@ -3733,18 +3733,18 @@
         <v>1</v>
       </c>
       <c r="L72" t="n">
-        <v>9.109999999999999</v>
+        <v>3.27</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>sh600691</t>
+          <t>sh600343</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>潞化科技</t>
+          <t>航天动力</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3753,13 +3753,13 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>3.29</v>
+        <v>33.08</v>
       </c>
       <c r="E73" t="n">
-        <v>3.29</v>
+        <v>33.14</v>
       </c>
       <c r="F73" t="n">
-        <v>3.16</v>
+        <v>31.76</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -3770,7 +3770,7 @@
         <v>52</v>
       </c>
       <c r="I73" t="n">
-        <v>1.231</v>
+        <v>0.731</v>
       </c>
       <c r="J73" t="n">
         <v>0</v>
@@ -3779,18 +3779,18 @@
         <v>1</v>
       </c>
       <c r="L73" t="n">
-        <v>1.39</v>
+        <v>3.43</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>sh600688</t>
+          <t>sh600340</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>上海石化</t>
+          <t>华夏幸福</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3799,13 +3799,13 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>2.81</v>
+        <v>1.28</v>
       </c>
       <c r="E74" t="n">
-        <v>2.79</v>
+        <v>1.26</v>
       </c>
       <c r="F74" t="n">
-        <v>2.7</v>
+        <v>1.2</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -3816,7 +3816,7 @@
         <v>52</v>
       </c>
       <c r="I74" t="n">
-        <v>1.444</v>
+        <v>3.226</v>
       </c>
       <c r="J74" t="n">
         <v>0</v>
@@ -3825,18 +3825,18 @@
         <v>1</v>
       </c>
       <c r="L74" t="n">
-        <v>0.85</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>sh600685</t>
+          <t>sh600337</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>中船防务</t>
+          <t>美克家居</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3845,13 +3845,13 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>32.04</v>
+        <v>2.8</v>
       </c>
       <c r="E75" t="n">
-        <v>31.47</v>
+        <v>2.77</v>
       </c>
       <c r="F75" t="n">
-        <v>29.95</v>
+        <v>2.61</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -3862,7 +3862,7 @@
         <v>52</v>
       </c>
       <c r="I75" t="n">
-        <v>4.263</v>
+        <v>2.941</v>
       </c>
       <c r="J75" t="n">
         <v>0</v>
@@ -3871,18 +3871,18 @@
         <v>1</v>
       </c>
       <c r="L75" t="n">
-        <v>8.5</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>sh600674</t>
+          <t>sh600328</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>川投能源</t>
+          <t>中盐化工</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3891,13 +3891,13 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>15.25</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="E76" t="n">
-        <v>15.17</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F76" t="n">
-        <v>14.75</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -3908,7 +3908,7 @@
         <v>52</v>
       </c>
       <c r="I76" t="n">
-        <v>1.262</v>
+        <v>0.6929999999999999</v>
       </c>
       <c r="J76" t="n">
         <v>0</v>
@@ -3917,18 +3917,18 @@
         <v>1</v>
       </c>
       <c r="L76" t="n">
-        <v>4.18</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>sh600664</t>
+          <t>sh600326</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>哈药股份</t>
+          <t>西藏天路</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3937,13 +3937,13 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>3.69</v>
+        <v>9.34</v>
       </c>
       <c r="E77" t="n">
-        <v>3.71</v>
+        <v>9.17</v>
       </c>
       <c r="F77" t="n">
-        <v>3.58</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -3954,7 +3954,7 @@
         <v>52</v>
       </c>
       <c r="I77" t="n">
-        <v>0.545</v>
+        <v>3.091</v>
       </c>
       <c r="J77" t="n">
         <v>0</v>
@@ -3963,18 +3963,18 @@
         <v>1</v>
       </c>
       <c r="L77" t="n">
-        <v>2.94</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>sh600642</t>
+          <t>sh600325</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>申能股份</t>
+          <t>华发股份</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3983,13 +3983,13 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>9.06</v>
+        <v>3.53</v>
       </c>
       <c r="E78" t="n">
-        <v>9</v>
+        <v>3.48</v>
       </c>
       <c r="F78" t="n">
-        <v>8.720000000000001</v>
+        <v>3.35</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -4000,7 +4000,7 @@
         <v>52</v>
       </c>
       <c r="I78" t="n">
-        <v>1.229</v>
+        <v>3.216</v>
       </c>
       <c r="J78" t="n">
         <v>0</v>
@@ -4009,18 +4009,18 @@
         <v>1</v>
       </c>
       <c r="L78" t="n">
-        <v>1.59</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>sh600641</t>
+          <t>sh600323</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>先导基电</t>
+          <t>瀚蓝环境</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -4029,13 +4029,13 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>27.6</v>
+        <v>32.43</v>
       </c>
       <c r="E79" t="n">
-        <v>26.95</v>
+        <v>31.96</v>
       </c>
       <c r="F79" t="n">
-        <v>24.99</v>
+        <v>30.78</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -4046,7 +4046,7 @@
         <v>52</v>
       </c>
       <c r="I79" t="n">
-        <v>4.072</v>
+        <v>3.511</v>
       </c>
       <c r="J79" t="n">
         <v>0</v>
@@ -4055,18 +4055,18 @@
         <v>1</v>
       </c>
       <c r="L79" t="n">
-        <v>11.51</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>sh600621</t>
+          <t>sh600316</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>华鑫股份</t>
+          <t>洪都航空</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4075,13 +4075,13 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>14.1</v>
+        <v>36.34</v>
       </c>
       <c r="E80" t="n">
-        <v>14.02</v>
+        <v>36.26</v>
       </c>
       <c r="F80" t="n">
-        <v>13.62</v>
+        <v>34.84</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -4092,7 +4092,7 @@
         <v>52</v>
       </c>
       <c r="I80" t="n">
-        <v>1.293</v>
+        <v>0.526</v>
       </c>
       <c r="J80" t="n">
         <v>0</v>
@@ -4101,18 +4101,18 @@
         <v>1</v>
       </c>
       <c r="L80" t="n">
-        <v>0.89</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>sh600619</t>
+          <t>sh600313</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>海立股份</t>
+          <t>农发种业</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4121,13 +4121,13 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>17.5</v>
+        <v>7.16</v>
       </c>
       <c r="E81" t="n">
-        <v>17.41</v>
+        <v>7.15</v>
       </c>
       <c r="F81" t="n">
-        <v>16.73</v>
+        <v>6.89</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -4138,7 +4138,7 @@
         <v>52</v>
       </c>
       <c r="I81" t="n">
-        <v>1.744</v>
+        <v>0.845</v>
       </c>
       <c r="J81" t="n">
         <v>0</v>
@@ -4147,18 +4147,18 @@
         <v>1</v>
       </c>
       <c r="L81" t="n">
-        <v>3.15</v>
+        <v>1.27</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>sh600617</t>
+          <t>sh600312</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>国新能源</t>
+          <t>平高电气</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4167,13 +4167,13 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>3.4</v>
+        <v>21.9</v>
       </c>
       <c r="E82" t="n">
-        <v>3.42</v>
+        <v>21.72</v>
       </c>
       <c r="F82" t="n">
-        <v>3.29</v>
+        <v>21.07</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -4184,7 +4184,7 @@
         <v>52</v>
       </c>
       <c r="I82" t="n">
-        <v>0.592</v>
+        <v>1.719</v>
       </c>
       <c r="J82" t="n">
         <v>0</v>
@@ -4193,7 +4193,7 @@
         <v>1</v>
       </c>
       <c r="L82" t="n">
-        <v>1.2</v>
+        <v>2.61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 实时报告更新 Wed Apr 29 04:51:05 UTC 2026
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>T:2026-04-29 10:46:24</t>
+          <t>T:2026-04-29 12:51:05</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -519,12 +519,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>sz301468</t>
+          <t>sz302132</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>博盈特焊</t>
+          <t>中航成飞</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -533,13 +533,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>50.6</v>
+        <v>67.84999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>50.6</v>
+        <v>67.28</v>
       </c>
       <c r="F3" t="n">
-        <v>48.34</v>
+        <v>65.37</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -550,7 +550,7 @@
         <v>52</v>
       </c>
       <c r="I3" t="n">
-        <v>0.576</v>
+        <v>1.602</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -559,18 +559,18 @@
         <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>0.8</v>
+        <v>2.61</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>sz301413</t>
+          <t>sz301498</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>安培龙</t>
+          <t>乖宝宠物</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -579,13 +579,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>97.66</v>
+        <v>55.83</v>
       </c>
       <c r="E4" t="n">
-        <v>97.67</v>
+        <v>55.25</v>
       </c>
       <c r="F4" t="n">
-        <v>94.67</v>
+        <v>53.21</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
         <v>52</v>
       </c>
       <c r="I4" t="n">
-        <v>0.525</v>
+        <v>3.007</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -605,18 +605,18 @@
         <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>sz301408</t>
+          <t>sz301487</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>华人健康</t>
+          <t>盟固利</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -625,13 +625,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>20.84</v>
+        <v>23.75</v>
       </c>
       <c r="E5" t="n">
-        <v>20.73</v>
+        <v>23.16</v>
       </c>
       <c r="F5" t="n">
-        <v>19.11</v>
+        <v>22.11</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
         <v>52</v>
       </c>
       <c r="I5" t="n">
-        <v>1.758</v>
+        <v>4.258</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -651,18 +651,18 @@
         <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>4.05</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>sz301392</t>
+          <t>sz301468</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>汇成真空</t>
+          <t>博盈特焊</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -671,13 +671,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>159.26</v>
+        <v>50.88</v>
       </c>
       <c r="E6" t="n">
-        <v>158.16</v>
+        <v>50.61</v>
       </c>
       <c r="F6" t="n">
-        <v>149.94</v>
+        <v>48.34</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         <v>52</v>
       </c>
       <c r="I6" t="n">
-        <v>1.783</v>
+        <v>1.133</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -697,18 +697,18 @@
         <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>3.35</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>sz301389</t>
+          <t>sz301428</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>隆扬电子</t>
+          <t>世纪恒通</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -717,13 +717,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>64.05</v>
+        <v>33.36</v>
       </c>
       <c r="E7" t="n">
-        <v>63.54</v>
+        <v>33.17</v>
       </c>
       <c r="F7" t="n">
-        <v>60.02</v>
+        <v>31.91</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -734,7 +734,7 @@
         <v>52</v>
       </c>
       <c r="I7" t="n">
-        <v>2.153</v>
+        <v>1.367</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -743,18 +743,18 @@
         <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>3.62</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>sz301382</t>
+          <t>sz301421</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>蜂助手</t>
+          <t>波长光电</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -763,13 +763,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>42.8</v>
+        <v>101.01</v>
       </c>
       <c r="E8" t="n">
-        <v>42.27</v>
+        <v>100.6</v>
       </c>
       <c r="F8" t="n">
-        <v>39.96</v>
+        <v>95.08</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -780,7 +780,7 @@
         <v>52</v>
       </c>
       <c r="I8" t="n">
-        <v>2.638</v>
+        <v>1.01</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -789,18 +789,18 @@
         <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>3.92</v>
+        <v>3.37</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>sz301378</t>
+          <t>sz301413</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>通达海</t>
+          <t>安培龙</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -809,13 +809,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>31.89</v>
+        <v>97.67</v>
       </c>
       <c r="E9" t="n">
-        <v>31.54</v>
+        <v>97.67</v>
       </c>
       <c r="F9" t="n">
-        <v>29.86</v>
+        <v>94.67</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -826,7 +826,7 @@
         <v>52</v>
       </c>
       <c r="I9" t="n">
-        <v>3.237</v>
+        <v>0.535</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -835,18 +835,18 @@
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>0.99</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>sz301377</t>
+          <t>sz301408</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>鼎泰高科</t>
+          <t>华人健康</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -855,13 +855,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>227.85</v>
+        <v>20.88</v>
       </c>
       <c r="E10" t="n">
-        <v>225.24</v>
+        <v>20.73</v>
       </c>
       <c r="F10" t="n">
-        <v>216.4</v>
+        <v>19.11</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -872,7 +872,7 @@
         <v>52</v>
       </c>
       <c r="I10" t="n">
-        <v>2.175</v>
+        <v>1.953</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -881,18 +881,18 @@
         <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>3.1</v>
+        <v>4.62</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>sz301373</t>
+          <t>sz301392</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>凌玮科技</t>
+          <t>汇成真空</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -901,13 +901,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>116.56</v>
+        <v>159.6</v>
       </c>
       <c r="E11" t="n">
-        <v>114.85</v>
+        <v>158.16</v>
       </c>
       <c r="F11" t="n">
-        <v>108.9</v>
+        <v>149.94</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -918,7 +918,7 @@
         <v>52</v>
       </c>
       <c r="I11" t="n">
-        <v>2.47</v>
+        <v>2</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -927,18 +927,18 @@
         <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>3.09</v>
+        <v>3.83</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>sz301372</t>
+          <t>sz301389</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>科净源</t>
+          <t>隆扬电子</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -947,13 +947,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>35.53</v>
+        <v>63.41</v>
       </c>
       <c r="E12" t="n">
-        <v>35</v>
+        <v>63.54</v>
       </c>
       <c r="F12" t="n">
-        <v>33.33</v>
+        <v>60.02</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         <v>52</v>
       </c>
       <c r="I12" t="n">
-        <v>4.408</v>
+        <v>1.132</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -973,18 +973,18 @@
         <v>1</v>
       </c>
       <c r="L12" t="n">
-        <v>0.95</v>
+        <v>4.23</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>sz301371</t>
+          <t>sz301382</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>敷尔佳</t>
+          <t>蜂助手</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -993,13 +993,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>29.45</v>
+        <v>43.25</v>
       </c>
       <c r="E13" t="n">
-        <v>29.13</v>
+        <v>42.42</v>
       </c>
       <c r="F13" t="n">
-        <v>27.6</v>
+        <v>39.96</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
         <v>52</v>
       </c>
       <c r="I13" t="n">
-        <v>2.506</v>
+        <v>3.717</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -1019,18 +1019,18 @@
         <v>1</v>
       </c>
       <c r="L13" t="n">
-        <v>0.95</v>
+        <v>5.23</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>sz301362</t>
+          <t>sz301378</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>民爆光电</t>
+          <t>通达海</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1039,13 +1039,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>142.82</v>
+        <v>32.13</v>
       </c>
       <c r="E14" t="n">
-        <v>140.19</v>
+        <v>31.54</v>
       </c>
       <c r="F14" t="n">
-        <v>130.69</v>
+        <v>29.86</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
         <v>52</v>
       </c>
       <c r="I14" t="n">
-        <v>3.854</v>
+        <v>4.014</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -1065,18 +1065,18 @@
         <v>1</v>
       </c>
       <c r="L14" t="n">
-        <v>2.15</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>sz301360</t>
+          <t>sz301377</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>荣旗科技</t>
+          <t>鼎泰高科</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1085,13 +1085,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>87.3</v>
+        <v>233</v>
       </c>
       <c r="E15" t="n">
-        <v>85.33</v>
+        <v>227.58</v>
       </c>
       <c r="F15" t="n">
-        <v>81.23</v>
+        <v>216.4</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1102,7 +1102,7 @@
         <v>52</v>
       </c>
       <c r="I15" t="n">
-        <v>4.314</v>
+        <v>4.484</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -1111,18 +1111,18 @@
         <v>1</v>
       </c>
       <c r="L15" t="n">
-        <v>0.8</v>
+        <v>5.52</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>sz301317</t>
+          <t>sz301373</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>鑫磊股份</t>
+          <t>凌玮科技</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1131,13 +1131,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>60.48</v>
+        <v>114.4</v>
       </c>
       <c r="E16" t="n">
-        <v>61.21</v>
+        <v>114.94</v>
       </c>
       <c r="F16" t="n">
-        <v>55.24</v>
+        <v>108.9</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
         <v>52</v>
       </c>
       <c r="I16" t="n">
-        <v>0.666</v>
+        <v>0.571</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1157,18 +1157,18 @@
         <v>1</v>
       </c>
       <c r="L16" t="n">
-        <v>3.96</v>
+        <v>3.97</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>sz301316</t>
+          <t>sz301372</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>慧博云通</t>
+          <t>科净源</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1177,13 +1177,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>47.47</v>
+        <v>35.52</v>
       </c>
       <c r="E17" t="n">
-        <v>47.37</v>
+        <v>35</v>
       </c>
       <c r="F17" t="n">
-        <v>44.98</v>
+        <v>33.33</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1194,7 +1194,7 @@
         <v>52</v>
       </c>
       <c r="I17" t="n">
-        <v>2.416</v>
+        <v>4.378</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1203,18 +1203,18 @@
         <v>1</v>
       </c>
       <c r="L17" t="n">
-        <v>3.86</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>sz301302</t>
+          <t>sz301371</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>华如科技</t>
+          <t>敷尔佳</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1223,13 +1223,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>24.25</v>
+        <v>29.34</v>
       </c>
       <c r="E18" t="n">
-        <v>24.13</v>
+        <v>29.13</v>
       </c>
       <c r="F18" t="n">
-        <v>23.46</v>
+        <v>27.6</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1240,7 +1240,7 @@
         <v>52</v>
       </c>
       <c r="I18" t="n">
-        <v>1.38</v>
+        <v>2.123</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1249,18 +1249,18 @@
         <v>1</v>
       </c>
       <c r="L18" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>sh600133</t>
+          <t>sz301365</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>东湖高新</t>
+          <t>矩阵股份</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1269,13 +1269,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>8.84</v>
+        <v>36.22</v>
       </c>
       <c r="E19" t="n">
-        <v>8.82</v>
+        <v>35.68</v>
       </c>
       <c r="F19" t="n">
-        <v>8.539999999999999</v>
+        <v>32.7</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1286,7 +1286,7 @@
         <v>52</v>
       </c>
       <c r="I19" t="n">
-        <v>0.569</v>
+        <v>4.894</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1295,18 +1295,18 @@
         <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>0.91</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>sh600131</t>
+          <t>sh600108</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>国网信通</t>
+          <t>亚盛集团</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1315,13 +1315,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>17.22</v>
+        <v>4.3</v>
       </c>
       <c r="E20" t="n">
-        <v>17.03</v>
+        <v>4.23</v>
       </c>
       <c r="F20" t="n">
-        <v>16.47</v>
+        <v>4.06</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1332,7 +1332,7 @@
         <v>52</v>
       </c>
       <c r="I20" t="n">
-        <v>2.439</v>
+        <v>2.871</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1341,18 +1341,18 @@
         <v>1</v>
       </c>
       <c r="L20" t="n">
-        <v>1.52</v>
+        <v>1.74</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>sh600127</t>
+          <t>sh600104</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>金健米业</t>
+          <t>上汽集团</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1361,13 +1361,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>6.84</v>
+        <v>13.68</v>
       </c>
       <c r="E21" t="n">
-        <v>6.81</v>
+        <v>13.64</v>
       </c>
       <c r="F21" t="n">
-        <v>6.59</v>
+        <v>13.28</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1378,7 +1378,7 @@
         <v>52</v>
       </c>
       <c r="I21" t="n">
-        <v>1.034</v>
+        <v>0.588</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1387,18 +1387,18 @@
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>0.82</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>sh600126</t>
+          <t>sh600103</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>杭钢股份</t>
+          <t>青山纸业</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1407,13 +1407,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>9.300000000000001</v>
+        <v>4.7</v>
       </c>
       <c r="E22" t="n">
-        <v>9.26</v>
+        <v>4.63</v>
       </c>
       <c r="F22" t="n">
-        <v>8.789999999999999</v>
+        <v>4.41</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1424,7 +1424,7 @@
         <v>52</v>
       </c>
       <c r="I22" t="n">
-        <v>1.639</v>
+        <v>3.524</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1433,18 +1433,18 @@
         <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>7.32</v>
+        <v>7.58</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>sh600121</t>
+          <t>sh600101</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>郑州煤电</t>
+          <t>明星电力</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1453,13 +1453,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>4.31</v>
+        <v>9.9</v>
       </c>
       <c r="E23" t="n">
-        <v>4.25</v>
+        <v>9.69</v>
       </c>
       <c r="F23" t="n">
-        <v>4.09</v>
+        <v>9.32</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1470,7 +1470,7 @@
         <v>52</v>
       </c>
       <c r="I23" t="n">
-        <v>2.619</v>
+        <v>3.665</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1479,18 +1479,18 @@
         <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>1.26</v>
+        <v>1.99</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>sh600116</t>
+          <t>sh600078</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>三峡水利</t>
+          <t>澄星股份</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1499,13 +1499,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>6.61</v>
+        <v>13.28</v>
       </c>
       <c r="E24" t="n">
-        <v>6.59</v>
+        <v>12.98</v>
       </c>
       <c r="F24" t="n">
-        <v>6.36</v>
+        <v>12.31</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1516,7 +1516,7 @@
         <v>52</v>
       </c>
       <c r="I24" t="n">
-        <v>0.916</v>
+        <v>4.321</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1525,18 +1525,18 @@
         <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>1.03</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>sh600114</t>
+          <t>sh600066</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>东睦股份</t>
+          <t>宇通客车</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1545,13 +1545,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>32.87</v>
+        <v>35.82</v>
       </c>
       <c r="E25" t="n">
-        <v>32.75</v>
+        <v>35.71</v>
       </c>
       <c r="F25" t="n">
-        <v>31.66</v>
+        <v>34.2</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1562,7 +1562,7 @@
         <v>52</v>
       </c>
       <c r="I25" t="n">
-        <v>0.828</v>
+        <v>0.533</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1571,18 +1571,18 @@
         <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>1.62</v>
+        <v>4.79</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sh600110</t>
+          <t>sh600063</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>诺德股份</t>
+          <t>皖维高新</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1591,13 +1591,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>10.74</v>
+        <v>7.18</v>
       </c>
       <c r="E26" t="n">
-        <v>10.67</v>
+        <v>7.05</v>
       </c>
       <c r="F26" t="n">
-        <v>10.19</v>
+        <v>6.75</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1608,7 +1608,7 @@
         <v>52</v>
       </c>
       <c r="I26" t="n">
-        <v>1.705</v>
+        <v>3.161</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1617,18 +1617,18 @@
         <v>1</v>
       </c>
       <c r="L26" t="n">
-        <v>9.44</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>sh600109</t>
+          <t>sh600060</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>国金证券</t>
+          <t>海信视像</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1637,13 +1637,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>8.949999999999999</v>
+        <v>24.88</v>
       </c>
       <c r="E27" t="n">
-        <v>8.880000000000001</v>
+        <v>24.77</v>
       </c>
       <c r="F27" t="n">
-        <v>8.6</v>
+        <v>23.84</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1654,7 +1654,7 @@
         <v>52</v>
       </c>
       <c r="I27" t="n">
-        <v>1.474</v>
+        <v>1.51</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1663,18 +1663,18 @@
         <v>1</v>
       </c>
       <c r="L27" t="n">
-        <v>1.68</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>sh600108</t>
+          <t>sh600057</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>亚盛集团</t>
+          <t>厦门象屿</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1683,13 +1683,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>4.27</v>
+        <v>7.3</v>
       </c>
       <c r="E28" t="n">
-        <v>4.23</v>
+        <v>7.23</v>
       </c>
       <c r="F28" t="n">
-        <v>4.06</v>
+        <v>6.96</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1700,7 +1700,7 @@
         <v>52</v>
       </c>
       <c r="I28" t="n">
-        <v>2.153</v>
+        <v>2.098</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1709,18 +1709,18 @@
         <v>1</v>
       </c>
       <c r="L28" t="n">
-        <v>1.38</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>sh600103</t>
+          <t>sh600056</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>青山纸业</t>
+          <t>中国医药</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1729,13 +1729,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>4.72</v>
+        <v>10.4</v>
       </c>
       <c r="E29" t="n">
-        <v>4.63</v>
+        <v>10.33</v>
       </c>
       <c r="F29" t="n">
-        <v>4.41</v>
+        <v>10.07</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1746,7 +1746,7 @@
         <v>52</v>
       </c>
       <c r="I29" t="n">
-        <v>3.965</v>
+        <v>1.167</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1755,18 +1755,18 @@
         <v>1</v>
       </c>
       <c r="L29" t="n">
-        <v>6.77</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>sh600101</t>
+          <t>sh600055</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>明星电力</t>
+          <t>万东医疗</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1775,13 +1775,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>9.880000000000001</v>
+        <v>15.02</v>
       </c>
       <c r="E30" t="n">
-        <v>9.69</v>
+        <v>14.95</v>
       </c>
       <c r="F30" t="n">
-        <v>9.32</v>
+        <v>14.27</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1792,7 +1792,7 @@
         <v>52</v>
       </c>
       <c r="I30" t="n">
-        <v>3.455</v>
+        <v>2.526</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1801,18 +1801,18 @@
         <v>1</v>
       </c>
       <c r="L30" t="n">
-        <v>1.81</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>sh600095</t>
+          <t>sh600054</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>湘财股份</t>
+          <t>黄山旅游</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1821,13 +1821,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>8.869999999999999</v>
+        <v>11.93</v>
       </c>
       <c r="E31" t="n">
-        <v>8.85</v>
+        <v>11.77</v>
       </c>
       <c r="F31" t="n">
-        <v>8.550000000000001</v>
+        <v>11.39</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1838,7 +1838,7 @@
         <v>52</v>
       </c>
       <c r="I31" t="n">
-        <v>0.5669999999999999</v>
+        <v>2.316</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1847,18 +1847,18 @@
         <v>1</v>
       </c>
       <c r="L31" t="n">
-        <v>0.83</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>sh600078</t>
+          <t>sh600048</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>澄星股份</t>
+          <t>保利发展</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1867,13 +1867,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>12.89</v>
+        <v>6.12</v>
       </c>
       <c r="E32" t="n">
-        <v>12.79</v>
+        <v>6.08</v>
       </c>
       <c r="F32" t="n">
-        <v>12.31</v>
+        <v>5.87</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         <v>52</v>
       </c>
       <c r="I32" t="n">
-        <v>1.257</v>
+        <v>1.493</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1893,18 +1893,18 @@
         <v>1</v>
       </c>
       <c r="L32" t="n">
-        <v>1.13</v>
+        <v>6.02</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>sh600063</t>
+          <t>sh600029</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>皖维高新</t>
+          <t>南方航空</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1913,13 +1913,13 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>7.1</v>
+        <v>5.48</v>
       </c>
       <c r="E33" t="n">
-        <v>7.01</v>
+        <v>5.46</v>
       </c>
       <c r="F33" t="n">
-        <v>6.75</v>
+        <v>5.3</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1930,7 +1930,7 @@
         <v>52</v>
       </c>
       <c r="I33" t="n">
-        <v>2.011</v>
+        <v>0.735</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1939,18 +1939,18 @@
         <v>1</v>
       </c>
       <c r="L33" t="n">
-        <v>1.32</v>
+        <v>2.33</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>sh600060</t>
+          <t>sh600026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>海信视像</t>
+          <t>中远海能</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1959,13 +1959,13 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>24.88</v>
+        <v>21.39</v>
       </c>
       <c r="E34" t="n">
-        <v>24.77</v>
+        <v>21.28</v>
       </c>
       <c r="F34" t="n">
-        <v>23.84</v>
+        <v>20.78</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1976,7 +1976,7 @@
         <v>52</v>
       </c>
       <c r="I34" t="n">
-        <v>1.51</v>
+        <v>1.615</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1985,18 +1985,18 @@
         <v>1</v>
       </c>
       <c r="L34" t="n">
-        <v>1.74</v>
+        <v>8.41</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>sh600219</t>
+          <t>sh600022</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>南山铝业</t>
+          <t>山东钢铁</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2005,13 +2005,13 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>5.34</v>
+        <v>1.47</v>
       </c>
       <c r="E35" t="n">
-        <v>5.31</v>
+        <v>1.45</v>
       </c>
       <c r="F35" t="n">
-        <v>5.1</v>
+        <v>1.4</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2022,7 +2022,7 @@
         <v>52</v>
       </c>
       <c r="I35" t="n">
-        <v>0.945</v>
+        <v>2.083</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -2031,18 +2031,18 @@
         <v>1</v>
       </c>
       <c r="L35" t="n">
-        <v>6.36</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>sh600211</t>
+          <t>sh600160</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>西藏药业</t>
+          <t>巨化股份</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2051,13 +2051,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>41.25</v>
+        <v>36.62</v>
       </c>
       <c r="E36" t="n">
-        <v>40.64</v>
+        <v>36.67</v>
       </c>
       <c r="F36" t="n">
-        <v>39.74</v>
+        <v>35.6</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2068,7 +2068,7 @@
         <v>52</v>
       </c>
       <c r="I36" t="n">
-        <v>2.996</v>
+        <v>1.104</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -2077,18 +2077,18 @@
         <v>1</v>
       </c>
       <c r="L36" t="n">
-        <v>1.53</v>
+        <v>10.96</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>sh600210</t>
+          <t>sh600158</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>紫江企业</t>
+          <t>中体产业</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2097,13 +2097,13 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>7.15</v>
+        <v>10.63</v>
       </c>
       <c r="E37" t="n">
-        <v>7.04</v>
+        <v>10.42</v>
       </c>
       <c r="F37" t="n">
-        <v>6.96</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -2114,7 +2114,7 @@
         <v>52</v>
       </c>
       <c r="I37" t="n">
-        <v>4.227</v>
+        <v>4.216</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -2123,18 +2123,18 @@
         <v>1</v>
       </c>
       <c r="L37" t="n">
-        <v>2.81</v>
+        <v>4.94</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>sh600208</t>
+          <t>sh600157</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>衢州发展</t>
+          <t>永泰能源</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2143,13 +2143,13 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>4.16</v>
+        <v>1.8</v>
       </c>
       <c r="E38" t="n">
-        <v>4.17</v>
+        <v>1.77</v>
       </c>
       <c r="F38" t="n">
-        <v>3.99</v>
+        <v>1.71</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -2160,7 +2160,7 @@
         <v>52</v>
       </c>
       <c r="I38" t="n">
-        <v>1.217</v>
+        <v>2.857</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -2169,18 +2169,18 @@
         <v>1</v>
       </c>
       <c r="L38" t="n">
-        <v>6.12</v>
+        <v>11.74</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>sh600206</t>
+          <t>sh600151</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>有研新材</t>
+          <t>航天机电</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2189,13 +2189,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>26.88</v>
+        <v>13.98</v>
       </c>
       <c r="E39" t="n">
-        <v>26.8</v>
+        <v>13.87</v>
       </c>
       <c r="F39" t="n">
-        <v>25.67</v>
+        <v>13.08</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -2206,7 +2206,7 @@
         <v>52</v>
       </c>
       <c r="I39" t="n">
-        <v>0.9389999999999999</v>
+        <v>2.044</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2215,18 +2215,18 @@
         <v>1</v>
       </c>
       <c r="L39" t="n">
-        <v>9.08</v>
+        <v>3.83</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>sh600201</t>
+          <t>sh600149</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>生物股份</t>
+          <t>廊坊发展</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2235,13 +2235,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>13.89</v>
+        <v>6.34</v>
       </c>
       <c r="E40" t="n">
-        <v>13.8</v>
+        <v>6.33</v>
       </c>
       <c r="F40" t="n">
-        <v>13.33</v>
+        <v>6.08</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -2252,7 +2252,7 @@
         <v>52</v>
       </c>
       <c r="I40" t="n">
-        <v>2.283</v>
+        <v>0.635</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2261,18 +2261,18 @@
         <v>1</v>
       </c>
       <c r="L40" t="n">
-        <v>2.18</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>sh600187</t>
+          <t>sh600143</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>国中水务</t>
+          <t>金发科技</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2281,13 +2281,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1.83</v>
+        <v>17</v>
       </c>
       <c r="E41" t="n">
-        <v>1.8</v>
+        <v>16.76</v>
       </c>
       <c r="F41" t="n">
-        <v>1.71</v>
+        <v>16.17</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -2298,7 +2298,7 @@
         <v>52</v>
       </c>
       <c r="I41" t="n">
-        <v>3.977</v>
+        <v>2.348</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2307,18 +2307,18 @@
         <v>1</v>
       </c>
       <c r="L41" t="n">
-        <v>0.95</v>
+        <v>4.29</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>sh600177</t>
+          <t>sh600141</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>雅戈尔</t>
+          <t>兴发集团</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2327,13 +2327,13 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>7.63</v>
+        <v>33.63</v>
       </c>
       <c r="E42" t="n">
-        <v>7.55</v>
+        <v>33.05</v>
       </c>
       <c r="F42" t="n">
-        <v>7.29</v>
+        <v>29.95</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -2344,7 +2344,7 @@
         <v>52</v>
       </c>
       <c r="I42" t="n">
-        <v>2.416</v>
+        <v>2.875</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
@@ -2353,18 +2353,18 @@
         <v>1</v>
       </c>
       <c r="L42" t="n">
-        <v>1.86</v>
+        <v>11.52</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>sh600172</t>
+          <t>sh600133</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>黄河旋风</t>
+          <t>东湖高新</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2373,13 +2373,13 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>8.26</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="E43" t="n">
-        <v>8.1</v>
+        <v>8.82</v>
       </c>
       <c r="F43" t="n">
-        <v>7.75</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -2390,7 +2390,7 @@
         <v>52</v>
       </c>
       <c r="I43" t="n">
-        <v>3.379</v>
+        <v>0.796</v>
       </c>
       <c r="J43" t="n">
         <v>0</v>
@@ -2399,18 +2399,18 @@
         <v>1</v>
       </c>
       <c r="L43" t="n">
-        <v>2.86</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>sh600170</t>
+          <t>sh600131</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>上海建工</t>
+          <t>国网信通</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2419,13 +2419,13 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>2.67</v>
+        <v>17.28</v>
       </c>
       <c r="E44" t="n">
-        <v>2.67</v>
+        <v>17.03</v>
       </c>
       <c r="F44" t="n">
-        <v>2.6</v>
+        <v>16.47</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -2436,7 +2436,7 @@
         <v>52</v>
       </c>
       <c r="I44" t="n">
-        <v>0.755</v>
+        <v>2.796</v>
       </c>
       <c r="J44" t="n">
         <v>0</v>
@@ -2445,18 +2445,18 @@
         <v>1</v>
       </c>
       <c r="L44" t="n">
-        <v>1.53</v>
+        <v>1.82</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>sh600160</t>
+          <t>sh600127</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>巨化股份</t>
+          <t>金健米业</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2465,13 +2465,13 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>36.79</v>
+        <v>6.84</v>
       </c>
       <c r="E45" t="n">
-        <v>36.67</v>
+        <v>6.81</v>
       </c>
       <c r="F45" t="n">
-        <v>35.6</v>
+        <v>6.59</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2482,7 +2482,7 @@
         <v>52</v>
       </c>
       <c r="I45" t="n">
-        <v>1.574</v>
+        <v>1.034</v>
       </c>
       <c r="J45" t="n">
         <v>0</v>
@@ -2491,18 +2491,18 @@
         <v>1</v>
       </c>
       <c r="L45" t="n">
-        <v>8.859999999999999</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>sh600158</t>
+          <t>sh600126</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>中体产业</t>
+          <t>杭钢股份</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2511,13 +2511,13 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>10.66</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="E46" t="n">
-        <v>10.42</v>
+        <v>9.26</v>
       </c>
       <c r="F46" t="n">
-        <v>9.859999999999999</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2528,7 +2528,7 @@
         <v>52</v>
       </c>
       <c r="I46" t="n">
-        <v>4.51</v>
+        <v>1.421</v>
       </c>
       <c r="J46" t="n">
         <v>0</v>
@@ -2537,18 +2537,18 @@
         <v>1</v>
       </c>
       <c r="L46" t="n">
-        <v>4.65</v>
+        <v>8.43</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>sh600157</t>
+          <t>sh600123</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>永泰能源</t>
+          <t>兰花科创</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2557,13 +2557,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1.79</v>
+        <v>6.89</v>
       </c>
       <c r="E47" t="n">
-        <v>1.77</v>
+        <v>6.88</v>
       </c>
       <c r="F47" t="n">
-        <v>1.71</v>
+        <v>6.64</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -2574,7 +2574,7 @@
         <v>52</v>
       </c>
       <c r="I47" t="n">
-        <v>2.286</v>
+        <v>0.584</v>
       </c>
       <c r="J47" t="n">
         <v>0</v>
@@ -2583,18 +2583,18 @@
         <v>1</v>
       </c>
       <c r="L47" t="n">
-        <v>10.94</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>sh600151</t>
+          <t>sh600121</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>航天机电</t>
+          <t>郑州煤电</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2603,13 +2603,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>13.98</v>
+        <v>4.32</v>
       </c>
       <c r="E48" t="n">
-        <v>13.87</v>
+        <v>4.25</v>
       </c>
       <c r="F48" t="n">
-        <v>13.08</v>
+        <v>4.09</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2620,7 +2620,7 @@
         <v>52</v>
       </c>
       <c r="I48" t="n">
-        <v>2.044</v>
+        <v>2.857</v>
       </c>
       <c r="J48" t="n">
         <v>0</v>
@@ -2629,18 +2629,18 @@
         <v>1</v>
       </c>
       <c r="L48" t="n">
-        <v>3.45</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>sh600143</t>
+          <t>sh600116</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>金发科技</t>
+          <t>三峡水利</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2649,13 +2649,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>16.91</v>
+        <v>6.64</v>
       </c>
       <c r="E49" t="n">
-        <v>16.73</v>
+        <v>6.59</v>
       </c>
       <c r="F49" t="n">
-        <v>16.17</v>
+        <v>6.36</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2666,7 +2666,7 @@
         <v>52</v>
       </c>
       <c r="I49" t="n">
-        <v>1.806</v>
+        <v>1.374</v>
       </c>
       <c r="J49" t="n">
         <v>0</v>
@@ -2675,18 +2675,18 @@
         <v>1</v>
       </c>
       <c r="L49" t="n">
-        <v>2.89</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>sh600141</t>
+          <t>sh600114</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>兴发集团</t>
+          <t>东睦股份</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2695,13 +2695,13 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>33.16</v>
+        <v>33.11</v>
       </c>
       <c r="E50" t="n">
-        <v>32.88</v>
+        <v>32.82</v>
       </c>
       <c r="F50" t="n">
-        <v>29.95</v>
+        <v>31.66</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2712,7 +2712,7 @@
         <v>52</v>
       </c>
       <c r="I50" t="n">
-        <v>1.438</v>
+        <v>1.564</v>
       </c>
       <c r="J50" t="n">
         <v>0</v>
@@ -2721,18 +2721,18 @@
         <v>1</v>
       </c>
       <c r="L50" t="n">
-        <v>9.19</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>sh600309</t>
+          <t>sh600109</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>万华化学</t>
+          <t>国金证券</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2741,13 +2741,13 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>90</v>
+        <v>8.94</v>
       </c>
       <c r="E51" t="n">
-        <v>89.81999999999999</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="F51" t="n">
-        <v>86.76000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2758,7 +2758,7 @@
         <v>52</v>
       </c>
       <c r="I51" t="n">
-        <v>0.581</v>
+        <v>1.361</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
@@ -2767,18 +2767,18 @@
         <v>1</v>
       </c>
       <c r="L51" t="n">
-        <v>10.11</v>
+        <v>1.99</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>sh600307</t>
+          <t>sh600230</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>酒钢宏兴</t>
+          <t>沧州大化</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2787,13 +2787,13 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>1.79</v>
+        <v>19.54</v>
       </c>
       <c r="E52" t="n">
-        <v>1.77</v>
+        <v>19.47</v>
       </c>
       <c r="F52" t="n">
-        <v>1.7</v>
+        <v>18.54</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2804,7 +2804,7 @@
         <v>52</v>
       </c>
       <c r="I52" t="n">
-        <v>2.286</v>
+        <v>1.612</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -2813,18 +2813,18 @@
         <v>1</v>
       </c>
       <c r="L52" t="n">
-        <v>0.89</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>sh600301</t>
+          <t>sh600226</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>华锡有色</t>
+          <t>亨通股份</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2833,13 +2833,13 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>49.49</v>
+        <v>5.28</v>
       </c>
       <c r="E53" t="n">
-        <v>49.34</v>
+        <v>5.27</v>
       </c>
       <c r="F53" t="n">
-        <v>47.63</v>
+        <v>5.05</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2850,7 +2850,7 @@
         <v>52</v>
       </c>
       <c r="I53" t="n">
-        <v>0.63</v>
+        <v>0.571</v>
       </c>
       <c r="J53" t="n">
         <v>0</v>
@@ -2859,18 +2859,18 @@
         <v>1</v>
       </c>
       <c r="L53" t="n">
-        <v>2.53</v>
+        <v>1.39</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>sh600299</t>
+          <t>sh600221</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>安迪苏</t>
+          <t>海航控股</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2879,13 +2879,13 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>13.87</v>
+        <v>1.45</v>
       </c>
       <c r="E54" t="n">
-        <v>13.95</v>
+        <v>1.44</v>
       </c>
       <c r="F54" t="n">
-        <v>13.43</v>
+        <v>1.39</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2896,7 +2896,7 @@
         <v>52</v>
       </c>
       <c r="I54" t="n">
-        <v>0.507</v>
+        <v>1.399</v>
       </c>
       <c r="J54" t="n">
         <v>0</v>
@@ -2905,18 +2905,18 @@
         <v>1</v>
       </c>
       <c r="L54" t="n">
-        <v>1.25</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>sh600298</t>
+          <t>sh600219</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>安琪酵母</t>
+          <t>南山铝业</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2925,13 +2925,13 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>38.5</v>
+        <v>5.33</v>
       </c>
       <c r="E55" t="n">
-        <v>38.44</v>
+        <v>5.31</v>
       </c>
       <c r="F55" t="n">
-        <v>37.45</v>
+        <v>5.1</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2942,7 +2942,7 @@
         <v>52</v>
       </c>
       <c r="I55" t="n">
-        <v>0.575</v>
+        <v>0.756</v>
       </c>
       <c r="J55" t="n">
         <v>0</v>
@@ -2951,18 +2951,18 @@
         <v>1</v>
       </c>
       <c r="L55" t="n">
-        <v>1.46</v>
+        <v>7.78</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>sh600282</t>
+          <t>sh600211</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>南钢股份</t>
+          <t>西藏药业</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2971,13 +2971,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>5.44</v>
+        <v>41.26</v>
       </c>
       <c r="E56" t="n">
-        <v>5.43</v>
+        <v>40.64</v>
       </c>
       <c r="F56" t="n">
-        <v>5.25</v>
+        <v>39.74</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2988,7 +2988,7 @@
         <v>52</v>
       </c>
       <c r="I56" t="n">
-        <v>1.493</v>
+        <v>3.021</v>
       </c>
       <c r="J56" t="n">
         <v>0</v>
@@ -2997,18 +2997,18 @@
         <v>1</v>
       </c>
       <c r="L56" t="n">
-        <v>1.34</v>
+        <v>1.64</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>sh600271</t>
+          <t>sh600210</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>航天信息</t>
+          <t>紫江企业</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3017,13 +3017,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>8.279999999999999</v>
+        <v>7.14</v>
       </c>
       <c r="E57" t="n">
-        <v>8.15</v>
+        <v>7.04</v>
       </c>
       <c r="F57" t="n">
-        <v>7.87</v>
+        <v>6.96</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -3034,7 +3034,7 @@
         <v>52</v>
       </c>
       <c r="I57" t="n">
-        <v>2.602</v>
+        <v>4.082</v>
       </c>
       <c r="J57" t="n">
         <v>0</v>
@@ -3043,18 +3043,18 @@
         <v>1</v>
       </c>
       <c r="L57" t="n">
-        <v>0.86</v>
+        <v>3.14</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>sh600268</t>
+          <t>sh600208</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>国电南自</t>
+          <t>衢州发展</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3063,13 +3063,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>15.11</v>
+        <v>4.23</v>
       </c>
       <c r="E58" t="n">
-        <v>14.86</v>
+        <v>4.17</v>
       </c>
       <c r="F58" t="n">
-        <v>14.39</v>
+        <v>3.99</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -3080,7 +3080,7 @@
         <v>52</v>
       </c>
       <c r="I58" t="n">
-        <v>2.999</v>
+        <v>2.92</v>
       </c>
       <c r="J58" t="n">
         <v>0</v>
@@ -3089,18 +3089,18 @@
         <v>1</v>
       </c>
       <c r="L58" t="n">
-        <v>1.83</v>
+        <v>6.96</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>sh600262</t>
+          <t>sh600206</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>北方股份</t>
+          <t>有研新材</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3109,13 +3109,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>24.36</v>
+        <v>26.89</v>
       </c>
       <c r="E59" t="n">
-        <v>23.91</v>
+        <v>26.8</v>
       </c>
       <c r="F59" t="n">
-        <v>23.63</v>
+        <v>25.67</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -3126,7 +3126,7 @@
         <v>52</v>
       </c>
       <c r="I59" t="n">
-        <v>4.281</v>
+        <v>0.976</v>
       </c>
       <c r="J59" t="n">
         <v>0</v>
@@ -3135,18 +3135,18 @@
         <v>1</v>
       </c>
       <c r="L59" t="n">
-        <v>2.23</v>
+        <v>10.73</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>sh600256</t>
+          <t>sh600201</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>广汇能源</t>
+          <t>生物股份</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3155,13 +3155,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>6.55</v>
+        <v>13.97</v>
       </c>
       <c r="E60" t="n">
-        <v>6.56</v>
+        <v>13.8</v>
       </c>
       <c r="F60" t="n">
-        <v>6.34</v>
+        <v>13.33</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -3172,7 +3172,7 @@
         <v>52</v>
       </c>
       <c r="I60" t="n">
-        <v>0.769</v>
+        <v>2.872</v>
       </c>
       <c r="J60" t="n">
         <v>0</v>
@@ -3181,18 +3181,18 @@
         <v>1</v>
       </c>
       <c r="L60" t="n">
-        <v>6.54</v>
+        <v>2.46</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>sh600251</t>
+          <t>sh600198</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>冠农股份</t>
+          <t>大唐电信</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3201,13 +3201,13 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>12.27</v>
+        <v>8.17</v>
       </c>
       <c r="E61" t="n">
-        <v>12.23</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="F61" t="n">
-        <v>11.76</v>
+        <v>7.71</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -3218,7 +3218,7 @@
         <v>52</v>
       </c>
       <c r="I61" t="n">
-        <v>1.91</v>
+        <v>2.897</v>
       </c>
       <c r="J61" t="n">
         <v>0</v>
@@ -3227,18 +3227,18 @@
         <v>1</v>
       </c>
       <c r="L61" t="n">
-        <v>1.26</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>sh600234</t>
+          <t>sh600187</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>科新发展</t>
+          <t>国中水务</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3247,13 +3247,13 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>24.35</v>
+        <v>1.83</v>
       </c>
       <c r="E62" t="n">
-        <v>24.25</v>
+        <v>1.8</v>
       </c>
       <c r="F62" t="n">
-        <v>22.89</v>
+        <v>1.71</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -3264,7 +3264,7 @@
         <v>52</v>
       </c>
       <c r="I62" t="n">
-        <v>2.397</v>
+        <v>3.977</v>
       </c>
       <c r="J62" t="n">
         <v>0</v>
@@ -3273,18 +3273,18 @@
         <v>1</v>
       </c>
       <c r="L62" t="n">
-        <v>1.24</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>sh600230</t>
+          <t>sh600185</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>沧州大化</t>
+          <t>珠免集团</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3293,13 +3293,13 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>19.6</v>
+        <v>5.96</v>
       </c>
       <c r="E63" t="n">
-        <v>19.47</v>
+        <v>5.89</v>
       </c>
       <c r="F63" t="n">
-        <v>18.54</v>
+        <v>5.69</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -3310,7 +3310,7 @@
         <v>52</v>
       </c>
       <c r="I63" t="n">
-        <v>1.924</v>
+        <v>2.055</v>
       </c>
       <c r="J63" t="n">
         <v>0</v>
@@ -3319,18 +3319,18 @@
         <v>1</v>
       </c>
       <c r="L63" t="n">
-        <v>1.76</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>sh600227</t>
+          <t>sh600184</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>赤天化</t>
+          <t>光电股份</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3339,13 +3339,13 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>4.25</v>
+        <v>22.88</v>
       </c>
       <c r="E64" t="n">
-        <v>4.15</v>
+        <v>22.46</v>
       </c>
       <c r="F64" t="n">
-        <v>3.92</v>
+        <v>21.54</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -3356,7 +3356,7 @@
         <v>52</v>
       </c>
       <c r="I64" t="n">
-        <v>4.938</v>
+        <v>3.249</v>
       </c>
       <c r="J64" t="n">
         <v>0</v>
@@ -3365,18 +3365,18 @@
         <v>1</v>
       </c>
       <c r="L64" t="n">
-        <v>11.08</v>
+        <v>5.18</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>sh600226</t>
+          <t>sh600177</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>亨通股份</t>
+          <t>雅戈尔</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3385,13 +3385,13 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>5.28</v>
+        <v>7.64</v>
       </c>
       <c r="E65" t="n">
-        <v>5.27</v>
+        <v>7.55</v>
       </c>
       <c r="F65" t="n">
-        <v>5.05</v>
+        <v>7.29</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -3402,7 +3402,7 @@
         <v>52</v>
       </c>
       <c r="I65" t="n">
-        <v>0.571</v>
+        <v>2.55</v>
       </c>
       <c r="J65" t="n">
         <v>0</v>
@@ -3411,18 +3411,18 @@
         <v>1</v>
       </c>
       <c r="L65" t="n">
-        <v>1.12</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>sh600221</t>
+          <t>sh600172</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>海航控股</t>
+          <t>黄河旋风</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3431,13 +3431,13 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>1.44</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="E66" t="n">
-        <v>1.44</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="F66" t="n">
-        <v>1.39</v>
+        <v>7.75</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
         <v>52</v>
       </c>
       <c r="I66" t="n">
-        <v>0.699</v>
+        <v>3.63</v>
       </c>
       <c r="J66" t="n">
         <v>0</v>
@@ -3457,18 +3457,18 @@
         <v>1</v>
       </c>
       <c r="L66" t="n">
-        <v>2.24</v>
+        <v>3.72</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>sh600376</t>
+          <t>sh600170</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>首开股份</t>
+          <t>上海建工</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3477,13 +3477,13 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>4.45</v>
+        <v>2.68</v>
       </c>
       <c r="E67" t="n">
-        <v>4.34</v>
+        <v>2.67</v>
       </c>
       <c r="F67" t="n">
-        <v>4.13</v>
+        <v>2.6</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -3494,7 +3494,7 @@
         <v>52</v>
       </c>
       <c r="I67" t="n">
-        <v>3.972</v>
+        <v>1.132</v>
       </c>
       <c r="J67" t="n">
         <v>0</v>
@@ -3503,18 +3503,18 @@
         <v>1</v>
       </c>
       <c r="L67" t="n">
-        <v>1.29</v>
+        <v>1.87</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>sh600372</t>
+          <t>sh600323</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>中航机载</t>
+          <t>瀚蓝环境</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3523,13 +3523,13 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>13</v>
+        <v>32.27</v>
       </c>
       <c r="E68" t="n">
-        <v>12.98</v>
+        <v>31.96</v>
       </c>
       <c r="F68" t="n">
-        <v>12.62</v>
+        <v>30.78</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -3540,7 +3540,7 @@
         <v>52</v>
       </c>
       <c r="I68" t="n">
-        <v>0.541</v>
+        <v>3</v>
       </c>
       <c r="J68" t="n">
         <v>0</v>
@@ -3549,18 +3549,18 @@
         <v>1</v>
       </c>
       <c r="L68" t="n">
-        <v>1.51</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>sh600366</t>
+          <t>sh600313</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>宁波韵升</t>
+          <t>农发种业</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3569,13 +3569,13 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>13.2</v>
+        <v>7.18</v>
       </c>
       <c r="E69" t="n">
-        <v>12.99</v>
+        <v>7.15</v>
       </c>
       <c r="F69" t="n">
-        <v>12.46</v>
+        <v>6.89</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -3586,7 +3586,7 @@
         <v>52</v>
       </c>
       <c r="I69" t="n">
-        <v>3.125</v>
+        <v>1.127</v>
       </c>
       <c r="J69" t="n">
         <v>0</v>
@@ -3595,18 +3595,18 @@
         <v>1</v>
       </c>
       <c r="L69" t="n">
-        <v>2.65</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>sh600362</t>
+          <t>sh600312</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>江西铜业</t>
+          <t>平高电气</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3615,13 +3615,13 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>44.89</v>
+        <v>22.26</v>
       </c>
       <c r="E70" t="n">
-        <v>44.61</v>
+        <v>21.81</v>
       </c>
       <c r="F70" t="n">
-        <v>43.07</v>
+        <v>21.07</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -3632,7 +3632,7 @@
         <v>52</v>
       </c>
       <c r="I70" t="n">
-        <v>1.378</v>
+        <v>3.391</v>
       </c>
       <c r="J70" t="n">
         <v>0</v>
@@ -3641,18 +3641,18 @@
         <v>1</v>
       </c>
       <c r="L70" t="n">
-        <v>7.23</v>
+        <v>3.68</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>sh600353</t>
+          <t>sh600307</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>旭光电子</t>
+          <t>酒钢宏兴</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3661,13 +3661,13 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>17.82</v>
+        <v>1.79</v>
       </c>
       <c r="E71" t="n">
-        <v>17.85</v>
+        <v>1.77</v>
       </c>
       <c r="F71" t="n">
-        <v>17.05</v>
+        <v>1.7</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -3678,7 +3678,7 @@
         <v>52</v>
       </c>
       <c r="I71" t="n">
-        <v>0.678</v>
+        <v>2.286</v>
       </c>
       <c r="J71" t="n">
         <v>0</v>
@@ -3687,18 +3687,18 @@
         <v>1</v>
       </c>
       <c r="L71" t="n">
-        <v>2.36</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>sh600348</t>
+          <t>sh600301</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>华阳股份</t>
+          <t>华锡有色</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3707,13 +3707,13 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>10.33</v>
+        <v>49.75</v>
       </c>
       <c r="E72" t="n">
-        <v>10.29</v>
+        <v>49.56</v>
       </c>
       <c r="F72" t="n">
-        <v>9.91</v>
+        <v>47.63</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -3724,7 +3724,7 @@
         <v>52</v>
       </c>
       <c r="I72" t="n">
-        <v>1.175</v>
+        <v>1.159</v>
       </c>
       <c r="J72" t="n">
         <v>0</v>
@@ -3733,18 +3733,18 @@
         <v>1</v>
       </c>
       <c r="L72" t="n">
-        <v>3.27</v>
+        <v>3.48</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>sh600343</t>
+          <t>sh600299</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>航天动力</t>
+          <t>安迪苏</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3753,13 +3753,13 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>33.08</v>
+        <v>14.15</v>
       </c>
       <c r="E73" t="n">
-        <v>33.14</v>
+        <v>13.95</v>
       </c>
       <c r="F73" t="n">
-        <v>31.76</v>
+        <v>13.43</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -3770,7 +3770,7 @@
         <v>52</v>
       </c>
       <c r="I73" t="n">
-        <v>0.731</v>
+        <v>2.536</v>
       </c>
       <c r="J73" t="n">
         <v>0</v>
@@ -3779,18 +3779,18 @@
         <v>1</v>
       </c>
       <c r="L73" t="n">
-        <v>3.43</v>
+        <v>1.92</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>sh600340</t>
+          <t>sh600282</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>华夏幸福</t>
+          <t>南钢股份</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3799,13 +3799,13 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>1.28</v>
+        <v>5.43</v>
       </c>
       <c r="E74" t="n">
-        <v>1.26</v>
+        <v>5.43</v>
       </c>
       <c r="F74" t="n">
-        <v>1.2</v>
+        <v>5.25</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -3816,7 +3816,7 @@
         <v>52</v>
       </c>
       <c r="I74" t="n">
-        <v>3.226</v>
+        <v>1.306</v>
       </c>
       <c r="J74" t="n">
         <v>0</v>
@@ -3825,18 +3825,18 @@
         <v>1</v>
       </c>
       <c r="L74" t="n">
-        <v>0.96</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>sh600337</t>
+          <t>sh600273</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>美克家居</t>
+          <t>嘉化能源</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3845,13 +3845,13 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>2.8</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="E75" t="n">
-        <v>2.77</v>
+        <v>8.32</v>
       </c>
       <c r="F75" t="n">
-        <v>2.61</v>
+        <v>8.07</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -3862,7 +3862,7 @@
         <v>52</v>
       </c>
       <c r="I75" t="n">
-        <v>2.941</v>
+        <v>1.209</v>
       </c>
       <c r="J75" t="n">
         <v>0</v>
@@ -3871,18 +3871,18 @@
         <v>1</v>
       </c>
       <c r="L75" t="n">
-        <v>1.05</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>sh600328</t>
+          <t>sh600271</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>中盐化工</t>
+          <t>航天信息</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3891,13 +3891,13 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>8.720000000000001</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="E76" t="n">
-        <v>8.699999999999999</v>
+        <v>8.15</v>
       </c>
       <c r="F76" t="n">
-        <v>8.359999999999999</v>
+        <v>7.87</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -3908,7 +3908,7 @@
         <v>52</v>
       </c>
       <c r="I76" t="n">
-        <v>0.6929999999999999</v>
+        <v>2.602</v>
       </c>
       <c r="J76" t="n">
         <v>0</v>
@@ -3917,18 +3917,18 @@
         <v>1</v>
       </c>
       <c r="L76" t="n">
-        <v>1.04</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>sh600326</t>
+          <t>sh600268</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>西藏天路</t>
+          <t>国电南自</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3937,13 +3937,13 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>9.34</v>
+        <v>15.16</v>
       </c>
       <c r="E77" t="n">
-        <v>9.17</v>
+        <v>14.87</v>
       </c>
       <c r="F77" t="n">
-        <v>8.880000000000001</v>
+        <v>14.39</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -3954,7 +3954,7 @@
         <v>52</v>
       </c>
       <c r="I77" t="n">
-        <v>3.091</v>
+        <v>3.34</v>
       </c>
       <c r="J77" t="n">
         <v>0</v>
@@ -3963,18 +3963,18 @@
         <v>1</v>
       </c>
       <c r="L77" t="n">
-        <v>2.45</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>sh600325</t>
+          <t>sh600266</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>华发股份</t>
+          <t>城建发展</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3983,13 +3983,13 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>3.53</v>
+        <v>4.88</v>
       </c>
       <c r="E78" t="n">
-        <v>3.48</v>
+        <v>4.81</v>
       </c>
       <c r="F78" t="n">
-        <v>3.35</v>
+        <v>4.67</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -4000,7 +4000,7 @@
         <v>52</v>
       </c>
       <c r="I78" t="n">
-        <v>3.216</v>
+        <v>2.521</v>
       </c>
       <c r="J78" t="n">
         <v>0</v>
@@ -4009,18 +4009,18 @@
         <v>1</v>
       </c>
       <c r="L78" t="n">
-        <v>1.68</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>sh600323</t>
+          <t>sh600262</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>瀚蓝环境</t>
+          <t>北方股份</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -4029,13 +4029,13 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>32.43</v>
+        <v>24.31</v>
       </c>
       <c r="E79" t="n">
-        <v>31.96</v>
+        <v>23.91</v>
       </c>
       <c r="F79" t="n">
-        <v>30.78</v>
+        <v>23.63</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -4046,7 +4046,7 @@
         <v>52</v>
       </c>
       <c r="I79" t="n">
-        <v>3.511</v>
+        <v>4.067</v>
       </c>
       <c r="J79" t="n">
         <v>0</v>
@@ -4055,18 +4055,18 @@
         <v>1</v>
       </c>
       <c r="L79" t="n">
-        <v>2.4</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>sh600316</t>
+          <t>sh600256</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>洪都航空</t>
+          <t>广汇能源</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4075,13 +4075,13 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>36.34</v>
+        <v>6.56</v>
       </c>
       <c r="E80" t="n">
-        <v>36.26</v>
+        <v>6.56</v>
       </c>
       <c r="F80" t="n">
-        <v>34.84</v>
+        <v>6.34</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -4092,7 +4092,7 @@
         <v>52</v>
       </c>
       <c r="I80" t="n">
-        <v>0.526</v>
+        <v>0.923</v>
       </c>
       <c r="J80" t="n">
         <v>0</v>
@@ -4101,18 +4101,18 @@
         <v>1</v>
       </c>
       <c r="L80" t="n">
-        <v>1.6</v>
+        <v>7.56</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>sh600313</t>
+          <t>sh600251</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>农发种业</t>
+          <t>冠农股份</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4121,13 +4121,13 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>7.16</v>
+        <v>12.3</v>
       </c>
       <c r="E81" t="n">
-        <v>7.15</v>
+        <v>12.23</v>
       </c>
       <c r="F81" t="n">
-        <v>6.89</v>
+        <v>11.76</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -4138,7 +4138,7 @@
         <v>52</v>
       </c>
       <c r="I81" t="n">
-        <v>0.845</v>
+        <v>2.159</v>
       </c>
       <c r="J81" t="n">
         <v>0</v>
@@ -4147,18 +4147,18 @@
         <v>1</v>
       </c>
       <c r="L81" t="n">
-        <v>1.27</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>sh600312</t>
+          <t>sh600246</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>平高电气</t>
+          <t>万通发展</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4167,13 +4167,13 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>21.9</v>
+        <v>10.33</v>
       </c>
       <c r="E82" t="n">
-        <v>21.72</v>
+        <v>10.29</v>
       </c>
       <c r="F82" t="n">
-        <v>21.07</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -4184,7 +4184,7 @@
         <v>52</v>
       </c>
       <c r="I82" t="n">
-        <v>1.719</v>
+        <v>1.076</v>
       </c>
       <c r="J82" t="n">
         <v>0</v>
@@ -4193,7 +4193,7 @@
         <v>1</v>
       </c>
       <c r="L82" t="n">
-        <v>2.61</v>
+        <v>4.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 实时报告更新 Thu Apr 30 02:22:32 UTC 2026
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -425,30 +425,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>系统诊断</t>
+          <t>诊断</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>故障原因</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>对策</t>
+          <t>原因</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>物理避封</t>
+          <t>系统静默</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -456,11 +451,6 @@
           <t>('Connection aborted.', RemoteDisconnected('Remote end closed connection without response'))</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>IP受限，静默6小时</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📊 实时报告更新 Thu Apr 30 02:48:13 UTC 2026
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -431,7 +431,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>诊断</t>
+          <t>状态</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -443,7 +443,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>系统静默</t>
+          <t>影子模式受限</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
📊 实时报告更新 Tue May  5 04:42:28 UTC 2026
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -488,7 +488,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>T:2026-05-04 13:01:23</t>
+          <t>T:2026-05-05 12:42:28</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -2343,12 +2343,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>603017</t>
+          <t>605066</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>中衡设计</t>
+          <t>天正电气</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2357,38 +2357,38 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>15.4</v>
+        <v>8.06</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="F49" t="n">
         <v>121.7</v>
       </c>
       <c r="G49" t="n">
-        <v>0.72</v>
+        <v>4.54</v>
       </c>
       <c r="H49" t="n">
-        <v>16.43</v>
+        <v>5.76</v>
       </c>
       <c r="I49" t="n">
-        <v>1.33</v>
+        <v>3.22</v>
       </c>
       <c r="J49" t="n">
-        <v>6.98</v>
+        <v>2.31</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>605066</t>
+          <t>603017</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>天正电气</t>
+          <t>中衡设计</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2397,27 +2397,27 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>8.06</v>
+        <v>15.4</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="F50" t="n">
         <v>121.7</v>
       </c>
       <c r="G50" t="n">
-        <v>4.54</v>
+        <v>0.72</v>
       </c>
       <c r="H50" t="n">
-        <v>5.76</v>
+        <v>16.43</v>
       </c>
       <c r="I50" t="n">
-        <v>3.22</v>
+        <v>1.33</v>
       </c>
       <c r="J50" t="n">
-        <v>2.31</v>
+        <v>6.98</v>
       </c>
     </row>
     <row r="51">
@@ -3583,12 +3583,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>300831</t>
+          <t>002725</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>派瑞股份</t>
+          <t>跃岭股份</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3597,38 +3597,38 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>20.22</v>
+        <v>16.9</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>潜伏蓄势</t>
+          <t>🔥 黄金堆积</t>
         </is>
       </c>
       <c r="F80" t="n">
         <v>113.1</v>
       </c>
       <c r="G80" t="n">
-        <v>3.75</v>
+        <v>5.16</v>
       </c>
       <c r="H80" t="n">
-        <v>14.8</v>
+        <v>7.88</v>
       </c>
       <c r="I80" t="n">
-        <v>1.16</v>
+        <v>1.8</v>
       </c>
       <c r="J80" t="n">
-        <v>5.51</v>
+        <v>2.84</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>002725</t>
+          <t>300831</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>跃岭股份</t>
+          <t>派瑞股份</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3637,27 +3637,27 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>16.9</v>
+        <v>20.22</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>🔥 黄金堆积</t>
+          <t>潜伏蓄势</t>
         </is>
       </c>
       <c r="F81" t="n">
         <v>113.1</v>
       </c>
       <c r="G81" t="n">
-        <v>5.16</v>
+        <v>3.75</v>
       </c>
       <c r="H81" t="n">
-        <v>7.88</v>
+        <v>14.8</v>
       </c>
       <c r="I81" t="n">
-        <v>1.8</v>
+        <v>1.16</v>
       </c>
       <c r="J81" t="n">
-        <v>2.84</v>
+        <v>5.51</v>
       </c>
     </row>
     <row r="82">

</xml_diff>